<commit_message>
S6: like-for-like digitalisation eval (federal >=2018): sample, baselines, corrected precision, review export
- sample digi-federal (150 pos / 250 neg, seed 42, grouped dev/test by title, first loop excluded) + meta (population counts)
- evaluate/digitalisation.py: CV-area + core-keyword baselines on full slice, dev threshold curve, test metrics with Wilson/bootstrap CIs, breakdowns; metrics.json/md
- review sheet filled blind (82 rows), key in results/adjudication_key.csv; make eval RUN=...
- decisions D36-D40

Verification (run 20261018T132629077874Z, 70B, adhoc_v3): baseline CV area P 40.9% R 80.2%, keyword P 41.3% R 56.4% (27,465 affairs).
Test: t=0.9 P_corr 77.6% (49-100) R 40.6% (32-50); t=0.5 P_corr 51.9% (35-84) R 63.4% (54-72). make test: 59 passed.
</commit_message>
<xml_diff>
--- a/data/gold/for_partner/adjudication.xlsx
+++ b/data/gold/for_partner/adjudication.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,6 +33,13 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -62,10 +69,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -74,10 +82,12 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -580,1204 +590,2945 @@
       </c>
     </row>
     <row r="2">
-      <c r="F2" s="4" t="n"/>
-      <c r="G2" s="4" t="n"/>
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="n">
+        <v>66198</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Qu'entreprend le Conseil fédéral pour protéger et promouvoir la biodiversité?</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Economiesuisse a souligné récemment l'énorme importance de la biodiversité pour la santé de l'économie et de la société. WSL et SCNAT viennent de publier un rapport concernant les subventions qui portent atteinte à la biodiversité et nuisent à long terme à l'économie du pays. Les associations environnementales ont déposé cette semaine une initiative en faveur de la biodiversité. Ces actions issues des milieux scientifiques, économiques et associatifs sont porteuses d'un message clair. Que fait le Conseil fédéral de son côté ?</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr"/>
+      <c r="G2" s="5" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="F3" s="4" t="n"/>
-      <c r="G3" s="4" t="n"/>
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="n">
+        <v>155716</v>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Coronavirus. Non scaricare i costi della pandemia sui premi di cassa malati</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Il Consiglio federale è incaricato di adottare le misure necessarie affinché negli anni 2021-2023 i premi dell'assicurazione malattie rimangano stabili e non siano innalzati in nessun caso.
+REASONING: La pandemia da coronavirus comporta un forte aumento dei costi della salute. Se da un lato dal 16 marzo al 27 aprile non sono stati eseguiti interventi elettivi, dall'altro non è dato sapere a quanto ne ammonteranno i costi effettivi sull'intero arco dell'anno né quanti di questi interventi, con i relativi costi, saranno rinviati ai prossimi anni. Gli assicuratori-malattie dispongono di riserve a cui possono attingere soltanto fino a un certo punto. Tuttavia i costi di una pandemia non devono sfociare in un aumento dei premi di cassa malati: vanno finanziati in maniera solidale e con un maggior coinvolgimento dei poteri pubblici (Confederazione e Cantoni). L'assicurazione malattie è finanziata con il sistema dei premi pro capite indipendenti dal reddito, che già oggi incidono in misura eccessiva sul budget di moltissime economie domestiche. L'incidenza media è del 14 per cento ed è destinata ad aumentare ulteriormente poiché durante la crisi del coronavirus i redditi sono dimin…</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="F4" s="4" t="n"/>
-      <c r="G4" s="4" t="n"/>
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="n">
+        <v>65463</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Im Interesse der Rechtsstaatlichkeit, der Souveränität und der Neutralität der Schweiz die Crypto-Leaks-Affäre mit einer PUK umfassend aufklären</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Das Parlament setzt eine Parlamentarische Untersuchungskommission PUK ein zur Aufarbeitung der Spionage-Affäre um die Firma Crypto AG.
+REASONING: Im Interesse der Rechtsstaatlichkeit, der Souveränität und der Neutralität der Schweiz muss die Cryptoleaks-Affäre umfassend aufgeklärt werden. Eine PUK hat dazu die notwendigen Ressourcen und kann insbesondere auch Untersuchungsbeauftragte i.S. von Artikel 166 ParIG einsetzen.</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="F5" s="4" t="n"/>
-      <c r="G5" s="4" t="n"/>
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="n">
+        <v>66518</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Rapporto sulla politica di sicurezza 2021</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="F6" s="4" t="n"/>
-      <c r="G6" s="4" t="n"/>
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="n">
+        <v>65226</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Zugang zu unterstützter Kommunikation</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Kommunikation dient dem sozialen Austausch, ermöglicht gesellschaftliche Teilhabe und ist damit ein menschliches Grundbedürfnis. Mit der Ratifizierung der UNO-Behindertenrechtskonvention verpflichtete sich die Schweiz, auf individuelle Bedürfnisse abgestimmte Kommunikationsformen und Kommunikationsmittel zu fördern. Für Menschen mit eingeschränkter Lautsprache gibt es die Unterstützte Kommunikation (UK). Das Gelingen der UK hängt u.a. davon ab, ob die passenden Methoden und Hilfsmittel zum Einsatz kommen, ob genügend UK-Fachpersonal in den Institutionen arbeitet und ob das Umfeld UK täglich und in möglichst vielen Lebensbereichen nutzt. Ich bitte den Bundesrat um die Beantwortung folgender Fragen: 1. Wie viele Menschen sind in der Schweiz auf UK angewiesen? Wie sieht die Verteilung aus zwischen Menschen mit leichten und Menschen mit schweren Kommunikationsbeeinträchtigungen u.a. aufgrund von schweren sowie mehrfachen Behinderungen? 2. Was tun Bund und Kantone, um sicherzustellen, dass alle Personen, Kinder und Erwachsene, mit eingeschränkten lautsprachlichen Fähigkeiten während ihres gesamten Lebens in verschiedenen Lebensbereichen wie u.a. Frühbereich, Bildung, Wohnen, Arbei…</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="F7" s="4" t="n"/>
-      <c r="G7" s="4" t="n"/>
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="n">
+        <v>234936</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Besteht die Gefahr, dass die Romandie bei den Offsets im Zusammenhang mit dem F-35A benachteiligt wird?</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Der Kauf der 36 Kampfflugzeuge des Typs F-35A bringt den Schweizer Unternehmen im Rahmen der Offsets rund 2,9 Milliarden Franken ein, wobei die Aufträge bis 2034 verteilt sein sollten. Dabei wurde vorgesehen, dass der Romandie 30 Prozent des Offsetvolumens zukommt, während 65 Prozent für die Deutschschweiz und 5 Prozent für das Tessin vorgesehen sind. Nun aber fürchten die Kantone der Romandie je länger je mehr, dass sie vergessen werden und dass die Zusagen, die beim Kauf der F-35A gemacht wurden, nicht eingehalten werden. Damit geht eine zunehmende Unzufriedenheit einher, sowohl in der Politik als auch in der Wirtschaft. Das Bundesunternehmen RUAG begehrt nämlich mehrere grosse Aufträge. Zur Instandhaltung der 36 Jets der Schweizer Armee sollen noch weitere Projekte dazukommen. Das Unternehmen ist jedoch vor allem in der Deutschschweiz angesiedelt, was nicht ohne Folgen für die Wirtschaft der Romandie bleiben würde, obwohl sie über zahlreiche Vorzüge verfügt. Insbesondere Genf, Freiburg und Neuenburg verfügen über viele Spezialistinnen und Spezialisten im Bereich der Luftfahrt. Mehr als siebzig grosse, mittlere und kleine Unternehmen der Romandie stellen der militärischen w…</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="F8" s="4" t="n"/>
-      <c r="G8" s="4" t="n"/>
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="n">
+        <v>156699</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Kommunikation zur Mitwirkung der Schweiz in der Allianz für Multilateralismus</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Im letzten Herbst ist im Rahmen der UNO die Allianz für Multilateralismus als Netzwerk entstanden. - Ist die Schweiz in diesem Netzwerk auch engagiert? - Wann gedenkt der Bundesrat öffentlich über das Engagement und die Projekte des Netzwerkes zu orientieren?</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr"/>
+      <c r="G8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="F9" s="4" t="n"/>
-      <c r="G9" s="4" t="n"/>
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="n">
+        <v>157177</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Mestieri del futuro. Sostegno pubblico alla riconversione professionale</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Il Consiglio federale è incaricato di illustrare in un rapporto in che modo è possibile creare nuove prospettive professionali in settori in fase di cambiamento strutturale tramite un maggiore investimento pubblico nella formazione continua e professionale.
+REASONING: La transizione ecologica causa la perdita di posti di lavoro in alcuni settori dell'industria e dei servizi, ma allo stesso tempo permette lo sviluppo di nuove professioni legate a un'economia più sostenibile: questo è quanto emerge da un rapporto realizzato dall'Organizzazione Internazionale del Lavoro (OIL) nel 2018. Lo studio mostra un fattore essenziale affinché la transizione ecologica possa portare alla creazione di posti di lavoro: una riconversione professionale efficace e mirata. È dunque necessario disporre di un piano a lungo termine e di dati chiari per identificare le esigenze attuali e future dell'economia e fornire i mezzi per formare (nuovamente) milioni di persone. Tuttavia in Svizzera manca un piano di questo genere. Allo stesso tempo, la digitalizzazione sta allargando il divario tra l'economia di produzione di ieri e l'economia digitale di domani, lasciando indietro dei dipendenti a causa de…</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr"/>
+      <c r="G9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="F10" s="4" t="n"/>
-      <c r="G10" s="4" t="n"/>
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="n">
+        <v>62663</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Quali rischi per la Confederazione comporta la strategia di convergenza di Swisscom?</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Chiedo al Consiglio federale di rispondere alle seguenti domande: 1. Il Consiglio federale ritiene che la strategia di convergenza di Swisscom e la posizione dominante sul mercato che ne deriva comportino nuovi rischi per la Confederazione e/o l'economia pubblica (in particolare per quanto riguarda la problematica "too big to fail" e gli attacchi informatici)? 2. La Confederazione, in quanto azionista di maggioranza, segue attivamente la strategia e analizza gli eventuali rischi per la Confederazione e/o l'economia pubblica insiti nei nuovi settori di attività? In caso affermativo, come avviene ciò concretamente? In caso negativo, perché non lo ritiene necessario? 3. Il Consiglio federale ritiene che Swisscom, che è quotata in borsa, possa fallire senza che ciò causi enormi danni collaterali al bilancio della Confederazione e/o all'intera economia svizzera? Se la risposta è "no", quali conseguenze trae dal rischio legato alla problematica "too big to fail"? Se la risposta è "sì", da dove trae questa convinzione? 4. Il Consiglio federale è disposto a far verificare le questioni di cui sopra nel quadro dell'esame esterno del governo d'impresa delle aziende parastatali e a infor…</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr"/>
+      <c r="G10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="F11" s="4" t="n"/>
-      <c r="G11" s="4" t="n"/>
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="n">
+        <v>154602</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Foglio informativo dell'UFAM sulla ristorazione sostenibile. Non abbiamo altri problemi?</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: In un nuovo foglio informativo, l'UFAM fornisce raccomandazioni per una ristorazione gustosa e rispettosa dell'ambiente in occasione di eventi. Tra le altre cose si raccomanda che almeno due terzi del cibo a buffet siano composti da prodotti vegetariani e che il cibo vegetariano sia collocato in primo piano. In merito chiedo al Consiglio federale di rispondere alle seguenti domande: 1. Il Consiglio federale ritiene veramente che in questo ambito sussista una necessità di intervento da parte della Confederazione? 2. Il Consiglio federale concorda sul fatto che con questo genere di "raccomandazioni" a favore del cibo vegetariano si penalizza il settore della carne e delle macellerie? 3. Quanti collaboratori dell'UFAM hanno partecipato all'elaborazione di questo foglio informativo? 4. Quanto tempo è stato necessario e a quanto ammontano i relativi costi? 5. Il Consiglio federale ritiene veramente che sia compito dello Stato educare i cittadini e dire loro cosa mangiare e bere? 6. Il Consiglio federale può confermare esplicitamente che queste raccomandazioni di oggi non saranno i divieti di domani?
+ANSWER: 1. Il rapporto Ambiente Svizzera 2018 del Consiglio federale indica che i…</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr"/>
+      <c r="G11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="F12" s="4" t="n"/>
-      <c r="G12" s="4" t="n"/>
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="n">
+        <v>235621</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Réforme de la valeur locative. Montant des déductions concernées</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Le 28 septembre 2025, la population se prononcera sur l'introduction d'un nouvel impôt immobilier cantonal sur les résidences secondaires. Ce projet est lié à la réforme fiscale qui supprime la valeur locative. Si la peuple se prononçait favorablement, la valeur locative ne serait plus imposée, mais un grand nombre de déductions aujourd'hui possibles, ne pourront plus être faites. En particulier, les intérêts hypothécaires (à part au tout début et de façon dégressive), les frais de rénovation y compris écologique, les frais d'entretien ne pourront plus être déduits du revenu. Le Conseil fédéral est prié de répondre aux questions suivantes: 1) Quel est le volume, en francs, des déductions octroyées au niveau fédéral qui sont aujourd'hui possible et qui ne seraient plus possibles si suppression de la valeur locative était acceptée 2) Quel est le montant d'impôt correspondant à ces déductions au niveau fédéral? 3) Si les cantons décident eux aussi de supprimer toutes les déductions qui ne sont plus possibles au niveau fédéral, quel serait le volume des déductions concernées, et le montant de l'impôt correspondant à ces déductions, cette fois-ci au niveau cantonal?
+ANSWER: Il es…</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr"/>
+      <c r="G12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="F13" s="4" t="n"/>
-      <c r="G13" s="4" t="n"/>
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="n">
+        <v>153348</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Online-Handel prüfen, überwachen und einschränken?</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Immer häufiger werden Fälle bekannt, wo in der Schweiz verbotene Waffen und andere illegale Gegenstände auf ausländischen Online-Handelsplattformen gekauft und auf dem Paketweg in die Schweiz gesendet wurden. Dabei werden unter anderem Waffen in Folien eingeschweisst, um den Detektoren der Zollverwaltung eine Entdeckung zu erschweren, oder Gegenstände als Muster bezeichnet, um Zollgebühren zu vermeiden. Bislang können für solche illegalen Praktiken allerdings nur die Empfänger belangt werden. Der Bundesrat wird gebeten, folgende Fragen zu beantworten: 1. Beabsichtigt er, der Eidgenössischen Zollverwaltung die nötigen Mittel zur Verfügung zu stellen, damit die grosse Mehrheit dieser illegalen Pakete künftig aus dem Verkehr gezogen werden kann? 2. Besteht aus seiner Sicht auch die Notwendigkeit, die verantwortlichen Online-Portale und die Versender in die Verantwortung zu nehmen? 3. Kann im Rahmen von Freihandelsabkommen die beschriebene Problematik zusammen mit unseren Handelspartnern wirkungsvoll angegangen werden? 4. Welche weiteren Mittel sieht er, um den transnationalen Versand illegaler Pakete wirkungsvoll einzudämmen?
+REASONING: Die Digitalisierung ermöglicht einen imme…</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr"/>
+      <c r="G13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="F14" s="4" t="n"/>
-      <c r="G14" s="4" t="n"/>
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="n">
+        <v>155827</v>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Crisi dovuta al coronavirus. Soluzione globale per stabilizzare le finanze federali e le opere sociali</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Il Consiglio federale è incaricato di presentare al Parlamento una soluzione globale che indichi come le prestazioni straordinarie fornite dalla Confederazione durante la crisi dovuta al coronavirus e le future perdite fiscali provocate dalla suddetta crisi debbano essere contabilizzate nei conti della Confederazione. Il Consiglio federale deve indicare in particolare come nei prossimi 6-8 anni dovrà essere coperto il disavanzo del fondo di compensazione stimato in 40 miliardi di franchi, come dovranno essere compensate le perdite fiscali stimate in cinque miliardi di franchi l'anno e quali misure dovranno essere adottate per consolidare le assicurazioni sociali del 1° e del 2° pilastro. Condizione: il freno all'indebitamento, che ha dato prova di efficacia, non deve essere allentato.
+REASONING: Il Consiglio federale ha espresso grande preoccupazione per le conseguenze economiche della crisi dovuta al coronavirus. Le prestazioni straordinarie graveranno le casse della Confederazione per un importo di circa 40 miliardi di franchi, che sarà trasferito a un fondo di compensazione. La base legale prevede che tale fondo sia riequilibrato entro 6-8 anni. Inoltre, a causa dell'immi…</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr"/>
+      <c r="G14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="F15" s="4" t="n"/>
-      <c r="G15" s="4" t="n"/>
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="n">
+        <v>235813</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Zentrales Informationssystem Digiflux. Was kostet die Umsetzung?</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Für die Verwendung von Pflanzenschutzmitteln und Nährstoffen wird ein zentrales Informationssystem (Digiflux) eingeführt. Der Bundesrat wird in diesem Zusammenhang gebeten, die folgenden Fragen zu beantworten: 1) Welche jährlichen Investitions-, Anwendungs- und Personalkosten sind mit dem Projekt verbunden? 2) Wie hoch ist der geschätzte zusätzliche administrative Aufwand für die Kantone, die Landwirtschaftsbetriebe und die anderen betroffenen Akteure? 3) Kann das Ziel der Transparenz auch erreicht werden, indem für die Landwirtschaftsbetriebe ein einfacheres System eingeführt wird, ein System, das beispielsweise auf Schätzungen und Befragungen beruht? 4) Ist der Bundesrat bereit, die Einführung der Digiflux-Anwendung zu verschieben, um den Anwenderinnen und Anwendern mehr Zeit für die Umsetzung zu gewähren?
+REASONING: Im Rahmen der parlamentarischen Initiative 19.475 wurden mehrere Gesetze geändert –dies mit dem Ziel, zur Verminderung der Risiken im Zusammenhang mit dem Einsatz von Pflanzenschutzmitteln und zur Reduktion der Nährstoffverluste Absenkpfade festzulegen. Das Landwirtschaftsgesetz wurde mit einer Mitteilungspflicht für Nährstofflieferungen, einschliesslich Kraft…</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr"/>
+      <c r="G15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="F16" s="4" t="n"/>
-      <c r="G16" s="4" t="n"/>
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="n">
+        <v>330749</v>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Intelligente Brillen: eine neue Dimension des Voyeurismus. Ist das Schweizer Recht den Anforderungen gewachsen?</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Intelligente Brillen vom Typ Ray-Ban Meta, von denen 2025 weltweit sieben Millionen Exemplare verkauft wurden und die nun bei Schweizer Optikern erhältlich sind, verfügen über einen Rahmen mit integrierter Kamera und integriertem Mikrofon, der von einer gewöhnlichen Brille nicht zu unterscheiden ist. Sie ermöglichen es, von anderen Personen unbemerkt und kontinuierlich Ton- und Bildaufnahmen zu machen. Jüngste Enthüllungen haben gezeigt, dass intime Bilder, die ohne Wissen der Betroffenen aufgenommen wurden – darunter Nacktszenen und besonders schützenswerte Personendaten –, für KI-Trainingszwecke an Subunternehmen weitergeleitet wurden. Der Hersteller plant zudem, die Gesichtserkennung zu integrieren. Eine neue Generation mit integriertem Bildschirm und Gestensteuerung ist in den Vereinigten Staaten bereits auf dem Markt und könnte bald auch in der Schweiz erhältlich sein. Das Schweizer Recht (Datenschutz, Schutz der Persönlichkeit, Strafbestimmungen zu Verletzungen der Privatsphäre) wurde mit Blick auf einen lokal begrenzten und wahrnehmbaren Voyeurismus konzipiert. Doch diese Technologien machen Voyeurismus allgegenwärtig, unsichtbar und sofort weltweit verbreitbar. Die Bü…</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr"/>
+      <c r="G16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="F17" s="4" t="n"/>
-      <c r="G17" s="4" t="n"/>
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="n">
+        <v>156561</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Verbot der Verwendung von Landessprachen bei nichtgewerbsmässigen Flügen. Warum lassen die vorübergehenden Ausnahmebestimmungen auf sich warten?</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Im Juni 2019 wurde das Monopol der englischen Sprache eingeführt, jedoch nicht für alle Flugplätze im Land, so etwa nicht für la Chaux-de-Fonds. Inzwischen wurde beschlossen, wieder zur Mehrsprachigkeit zurückzukehren. In seiner Antwort auf meine Frage 19.5691 sagte der Bundesrat, dass das BAZL neue Ausnahmen prüfe. Er will aber vorderhand nichts entscheiden und verweist auf hängige Rekurse. Sitten und Payerne sind in erster Linie betroffen. Was unternimmt der Bundesrat, damit alle Flugplätze gleich und gerecht behandelt werden und die verlangten Ausnahmen sofort gewährt werden können?
+ANSWER: Die Antwort des Bundesrates existiert nur in französischer Sprache. (Bitte wechseln Sie auf der Homepage oben rechts die Sprache)</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr"/>
+      <c r="G17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="F18" s="4" t="n"/>
-      <c r="G18" s="4" t="n"/>
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="n">
+        <v>201868</v>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Coopération internationale des autorités pénales dans la lutte contre la cybercriminalité</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Au vu de la forte hausse des cyberattaques d'origine étrangère contre des personnes physiques et morales en Suisse, je pose les questions suivantes au Conseil fédéral : 1. Y a-t-il une bonne coopération avec les autorités pénales étrangères lorsque les enquêtes de police sur des plaintes pénales déposées par des victimes suisses révèlent que les malfaiteurs opèrent de manière ciblée depuis l'étranger ? 2. Y a-t-il des pays qui ne coopèrent pas suffisamment avec la Suisse et qui sont donc souvent utilisés comme base par les cybercriminels ? 3. À combien le Conseil fédéral estime-t-il le nombre de cas où il est impossible de déterminer où se trouvent les auteurs ? 4. La présente interpellation fait écho aux cyberattaques menées depuis des mois contre des clients de PostFinance et d'autres entreprises suisses, qui, attirés par un site Internet falsifié (hameçonnage), permettent aux malfaiteurs d'accéder directement à leurs comptes et dépôts. Le Ministère public de la Confédération, chargé de l'enquête, a pu remonter la trace des auteurs jusqu'en Inde, à qui les cas traités ont été transmis pour qu'elle les poursuive. Le Conseil fédéral peut-il donner des informations plus détail…</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr"/>
+      <c r="G18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="F19" s="4" t="n"/>
-      <c r="G19" s="4" t="n"/>
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="n">
+        <v>66100</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Vaterschaftsurlaub. Beeinflussung der Volksabstimmung durch den Bund?</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Anfang Mai 2020 wurde darüber berichtet, dass die Post, Postfinance und PostAuto Schweiz AG ab 2021 den Vätern neu 4 Wochen Vaterschaftsurlaub gewähren. In kürze nimmt das Volk in einer Referendumsabstimmung zum staatlichen Vaterschaftsurlaub von 2 Wochen Stellung. Wie beurteilt der Bundesrat seine Rolle und seine Wirkung im Abstimmungskampf, wenn ein Unternehmen des Bundes - der Bund ist alleiniger Aktionär der Schweizerischen Post AG - kurz vor dem Urnengang einen solchen Entscheid fällt?
+ANSWER: Die Post hat kürzlich den Abschluss der Verhandlungen mit syndicom und transfair zum neuen Dach-Gesamtarbeitsvertrag der Post bekanntgegeben. Dieser GAV tritt per 1. Januar 2021 in Kraft und beinhaltet neu einen Vaterschaftsurlaub von vier Wochen (bisher 2 Wochen). Die Personalpolitik liegt uneingeschränkt in der Verantwortung der bundesnahen Unternehmen. Dennoch formuliert der Bundesrat in seinen strategischen Zielvorgaben auch personalpolitische Ziele und trägt damit dem Umstand Rechnung, dass diese Unternehmen wichtige Arbeitgeber sind und eine Vorbildrolle einnehmen. Der Bundesrat mischt sich aber nicht in die Sozialpartnerschaft ein und beschränkt die personalpolitischen Ziel…</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr"/>
+      <c r="G19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="F20" s="4" t="n"/>
-      <c r="G20" s="4" t="n"/>
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="n">
+        <v>155280</v>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Rechtshilfe gegenüber Griechenland. Zu neuen Ersuchen ermuntern</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Das Bundesstrafgericht und danach das Bundesgericht haben vorläufig die Herausgabe von Bankdaten an die griechischen Strafverfolgungsbehörden durch die Bundesanwaltschaft blockiert. Der Entscheid schockiert in einem krassen Korruptionsfall, der im Jahr 2013 bereits zur Verurteilung des ehemaligen Verteidigungsministers Tsochatzopoulos zu einer Freiheitsstrafe von 20 Jahren führte. Als Grund nannten die Gerichte den Verdacht, dass das Rechtshilfeersuchen auf den Bankdaten der Falciani-Liste beruhe. Wird das Bundesamt für Justiz den griechischen Behörden nahelegen, ihr Anliegen noch einmal vorzubringen und dabei zu belegen, dass das Ersuchen nicht auf den Daten der Falciani-Liste beruht?
+ANSWER: Die Antwort des Bundesrates existiert nur in französischer Sprache. (Bitte wechseln Sie auf der Homepage oben rechts die Sprache)</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr"/>
+      <c r="G20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="F21" s="4" t="n"/>
-      <c r="G21" s="4" t="n"/>
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="n">
+        <v>69536</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Nouvelle édition des Principes directeurs de l'OCDE à l'intention des entreprises multinationales</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Le 8 juin, l'OCDE a, lors de sa conférence ministérielle (qui s'est tenue à Paris et à laquelle la Suisse participait), adopté une nouvelle édition de ses principes directeurs à l’intention des entreprises multinationales. La révision visait à intégrer dans les principes directeurs des précisions concernant le devoir de diligence, précisions qui avaient été élaborées dans le cadre de différents guides depuis la dernière révision (laquelle datait de 2011). 1. Les ministres de l'OCDE ont exigé, dans leurs précédentes recommandations relatives au rôle des États (OECD/LEGAL/0486), que les États membres édictent les lois nécessaires et vérifient régulièrement que celles-ci ne contiennent pas de lacunes, notamment en lien avec la mise en œuvre effective de ces lois et l'accès aux voies de recours. Ils recommandent aux États membres de combler les lacunes existantes en légiférant et de veiller à ce que les normes qu'ils édictent soient conformes aux nouveaux principes directeurs. Quelles mesures le Conseil fédéral a-t-il prises pour mettre en œuvre cette recommandation ? 2. La nouvelle édition des principes directeurs de l'OCDE prévoit un renforcement substantiel du devoir de dilige…</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr"/>
+      <c r="G21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="F22" s="4" t="n"/>
-      <c r="G22" s="4" t="n"/>
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="n">
+        <v>65791</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Conoscere meglio il bullismo in Svizzera per proteggere meglio i bambini</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Il Consiglio federale è incaricato di redigere un rapporto sul bullismo che permetta di ottenere i dati quantitativi e qualitativi necessari per mettere a punto misure contro la reiterazione delle violenze verbali, fisiche e piscologiche in ambito scolastico. Il rapporto conterrà in particolare: 1. alcune statistiche specifiche sul bullismo in Svizzera, 2. un bilancio degli attuali strumenti di sostegno della Confederazione, 3. un elenco esaustivo delle misure contro il bullismo messe in campo dalla Confederazione e dai Cantoni, 4. una valutazione della possibilità di predisporre degli aiuti per finanziare misure di prevenzione del bullismo, in analogia con le misure finanziarie varate per contrastare la violenza sulle donne e la violenza domestica.
+REASONING: Il bullismo nelle scuole è un problema sociale spesso banalizzato ma ampiamente diffuso e con risvolti molto pesanti. Le persone bullizzate, infatti, vengono minate nella loro autostima e corrono un rischio maggiore di cadere in depressione e sviluppare comportamenti antisociali, sintomi psicotici e persino idee suicidarie. Dall'altro lato le persone che commettono bullismo possono essere affette da disturbi psicologic…</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr"/>
+      <c r="G22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="F23" s="4" t="n"/>
-      <c r="G23" s="4" t="n"/>
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="n">
+        <v>214635</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Transparence de la publicité politique diffusée sur les médias sociaux</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Le Conseil fédéral est chargé de présenter un projet de loi qui permettra aux utilisateurs de reconnaître en tant que telle la publicité politique dans les médias.
+REASONING: Dans sa réponse à l'ip. 21.4086, le Conseil fédéral déclare que " pour le moment, les éventuelles conséquences négatives [de la publicité politique numérique] sur la formation de l'opinion publique devraient être négligeables ". Simultanément, il reconnaît que les plateformes de communication numériques jouent " un rôle de plus en plus important " (71 % de la population suisse les ont utilisées en 2019) et " qu'elles revêtent une importance croissante pour la formation de l'opinion ". Le rapport du Conseil fédéral sur l'activité des opérateurs de plateformes numériques reconnaît en outre que le manque de transparence de la publicité politique sur ces plateformes est problématique. Il semble dès lors opportun de régler la publicité politique sur les plateformes numériques tant qu'elle n'est pas encore très répandue et avant qu'elle ne devienne effectivement problématique. Toute la publicité diffusée sur les médias sociaux devraient être signalée comme telle, afin que tous les utilisateurs comprennent qu'…</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr"/>
+      <c r="G23" s="5" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="F24" s="4" t="n"/>
-      <c r="G24" s="4" t="n"/>
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="n">
+        <v>64898</v>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Modification de l'article 697l du code des obligations et accès à liste des ayants droit économiques</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: La loi fédérale du 21 juin 2019 sur la mise en oeuvre des recommandations du Forum mondial sur la transparence et l'échange de renseignements à des fins fiscales entraîne la disparition des actions au porteur. L'art. 697l du code des obligations (CO) est simplifié en conséquence et ne prévoit plus pour la société que l'obligation de tenir une liste des ayants droit économiques qui lui ont été annoncés. Conformément à la recommandation 24 du GAFI, l'art. 697l, al. 4, CO prévoit que la liste doit être tenue de manière à ce qu'il soit possible d'y accéder en tout temps en Suisse. La loi ne règle toutefois pas qui peut accéder à la liste. Le message concernant la mise en oeuvre des recommandations du GAFI révisées en 2012 n'imposait pas au conseil d'administration d'une société suisse de fournir de telles listes à l'autorité suisse compétente, sauf dans le cas de vérifications particulières dans le cadre d'une enquête du Ministère public, dans le domaine du droit pénal administratif ou en cas d'infraction fiscale (fraude fiscale). L'Administration fédérale des contributions (AFC) procède actuellement à la collecte systématique de ces listes par l'envoi d'une lettre-type aux contr…</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr"/>
+      <c r="G24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="F25" s="4" t="n"/>
-      <c r="G25" s="4" t="n"/>
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="n">
+        <v>235223</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Le caratteristiche e i dispositivi di sicurezza del sistema svizzero di verifica dei medicamenti (SMVS) sono inadatti per il monitoraggio degli agenti terapeutici?</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Il Consiglio federale condivide l’opinione secondo cui non esiste una base legale che consenta di attuare mediante l’articolo 17a LATer, approvato ma non in vigore, la gestione digitale delle penurie di medicamenti per uso umano richiesta dalla mozione Ettlin e che è necessario elaborare una specifica base legale all’interno della LATer? L’introduzione del SMVS fa parte delle otto raccomandazioni proposte al Consiglio federale dalla task force per gli agenti terapeutici? Il monitoraggio necessita di un’ulteriore base legale o è sufficiente il sistema di preallarme dell’Ufficio federale dell’approvvigionamento economico del Paese (UFAE)? È vero che l’UFAE non intende servirsi del SMVS per la gestione digitale delle penurie di medicamenti per uso umano? Il Consiglio federale ritiene che esista un rischio significativo che in Svizzera entrino in commercio medicamenti contraffatti? Se sì, in quali casi? Il Consiglio federale condivide la posizione dei fornitori di servizi, secondo cui i costi di attuazione dei requisiti SMVS sono troppo elevati rispetto ai potenziali benefici?
+REASONING: Il 26 settembre 2023 il Parlamento ha approvato, con un adattamento del punto 2, la mozione …</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr"/>
+      <c r="G25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="F26" s="4" t="n"/>
-      <c r="G26" s="4" t="n"/>
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="n">
+        <v>337367</v>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Legge sul sostegno alla banda larga (LSBL)</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="5" t="inlineStr"/>
+      <c r="G26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="F27" s="4" t="n"/>
-      <c r="G27" s="4" t="n"/>
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="n">
+        <v>214312</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Centovalliexpress. Quo vadis?</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Abbiamo recentemente potuto prendere atto con piacere dell'ordinazione da parte delle FART di nuovi elettrotreni per 94 mio a dimostrazione dell'impegno svizzero a voler mantenere viva la linea Locarno Domodossola anche per il traffico internazionale, sono anche previsti potenziamenti sul segmento svizzero finanziati nell'ambito Prossif 2035. Purtroppo questi investimenti non fanno da pari con il servizio offerto che è diventato negli anni sempre più scadente, oltretutto tassato extra sui convogli "panoramici" della SSIF . Tempi di percorrenza in crescita, infrastruttura ferroviaria sul segmento italiano con tratte percorse a passo d'uomo o quasi. Tempi di percorrenza attualmente attorno a 1h50' (erano a 1h45' nel 2010, stessi tempi negli anni 80 del secolo scorso prima dell'interramento a Locarno e con trasbordo per frana a Ré), in generale il Centovalliexpress percorre Locarno Domodossola a una velocità media inferiore a 30 km/h. Le ultime corse partono alle 17:45 da Locarno alle 19 da Domodossola! Nel 2010 l'Ata aveva presentato un progetto per la sistemazione della tratta che permetteva di ridurre i tempi fino a circa 1h30'. Questa linea rappresenterebbe un ideale collega…</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr"/>
+      <c r="G27" s="5" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="F28" s="4" t="n"/>
-      <c r="G28" s="4" t="n"/>
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="n">
+        <v>156261</v>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Istituzione delle basi legali per un'attività parlamentare digitale e per la partecipazione digitale all'attività parlamentare fisica</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Occorre istituire le basi legali per un'attività parlamentare digitale e per la partecipazione digitale all'attività parlamentare fisica.
+REASONING: Con la crisi del Coronavirus l'attività parlamentare si è arrestata. La sessione primaverile è stata interrotta anzitempo e anche le Commissioni, su ordine degli Uffici delle rispettive Camere, non hanno più potuto riunirsi. Da molte parti ci si è chiesti come sarebbe stato possibile mantenere l'attività delle Camere in caso di crisi prolungata. La Costituzione prevede esplicitamente che i parlamentari siano presenti fisicamente e la legge sul Parlamento stabilisce che le Camere si riuniscono a Berna. Una perizia dell'Università di Zurigo giunge tuttavia alla conclusione che un funzionamento digitale del Parlamento sia del tutto possibile. I requisiti tecnici dovrebbero ovviamente essere elevati al fine di escludere qualsiasi abuso, fra cui la partecipazione di persone non autorizzate in vece dei membri preposti. Anche le condizioni per lo svolgimento dell'attività parlamentare dovranno essere definite severamente e valere solo in situazioni eccezionali, oltre ad essere assoggettate all'obbligo di autorizzazione (p. es. da parte…</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr"/>
+      <c r="G28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="F29" s="4" t="n"/>
-      <c r="G29" s="4" t="n"/>
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="n">
+        <v>337362</v>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Commissioni extraparlamentari. Riorganizzazione nel quadro della verifica 2025</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr"/>
+      <c r="F29" s="5" t="inlineStr"/>
+      <c r="G29" s="5" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="F30" s="4" t="n"/>
-      <c r="G30" s="4" t="n"/>
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="n">
+        <v>153188</v>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Stärkung der Volksrechte. Unterschriftensammlung für Initiativen und Referenden im Internet</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Der Bundesrat wird aufgefordert, die gesetzlichen Grundlagen zu schaffen, um das elektronische Sammeln von Unterschriften für Initiativen und Referenden zu erlauben. Dazu zählt auch die Unterschrift über Touchscreens. Der Bund soll in diesem Zusammenhang die digitale Partizipation der stimmberechtigten Schweizerinnen und Schweizer im In- und Ausland stärken.
+REASONING: E-Collecting war ein fester Bestandteil der "Vote électronique"-Strategie des Bundesrates, um die Volksrechte der Schweiz zu modernisieren (vgl. BK, Strategische Planung Vote électronique, 18. März 2011). Im April 2015 kündigte der Bundesrat überraschend an, auf die Weiterführung im Bereich des E-Collectings zu verzichten. Die Folge davon ist eine Schwächung der direkten Demokratie, da wachsende Teile der Stimmberechtigten bei Unterschriftensammlungen ausgeschlossen und immer höhere finanzielle und personelle Ressourcen für die Komitees nötig werden. Eine Ergänzung des Bundesgesetzes über die politischen Rechte (BPR) soll daher digitale Unterschriften erlauben - etwa auf Touchscreens, so wie seit geraumer Zeit der Empfang von Paketen und Einschreiben bestätigt wird. Dies würde es einer breiteren Bevölkerungsgr…</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr"/>
+      <c r="G30" s="5" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="F31" s="4" t="n"/>
-      <c r="G31" s="4" t="n"/>
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="n">
+        <v>154613</v>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Lancio del 5G in Svizzera. Onere supplementare per i cantoni. Quale compensazione da parte della Confederazione?</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Recentemente la Commissione federale delle comunicazioni (Comcom) ha attribuito nuove frequenze di radiocomunicazione a tre operatori svizzeri. I ricavi realizzati con questa operazione si aggirano sui 380 milioni di franchi e sono stati versati nelle casse federali a titolo di ricavi straordinari. Siccome le concessioni sono state attribuite per una durata di 15 anni, per i prossimi anni si prevede un numero significativo di domande di costruzione per nuove antenne. A titolo esemplificativo, nell'arco dei prossimi due a tre anni l'operatore Swisscom progetta di installare una ventina di piloni nel Cantone del Giura. Qualsiasi nuova costruzione o modifica di impianti preesistenti è sottoposta al rilascio di un'autorizzazione. L'introduzione del 5G in Svizzera implicherà pertanto inevitabilmente un incremento del carico di lavoro e costi supplementari per i Cantoni. Anche se le autorizzazioni rilasciate dalle amministrazioni cantonali sono soggette al versamento di tasse, altre prestazioni legate al trattamento di questi dossier (segnatamente i lavori generati dalle procedure di opposizione e di ricorso) sono particolarmente laboriose e non generano alcun introito. Le domande …</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr"/>
+      <c r="G31" s="5" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="F32" s="4" t="n"/>
-      <c r="G32" s="4" t="n"/>
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="n">
+        <v>236031</v>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Renvois vers l’Afghanistan. Un flop ?</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Depuis l’automne 2024, les renvois de ressortissants afghans ont repris graduellement, mais ils se limitent pour l’instant aux personnes qui ont commis des crimes graves. En avril 2025, le Conseil fédéral a décidé d’ajuster sa pratique pour les hommes seuls qui ne présentent pas de vulnérabilités. Les conditions à remplir pour un renvoi sont les suivantes : ces hommes doivent séjourner en Suisse sans famille, être majeurs et en bonne santé et disposer en Afghanistan d’un réseau relationnel stable et solide qui leur permet de se réintégrer dans la société. On a pu lire dans la presse que cette nouvelle pratique n’avait conduit à aucun renvoi et qu’un migrant renvoyé en Afghanistan avait même dû être ramené en Suisse parce que les autorités afghanes avaient refusé de le réadmettre, à l’aéroport de Kaboul. On a appris dans le même temps que la Suisse versait à nouveau une aide au développement à l’Afghanistan, d’un montant annuel de 27 millions de francs. Je pose au Conseil fédéral les questions suivantes : Que pense-t-il des résultats de la nouvelle pratique appliquée pour le renvoi des migrants afghans qui n’ont pas le droit de rester en Suisse ? Ne considère-t-il pas que les …</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr"/>
+      <c r="G32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="F33" s="4" t="n"/>
-      <c r="G33" s="4" t="n"/>
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="n">
+        <v>159478</v>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Étendre les compétences du SRC alors qu’il fiche les partis ?</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Les médias ont révélé que le SRC continuait de collecter beaucoup trop de données et ne respectait pas les conditions de l'art. 5 LRens, qui lui interdit de rechercher et de traiter des informations relatives aux activités politiques. Cette pratique est extrêmement dommageable pour la démocratie et soulève des questions fondamentales en matière de gouvernance. - Dans ce contexte, est-il légitime de prévoir une extension des compétences du SRC ? - Le Conseil fédéral n'estimerait-il pas préférable de suspendre la révision de la LRens ?</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr"/>
+      <c r="G33" s="5" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="F34" s="4" t="n"/>
-      <c r="G34" s="4" t="n"/>
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="n">
+        <v>67332</v>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Weg von Fast Fashion, aber wie?</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: In den letzten 20 Jahren sind Textilien von einem Gebrauchsgegenstand zum Wegwerf-Artikel geworden. Die Tragedauer von Kleidern ist um 40 Prozent gesunken. Dafür hat sich die weltweite Produktion verdoppelt. Die billige und schnelllebige Fast-Fashion-Industrie hat immense Schattenseiten. Prekäre Arbeitsbedingungen und gesundheitsschädigende Umweltbelastungen prägen die globalen Lieferketten. 2018 haben deshalb das Bundesamt für Umwelt (BAFU) gemeinsam mit dem Staatssekretariat für Wirtschaft (SECO) sowie den Verbänden Swiss Textiles und amfori die Initiative "Nachhaltige Textilien Schweiz" als Multi-Stakeholder-Dialog gestartet. Daraus ist das Programm "Sustainable Textiles Switzerland 2030 (STS 2030)" entstanden, das einen wesentlichen Beitrag zur Erreichung der Nachhaltigen Entwicklungsziele (SDGs) im Schweizer Textil- und Bekleidungssektor entlang der gesamten Wertschöpfungskette leisten will. Die am Programm beteiligten Unternehmungen und Verbände setzen sich im Rahmen ihrer Eigenverantwortung in einem vorbildlichen Prozess für die Reduktion der Treibhausgasemissionen, die Förderung fairer Löhne und menschenwürdiger Arbeitsbedingungen, die Förderung innovativer Geschäftsm…</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr"/>
+      <c r="G34" s="5" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="F35" s="4" t="n"/>
-      <c r="G35" s="4" t="n"/>
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="n">
+        <v>66800</v>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Mesures contre l'immigration illégale (8/9). Systématiser l'échange des données concernant les immigrés illégaux</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Afin de lutter durablement contre l'immigration illégale en Suisse et si possible d'y mettre un terme, il faut que l'échange des données sur les personnes concernées entre les cantons, les communes, les autorités sociales, les caisses-maladie, l'AVS, l'AI et d'autres assurances sociales devienne systématique. Il s'agit d'échanger et de comparer toutes les données relatives au statut de séjour, au lieu de domicile, à la couverture d'assurance, aux paiements des primes, aux réductions de primes, aux prestations des caisses-maladie, à l'AVS, à l'AI et à d'autres assurances sociales.
+REASONING: En fonction des estimations et des sources d'information, jusqu'à 100 000 immigrés illégaux - banalement appelés " sans-papiers " - seraient en Suisse. Afin de réduire l'attrait de notre pays à cet égard, il importe que ces personnes puissent être identifiées et renvoyées grâce à un échange systématique des données les concernant. Selon le rapport du Conseil fédéral " Pour un examen global de la problématique des sans-papiers " en réponse au postulat de la Commission des institutions politiques du Conseil national du 12 avril 2018 (18.3381), les assurances et les caisses-maladie surtout n…</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr"/>
+      <c r="G35" s="5" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="F36" s="4" t="n"/>
-      <c r="G36" s="4" t="n"/>
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="n">
+        <v>331084</v>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Finanzierung und Rüstungsplanung der Armee</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Laut Vernehmlassungsunterlagen plant das VBS ab 2028 mit zusätzlichen jährlichen Ausgaben von 3,1 Milliarden Franken, die in den ersten Jahren durch Verschuldung des Rüstungsfonds finanziert werden sollen. 1. Finden diese zusätzlichen Milliardenausgaben Eingang in die Finanzplanung des Bundes? 2. Wie hoch ist der maximale «Bereinigungsbedarf» im Falle einer Ablehnung der Vorlage? 3. Welche Ausgaben wären von dieser «Bereinigung» betroffen? 4. Wären auch sicherheitsrelevante Ausgabenbereiche (FedPol, BACS, NDB, SEPOS usw.) von dieser «Bereinigung» betroffen? 5. In welchem Verhältnis steht die Höhe des maximalen «Bereinigungsbedarfs» zur Höhe der Ausgaben, die im Falle einer Ablehnung der Vorlage kurzfristig gekürzt werden müssen? Hat der Bundesrat das grösstmögliche Risiko berechnet und darf dieses wirklich eingegangen werden? 6. Welche Finanzmittel können für dringende Beschaffungen in den Jahren 2027, 2028 und 2029 freigespielt werden, wenn bereits bewilligte Beschaffungsvorhaben, die auf Bedrohungen mit einer geringen Eintretenswahrscheinlichkeit ausgerichtet sind, frühestens ab 2030 finanzwirksam würden?
+ANSWER: Der Bundesrat hat nach Abschluss der Vernehmlassung die Eckw…</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr"/>
+      <c r="G36" s="5" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="F37" s="4" t="n"/>
-      <c r="G37" s="4" t="n"/>
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="n">
+        <v>62377</v>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Rete nazionale di dati sicura. Credito d’impegno</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr"/>
+      <c r="F37" s="5" t="inlineStr"/>
+      <c r="G37" s="5" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="F38" s="4" t="n"/>
-      <c r="G38" s="4" t="n"/>
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="n">
+        <v>65819</v>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Chiusura dell'ultimo ufficio postale a Chêne-Bougeries</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: La Posta sta valutando di chiudere l'ufficio postale del Comune di Chêne-Bougeries. Questo comune di oltre 11 000 abitanti perderebbe così il suo ultimo ufficio postale dopo la soppressione di quello di Conches nel 2015. Vi è una forte domanda e questa chiusura è incomprensibile. Infatti, in questo Comune nascono nuovi quartieri. Inoltre, un quarto della popolazione ha superato l'età di pensionamento e quasi il 10 per cento ha più di 80 anni. Queste persone fanno spesso capo agli uffici postali. In aggiunta questo ufficio postale è uno degli elementi strutturali preso in considerazione per lo sviluppo del Comune, in particolare per l'allestimento dell'infrastruttura dei trasporti pubblici. Una petizione era stata lanciata nel 2017 da un gruppo politico, sindacati e utenti; all'inizio del 2018 sono state raccolte 1251 firme, che sono state inviate alla direzione della Posta. Invito pertanto il Consiglio federale a rispondere alle seguenti domande: 1. Quante persone fanno capo all'ufficio postale di Chêne-Bougeries dal 2015? 2. Come intende garantire un servizio postale pubblico di qualità per gli abitanti di Chêne-Bougeries? 3. Se la Posta intende sostituire l'ufficio di Chêne…</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr"/>
+      <c r="G38" s="5" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="F39" s="4" t="n"/>
-      <c r="G39" s="4" t="n"/>
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="n">
+        <v>153731</v>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Stromspeicher bezüglich Netznutzung technologieneutral und somit gleichbehandeln</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Ich bitte den Bundesrat, folgende Fragen zu beantworten: 1. Warum beabsichtigt der Bundesrat, Stromspeicher hinsichtlich der Verrechnung von Netznutzungsentgelten für den Bezug von Elektrizität aus dem Netz gegenüber Pumpspeicherkraftwerken zu diskriminieren - Regulierungsvorgaben sollten technologieneutral sein -? 2. Ist er sich bewusst, dass Stromspeicher beim Umbau des Energiesystems zukünftig eine wichtige Rolle für den Ausgleich zwischen stark fluktuierender und wetterabhängiger erneuerbarer Energie und dem Verbrauch übernehmen müssen? 3. Ist er nicht der Ansicht, dass mit der Belastung von Speichern mit Netznutzungsentgelten auch die Ausnahmeregelung für Pumpspeicherkraftwerke hinterfragt werden muss und gefährdet ist? 4. Ist er sich bewusst, dass er mit dem neuen Artikel 2 Absatz 3 der Stromversorgungsverordnung (StromVV; Speicher gelten für den Bezug als Endverbraucher) einen Widerspruch zu Artikel 4 Absatz 1 Litera b schafft, worin ein Endverbraucher definiert ist als Kunde, der Elektrizität für den eigenen Verbrauch kauft, und somit eine Rechtsunsicherheit?
+REASONING: In der Vernehmlassungsvorlage zu den Verordnungen der Strategie Stromnetze ist vorgesehen, dass, w…</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr"/>
+      <c r="G39" s="5" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="F40" s="4" t="n"/>
-      <c r="G40" s="4" t="n"/>
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="n">
+        <v>157707</v>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Ordinanza sull’indicazione dei prezzi. Semplificare l’autocomparazione</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Il Consiglio federale è incaricato di semplificare le disposizioni dell'ordinanza sull'indicazione dei prezzi (OIP; RS 942.211) riguardanti l'indicazione fallace dei prezzi (art. 16 cpv. 1 lett. a e cpv. 3 OIP) in modo da consentire l'autocomparazione senza che siano fissati limiti di tempo, in particolare per gli articoli di stagione come capi di abbigliamento, calzature, articoli sportivi, ecc., se la merce in questione è stata effettivamente proposta in precedenza, per almeno quattro settimane consecutive, al prezzo più alto indicato.
+REASONING: Le disposizioni piuttosto complesse dell'OIP sull'autocomparazione, che regolamentano le indicazioni di riduzione dei prezzi e le comparazioni con il prezzo di vendita iniziale, erano state introdotte per evitare che i consumatori fossero tratti in inganno, ma oggi sono superate. Più in particolare, la cosiddetta regola del dimezzamento secondo cui il "prezzo comparativo" può essere indicato solo per la metà del periodo durante il quale è stato o sarà praticato, e al massimo per due mesi, comporta per i venditori e per le autorità di controllo un onere sproporzionato rispetto al vantaggio che ne risulta per il cliente. Questa rego…</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr"/>
+      <c r="G40" s="5" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="F41" s="4" t="n"/>
-      <c r="G41" s="4" t="n"/>
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="n">
+        <v>63936</v>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Renforcement de la Division Sécurité humaine au niveau de la coopération internationale</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Le Conseil fédéral est chargé de prendre des mesures afin de renforcer les moyens financiers de la Division sécurité humaine dans le cadre de nos actions de coopération internationale.
+REASONING: Au sein des activités de coopération internationale réalisées par notre pays, figure celles de la Division sécurité humaine. Pour leur réalisation, cette division dispose d'un budget de 2,3 % du crédit-cadre de la coopération internationale 2021-2024. Ce pourcentage m'apparaît nettement insuffisant. Dans la perspective "mieux vaut prévenir que guérir", il me semble plus logique de prendre toutes les mesures utiles avant l'éclatement de conflits, de tenter toutes les démarches visant à les désamorcer plutôt que de venir réparer les dégâts après. L'actualité et les échos que nous en donnent les médias montrent que de nombreuses populations et régions du globe souffrent de conflits qui auraient pu, et dû, être évités. Renforcer ce secteur de la sécurité humaine permettrait d'obtenir des "économies" en vies humaines et en catastrophes de tous genres. La Suisse est crédible dans les domaines des droits humains, du désarmement, du droit humanitaire. Son statut et sa réputation de pays neu…</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="inlineStr"/>
+      <c r="G41" s="5" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="F42" s="4" t="n"/>
-      <c r="G42" s="4" t="n"/>
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="n">
+        <v>340056</v>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Jetzt handeln: Kriterien für Ausnahmebewilligungen nach Art. 5 WG überarbeiten</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Der Bundesrat wird beauftragt, die gesetzlichen Grundlagen so anzupassen, dass Ausnahmebewilligungen für verbotene Waffen nach Artikel 5 WG künftig restriktiver und nach einheitlichen, nachvollziehbaren Kriterien erteilt werden und der Ausnahmecharakter dieser Bewilligungen gewahrt bleibt.
+REASONING: Verbotene Waffen dürfen gemäss Waffengesetz nur ausnahmsweise und unter bestimmten Voraussetzungen erworben und besessen werden. Im Kanton Zürich wurden in den letzten sieben Jahren fast 20'000 verbotene Waffen mit einer Ausnahmebewilligung zugelassen, im Kanton Thurgau gut 5'300 und im Kanton Aargau mehr als 6'000. Im Kanton Basel-Landschaft wurden in dieser Zeit fast 1'900, in Genf knapp 1'300 Ausnahmebewilligungen ausgestellt und im Kanton Wallis sind es alleine dieses Jahr fast 400. Dies wirft die Frage auf, ob die heutige Bewilligungspraxis dem gesetzlich vorgesehenen Ausnahmecharakter noch ausreichend Rechnung trägt. Angesichts der Fälle, in denen Waffen zur Tötung oder schweren Gefährdung von Menschen eingesetzt werden, ist eine sorgfältige und restriktive Bewilligungspraxis von besonderer Bedeutung. Es muss gewährleistet sein, dass vor der Erteilung einer Ausnahmebewilli…</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="inlineStr"/>
+      <c r="G42" s="5" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="F43" s="4" t="n"/>
-      <c r="G43" s="4" t="n"/>
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="n">
+        <v>202440</v>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Inkassounternehmen. Für eine bessere Information der Konsumentinnen und Konsumenten</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Der Bundesrat wird beauftragt, eine Einrichtung zur Entgegennahme von Beschwerden zu schaffen, damit Konsumentinnen und Konsumenten die Verarbeitung ihrer Daten durch private Inkassounternehmen und Kreditauskunfteien wenn nötig anfechten können. Die Einrichtung wäre dem Eidgenössischen Datenschutz- und Öffentlichkeitsbeauftragten (EDÖB) angegliedert, würde über ein eigenes Budget verfügen und auch Sensibilisierungs- und Informationsarbeit leisten.
+REASONING: Unternehmen, die im Bereich Inkasso tätig sind, geben Auskünfte über die Zahlungsfähigkeit der ihnen bekannten Debitorinnen und Debitoren, ohne dabei den gesetzlichen Rahmen immer einzuhalten. Die Art, wie die Daten gesammelt werden, ist undurchsichtig, insbesondere bei Online-Einkäufen oder wenn die Daten basierend auf Algorithmen gesammelt werden, die eine Person aufgrund von Verhaltensdaten bewerten. Die Konsumentinnen und Konsumenten haben so gut wie keine Kontrolle darüber, wie ihre persönlichen Daten und Informationen zu ihren Zahlungsgewohnheiten gesammelt und weitergegeben werden. Doch auf dieser Grundlage getroffene Entscheidungen können schwerwiegende Folgen haben: Es kann soweit kommen, dass Konsumentinnen und…</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="inlineStr"/>
+      <c r="G43" s="5" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="F44" s="4" t="n"/>
-      <c r="G44" s="4" t="n"/>
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="n">
+        <v>213693</v>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Entreprises plates-formes et économie à la tâche ou "gig economy". Mieux protéger les travailleurs indépendants</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Le Conseil fédéral est chargé d'élaborer un rapport dans lequel il propose des pistes pour améliorer la protection sociale des indépendants travaillant à la tâche. Il devra en particulier examiner comment les entreprises plateformes pourraient contribuer à assurer une meilleure couverture sociale aux personnes participant à cette économie dite collaborative ou de partage.
+REASONING: Déjà en plein essor, les modèles de travail flexible vont se développer encore sous l'effet d'une numérisation galopante. Ils consistent à proposer de brèves missions à des indépendants ou des personnes employées à temps très partiel. On peut s'attendre à ce que la tendance à l'ubérisation, dominée par les entreprises plateformes, prenne encore de l'ampleur. Cette évolution propose de nouveaux modèles d'entreprises mais elle ouvre aussi de nouvelles possibilités qui, à certaines conditions, peuvent tout à fait séduire les indépendants. Le problème est que ceux-ci se voient moins bien protégés contre les risques sociaux. Les acteurs politiques sont donc appelés à examiner les conditions de cette nouvelle économie et à les adapter si nécessaire afin qu'elle ne soit pas synonyme de réduction de la p…</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="inlineStr"/>
+      <c r="G44" s="5" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="F45" s="4" t="n"/>
-      <c r="G45" s="4" t="n"/>
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="n">
+        <v>71679</v>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Jeu vidéo à caractère islamiste vendu sur « Steam » : le Conseil fédéral va-t-il réagir en conséquence ?</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Nous avons appris avec stupeur qu’un jeu vidéo est en vente sur la très populaire plateforme « Steam », intitulé « Fursan al-Aqsa: The Knights of the Al-Aqsa Mosque », glorifiant explicitement les abominables attaques terroristes du 7 octobre 2023 en Israël lors desquelles plus de 1000 personnes, principalement des civils sans défense, ont été massacrées. Ce jeu est une promotion explicite de l’idéologie islamiste et des crimes contre l’humanité commis lors de l’attaque du Hamas contre Israël en 2023. Le 29 novembre dernier, nous apprenions par voie de presse que le Royaume-Uni a interdit et banni ce « jeu » de la plateforme « Steam » et de tout support officiel permettant de se le procurer. L’apologie du terrorisme islamiste, de la haine et des crimes de guerre et crimes contre l’humanité n’étant pas tolérable dans notre pays, la Confédération compte-t-elle aussi intervenir afin d’interdire ce « jeu » vidéo abjecte ?
+ANSWER: L'incitation à la violence ou la discrimination envers une personne ou un groupe de personnes en raison de leur appartenance religieuse ou ethnique ainsi que la négation d'un génocide sont largement couverts par le Code pénal. La répression pénale de ce…</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr"/>
+      <c r="G45" s="5" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="F46" s="4" t="n"/>
-      <c r="G46" s="4" t="n"/>
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="n">
+        <v>155922</v>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Atténuer la crise du coronavirus pour les personnes à faibles revenus</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Le Conseil fédéral est chargé avec les cantons d'augmenter le montant des subsides aux primes d'assurance-maladie de 50 % pendant deux ans pour les personnes ayant de faibles revenus afin d'éviter que davantage de personnes en Suisse ne sombrent dans la précarité.
+REASONING: Dans notre pays, près d'un million de personnes vivent dans la précarité ou juste au-dessus du seuil de pauvreté selon les derniers chiffres de l'Office fédéral de la statistique, soit une personne sur sept. La situation s'est considérablement aggravée depuis avec la pandémie, qui a privé de nombreux ménages de leur revenu principal. Un nombre croissant de personnes ne peuvent plus payer leurs primes d'assurance-maladie, qui déjà avant la crise représentaient une charge très importante pour les familles. Dans cette situation extraordinaire, la Confédération et les cantons doivent augmenter de 50 %, pour une durée de deux ans le montant des subsides aux primes d'assurance-maladie. Les finances fédérales et cantonales permettent de supporter cette charge supplémentaire. Elle permettra d'éviter la précarisation d'une partie de la population, qui coûterait très cher à l'État à long terme. Agir maintenant, po…</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="inlineStr"/>
+      <c r="G46" s="5" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="F47" s="4" t="n"/>
-      <c r="G47" s="4" t="n"/>
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="n">
+        <v>288093</v>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Sicurezza dei prodotti: rafforzare la libera concorrenza tra attori svizzeri e stranieri del commercio online</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: I recenti avvenimenti che hanno coinvolto la piattaforma di e-commerce cinese Shein nella vicina Francia sollevano interrogativi legittimi anche in Svizzera. Se si considera che ogni giorno arrivano a Zurigo circa 500 000 pacchi dalla Cina, risulta difficile stabilire se i controlli di qualità imposti ai prodotti svizzeri siano applicati nella stessa misura anche ai prodotti cinesi. Alcuni degli articoli in vendita sulle piattaforme cinesi stanno suscitando un certo scalpore. Su Temu, ad esempio, è possibile trovare puntatori laser il cui uso è severamente vietato in Svizzera a causa dei possibili rischi per la vista associati. Inoltre, un recente studio dimostra che l'86 per cento dei giocattoli disponibili sulle principali piattaforme di commercio online straniere (Temu, Shein, Amazon) sono considerati pericolosi per la salute dei bambini. Come giustifica il Consiglio federale il fatto che i prodotti in vendita sulle piattaforme cinesi non soddisfino gli stessi requisiti di qualità dei prodotti svizzeri, soprattutto in termini di sicurezza? Come intende obbligare le piattaforme straniere a rispettare le stesse regole imposte ai loro concorrenti svizzeri? Quali misure intend…</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr"/>
+      <c r="G47" s="5" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="F48" s="4" t="n"/>
-      <c r="G48" s="4" t="n"/>
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="n">
+        <v>63574</v>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Adeguamento del diritto federale agli sviluppi della tecnologia di registro distribuito. Legge federale</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr"/>
+      <c r="F48" s="5" t="inlineStr"/>
+      <c r="G48" s="5" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="F49" s="4" t="n"/>
-      <c r="G49" s="4" t="n"/>
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="n">
+        <v>65002</v>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Coronavirus. Un Parlement virtuel serait-il une solution?</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Alors que la Suisse risque elle aussi de se retrouver dans une situation de crise en raison de la propagation du coronavirus, je prie le Bureau de répondre aux questions suivantes : 1. Comment le bon fonctionnement des institutions peut-il être garanti en période de crise ? 2. Le Parlement aurait-il la possibilité à l'heure actuelle de prendre des décisions dans une situation de crise sans avoir à se réunir physiquement ? 3. Dans la négative, quelles bases légales ou constitutionnelles faudrait-il créer pour que le travail parlementaire puisse avoir lieu en situation de crise sans que le Parlement ait à se réunir physiquement ? 4. Quelles mesures techniques y aurait-il lieu de prendre (identités électroniques, logiciels permettant de conduire de bout en bout les processus politiques, etc.) pour que le travail parlementaire puisse être effectué en ligne avec toute l'efficacité et toute la sécurité requises ?
+REASONING: Les défis que les parlementaires de milice doivent relever dans leur quotidien parlementaire sont déjà nombreux. Mais dans des situations de crise telles que celle qui s'annonce avec l'épidémie de coronavirus, il est encore plus difficile de garantir le bon dér…</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr"/>
+      <c r="G49" s="5" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="F50" s="4" t="n"/>
-      <c r="G50" s="4" t="n"/>
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="n">
+        <v>340378</v>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Weiteres IT - Experimentierfeld beim Bund mit Microsoft 365?</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Kaum ist die Einführung von Microsoft 365 in der Bundesverwaltung abgeschlossen, wird bereits an einer Open-Source-Alternative gearbeitet. Grundsätzlich ist es richtig, Abhängigkeiten zu prüfen. Es stellt sich jedoch die Frage, ob der Bund hier erneut Gefahr läuft, ein funktionierendes System zum kostspieligen IT-Experimentierfeld zu machen. Microsoft 365 ist etabliert und wird in der Bundesverwaltung breit eingesetzt. Microsoft verfügt zudem über Rechenzentrumsregionen in der Schweiz und arbeitet eng mit Schweizer Partnern zusammen. Für besonders schützenswerte Daten hat der Bund zusätzliche Vorgaben und eigene Infrastrukturen. Vor diesem Hintergrund muss nachvollziehbar dargelegt werden, welchen konkreten Mehrwert ein paralleles oder neues System tatsächlich bringt. Die Vergangenheit zeigt, dass IT-Projekte des Bundes immer wieder durch Verzögerungen, Kostenüberschreitungen, Schnittstellenprobleme oder mangelnde Praxistauglichkeit aufgefallen sind. Umso weniger verständlich wäre es, ein funktionierendes und erst kürzlich eingeführtes System aus politischen Überlegungen abzustellen, ohne Kosten, Risiken und Nutzen vollständig offenzulegen. Der Bundesrat wird gebeten, folgend…</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr"/>
+      <c r="G50" s="5" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="F51" s="4" t="n"/>
-      <c r="G51" s="4" t="n"/>
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="n">
+        <v>68304</v>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Les règles sur la transparence du financement de la vie politique doivent être mises en oeuvre de manière conforme à la volonté du Parlement</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: 1. Que pense le Conseil fédéral des critiques émises au sujet de l'ordonnance par plusieurs participants à la procédure de consultation, et de quelle manière entend-il en tenir compte dans la version définitive de l'ordonnance ? 2. Est-il problématique selon lui de vouloir contraindre le Contrôle fédéral des finances (CDF), contre la volonté de son directeur, à contrôler si les règles sur la transparence du financement des partis sont respectées ? 3. En adoptant le contre-projet, le Parlement a montré clairement qu'il souhaitait la plus grande transparence possible dans le financement de la vie politique et la mise en place de règles uniformes et contrôlables applicables à tous, afin de favoriser la libre formation de l'opinion des citoyens avant les votations et les élections. Quelle serait la réglementation nécessaire, selon le Conseil fédéral, pour que la loi et l'ordonnance garantissent la transparence du financement des partis ? 4. La mesure prévoyant que l'autorité compétente effectue des contrôles par échantillonnage pour vérifier si les règles sur la transparence sont mises en oeuvre correctement a été ajoutée par les Chambres lors des délibérations parlementaires, et…</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr"/>
+      <c r="G51" s="5" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="F52" s="4" t="n"/>
-      <c r="G52" s="4" t="n"/>
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" t="n">
+        <v>331167</v>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>G7-Gipfel: Vom 10. bis 19. Juni 2026 lässt der Bundesrat an der Grenze zu Frankreich verstärkte Grenzkontrollen durchführen. Was macht er bei grenzüberschreitender Kriminalität?</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Polizeimeldungen bestätigen, dass Tätergruppen aus Frankreich wiederholt Fahrzeugdiebstähle und weitere Delikte in der Schweiz begehen. - Ist der Bundesrat der Ansicht, dass verstärkte Grenzkontrollen nicht nur zum Schutz des G7-Gipfels, sondern auch zur Bekämpfung der grenzüberschreitenden Kriminalität beitragen können? - Bestehen die notwendigen rechtlichen und operativen Möglichkeiten, um die Kontrolldichte an der Grenze zu Frankreich (analog zu den Massnahmen zum G7-Gipfel) zu erhöhen?
+ANSWER: Bei früheren G8-Treffen ist es zu gewaltsamen Auseinandersetzungen, Stör- und Sabotageaktionen sowie zu Sachbeschädigungen gekommen. Vor diesem Hintergrund hat der Kanton Genf beim Bundesrat für die Dauer des G7-Gipfels ein Gesuch um temporäre Wiedereinführung von Binnengrenzkontrollen an den Land- und Seegrenze eingereicht. Dieses hat der Bundesrat gutgeheissen. Für die Bekämpfung von grenzüberschreitender Kriminalität setzen Bund und Kantone aber grundsätzlich auf andere Instrumente: Das Bundesamt für Zoll und Grenzsicherheit (BAZG) ist an der Grenze und im Grenzraum präsent und kontrolliert im Rahmen seines Auftrages lage- und risikobasiert den grenzüberschreitenden Waren- und P…</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr"/>
+      <c r="G52" s="5" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="F53" s="4" t="n"/>
-      <c r="G53" s="4" t="n"/>
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="n">
+        <v>159482</v>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Steigende Heizkosten: Wie rasch kann der Bundesrat handeln?</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Gemäss Antwort auf 22.7358 hat der Bundesrat Massnahmen betreffend steigende Heizkosten geprüft, die rasch umsetzbar sein sollen und an die Ergänzungsleistungen oder Prämienverbilligung anknüpfen. Er hat aber keine Entscheide getroffen. - Mit welchen Fristen rechnet der Bundesrat für die Umsetzung dieser Massnahmen nach einem Entscheid? - Können diese spätestens auf den Zeitpunkt der Abrechnung Heizkostenperiode Juni 2023 in Kraft treten?</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="inlineStr"/>
+      <c r="G53" s="5" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="F54" s="4" t="n"/>
-      <c r="G54" s="4" t="n"/>
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="n">
+        <v>235974</v>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Le prospettive dell'AVS erano errate. Lo sono anche quelle dell'AI?</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Chiedo al Consiglio federale di rispondere alle seguenti domande: È noto che sono stati commessi errori nelle previsioni dell’AVS. Sono stati commessi gli stessi errori anche per quanto riguarda le cifre dell’AI? I debiti dell’AI gravano l’AVS. L’Amministrazione federale ha ripetutamente comunicato a partire da quando l’AI potrà ridurre il debito nel bilancio dell’AVS. Quali dati sono stati comunicati dal 2012? Quali motivazioni sono state addotte dal 2012 per la costante posticipazione di questo momento? Quando saranno presentate al Parlamento nuove basi di dati che contengano anche la crescita delle nuove rendite e la diminuzione dei tassi di uscita, fattori menzionati da Compenswiss? Il Consiglio federale come garantisce una maggiore attendibilità delle previsioni dell’AI affinché si disponga di basi sicure per una prossima revisione dell’AI?
+REASONING: Il 18 febbraio 2025 il Consiglio di amministrazione di Compenswiss ha comunicato che «[a]nche per il fondo AI le prospettive finanziarie sono peggiorate a causa dell’aumento delle nuove rendite e della diminuzione dei tassi di uscita» e avvertito che «[d]ata la sua situazione finanziaria, è improbabile che l’AI possa ridur…</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr"/>
+      <c r="G54" s="5" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="F55" s="4" t="n"/>
-      <c r="G55" s="4" t="n"/>
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" t="n">
+        <v>153874</v>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Vorstösse verbindlich behandeln</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Gestützt auf Artikel 160 Absatz 1 der Bundesverfassung und Artikel 107 des Parlamentsgesetzes reiche ich folgende parlamentarische Initiative ein: Im Bundesgesetz über die Bundesversammlung (Parlamentsgesetz, ParlG) ist eine Frist zur Behandlung von Motionen und Postulaten vorzusehen ähnlich wie für parlamentarische Initiativen. Motionen und Postulate dürfen nicht mehr unbehandelt abgeschrieben werden. Es darf jedoch keine Einschränkung der Anzahl eingereichter Vorstösse geben. Stattdessen könnte das Büro beispielsweise verpflichtet werden, ältere Vorstösse prioritär zu behandeln.
+REASONING: Motionen und Postulate sind wichtige Instrumente der Parlamentsarbeit. Wir als gewählte Vertreterinnen und Vertreter des Volkes können über diese Instrumente unsere politischen Anliegen zielgerichtet einbringen und nehmen so auch massgeblich unseren Wählerauftrag wahr. Nur leider geht es im Schnitt über ein Jahr, bis die Vorstösse überhaupt im Rat behandelt werden. Dies führt dazu, dass wichtige Anliegen verschleppt werden oder sogar verloren gehen. Dies zeugt nicht von einem effizienten Ratsbetrieb. Das entspricht auch nicht dem Tempo, in dem unsere Welt funktioniert oder unsere Wirtsch…</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr"/>
+      <c r="G55" s="5" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="F56" s="4" t="n"/>
-      <c r="G56" s="4" t="n"/>
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" t="n">
+        <v>71286</v>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Opposition locale contre les centres fédéraux pour requérants d’asile</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: - Lorsqu’un centre fédéral pour requérants d’asile est prévu, l’opposition de la population locale a-t-elle une influence sur sa réalisation et son exploitation ? - La Confédération pense-t-elle que cette opposition disparaîtra d’elle-même avec le temps ?
+ANSWER: La réponse du Conseil fédéral n'existe qu'en allemand. (Veuillez changer la langue en haut à droite de la page d'accueil)</t>
+        </is>
+      </c>
+      <c r="F56" s="5" t="inlineStr"/>
+      <c r="G56" s="5" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="F57" s="4" t="n"/>
-      <c r="G57" s="4" t="n"/>
+      <c r="A57" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" t="n">
+        <v>251354</v>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Sanzioni contro le opposizioni abusive nel settore edilizio</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Il Consiglio federale è incaricato di creare una base legale che permetta di sanzionare le opposizioni abusive. In futuro, coloro che presenteranno opposizione senza un interesse da proteggere o con intenzioni palesemente abusive dovranno poter essere obbligati ad assumere i costi ed eventualmente a risarcire i danni. Il Consiglio federale è tenuto a illustrare come disposizioni in tal senso possano essere disciplinate nella legge sulla pianificazione del territorio (LPT) o in altre leggi federali pertinenti senza compromettere i legittimi diritti di partecipazione della popolazione.
+REASONING: La situazione giuridica attuale consente di protrarre per anni o addirittura di impedire del tutto progetti di costruzione e sviluppo presentando opposizioni di modesta entità o pretestuose. Uno studio recentemente pubblicato dall’Ufficio federale delle abitazioni (UFAB) e dall’Ufficio federale dello sviluppo territoriale (ARE) dimostra chiaramente che le opposizioni sono il motivo più frequente alla base di ritardi e annullamenti di progetti di costruzione di abitazioni. Ne conseguono un aumento dei costi di costruzione, un calo dell’attività edilizia e un’accentuazione della penuria…</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr"/>
+      <c r="G57" s="5" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="F58" s="4" t="n"/>
-      <c r="G58" s="4" t="n"/>
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" t="n">
+        <v>334999</v>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Proteggere i minori dalle immagini intime generate con l'intelligenza artificiale</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Il Consiglio federale è incaricato di presentare, nell’ambito dei progetti legislativi in corso, modifiche giuridiche e misure concrete di attuazione per proteggere i minori dalle immagini sintetiche non consensuali (deepfake sessuali e «nudificazione»), assicurarne la rapida rimozione, permettere un perseguimento penale efficace e garantire un sostegno coordinato alle scuole. Si tratta di adeguare il diritto penale e la legge sulle piattaforme nonché d’instaurare un coordinamento federale con i Cantoni per prevenire e reprimere efficacemente la creazione, la diffusione e lo sfruttamento di immagini intime sintetiche non consensuali che coinvolgono minori, con meccanismi rapidi di segnalazione, conservazione delle prove e sostegno alle vittime.
+REASONING: Le prove si moltiplicano: i deepfake sessuali sono utilizzati prevalentemente a fini pornografici o degradanti, e i minori sono esposti a rischi maggiori rispetto agli adulti. L’UNICEF ha di recente affermato che l’abuso tramite deepfake è un abuso, e ha esortato i governi e l’industria a intervenire per contrastare le immagini sessualizzate generate con l’intelligenza artificiale che coinvolgono minori. Anche le politiche …</t>
+        </is>
+      </c>
+      <c r="F58" s="5" t="inlineStr"/>
+      <c r="G58" s="5" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="F59" s="4" t="n"/>
-      <c r="G59" s="4" t="n"/>
+      <c r="A59" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" t="n">
+        <v>65774</v>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Utiliser "Government Technology" dans l'administration</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Lors de la session d'automne 2020, le Conseil national a suivi la proposition du Conseil fédéral d'adopter le postulat 20.3240 " Création d'un centre d'innovation dans l'administration fédérale ". Le progrès technologique, la numérisation et les nouveaux processus qui y sont associés se sont déjà implantés dans la plupart des secteurs de l'économie privée et ont entraîné de nombreux changements. La plateforme Government Technology (GovTech) élargit la palette numérique pour y inclure la collaboration du secteur public avec des entreprises innovantes du secteur privé, y compris des jeunes pousses technologiques. Dans ce contexte, je prie le Conseil fédéral de répondre aux questions suivantes. 1. Le rapport qui sera établi en réponse au postulat 20.3240 pourra-t-il aussi mettre en évidence des aspects qui pourraient être favorisés par l'utilisation ciblée de GovTech dans la coopération avec des jeunes pousses technologiques ? 2. Quels sont les domaines d'application dans lesquels le Conseil fédéral voit des possibilités de tester et d'appliquer les solutions de ces jeunes pousses ? 3. Peut-il envisager d'impliquer spécifiquement ces jeunes pousses dans l'administration ? Si oui…</t>
+        </is>
+      </c>
+      <c r="F59" s="5" t="inlineStr"/>
+      <c r="G59" s="5" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="F60" s="4" t="n"/>
-      <c r="G60" s="4" t="n"/>
+      <c r="A60" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" t="n">
+        <v>67123</v>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Zugang zu Angeboten der Kinder- und Jugendarbeit für bis 25-Jährige und kinder- und jugendgerechte Informationen in der Corona-Krise</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Seit dem 13. September 2021 gilt für weite Bereiche des öffentlichen Lebens für Personen ab 16 Jahren die Pflicht, ein Covid-Zertifikat vorzuweisen. Diese Neuerung bringt für Jugendliche ab 16 Jahren erneut eine deutliche Einschränkung ihres Lebens. Ausserschulische Angebote bieten Lernorte, die für umfassende Bildung, physisches und psychisches Wohlbefinden sowie gesunde Entwicklung zentral sind. Die Angebote der Offenen Kinder- und Jugendarbeit (OKJA) gehören zum Grundangebot für Kinder und Jugendliche. Um ihre zentralen Funktionen der Früherkennung und -intervention sowie der Förderung der gesunden Entwicklung leisten zu können, müssen die Einrichtungen einen niederschwelligen Zugang gewährleisten können. Die Zertifikatspflicht ab 16 Jahren führt zu einer unangemessenen Hürde bei diesem Zugang. Erste Rückmeldungen aus der Praxis zeigen, dass ein Teil der Jugendlichen und Familien die Angebote gar nicht mehr besuchen - obwohl gerade unter ihnen viele die Freiräume und Unterstützung dringend nötig hätten. In Zusammenhang mit der Coronakrise und der damit verbundenen, zum Teil widersprüchlichen und nicht kinder- und jugendgerechten Kommunikation, ist das Recht auf Information…</t>
+        </is>
+      </c>
+      <c r="F60" s="5" t="inlineStr"/>
+      <c r="G60" s="5" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="F61" s="4" t="n"/>
-      <c r="G61" s="4" t="n"/>
+      <c r="A61" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" t="n">
+        <v>70545</v>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Deklaration von Werbung bei Influencern in der Schweiz</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Der Bundesrat wird beauftragt eine gesetzliche Grundlage zu schaffen, welche die Transparenz und Fairness im Bereich der Influencer-Werbung in der Schweiz fördert. Angesichts der aktuellen Situation, ist nur eine Minderheit der kommerziellen Partnerschaften von Influencer:innen transparent deklariert. Deshalb ist es von entscheidender Bedeutung, klare und verbindliche Regeln zu etablieren.
+REASONING: Mit der Verbreitung sozialer Medien wie Instagram kam auch der Aufstieg der Influencer:innen (Deutsch: Beeinflusser:innen). Solche Influencer:innen sind für ihre Fans Vorbilder in Sachen Mode, Fitness, Entschlackungstees, Nahrungsergänzungsmittel, Schönheit bzw. Schönheitsprodukte, Kochen etc. Deren Empfehlungen gelten viel und sind der Werbeindustrie darum viel Geld wert. Gemäss einer EU-Untersuchung veröffentlichen 97 Prozent der Influencer:innen kommerzielle Inhalte, jedoch deklarieren nur 20 Prozent diese Partnerschaften transparent. Konsumenten dürfen nicht durch versteckte Werbung getäuscht werden. Umso mehr, wenn die Zielgruppe sehr jung und leicht beeinflussbar ist. Die fehlende Deklaration von Werbung zeigt auf, dass in der aktuellen Situation Handlungsbedarf besteht. D…</t>
+        </is>
+      </c>
+      <c r="F61" s="5" t="inlineStr"/>
+      <c r="G61" s="5" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="F62" s="4" t="n"/>
-      <c r="G62" s="4" t="n"/>
+      <c r="A62" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" t="n">
+        <v>65119</v>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Chasser sans preuve de la sûreté du tir est-il sûr, respectueux des animaux et efficace?</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Depuis le 1er janvier 2017, fournir la preuve de la sûreté du tir est obligatoire dans toute la Suisse pour pouvoir s'adonner à la chasse. La conférence des services de la faune, de la chasse et de la pêche de la Suisse et de la Principauté de Liechtenstein a présenté le principe applicable : " La sécurité de la manipulation de l'arme de chasse et la précision du tir sont des éléments indispensables pour une chasse responsable et respectueuse envers la protection des animaux. Pour des raisons de protection des animaux, de sécurité, de valorisation du gibier mais aussi pour une chasse efficace, l'artisanat de base des chasseurs, la sûreté du tir revêt une importance capitale. Un entraînement régulier de tir et une attestation valable sur la sûreté du tir devraient être évidents pour chaque chasseur ". En raison du coronavirus, les stands de tir sont fermés dans toute la Suisse jusqu'à nouvel ordre. Les services cantonaux de la chasse réagissent manifestement de façon très différente. Certains prolongent automatiquement jusqu'au 30 septembre 2020 les permis de tir échus, d'autres exigent un renouvellement de la preuve de la sûreté du tir dans les deux mois à compter de la levée…</t>
+        </is>
+      </c>
+      <c r="F62" s="5" t="inlineStr"/>
+      <c r="G62" s="5" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="F63" s="4" t="n"/>
-      <c r="G63" s="4" t="n"/>
+      <c r="A63" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" t="n">
+        <v>159211</v>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>Soumettre la Société suisse de radiodiffusion et télévision au Contrôle fédéral des finances</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: La loi fédérale sur la radio et la télévision est modifiée de sorte que la Société suisse de radiodiffusion et télévision (SSR) soit soumise au Contrôle fédéral des finances (CDF) en tant qu'autorité de surveillance financière.
+REASONING: La SSR remplit un mandat de prestations global au niveau national et au niveau des régions linguistiques. Elle est principalement financée par la redevance, dont le montant total s'élève à plus d'un milliard de francs. Compte tenu de cette somme, du volume important des activités, du très grand intérêt public et des discussions politiques en cours, la SSR devrait être soumise à la surveillance financière du CDF, comme les autres organisations auxquelles la Confédération confie l'exécution de tâches publiques (voir art. 8, al. 1, let. d, LCF). En tant qu'organe indépendant, le CDF devrait pouvoir examiner les finances de la SSR du point de vue des risques et de la gestion des activités, en étroite collaboration avec les autres autorités et organes chargés de contrôler la société. L'autonomie dans la conception et la gestion des programmes de radio et de télévision, garantie par l'art. 93, al. 3, Cst., resterait opposable au CDF. D'autres org…</t>
+        </is>
+      </c>
+      <c r="F63" s="5" t="inlineStr"/>
+      <c r="G63" s="5" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="F64" s="4" t="n"/>
-      <c r="G64" s="4" t="n"/>
+      <c r="A64" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" t="n">
+        <v>64883</v>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Luftfahrtgesetz. Änderung</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr"/>
+      <c r="F64" s="5" t="inlineStr"/>
+      <c r="G64" s="5" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="F65" s="4" t="n"/>
-      <c r="G65" s="4" t="n"/>
+      <c r="A65" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" t="n">
+        <v>297761</v>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Chiarimenti giuridici e potenzialità dell'impiego dell'intelligenza artificiale nei settori della polizia e della sicurezza interna</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Il Consiglio federale è incaricato di presentare un rapporto sull’impiego dell’intelligenza artificiale (IA) nei settori della polizia, della sicurezza interna e del perseguimento penale, illustrandone il potenziale, le basi legali e i limiti costituzionali, in particolare per la protezione della vita privata. Sulla base di queste conclusioni, dovrà sottoporre al Parlamento linee guida per un utilizzo dell’IA coerente e conforme ai diritti fondamentali nei settori della polizia, della sicurezza interna e del perseguimento penale, che tenga conto della sovranità digitale della Svizzera. Il rapporto dovrà in particolare: 1. illustrare il potenziale e gli ambiti d’applicazione delle tecnologie di IA per rendere più efficace la lotta alla criminalità e contribuire alla salvaguardia della sicurezza interna; 2. analizzare il quadro giuridico esistente per l’utilizzo delle tecnologie di IA nel settore della sicurezza e identificare le eventuali lacune; 3. esporre i limiti costituzionali all’impiego delle tecnologie di IA nei settori della polizia e della sicurezza, e definire le condizioni quadro e le linee guida per l’utilizzo di queste tecnologie; 4. mostrare come i requisiti in m…</t>
+        </is>
+      </c>
+      <c r="F65" s="5" t="inlineStr"/>
+      <c r="G65" s="5" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="F66" s="4" t="n"/>
-      <c r="G66" s="4" t="n"/>
+      <c r="A66" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" t="n">
+        <v>153475</v>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Web 3.0 - Quelle place pour la Suisse dans un web décentralisé?</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Le Conseil fédéral est prié d'étudier les perspectives du Web 3.0, les opportunités économiques pour la Suisse et les possibilités d'y promouvoir nos valeurs. Le Web actuel est très centralisé. L'essor de la technologie "blockchain" pourrait remettre en cause la suprématie des GAFA et permettre une redistribution du pouvoir vers les internautes et de nouveaux acteurs. Le potentiel de la "blockchain" est tel que l'Europe et la Suisse pourraient retrouver une capacité d'influence sur Internet. Nous sommes à un moment charnière : c'est maintenant qu'il faut agir. Cette étude précisera les enjeux du Web 3.0 ; définira notre stratégie en matière de Web 3.0 et de "blockchain" (puisque la Suisse est dans le top 3 mondial); déterminera les talents nécessaires ; se demandera s'il faudrait créer des "blockchain" publiques ; évaluera ce que nous sommes prêts à faire pour protéger la sphère privée, favoriser une concurrence plus juste, répartir le pouvoir de manière plus équilibrée : trois promesses du Web 3.0.
+REASONING: La technologie "blockchain" pourrait bouleverser la structure sous-jacente d'Internet. La sécurité quasiment inviolable qu'elle apporte transformerait profondément la …</t>
+        </is>
+      </c>
+      <c r="F66" s="5" t="inlineStr"/>
+      <c r="G66" s="5" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="F67" s="4" t="n"/>
-      <c r="G67" s="4" t="n"/>
+      <c r="A67" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" t="n">
+        <v>64326</v>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Stopp der Datensammelwut in der Armee!</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Der Bundesrat wird beauftragt das Bundesgesetz über die Archivierung (BGA) so abzuändern, dass die Armee nicht mehr gegenüber dem Bundesarchiv angebotspflichtig ist.
+REASONING: Das Bundesarchiv sieht in einer Vielzahl von Daten der Armeeformationen eine wichtige Quellengrundlage für die Militär-, Sozial-, und Kulturgeschichte der Schweiz. Deshalb ist die Armee gemäss dem Bundesgesetz über die Archivierung Artikel 1 Absatz 1 litera b gegenüber dem Bundesarchiv angebotspflichtig. Dies bedeutet, dass Einheiten und Truppenkörper heikle Personendaten, welche nicht anonymisiert werden (z. Bsp. Disziplinarstrafdossiers) via das Bundesarchiv nach Ablauf einer Schutzfrist der Öffentlichkeit zugänglich machen muss. Im Falle der Überweisung der Disziplinarstrafdossiers bedeutet dies einen Verstoss gegen Artikel 205 des Militärstrafgesetzes, welches die Vernichtung der Unterlagen nach 5 Jahren vorschreibt. Angehörige der Armee können mit der Datenübermittlung an das Bundesarchiv, ohne ihr Wissen und ohne ihr ausdrückliches Einverständnis, zu Personen des öffentlichen Interesses werden. Kein Angehöriger der Armee kann deshalb kontrollieren, welche Daten an das Bundesarchiv gesendet werde…</t>
+        </is>
+      </c>
+      <c r="F67" s="5" t="inlineStr"/>
+      <c r="G67" s="5" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="F68" s="4" t="n"/>
-      <c r="G68" s="4" t="n"/>
+      <c r="A68" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" t="n">
+        <v>67184</v>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Dazit e controllo delle frontiere</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Nel quadro del Rapporto del Consiglio federale in adempimento del postulato 17.4177 del 14.12.2017, l'approccio risulta essere piuttosto teorico e poco orientato alla reale operatività quotidiana del personale che opera ai valichi ferroviari. In considerazione degli importanti cambiamenti previsti, è opportuno conoscere maggiori informazioni operative che toccano la quotidianità dei dipendenti e dei cittadini. 1. Sono previsti investimenti infrastrutturali utili alle attività di controllo, soprattutto merci, in tutte le stazioni di confine (Basilea, Buchs, Vallorbe, Ginevra, Domodossola, Luino, Chiasso)? Sono di competenza dell'AfD o direttamente delle FFS? Come è garantito il finanziamento e il coordinamento delle procedure? 2. Si prevede di installare scanner fissi per il traffico ferroviario merci? In quali stazioni? 3. La riforma in corso prevede un aggiornamento degli accordi internazionali vigenti per le stazioni di frontiera? Quali accordi si prevede di aggiornare con le rispettive controparti? 4. Il progetto Dazit prevede un coinvolgimento attivo - per ottimizzare i flussi di lavoro e i controlli - delle aziende ferroviarie svizzere leader nel traffico delle merci? Se…</t>
+        </is>
+      </c>
+      <c r="F68" s="5" t="inlineStr"/>
+      <c r="G68" s="5" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="F69" s="4" t="n"/>
-      <c r="G69" s="4" t="n"/>
+      <c r="A69" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" t="n">
+        <v>339430</v>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Technologies quantiques : pour une stratégie nationale d’anticipation</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>OTHER (Texte déposé): Le Conseil fédéral est chargé de présenter un rapport analysant : a) les principaux impacts prévisibles de la révolution quantique sur les grands domaines de l'action publique, ainsi que les principales mesures à envisager ; b) le positionnement stratégique de la Suisse pour saisir les opportunités et limiter les risques ; c) les conditions-cadres nécessaires pour développer, attirer et retenir en Suisse les entreprises et les talents à la pointe de ces technologies. Il formulera des propositions pour atteindre ces objectifs et posera les bases d'une stratégie nationale quantique.
+OTHER (Développement): La révolution quantique n'est plus une hypothèse de long terme. En 2026, les ordinateurs quantiques sortent des laboratoires et commencent à surpasser les systèmes classiques dans des domaines stratégiques. Leur convergence avec l'intelligence artificielle ouvre une ère de puissance de calcul sans précédent, avec des implications majeures, notamment pour la sécurité, la santé, la finance, la formation et la souveraineté numérique. La Suisse a eu la sagesse d'anticiper ces ruptures. La Swiss Quantum Initiative, dotée de 82,1 millions de francs pour la période F…</t>
+        </is>
+      </c>
+      <c r="F69" s="5" t="inlineStr"/>
+      <c r="G69" s="5" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="F70" s="4" t="n"/>
-      <c r="G70" s="4" t="n"/>
+      <c r="A70" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" t="n">
+        <v>339887</v>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Datencenter und Energiespeicher in militärischen Bunkern und Kavernen ermöglichen!</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Der Bundesrat wird beauftragt, die notwendigen gesetzlichen und organisatorischen Voraussetzungen zu schaffen, damit geeignete, militärisch nicht oder nur teilweise genutzte Bunker, Kavernen und andere geschützte Untertageanlagen für sicherheitsrelevante zivile und kommerzielle Zwecke genutzt werden können. Insbesondere sollen folgende Nutzungen ermöglicht werden: – geschützte Rechen- und Datencenter – Batterie- und Energiespeicher – kritische Kommunikations- und Versorgungsinfrastrukturen; – weitere Nutzungen, welche gleichzeitig die Resilienz und Versorgungssicherheit der Schweiz stärken. Die militärischen und sicherheitspolitischen Interessen haben jederzeit Vorrang. Strategisch wichtige Anlagen sollen im Eigentum des Bundes verbleiben und bei Bedarf wieder vollständig für militärische Zwecke zur Verfügung stehen. Dazu sind geeignete Vermietungs-, Nutzungs- und Zusammenarbeitsmodelle mit öffentlichen und privaten Partnern zu schaffen sowie bestehende rechtliche Hindernisse für eine solche Doppelnutzung soweit möglich zu beseitigen.
+REASONING: Die Armee verfügt über zahlreiche Bunker, Kavernen und andere hochwertige geschützte Untertageanlagen. Ein Teil davon wird heute ni…</t>
+        </is>
+      </c>
+      <c r="F70" s="5" t="inlineStr"/>
+      <c r="G70" s="5" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="F71" s="4" t="n"/>
-      <c r="G71" s="4" t="n"/>
+      <c r="A71" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" t="n">
+        <v>70317</v>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>Doppelbesteuerung. Abkommen mit Serbien</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr"/>
+      <c r="F71" s="5" t="inlineStr"/>
+      <c r="G71" s="5" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="F72" s="4" t="n"/>
-      <c r="G72" s="4" t="n"/>
+      <c r="A72" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" t="n">
+        <v>154501</v>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Come incoraggiare lo spirito pionieristico svizzero?</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Le buone condizioni quadro per la ricerca presto non saranno più sufficienti a garantire alla Svizzera il suo posto di leader mondiale nel campo dell'innovazione, dei brevetti e delle blockchain. I nuovi giganti del digitale stanno nascendo altrove. In 18 mesi, l'utile della piattaforma cinese blockchain Binance è passato da zero a un miliardo di fanchi e l'impresa sta sviluppando un intero ecosistema a tempo di record: Binance Labs, Binance Info, Binance Chian, Binance Uganda ecc. Quella delle blockchain è una "tecnologia di frontiera" che permette di superare i limiti conosciuti della tecnologia. La padronanza tecnologica non basta più per essere concorrenziale in questo settore: è necessario sviluppare in Svizzera uno spirito pionieristico paragonabile a quello della Silicon Valley. Qual è la posizione del Consiglio federale al riguardo?
+REASONING: La Svizzera sostiene attivamente l'innovazione con l'agenzia Innosuisse, i suoi cinque parchi dell'innovazione, gli intensi scambi tra economia e formazione superiore, il dinamismo delle sue università e numerose start-up. Ma il nostro deve diventare un vero Paese delle opportunità. Trovare un finanziamento per un prototipo è r…</t>
+        </is>
+      </c>
+      <c r="F72" s="5" t="inlineStr"/>
+      <c r="G72" s="5" t="inlineStr"/>
     </row>
     <row r="73">
-      <c r="F73" s="4" t="n"/>
-      <c r="G73" s="4" t="n"/>
+      <c r="A73" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" t="n">
+        <v>156405</v>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>Misure per potenziare l'agricoltura alpestre e di montagna</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Il Consiglio federale è incaricato di valutare quali misure possono essere adottate nell'ambito della politica agricola al fine di potenziare l'agricoltura alpestre e di montagna in seguito all'affossamento della revisione della legge sulla caccia
+REASONING: La popolazione di lupi in rapida crescita nelle aree di montagna aumenta ulteriormente la pressione sull'agricoltura e sull'economia alpestre nonché sul turismo alpino. La situazione è già oggi talmente precaria che alcuni alpi non vengono più caricati o viene anticipata la discesa dall'alpe. Il rigetto della revisione della legge sulla caccia in occasione della votazione popolare di settembre 2020 ha inasprito ulteriormente la situazione. È elevato il rischio che venga abbandonata la gestione di numerose aziende dedite all'agricoltura di montagna. Senza contromisure incombe la minaccia di un'accelerazione dell'esodo e dell'abbandono di intere vallate. Inoltre, sono da attendersi sempre più conflitti con le attività turistiche, da un lato a causa delle misure per la protezione delle greggi, dall'altro perché i bovini dopo gli attacchi dei lupi diventano paurosi e aggressivi. Entrambe le situazioni causano già grandi prob…</t>
+        </is>
+      </c>
+      <c r="F73" s="5" t="inlineStr"/>
+      <c r="G73" s="5" t="inlineStr"/>
     </row>
     <row r="74">
-      <c r="F74" s="4" t="n"/>
-      <c r="G74" s="4" t="n"/>
+      <c r="A74" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" t="n">
+        <v>155864</v>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>Modification de la loi sur l'assurance-chômage</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Le Conseil fédéral est chargé de revoir certaines dispositions de la loi sur l'assurance chômage, en particulier l'art. 31, al. 3, let. b, afin que dans une PME familiale le conjoint de l'employeur, occupé dans l'entreprise de celui-ci, puisse bénéficier d'une indemnité plafonnée en cas de réduction de l'horaire de travail (RHT) consécutive à des circonstances non imputables à l'employeur (cas de rigueur selon l'art. 32, al. 3). Une minorité de la commission (Aeschi Thomas, Amaudruz, de Courten, Dobler, Glarner, Herzog Verena, Riniker, Rösti, Sauter, Schläpfer) propose de rejeter la motion.
+REASONING: La crise Covid-19 a démontré la précarité des petites entreprises familiales, notamment celles où le conjoint est exclu du droit à l'indemnité en cas de réduction de l'horaire de travail (RHT), au même titre qu'une personne exerçant une influence sur l'entreprise (art. 31 ch. 3 al b et c). L'ordonnance 2 Covid-19 a corrigé pour la durée de la crise cette lacune de la loi sur l'assurance chômage en octroyant à ces personnes des mesures RHT. Il s'agit de prolonger cette mesure par une modification de la loi afin que le Conseil fédéral n'ait pas à édicter de nouvelles règles pour …</t>
+        </is>
+      </c>
+      <c r="F74" s="5" t="inlineStr"/>
+      <c r="G74" s="5" t="inlineStr"/>
     </row>
     <row r="75">
-      <c r="F75" s="4" t="n"/>
-      <c r="G75" s="4" t="n"/>
+      <c r="A75" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" t="n">
+        <v>214904</v>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>Abbau von Handelshemmnissen beim Import von Gebrauchtwagen</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Der Bundesrat wird beauftragt, auf Verordnungsstufe rechtliche Grundlagen für den weltweiten Import von Gebrauchtwagen zu schaffen. Heute können insbesondere amerikanische Fahrzeuge, die als Gebrauchtwagen in die Schweiz importiert werden, in der Schweiz nicht zugelassen werden, weil das Datum der 1. Inverkehrsetzung (1. Inv.) in den amerikanischen Fahrzeugpapieren nicht immer vermerkt ist. Nordamerika registriert primär den Modelljahrgang eines Personenwagens oder eines Nutzfahrzeuges. Dennoch verlangen die Schweizer Behörden von der amerikanischen Verkehrsbehörde einen Nachweis über die 1. Inv., was in der Praxis nahezu unmöglich ist. Der Handel mit Gebrauchtwagen ist aufgrund dieses Handelshemmnisses praktisch inexistent, was der Volkswirtschaft schadet. Die Motion bezweckt nur den Abbau einer bürokratischen Formalität, Lärm-, Abgas- und Sicherheitsvorschriften sind davon nicht betroffen.
+REASONING: Amerikanische Fahrzeuge erhalten bei der 1. Inv. in den USA als Zulassungsdokument ein sogenanntes "Certificate of Title", welches vom National Motor Vehicle Title Informations System (NMVTIS) ausgestellt wird. In diesem offiziellen Dokument wird ausschliesslich das Modell-Jah…</t>
+        </is>
+      </c>
+      <c r="F75" s="5" t="inlineStr"/>
+      <c r="G75" s="5" t="inlineStr"/>
     </row>
     <row r="76">
-      <c r="F76" s="4" t="n"/>
-      <c r="G76" s="4" t="n"/>
+      <c r="A76" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" t="n">
+        <v>155776</v>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>Covid-19. Eine Grundlage, um in der Bundesverwaltung die Verbreitung von Homeoffice zu beschleunigen?</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Der Umgang mit der Covid-19-Notlage hat allen Gesellschaftsschichten grosse Anpassungen abverlangt. Sehr deutlich zeigte sich dies bei der weit verbreiteten Nutzung des Homeoffice. Auch zahlreiche Bundesangestellte arbeiten zurzeit im Homeoffice. Diesbezüglich stellen die gegenwärtigen Umstände einen wichtigen Test dar, aus dem für die Zukunft Erfahrungen gesammelt werden können und der dazu genutzt werden kann, die Verbreitung des Homeoffice zu beschleunigen. Wie in anderen Bereichen könnte die Einführung von erleichterten Bedingungen für das Homeoffice auch in der Bundesverwaltung positive Auswirkungen auf verschiedene Bereiche haben, z. B. den Verkehr (weniger überfüllte öffentliche Verkehrsmittel und weniger Stau auf den Strassen), die Lebensqualität der Angestellten (bessere Vereinbarkeit von Berufs- und Familienleben, weniger Stress) und die Arbeitsleistung (grössere Flexibilität und Produktivität, geringeres Risiko eines Burnout). Weiter könnten solche Massnahme sich auch positiv auf die Bundesfinanzen auswirken dank einer effizienteren Verwaltung der gemieteten Räumlichkeiten und einem gezielteren Ressourceneinsatz. Unterstrichen werden muss zudem, dass eine flexibler…</t>
+        </is>
+      </c>
+      <c r="F76" s="5" t="inlineStr"/>
+      <c r="G76" s="5" t="inlineStr"/>
     </row>
     <row r="77">
-      <c r="F77" s="4" t="n"/>
-      <c r="G77" s="4" t="n"/>
+      <c r="A77" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" t="n">
+        <v>215214</v>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>TVA. État des lieux de la nouvelle imposition des plateformes numériques</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Depuis le 1er janvier 2025, les plateformes numériques sont assujetties à la TVA en Suisse. Comment le nombre d’inscriptions à la TVA et de taxations fiscales a-t-il évolué depuis l’instauration des nouvelles règles ? Comment l’augmentation des inscriptions à la TVA se répartit-elle entre les entreprises nationales et les entreprises étrangères ? Quelles mesures l’AFC prend-elle cette année pour s’assurer que toutes les entreprises disposant d’un IDE remplissent bel et bien leurs obligations en matière de TVA ?
+ANSWER: Questions 1 et 2 : les inscriptions à la TVA en tant que plateforme au sens de l’art. 20a, al. 1 de la loi fédérale du 12 juin 2009 sur la taxe sur la valeur ajoutée (LTVA ; RS 641.20) se répartissent à mi-mars entre vingt plateformes sises à l’étranger et quatre plateformes sises sur le territoire suisse. Toutefois, ces chiffres doivent être interprétés avec prudence pour les raisons suivantes : l’inscription en ligne en tant que plateforme pour les nouveaux assujettis n’est disponible que depuis novembre 2024 pour les plateformes étrangères et mars 2025 pour celles situées sur le territoire suisse ; par ailleurs, certaines entreprises ont pu omettre de décla…</t>
+        </is>
+      </c>
+      <c r="F77" s="5" t="inlineStr"/>
+      <c r="G77" s="5" t="inlineStr"/>
     </row>
     <row r="78">
-      <c r="F78" s="4" t="n"/>
-      <c r="G78" s="4" t="n"/>
+      <c r="A78" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" t="n">
+        <v>280488</v>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>Combler les lacunes en matière de capacité de défense</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Le Conseil fédéral est chargé de montrer sans attendre au Parlement comment l’armée peut – compte tenu de la dégradation croissante de la situation sécuritaire en Europe – combler le plus rapidement possible les plus grandes lacunes en matière de capacité de défense et quels sont les moyens financiers nécessaires à cet effet. Une minorité de la commission (Roth Franziska, Zopfi) propose de rejeter la motion.
+ANSWER: Compte tenu de la détérioration de la situation en matière de politique de sécurité, le Conseil fédéral a décidé, le 28 janvier 2026, de renforcer de manière substantielle la sécurité et la défense de la Suisse. Les moyens supplémentaires nécessaires, d’un montant d’environ 31 milliards de francs, doivent être couverts par une augmentation temporaire et affectée de la taxe sur la valeur ajoutée de 0,8 point de pourcentage à partir de 2028, pour une durée de dix ans. Ces recettes supplémentaires seront versées dans un fonds pour l’armement ayant une capacité d’endettement, qui doit permettre de couvrir de manière flexible les concentrations de paiements et le versement rapide des acomptes nécessaires dans le cadre des acquisitions d’armement. Afin de combler plus …</t>
+        </is>
+      </c>
+      <c r="F78" s="5" t="inlineStr"/>
+      <c r="G78" s="5" t="inlineStr"/>
     </row>
     <row r="79">
-      <c r="F79" s="4" t="n"/>
-      <c r="G79" s="4" t="n"/>
+      <c r="A79" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" t="n">
+        <v>161136</v>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>EU-Richtlinie über Plattformarbeit. Will sich die Schweiz daran orientieren?</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Kürzlich hat die EU eine Richtlinie über die Plattformarbeit angenommen. Diese Richtlinie ist ein wichtiger Fortschritt für Arbeitnehmerinnen und Arbeitnehmer, die in der Plattformwirtschaft tätig sind. Damit werden zwei wichtige Prinzipien eingeführt: 1. Plattformunternehmen gelten automatisch als Arbeitgeber. 2. Bei der Verwendung von Algorithmen in der Arbeitsplanung wird mehr Transparenz verlangt. Aufgrund der Annahme der EU-Richtlinie über Plattformarbeit bitten wir den Bundesrat, die folgenden Fragen zu beantworten: Welche Anpassungen wären nötig und wie könnte die Beweislastumkehr gesetzlich verankert werden? Gibt es Überlegungen in diese Richtung? Welche Massnahmen haben Bund und Kantone ergriffen, um Gerichtsurteile durchzusetzen, die Plattformen wie Uber oder Uber Eats als Arbeitgeber qualifizieren, um diese Unternehmen dem Arbeitsgesetz zu unterstellen und um sicherzustellen, dass Uber oder Uber Eats den Verpflichtungen als Arbeitgeber nachkommt? Wie viel Aufwand haben die Sozialversicherungen bisher betrieben, um die neuen Verträge der Plattformen, die eine selbstständige Tätigkeit vorsehen, zu bearbeiten und gerichtlich vorzugehen? Wie beurteilt der Bund die Rich…</t>
+        </is>
+      </c>
+      <c r="F79" s="5" t="inlineStr"/>
+      <c r="G79" s="5" t="inlineStr"/>
     </row>
     <row r="80">
-      <c r="F80" s="4" t="n"/>
-      <c r="G80" s="4" t="n"/>
+      <c r="A80" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" t="n">
+        <v>253526</v>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>Unabhängigere Regulierungskostenschätzung</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Der Bundesrat wird beauftragt, das Bundesgesetz über die Entlastung der Unternehmen von Regulierungskosten (Unternehmensentlastungsgesetz, UEG) zu ändern, sodass die Federführung bei den nach Artikel 5 UEG sowie nach Artikel 111 Absatz 4 des Bundesgesetzes über die Bundesversammlung zu erstellenden Regulierungskostenschätzungen künftig beim Eidgenössischen Departement für Wirtschaft, Bildung und Forschung liegt.
+REASONING: Gemäss Artikel 5 Absatz 1 UEG schätzen die verantwortlichen Einheiten der Bundesverwaltung bei der Ausarbeitung von rechtsetzenden Erlassen des Bundes die einmaligen und wiederkehrenden Kosten, die den Unternehmen als Folge der Auferlegung von Handlungs-, Duldungs- oder Unterlassungspflichten entstehen. Das Eidgenössische Departement für Wirtschaft, Bildung und Forschung WBF stellt dazu die methodischen Grundlagen zur Verfügung. In der Praxis zeigt sich aber folgendes Problem: Die Regulierungskosten werden in den Verlautbarungen der für den jeweiligen Erlass zuständigen Verwaltungseinheit oft kleingeredet. Das Beispiel der vom Bundesamt für Lebensmittelsicherheit und Veterinärwesen (BLV) in Auftrag gegebenen Regulierungsfolgenabschätzung (RFA) zu einer Wer…</t>
+        </is>
+      </c>
+      <c r="F80" s="5" t="inlineStr"/>
+      <c r="G80" s="5" t="inlineStr"/>
     </row>
     <row r="81">
-      <c r="F81" s="4" t="n"/>
-      <c r="G81" s="4" t="n"/>
+      <c r="A81" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" t="n">
+        <v>213749</v>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>Explosion des coûts de la santé. A quand des mesures efficaces contre le gaspillage de l'argent des primes et pour freiner la hausse des coûts?</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Comme chaque année à cette même période, le jeu des caisses-maladie bat son plein. Les assureurs font parvenir de la publicité aux ménages par les canaux les plus divers : certaines caisses-maladie proposent des rabais et d'autres promettent des baisses de primes pour l'année prochaine, alors que l'association des assureurs-maladie Santésuisse a annoncé cet été une hausse générale des primes de l'ordre de 3 %. 1. Tout laisse à penser dans ce contexte que, comme lors des précédentes années électorales, les caisses-maladie puisent plus profondément dans leurs réserves qu'à l'ordinaire pour réduire au maximum la hausse des primes. Que pense l'Office fédéral de la santé publique de ce soupçon en sa qualité d'autorité d'approbation des primes ? Des réserves ont-elles dû ou devraient-elles être réduites pour obtenir des primes plus basses ? 2. La numérisation doit profiter au système de santé : elle améliore l'efficacité et la qualité des soins ainsi que l'information des assurés et des patients. Il y a un an, le Conseil fédéral a proposé le rejet d'une intervention qui visait à créer une base légale garantissant que la documentation médicale du patient soit tenue de manière struct…</t>
+        </is>
+      </c>
+      <c r="F81" s="5" t="inlineStr"/>
+      <c r="G81" s="5" t="inlineStr"/>
     </row>
     <row r="82">
-      <c r="F82" s="4" t="n"/>
-      <c r="G82" s="4" t="n"/>
+      <c r="A82" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" t="n">
+        <v>154878</v>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>Ist die Zukunft einer vielfältigen und qualitativ hochstehenden Kulturberichterstattung gefährdet?</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Sowohl das Informations- und Kommunikationsverhalten der Bevölkerung als auch die Medienlandschaft wandeln sich stark und rasch. Dies wirkt sich insbesondere auch auf die mediale Kulturberichterstattung aus. Es gibt immer weniger selbstständige Kulturredaktionen, sowohl in den Printmedien wie in den elektronischen Medien nimmt der Raum, der der Kultur zur Verfügung steht, ab. Mediale Kulturinformation konzentriert sich zunehmend entweder auf Grossereignisse wie Premieren auf grossen Bühnen oder Neuerscheinungen prominenter Autorinnen und Autoren oder auf kulturelle Anlässe von lokaler oder regionaler Bedeutung. So verliert die Schweiz an Vielfalt der Themen und der kritischen Stimmen und an überregionalen Kulturinformationen insbesondere über die Sprachregionen hinaus. So verliert immer mehr wertvolles Kulturschaffen an Aufmerksamkeit. Denn das Kulturschaffen ist auf eine kompetente, rege und vielfältige öffentliche Kulturkritik angewiesen. Sie ist es auch, die in der Bevölkerung das Interesse am kulturellen Schaffen und Darbieten des ganzen Landes weckt und wachhält. Wenn Kultur gefördert wird, ist es auch im Interesse der Förderung, dass sie auch Beachtung findet. In diesem…</t>
+        </is>
+      </c>
+      <c r="F82" s="5" t="inlineStr"/>
+      <c r="G82" s="5" t="inlineStr"/>
     </row>
     <row r="83">
-      <c r="F83" s="4" t="n"/>
-      <c r="G83" s="4" t="n"/>
+      <c r="A83" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" t="n">
+        <v>153461</v>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>Jeux vidéo. Prévenir les abus des microtransactions apparentées aux jeux d'argent</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Le Conseil fédéral est chargé de proposer un système pour réguler l'emploi des microtransactions avec de l'argent réel dans les jeux vidéos, quelle que soit la plateforme. En particulier, le Conseil fédéral est chargé de déterminer quels types de microtransactions sont apparentées à des jeux d'argent et doivent être régulées comme telles, et de garantir la protection des joueurs, en particulier mineurs. Les pratiques posant le plus de problèmes et devant faire appel à régulation sont : 1. les microtransactions avec de l'argent réel donnant un avantage aux joueurs, mais où la récompense est aléatoire ; 2. les systèmes de microtransactions particulièrement conçus pour générer de l'addiction chez les joueurs ; 3. les microtransactions ciblant en particulier les mineurs.
+REASONING: De nombreux jeux vidéos pour appareils mobiles, consoles de jeux ou sur PC comportent, parfois au delà d'un prix d'achat élevé, un système de microtransaction. Dans des modèles "free to play", ce système peut être le seul moyen de rentabiliser le jeu, mais dans d'autres cas, il s'agit de sources de recettes supplémentaires. Ces microtransactions permettent aux joueurs qui dépensent de l'argent réel, d…</t>
+        </is>
+      </c>
+      <c r="F83" s="5" t="inlineStr"/>
+      <c r="G83" s="5" t="inlineStr"/>
     </row>
     <row r="84">
-      <c r="F84" s="4" t="n"/>
-      <c r="G84" s="4" t="n"/>
+      <c r="F84" s="5" t="n"/>
+      <c r="G84" s="5" t="n"/>
     </row>
     <row r="85">
-      <c r="F85" s="4" t="n"/>
-      <c r="G85" s="4" t="n"/>
+      <c r="F85" s="5" t="n"/>
+      <c r="G85" s="5" t="n"/>
     </row>
     <row r="86">
-      <c r="F86" s="4" t="n"/>
-      <c r="G86" s="4" t="n"/>
+      <c r="F86" s="5" t="n"/>
+      <c r="G86" s="5" t="n"/>
     </row>
     <row r="87">
-      <c r="F87" s="4" t="n"/>
-      <c r="G87" s="4" t="n"/>
+      <c r="F87" s="5" t="n"/>
+      <c r="G87" s="5" t="n"/>
     </row>
     <row r="88">
-      <c r="F88" s="4" t="n"/>
-      <c r="G88" s="4" t="n"/>
+      <c r="F88" s="5" t="n"/>
+      <c r="G88" s="5" t="n"/>
     </row>
     <row r="89">
-      <c r="F89" s="4" t="n"/>
-      <c r="G89" s="4" t="n"/>
+      <c r="F89" s="5" t="n"/>
+      <c r="G89" s="5" t="n"/>
     </row>
     <row r="90">
-      <c r="F90" s="4" t="n"/>
-      <c r="G90" s="4" t="n"/>
+      <c r="F90" s="5" t="n"/>
+      <c r="G90" s="5" t="n"/>
     </row>
     <row r="91">
-      <c r="F91" s="4" t="n"/>
-      <c r="G91" s="4" t="n"/>
+      <c r="F91" s="5" t="n"/>
+      <c r="G91" s="5" t="n"/>
     </row>
     <row r="92">
-      <c r="F92" s="4" t="n"/>
-      <c r="G92" s="4" t="n"/>
+      <c r="F92" s="5" t="n"/>
+      <c r="G92" s="5" t="n"/>
     </row>
     <row r="93">
-      <c r="F93" s="4" t="n"/>
-      <c r="G93" s="4" t="n"/>
+      <c r="F93" s="5" t="n"/>
+      <c r="G93" s="5" t="n"/>
     </row>
     <row r="94">
-      <c r="F94" s="4" t="n"/>
-      <c r="G94" s="4" t="n"/>
+      <c r="F94" s="5" t="n"/>
+      <c r="G94" s="5" t="n"/>
     </row>
     <row r="95">
-      <c r="F95" s="4" t="n"/>
-      <c r="G95" s="4" t="n"/>
+      <c r="F95" s="5" t="n"/>
+      <c r="G95" s="5" t="n"/>
     </row>
     <row r="96">
-      <c r="F96" s="4" t="n"/>
-      <c r="G96" s="4" t="n"/>
+      <c r="F96" s="5" t="n"/>
+      <c r="G96" s="5" t="n"/>
     </row>
     <row r="97">
-      <c r="F97" s="4" t="n"/>
-      <c r="G97" s="4" t="n"/>
+      <c r="F97" s="5" t="n"/>
+      <c r="G97" s="5" t="n"/>
     </row>
     <row r="98">
-      <c r="F98" s="4" t="n"/>
-      <c r="G98" s="4" t="n"/>
+      <c r="F98" s="5" t="n"/>
+      <c r="G98" s="5" t="n"/>
     </row>
     <row r="99">
-      <c r="F99" s="4" t="n"/>
-      <c r="G99" s="4" t="n"/>
+      <c r="F99" s="5" t="n"/>
+      <c r="G99" s="5" t="n"/>
     </row>
     <row r="100">
-      <c r="F100" s="4" t="n"/>
-      <c r="G100" s="4" t="n"/>
+      <c r="F100" s="5" t="n"/>
+      <c r="G100" s="5" t="n"/>
     </row>
     <row r="101">
-      <c r="F101" s="4" t="n"/>
-      <c r="G101" s="4" t="n"/>
+      <c r="F101" s="5" t="n"/>
+      <c r="G101" s="5" t="n"/>
     </row>
     <row r="102">
-      <c r="F102" s="4" t="n"/>
-      <c r="G102" s="4" t="n"/>
+      <c r="F102" s="5" t="n"/>
+      <c r="G102" s="5" t="n"/>
     </row>
     <row r="103">
-      <c r="F103" s="4" t="n"/>
-      <c r="G103" s="4" t="n"/>
+      <c r="F103" s="5" t="n"/>
+      <c r="G103" s="5" t="n"/>
     </row>
     <row r="104">
-      <c r="F104" s="4" t="n"/>
-      <c r="G104" s="4" t="n"/>
+      <c r="F104" s="5" t="n"/>
+      <c r="G104" s="5" t="n"/>
     </row>
     <row r="105">
-      <c r="F105" s="4" t="n"/>
-      <c r="G105" s="4" t="n"/>
+      <c r="F105" s="5" t="n"/>
+      <c r="G105" s="5" t="n"/>
     </row>
     <row r="106">
-      <c r="F106" s="4" t="n"/>
-      <c r="G106" s="4" t="n"/>
+      <c r="F106" s="5" t="n"/>
+      <c r="G106" s="5" t="n"/>
     </row>
     <row r="107">
-      <c r="F107" s="4" t="n"/>
-      <c r="G107" s="4" t="n"/>
+      <c r="F107" s="5" t="n"/>
+      <c r="G107" s="5" t="n"/>
     </row>
     <row r="108">
-      <c r="F108" s="4" t="n"/>
-      <c r="G108" s="4" t="n"/>
+      <c r="F108" s="5" t="n"/>
+      <c r="G108" s="5" t="n"/>
     </row>
     <row r="109">
-      <c r="F109" s="4" t="n"/>
-      <c r="G109" s="4" t="n"/>
+      <c r="F109" s="5" t="n"/>
+      <c r="G109" s="5" t="n"/>
     </row>
     <row r="110">
-      <c r="F110" s="4" t="n"/>
-      <c r="G110" s="4" t="n"/>
+      <c r="F110" s="5" t="n"/>
+      <c r="G110" s="5" t="n"/>
     </row>
     <row r="111">
-      <c r="F111" s="4" t="n"/>
-      <c r="G111" s="4" t="n"/>
+      <c r="F111" s="5" t="n"/>
+      <c r="G111" s="5" t="n"/>
     </row>
     <row r="112">
-      <c r="F112" s="4" t="n"/>
-      <c r="G112" s="4" t="n"/>
+      <c r="F112" s="5" t="n"/>
+      <c r="G112" s="5" t="n"/>
     </row>
     <row r="113">
-      <c r="F113" s="4" t="n"/>
-      <c r="G113" s="4" t="n"/>
+      <c r="F113" s="5" t="n"/>
+      <c r="G113" s="5" t="n"/>
     </row>
     <row r="114">
-      <c r="F114" s="4" t="n"/>
-      <c r="G114" s="4" t="n"/>
+      <c r="F114" s="5" t="n"/>
+      <c r="G114" s="5" t="n"/>
     </row>
     <row r="115">
-      <c r="F115" s="4" t="n"/>
-      <c r="G115" s="4" t="n"/>
+      <c r="F115" s="5" t="n"/>
+      <c r="G115" s="5" t="n"/>
     </row>
     <row r="116">
-      <c r="F116" s="4" t="n"/>
-      <c r="G116" s="4" t="n"/>
+      <c r="F116" s="5" t="n"/>
+      <c r="G116" s="5" t="n"/>
     </row>
     <row r="117">
-      <c r="F117" s="4" t="n"/>
-      <c r="G117" s="4" t="n"/>
+      <c r="F117" s="5" t="n"/>
+      <c r="G117" s="5" t="n"/>
     </row>
     <row r="118">
-      <c r="F118" s="4" t="n"/>
-      <c r="G118" s="4" t="n"/>
+      <c r="F118" s="5" t="n"/>
+      <c r="G118" s="5" t="n"/>
     </row>
     <row r="119">
-      <c r="F119" s="4" t="n"/>
-      <c r="G119" s="4" t="n"/>
+      <c r="F119" s="5" t="n"/>
+      <c r="G119" s="5" t="n"/>
     </row>
     <row r="120">
-      <c r="F120" s="4" t="n"/>
-      <c r="G120" s="4" t="n"/>
+      <c r="F120" s="5" t="n"/>
+      <c r="G120" s="5" t="n"/>
     </row>
     <row r="121">
-      <c r="F121" s="4" t="n"/>
-      <c r="G121" s="4" t="n"/>
+      <c r="F121" s="5" t="n"/>
+      <c r="G121" s="5" t="n"/>
     </row>
     <row r="122">
-      <c r="F122" s="4" t="n"/>
-      <c r="G122" s="4" t="n"/>
+      <c r="F122" s="5" t="n"/>
+      <c r="G122" s="5" t="n"/>
     </row>
     <row r="123">
-      <c r="F123" s="4" t="n"/>
-      <c r="G123" s="4" t="n"/>
+      <c r="F123" s="5" t="n"/>
+      <c r="G123" s="5" t="n"/>
     </row>
     <row r="124">
-      <c r="F124" s="4" t="n"/>
-      <c r="G124" s="4" t="n"/>
+      <c r="F124" s="5" t="n"/>
+      <c r="G124" s="5" t="n"/>
     </row>
     <row r="125">
-      <c r="F125" s="4" t="n"/>
-      <c r="G125" s="4" t="n"/>
+      <c r="F125" s="5" t="n"/>
+      <c r="G125" s="5" t="n"/>
     </row>
     <row r="126">
-      <c r="F126" s="4" t="n"/>
-      <c r="G126" s="4" t="n"/>
+      <c r="F126" s="5" t="n"/>
+      <c r="G126" s="5" t="n"/>
     </row>
     <row r="127">
-      <c r="F127" s="4" t="n"/>
-      <c r="G127" s="4" t="n"/>
+      <c r="F127" s="5" t="n"/>
+      <c r="G127" s="5" t="n"/>
     </row>
     <row r="128">
-      <c r="F128" s="4" t="n"/>
-      <c r="G128" s="4" t="n"/>
+      <c r="F128" s="5" t="n"/>
+      <c r="G128" s="5" t="n"/>
     </row>
     <row r="129">
-      <c r="F129" s="4" t="n"/>
-      <c r="G129" s="4" t="n"/>
+      <c r="F129" s="5" t="n"/>
+      <c r="G129" s="5" t="n"/>
     </row>
     <row r="130">
-      <c r="F130" s="4" t="n"/>
-      <c r="G130" s="4" t="n"/>
+      <c r="F130" s="5" t="n"/>
+      <c r="G130" s="5" t="n"/>
     </row>
     <row r="131">
-      <c r="F131" s="4" t="n"/>
-      <c r="G131" s="4" t="n"/>
+      <c r="F131" s="5" t="n"/>
+      <c r="G131" s="5" t="n"/>
     </row>
     <row r="132">
-      <c r="F132" s="4" t="n"/>
-      <c r="G132" s="4" t="n"/>
+      <c r="F132" s="5" t="n"/>
+      <c r="G132" s="5" t="n"/>
     </row>
     <row r="133">
-      <c r="F133" s="4" t="n"/>
-      <c r="G133" s="4" t="n"/>
+      <c r="F133" s="5" t="n"/>
+      <c r="G133" s="5" t="n"/>
     </row>
     <row r="134">
-      <c r="F134" s="4" t="n"/>
-      <c r="G134" s="4" t="n"/>
+      <c r="F134" s="5" t="n"/>
+      <c r="G134" s="5" t="n"/>
     </row>
     <row r="135">
-      <c r="F135" s="4" t="n"/>
-      <c r="G135" s="4" t="n"/>
+      <c r="F135" s="5" t="n"/>
+      <c r="G135" s="5" t="n"/>
     </row>
     <row r="136">
-      <c r="F136" s="4" t="n"/>
-      <c r="G136" s="4" t="n"/>
+      <c r="F136" s="5" t="n"/>
+      <c r="G136" s="5" t="n"/>
     </row>
     <row r="137">
-      <c r="F137" s="4" t="n"/>
-      <c r="G137" s="4" t="n"/>
+      <c r="F137" s="5" t="n"/>
+      <c r="G137" s="5" t="n"/>
     </row>
     <row r="138">
-      <c r="F138" s="4" t="n"/>
-      <c r="G138" s="4" t="n"/>
+      <c r="F138" s="5" t="n"/>
+      <c r="G138" s="5" t="n"/>
     </row>
     <row r="139">
-      <c r="F139" s="4" t="n"/>
-      <c r="G139" s="4" t="n"/>
+      <c r="F139" s="5" t="n"/>
+      <c r="G139" s="5" t="n"/>
     </row>
     <row r="140">
-      <c r="F140" s="4" t="n"/>
-      <c r="G140" s="4" t="n"/>
+      <c r="F140" s="5" t="n"/>
+      <c r="G140" s="5" t="n"/>
     </row>
     <row r="141">
-      <c r="F141" s="4" t="n"/>
-      <c r="G141" s="4" t="n"/>
+      <c r="F141" s="5" t="n"/>
+      <c r="G141" s="5" t="n"/>
     </row>
     <row r="142">
-      <c r="F142" s="4" t="n"/>
-      <c r="G142" s="4" t="n"/>
+      <c r="F142" s="5" t="n"/>
+      <c r="G142" s="5" t="n"/>
     </row>
     <row r="143">
-      <c r="F143" s="4" t="n"/>
-      <c r="G143" s="4" t="n"/>
+      <c r="F143" s="5" t="n"/>
+      <c r="G143" s="5" t="n"/>
     </row>
     <row r="144">
-      <c r="F144" s="4" t="n"/>
-      <c r="G144" s="4" t="n"/>
+      <c r="F144" s="5" t="n"/>
+      <c r="G144" s="5" t="n"/>
     </row>
     <row r="145">
-      <c r="F145" s="4" t="n"/>
-      <c r="G145" s="4" t="n"/>
+      <c r="F145" s="5" t="n"/>
+      <c r="G145" s="5" t="n"/>
     </row>
     <row r="146">
-      <c r="F146" s="4" t="n"/>
-      <c r="G146" s="4" t="n"/>
+      <c r="F146" s="5" t="n"/>
+      <c r="G146" s="5" t="n"/>
     </row>
     <row r="147">
-      <c r="F147" s="4" t="n"/>
-      <c r="G147" s="4" t="n"/>
+      <c r="F147" s="5" t="n"/>
+      <c r="G147" s="5" t="n"/>
     </row>
     <row r="148">
-      <c r="F148" s="4" t="n"/>
-      <c r="G148" s="4" t="n"/>
+      <c r="F148" s="5" t="n"/>
+      <c r="G148" s="5" t="n"/>
     </row>
     <row r="149">
-      <c r="F149" s="4" t="n"/>
-      <c r="G149" s="4" t="n"/>
+      <c r="F149" s="5" t="n"/>
+      <c r="G149" s="5" t="n"/>
     </row>
     <row r="150">
-      <c r="F150" s="4" t="n"/>
-      <c r="G150" s="4" t="n"/>
+      <c r="F150" s="5" t="n"/>
+      <c r="G150" s="5" t="n"/>
     </row>
     <row r="151">
-      <c r="F151" s="4" t="n"/>
-      <c r="G151" s="4" t="n"/>
+      <c r="F151" s="5" t="n"/>
+      <c r="G151" s="5" t="n"/>
     </row>
     <row r="152">
-      <c r="F152" s="4" t="n"/>
-      <c r="G152" s="4" t="n"/>
+      <c r="F152" s="5" t="n"/>
+      <c r="G152" s="5" t="n"/>
     </row>
     <row r="153">
-      <c r="F153" s="4" t="n"/>
-      <c r="G153" s="4" t="n"/>
+      <c r="F153" s="5" t="n"/>
+      <c r="G153" s="5" t="n"/>
     </row>
     <row r="154">
-      <c r="F154" s="4" t="n"/>
-      <c r="G154" s="4" t="n"/>
+      <c r="F154" s="5" t="n"/>
+      <c r="G154" s="5" t="n"/>
     </row>
     <row r="155">
-      <c r="F155" s="4" t="n"/>
-      <c r="G155" s="4" t="n"/>
+      <c r="F155" s="5" t="n"/>
+      <c r="G155" s="5" t="n"/>
     </row>
     <row r="156">
-      <c r="F156" s="4" t="n"/>
-      <c r="G156" s="4" t="n"/>
+      <c r="F156" s="5" t="n"/>
+      <c r="G156" s="5" t="n"/>
     </row>
     <row r="157">
-      <c r="F157" s="4" t="n"/>
-      <c r="G157" s="4" t="n"/>
+      <c r="F157" s="5" t="n"/>
+      <c r="G157" s="5" t="n"/>
     </row>
     <row r="158">
-      <c r="F158" s="4" t="n"/>
-      <c r="G158" s="4" t="n"/>
+      <c r="F158" s="5" t="n"/>
+      <c r="G158" s="5" t="n"/>
     </row>
     <row r="159">
-      <c r="F159" s="4" t="n"/>
-      <c r="G159" s="4" t="n"/>
+      <c r="F159" s="5" t="n"/>
+      <c r="G159" s="5" t="n"/>
     </row>
     <row r="160">
-      <c r="F160" s="4" t="n"/>
-      <c r="G160" s="4" t="n"/>
+      <c r="F160" s="5" t="n"/>
+      <c r="G160" s="5" t="n"/>
     </row>
     <row r="161">
-      <c r="F161" s="4" t="n"/>
-      <c r="G161" s="4" t="n"/>
+      <c r="F161" s="5" t="n"/>
+      <c r="G161" s="5" t="n"/>
     </row>
     <row r="162">
-      <c r="F162" s="4" t="n"/>
-      <c r="G162" s="4" t="n"/>
+      <c r="F162" s="5" t="n"/>
+      <c r="G162" s="5" t="n"/>
     </row>
     <row r="163">
-      <c r="F163" s="4" t="n"/>
-      <c r="G163" s="4" t="n"/>
+      <c r="F163" s="5" t="n"/>
+      <c r="G163" s="5" t="n"/>
     </row>
     <row r="164">
-      <c r="F164" s="4" t="n"/>
-      <c r="G164" s="4" t="n"/>
+      <c r="F164" s="5" t="n"/>
+      <c r="G164" s="5" t="n"/>
     </row>
     <row r="165">
-      <c r="F165" s="4" t="n"/>
-      <c r="G165" s="4" t="n"/>
+      <c r="F165" s="5" t="n"/>
+      <c r="G165" s="5" t="n"/>
     </row>
     <row r="166">
-      <c r="F166" s="4" t="n"/>
-      <c r="G166" s="4" t="n"/>
+      <c r="F166" s="5" t="n"/>
+      <c r="G166" s="5" t="n"/>
     </row>
     <row r="167">
-      <c r="F167" s="4" t="n"/>
-      <c r="G167" s="4" t="n"/>
+      <c r="F167" s="5" t="n"/>
+      <c r="G167" s="5" t="n"/>
     </row>
     <row r="168">
-      <c r="F168" s="4" t="n"/>
-      <c r="G168" s="4" t="n"/>
+      <c r="F168" s="5" t="n"/>
+      <c r="G168" s="5" t="n"/>
     </row>
     <row r="169">
-      <c r="F169" s="4" t="n"/>
-      <c r="G169" s="4" t="n"/>
+      <c r="F169" s="5" t="n"/>
+      <c r="G169" s="5" t="n"/>
     </row>
     <row r="170">
-      <c r="F170" s="4" t="n"/>
-      <c r="G170" s="4" t="n"/>
+      <c r="F170" s="5" t="n"/>
+      <c r="G170" s="5" t="n"/>
     </row>
     <row r="171">
-      <c r="F171" s="4" t="n"/>
-      <c r="G171" s="4" t="n"/>
+      <c r="F171" s="5" t="n"/>
+      <c r="G171" s="5" t="n"/>
     </row>
     <row r="172">
-      <c r="F172" s="4" t="n"/>
-      <c r="G172" s="4" t="n"/>
+      <c r="F172" s="5" t="n"/>
+      <c r="G172" s="5" t="n"/>
     </row>
     <row r="173">
-      <c r="F173" s="4" t="n"/>
-      <c r="G173" s="4" t="n"/>
+      <c r="F173" s="5" t="n"/>
+      <c r="G173" s="5" t="n"/>
     </row>
     <row r="174">
-      <c r="F174" s="4" t="n"/>
-      <c r="G174" s="4" t="n"/>
+      <c r="F174" s="5" t="n"/>
+      <c r="G174" s="5" t="n"/>
     </row>
     <row r="175">
-      <c r="F175" s="4" t="n"/>
-      <c r="G175" s="4" t="n"/>
+      <c r="F175" s="5" t="n"/>
+      <c r="G175" s="5" t="n"/>
     </row>
     <row r="176">
-      <c r="F176" s="4" t="n"/>
-      <c r="G176" s="4" t="n"/>
+      <c r="F176" s="5" t="n"/>
+      <c r="G176" s="5" t="n"/>
     </row>
     <row r="177">
-      <c r="F177" s="4" t="n"/>
-      <c r="G177" s="4" t="n"/>
+      <c r="F177" s="5" t="n"/>
+      <c r="G177" s="5" t="n"/>
     </row>
     <row r="178">
-      <c r="F178" s="4" t="n"/>
-      <c r="G178" s="4" t="n"/>
+      <c r="F178" s="5" t="n"/>
+      <c r="G178" s="5" t="n"/>
     </row>
     <row r="179">
-      <c r="F179" s="4" t="n"/>
-      <c r="G179" s="4" t="n"/>
+      <c r="F179" s="5" t="n"/>
+      <c r="G179" s="5" t="n"/>
     </row>
     <row r="180">
-      <c r="F180" s="4" t="n"/>
-      <c r="G180" s="4" t="n"/>
+      <c r="F180" s="5" t="n"/>
+      <c r="G180" s="5" t="n"/>
     </row>
     <row r="181">
-      <c r="F181" s="4" t="n"/>
-      <c r="G181" s="4" t="n"/>
+      <c r="F181" s="5" t="n"/>
+      <c r="G181" s="5" t="n"/>
     </row>
     <row r="182">
-      <c r="F182" s="4" t="n"/>
-      <c r="G182" s="4" t="n"/>
+      <c r="F182" s="5" t="n"/>
+      <c r="G182" s="5" t="n"/>
     </row>
     <row r="183">
-      <c r="F183" s="4" t="n"/>
-      <c r="G183" s="4" t="n"/>
+      <c r="F183" s="5" t="n"/>
+      <c r="G183" s="5" t="n"/>
     </row>
     <row r="184">
-      <c r="F184" s="4" t="n"/>
-      <c r="G184" s="4" t="n"/>
+      <c r="F184" s="5" t="n"/>
+      <c r="G184" s="5" t="n"/>
     </row>
     <row r="185">
-      <c r="F185" s="4" t="n"/>
-      <c r="G185" s="4" t="n"/>
+      <c r="F185" s="5" t="n"/>
+      <c r="G185" s="5" t="n"/>
     </row>
     <row r="186">
-      <c r="F186" s="4" t="n"/>
-      <c r="G186" s="4" t="n"/>
+      <c r="F186" s="5" t="n"/>
+      <c r="G186" s="5" t="n"/>
     </row>
     <row r="187">
-      <c r="F187" s="4" t="n"/>
-      <c r="G187" s="4" t="n"/>
+      <c r="F187" s="5" t="n"/>
+      <c r="G187" s="5" t="n"/>
     </row>
     <row r="188">
-      <c r="F188" s="4" t="n"/>
-      <c r="G188" s="4" t="n"/>
+      <c r="F188" s="5" t="n"/>
+      <c r="G188" s="5" t="n"/>
     </row>
     <row r="189">
-      <c r="F189" s="4" t="n"/>
-      <c r="G189" s="4" t="n"/>
+      <c r="F189" s="5" t="n"/>
+      <c r="G189" s="5" t="n"/>
     </row>
     <row r="190">
-      <c r="F190" s="4" t="n"/>
-      <c r="G190" s="4" t="n"/>
+      <c r="F190" s="5" t="n"/>
+      <c r="G190" s="5" t="n"/>
     </row>
     <row r="191">
-      <c r="F191" s="4" t="n"/>
-      <c r="G191" s="4" t="n"/>
+      <c r="F191" s="5" t="n"/>
+      <c r="G191" s="5" t="n"/>
     </row>
     <row r="192">
-      <c r="F192" s="4" t="n"/>
-      <c r="G192" s="4" t="n"/>
+      <c r="F192" s="5" t="n"/>
+      <c r="G192" s="5" t="n"/>
     </row>
     <row r="193">
-      <c r="F193" s="4" t="n"/>
-      <c r="G193" s="4" t="n"/>
+      <c r="F193" s="5" t="n"/>
+      <c r="G193" s="5" t="n"/>
     </row>
     <row r="194">
-      <c r="F194" s="4" t="n"/>
-      <c r="G194" s="4" t="n"/>
+      <c r="F194" s="5" t="n"/>
+      <c r="G194" s="5" t="n"/>
     </row>
     <row r="195">
-      <c r="F195" s="4" t="n"/>
-      <c r="G195" s="4" t="n"/>
+      <c r="F195" s="5" t="n"/>
+      <c r="G195" s="5" t="n"/>
     </row>
     <row r="196">
-      <c r="F196" s="4" t="n"/>
-      <c r="G196" s="4" t="n"/>
+      <c r="F196" s="5" t="n"/>
+      <c r="G196" s="5" t="n"/>
     </row>
     <row r="197">
-      <c r="F197" s="4" t="n"/>
-      <c r="G197" s="4" t="n"/>
+      <c r="F197" s="5" t="n"/>
+      <c r="G197" s="5" t="n"/>
     </row>
     <row r="198">
-      <c r="F198" s="4" t="n"/>
-      <c r="G198" s="4" t="n"/>
+      <c r="F198" s="5" t="n"/>
+      <c r="G198" s="5" t="n"/>
     </row>
     <row r="199">
-      <c r="F199" s="4" t="n"/>
-      <c r="G199" s="4" t="n"/>
+      <c r="F199" s="5" t="n"/>
+      <c r="G199" s="5" t="n"/>
     </row>
     <row r="200">
-      <c r="F200" s="4" t="n"/>
-      <c r="G200" s="4" t="n"/>
+      <c r="F200" s="5" t="n"/>
+      <c r="G200" s="5" t="n"/>
     </row>
     <row r="201">
-      <c r="F201" s="4" t="n"/>
-      <c r="G201" s="4" t="n"/>
+      <c r="F201" s="5" t="n"/>
+      <c r="G201" s="5" t="n"/>
     </row>
     <row r="202">
-      <c r="F202" s="4" t="n"/>
-      <c r="G202" s="4" t="n"/>
+      <c r="F202" s="5" t="n"/>
+      <c r="G202" s="5" t="n"/>
     </row>
     <row r="203">
-      <c r="F203" s="4" t="n"/>
-      <c r="G203" s="4" t="n"/>
+      <c r="F203" s="5" t="n"/>
+      <c r="G203" s="5" t="n"/>
     </row>
     <row r="204">
-      <c r="F204" s="4" t="n"/>
-      <c r="G204" s="4" t="n"/>
+      <c r="F204" s="5" t="n"/>
+      <c r="G204" s="5" t="n"/>
     </row>
     <row r="205">
-      <c r="F205" s="4" t="n"/>
-      <c r="G205" s="4" t="n"/>
+      <c r="F205" s="5" t="n"/>
+      <c r="G205" s="5" t="n"/>
     </row>
     <row r="206">
-      <c r="F206" s="4" t="n"/>
-      <c r="G206" s="4" t="n"/>
+      <c r="F206" s="5" t="n"/>
+      <c r="G206" s="5" t="n"/>
     </row>
     <row r="207">
-      <c r="F207" s="4" t="n"/>
-      <c r="G207" s="4" t="n"/>
+      <c r="F207" s="5" t="n"/>
+      <c r="G207" s="5" t="n"/>
     </row>
     <row r="208">
-      <c r="F208" s="4" t="n"/>
-      <c r="G208" s="4" t="n"/>
+      <c r="F208" s="5" t="n"/>
+      <c r="G208" s="5" t="n"/>
     </row>
     <row r="209">
-      <c r="F209" s="4" t="n"/>
-      <c r="G209" s="4" t="n"/>
+      <c r="F209" s="5" t="n"/>
+      <c r="G209" s="5" t="n"/>
     </row>
     <row r="210">
-      <c r="F210" s="4" t="n"/>
-      <c r="G210" s="4" t="n"/>
+      <c r="F210" s="5" t="n"/>
+      <c r="G210" s="5" t="n"/>
     </row>
     <row r="211">
-      <c r="F211" s="4" t="n"/>
-      <c r="G211" s="4" t="n"/>
+      <c r="F211" s="5" t="n"/>
+      <c r="G211" s="5" t="n"/>
     </row>
     <row r="212">
-      <c r="F212" s="4" t="n"/>
-      <c r="G212" s="4" t="n"/>
+      <c r="F212" s="5" t="n"/>
+      <c r="G212" s="5" t="n"/>
     </row>
     <row r="213">
-      <c r="F213" s="4" t="n"/>
-      <c r="G213" s="4" t="n"/>
+      <c r="F213" s="5" t="n"/>
+      <c r="G213" s="5" t="n"/>
     </row>
     <row r="214">
-      <c r="F214" s="4" t="n"/>
-      <c r="G214" s="4" t="n"/>
+      <c r="F214" s="5" t="n"/>
+      <c r="G214" s="5" t="n"/>
     </row>
     <row r="215">
-      <c r="F215" s="4" t="n"/>
-      <c r="G215" s="4" t="n"/>
+      <c r="F215" s="5" t="n"/>
+      <c r="G215" s="5" t="n"/>
     </row>
     <row r="216">
-      <c r="F216" s="4" t="n"/>
-      <c r="G216" s="4" t="n"/>
+      <c r="F216" s="5" t="n"/>
+      <c r="G216" s="5" t="n"/>
     </row>
     <row r="217">
-      <c r="F217" s="4" t="n"/>
-      <c r="G217" s="4" t="n"/>
+      <c r="F217" s="5" t="n"/>
+      <c r="G217" s="5" t="n"/>
     </row>
     <row r="218">
-      <c r="F218" s="4" t="n"/>
-      <c r="G218" s="4" t="n"/>
+      <c r="F218" s="5" t="n"/>
+      <c r="G218" s="5" t="n"/>
     </row>
     <row r="219">
-      <c r="F219" s="4" t="n"/>
-      <c r="G219" s="4" t="n"/>
+      <c r="F219" s="5" t="n"/>
+      <c r="G219" s="5" t="n"/>
     </row>
     <row r="220">
-      <c r="F220" s="4" t="n"/>
-      <c r="G220" s="4" t="n"/>
+      <c r="F220" s="5" t="n"/>
+      <c r="G220" s="5" t="n"/>
     </row>
     <row r="221">
-      <c r="F221" s="4" t="n"/>
-      <c r="G221" s="4" t="n"/>
+      <c r="F221" s="5" t="n"/>
+      <c r="G221" s="5" t="n"/>
     </row>
     <row r="222">
-      <c r="F222" s="4" t="n"/>
-      <c r="G222" s="4" t="n"/>
+      <c r="F222" s="5" t="n"/>
+      <c r="G222" s="5" t="n"/>
     </row>
     <row r="223">
-      <c r="F223" s="4" t="n"/>
-      <c r="G223" s="4" t="n"/>
+      <c r="F223" s="5" t="n"/>
+      <c r="G223" s="5" t="n"/>
     </row>
     <row r="224">
-      <c r="F224" s="4" t="n"/>
-      <c r="G224" s="4" t="n"/>
+      <c r="F224" s="5" t="n"/>
+      <c r="G224" s="5" t="n"/>
     </row>
     <row r="225">
-      <c r="F225" s="4" t="n"/>
-      <c r="G225" s="4" t="n"/>
+      <c r="F225" s="5" t="n"/>
+      <c r="G225" s="5" t="n"/>
     </row>
     <row r="226">
-      <c r="F226" s="4" t="n"/>
-      <c r="G226" s="4" t="n"/>
+      <c r="F226" s="5" t="n"/>
+      <c r="G226" s="5" t="n"/>
     </row>
     <row r="227">
-      <c r="F227" s="4" t="n"/>
-      <c r="G227" s="4" t="n"/>
+      <c r="F227" s="5" t="n"/>
+      <c r="G227" s="5" t="n"/>
     </row>
     <row r="228">
-      <c r="F228" s="4" t="n"/>
-      <c r="G228" s="4" t="n"/>
+      <c r="F228" s="5" t="n"/>
+      <c r="G228" s="5" t="n"/>
     </row>
     <row r="229">
-      <c r="F229" s="4" t="n"/>
-      <c r="G229" s="4" t="n"/>
+      <c r="F229" s="5" t="n"/>
+      <c r="G229" s="5" t="n"/>
     </row>
     <row r="230">
-      <c r="F230" s="4" t="n"/>
-      <c r="G230" s="4" t="n"/>
+      <c r="F230" s="5" t="n"/>
+      <c r="G230" s="5" t="n"/>
     </row>
     <row r="231">
-      <c r="F231" s="4" t="n"/>
-      <c r="G231" s="4" t="n"/>
+      <c r="F231" s="5" t="n"/>
+      <c r="G231" s="5" t="n"/>
     </row>
     <row r="232">
-      <c r="F232" s="4" t="n"/>
-      <c r="G232" s="4" t="n"/>
+      <c r="F232" s="5" t="n"/>
+      <c r="G232" s="5" t="n"/>
     </row>
     <row r="233">
-      <c r="F233" s="4" t="n"/>
-      <c r="G233" s="4" t="n"/>
+      <c r="F233" s="5" t="n"/>
+      <c r="G233" s="5" t="n"/>
     </row>
     <row r="234">
-      <c r="F234" s="4" t="n"/>
-      <c r="G234" s="4" t="n"/>
+      <c r="F234" s="5" t="n"/>
+      <c r="G234" s="5" t="n"/>
     </row>
     <row r="235">
-      <c r="F235" s="4" t="n"/>
-      <c r="G235" s="4" t="n"/>
+      <c r="F235" s="5" t="n"/>
+      <c r="G235" s="5" t="n"/>
     </row>
     <row r="236">
-      <c r="F236" s="4" t="n"/>
-      <c r="G236" s="4" t="n"/>
+      <c r="F236" s="5" t="n"/>
+      <c r="G236" s="5" t="n"/>
     </row>
     <row r="237">
-      <c r="F237" s="4" t="n"/>
-      <c r="G237" s="4" t="n"/>
+      <c r="F237" s="5" t="n"/>
+      <c r="G237" s="5" t="n"/>
     </row>
     <row r="238">
-      <c r="F238" s="4" t="n"/>
-      <c r="G238" s="4" t="n"/>
+      <c r="F238" s="5" t="n"/>
+      <c r="G238" s="5" t="n"/>
     </row>
     <row r="239">
-      <c r="F239" s="4" t="n"/>
-      <c r="G239" s="4" t="n"/>
+      <c r="F239" s="5" t="n"/>
+      <c r="G239" s="5" t="n"/>
     </row>
     <row r="240">
-      <c r="F240" s="4" t="n"/>
-      <c r="G240" s="4" t="n"/>
+      <c r="F240" s="5" t="n"/>
+      <c r="G240" s="5" t="n"/>
     </row>
     <row r="241">
-      <c r="F241" s="4" t="n"/>
-      <c r="G241" s="4" t="n"/>
+      <c r="F241" s="5" t="n"/>
+      <c r="G241" s="5" t="n"/>
     </row>
     <row r="242">
-      <c r="F242" s="4" t="n"/>
-      <c r="G242" s="4" t="n"/>
+      <c r="F242" s="5" t="n"/>
+      <c r="G242" s="5" t="n"/>
     </row>
     <row r="243">
-      <c r="F243" s="4" t="n"/>
-      <c r="G243" s="4" t="n"/>
+      <c r="F243" s="5" t="n"/>
+      <c r="G243" s="5" t="n"/>
     </row>
     <row r="244">
-      <c r="F244" s="4" t="n"/>
-      <c r="G244" s="4" t="n"/>
+      <c r="F244" s="5" t="n"/>
+      <c r="G244" s="5" t="n"/>
     </row>
     <row r="245">
-      <c r="F245" s="4" t="n"/>
-      <c r="G245" s="4" t="n"/>
+      <c r="F245" s="5" t="n"/>
+      <c r="G245" s="5" t="n"/>
     </row>
     <row r="246">
-      <c r="F246" s="4" t="n"/>
-      <c r="G246" s="4" t="n"/>
+      <c r="F246" s="5" t="n"/>
+      <c r="G246" s="5" t="n"/>
     </row>
     <row r="247">
-      <c r="F247" s="4" t="n"/>
-      <c r="G247" s="4" t="n"/>
+      <c r="F247" s="5" t="n"/>
+      <c r="G247" s="5" t="n"/>
     </row>
     <row r="248">
-      <c r="F248" s="4" t="n"/>
-      <c r="G248" s="4" t="n"/>
+      <c r="F248" s="5" t="n"/>
+      <c r="G248" s="5" t="n"/>
     </row>
     <row r="249">
-      <c r="F249" s="4" t="n"/>
-      <c r="G249" s="4" t="n"/>
+      <c r="F249" s="5" t="n"/>
+      <c r="G249" s="5" t="n"/>
     </row>
     <row r="250">
-      <c r="F250" s="4" t="n"/>
-      <c r="G250" s="4" t="n"/>
+      <c r="F250" s="5" t="n"/>
+      <c r="G250" s="5" t="n"/>
     </row>
     <row r="251">
-      <c r="F251" s="4" t="n"/>
-      <c r="G251" s="4" t="n"/>
+      <c r="F251" s="5" t="n"/>
+      <c r="G251" s="5" t="n"/>
     </row>
     <row r="252">
-      <c r="F252" s="4" t="n"/>
-      <c r="G252" s="4" t="n"/>
+      <c r="F252" s="5" t="n"/>
+      <c r="G252" s="5" t="n"/>
     </row>
     <row r="253">
-      <c r="F253" s="4" t="n"/>
-      <c r="G253" s="4" t="n"/>
+      <c r="F253" s="5" t="n"/>
+      <c r="G253" s="5" t="n"/>
     </row>
     <row r="254">
-      <c r="F254" s="4" t="n"/>
-      <c r="G254" s="4" t="n"/>
+      <c r="F254" s="5" t="n"/>
+      <c r="G254" s="5" t="n"/>
     </row>
     <row r="255">
-      <c r="F255" s="4" t="n"/>
-      <c r="G255" s="4" t="n"/>
+      <c r="F255" s="5" t="n"/>
+      <c r="G255" s="5" t="n"/>
     </row>
     <row r="256">
-      <c r="F256" s="4" t="n"/>
-      <c r="G256" s="4" t="n"/>
+      <c r="F256" s="5" t="n"/>
+      <c r="G256" s="5" t="n"/>
     </row>
     <row r="257">
-      <c r="F257" s="4" t="n"/>
-      <c r="G257" s="4" t="n"/>
+      <c r="F257" s="5" t="n"/>
+      <c r="G257" s="5" t="n"/>
     </row>
     <row r="258">
-      <c r="F258" s="4" t="n"/>
-      <c r="G258" s="4" t="n"/>
+      <c r="F258" s="5" t="n"/>
+      <c r="G258" s="5" t="n"/>
     </row>
     <row r="259">
-      <c r="F259" s="4" t="n"/>
-      <c r="G259" s="4" t="n"/>
+      <c r="F259" s="5" t="n"/>
+      <c r="G259" s="5" t="n"/>
     </row>
     <row r="260">
-      <c r="F260" s="4" t="n"/>
-      <c r="G260" s="4" t="n"/>
+      <c r="F260" s="5" t="n"/>
+      <c r="G260" s="5" t="n"/>
     </row>
     <row r="261">
-      <c r="F261" s="4" t="n"/>
-      <c r="G261" s="4" t="n"/>
+      <c r="F261" s="5" t="n"/>
+      <c r="G261" s="5" t="n"/>
     </row>
     <row r="262">
-      <c r="F262" s="4" t="n"/>
-      <c r="G262" s="4" t="n"/>
+      <c r="F262" s="5" t="n"/>
+      <c r="G262" s="5" t="n"/>
     </row>
     <row r="263">
-      <c r="F263" s="4" t="n"/>
-      <c r="G263" s="4" t="n"/>
+      <c r="F263" s="5" t="n"/>
+      <c r="G263" s="5" t="n"/>
     </row>
     <row r="264">
-      <c r="F264" s="4" t="n"/>
-      <c r="G264" s="4" t="n"/>
+      <c r="F264" s="5" t="n"/>
+      <c r="G264" s="5" t="n"/>
     </row>
     <row r="265">
-      <c r="F265" s="4" t="n"/>
-      <c r="G265" s="4" t="n"/>
+      <c r="F265" s="5" t="n"/>
+      <c r="G265" s="5" t="n"/>
     </row>
     <row r="266">
-      <c r="F266" s="4" t="n"/>
-      <c r="G266" s="4" t="n"/>
+      <c r="F266" s="5" t="n"/>
+      <c r="G266" s="5" t="n"/>
     </row>
     <row r="267">
-      <c r="F267" s="4" t="n"/>
-      <c r="G267" s="4" t="n"/>
+      <c r="F267" s="5" t="n"/>
+      <c r="G267" s="5" t="n"/>
     </row>
     <row r="268">
-      <c r="F268" s="4" t="n"/>
-      <c r="G268" s="4" t="n"/>
+      <c r="F268" s="5" t="n"/>
+      <c r="G268" s="5" t="n"/>
     </row>
     <row r="269">
-      <c r="F269" s="4" t="n"/>
-      <c r="G269" s="4" t="n"/>
+      <c r="F269" s="5" t="n"/>
+      <c r="G269" s="5" t="n"/>
     </row>
     <row r="270">
-      <c r="F270" s="4" t="n"/>
-      <c r="G270" s="4" t="n"/>
+      <c r="F270" s="5" t="n"/>
+      <c r="G270" s="5" t="n"/>
     </row>
     <row r="271">
-      <c r="F271" s="4" t="n"/>
-      <c r="G271" s="4" t="n"/>
+      <c r="F271" s="5" t="n"/>
+      <c r="G271" s="5" t="n"/>
     </row>
     <row r="272">
-      <c r="F272" s="4" t="n"/>
-      <c r="G272" s="4" t="n"/>
+      <c r="F272" s="5" t="n"/>
+      <c r="G272" s="5" t="n"/>
     </row>
     <row r="273">
-      <c r="F273" s="4" t="n"/>
-      <c r="G273" s="4" t="n"/>
+      <c r="F273" s="5" t="n"/>
+      <c r="G273" s="5" t="n"/>
     </row>
     <row r="274">
-      <c r="F274" s="4" t="n"/>
-      <c r="G274" s="4" t="n"/>
+      <c r="F274" s="5" t="n"/>
+      <c r="G274" s="5" t="n"/>
     </row>
     <row r="275">
-      <c r="F275" s="4" t="n"/>
-      <c r="G275" s="4" t="n"/>
+      <c r="F275" s="5" t="n"/>
+      <c r="G275" s="5" t="n"/>
     </row>
     <row r="276">
-      <c r="F276" s="4" t="n"/>
-      <c r="G276" s="4" t="n"/>
+      <c r="F276" s="5" t="n"/>
+      <c r="G276" s="5" t="n"/>
     </row>
     <row r="277">
-      <c r="F277" s="4" t="n"/>
-      <c r="G277" s="4" t="n"/>
+      <c r="F277" s="5" t="n"/>
+      <c r="G277" s="5" t="n"/>
     </row>
     <row r="278">
-      <c r="F278" s="4" t="n"/>
-      <c r="G278" s="4" t="n"/>
+      <c r="F278" s="5" t="n"/>
+      <c r="G278" s="5" t="n"/>
     </row>
     <row r="279">
-      <c r="F279" s="4" t="n"/>
-      <c r="G279" s="4" t="n"/>
+      <c r="F279" s="5" t="n"/>
+      <c r="G279" s="5" t="n"/>
     </row>
     <row r="280">
-      <c r="F280" s="4" t="n"/>
-      <c r="G280" s="4" t="n"/>
+      <c r="F280" s="5" t="n"/>
+      <c r="G280" s="5" t="n"/>
     </row>
     <row r="281">
-      <c r="F281" s="4" t="n"/>
-      <c r="G281" s="4" t="n"/>
+      <c r="F281" s="5" t="n"/>
+      <c r="G281" s="5" t="n"/>
     </row>
     <row r="282">
-      <c r="F282" s="4" t="n"/>
-      <c r="G282" s="4" t="n"/>
+      <c r="F282" s="5" t="n"/>
+      <c r="G282" s="5" t="n"/>
     </row>
     <row r="283">
-      <c r="F283" s="4" t="n"/>
-      <c r="G283" s="4" t="n"/>
+      <c r="F283" s="5" t="n"/>
+      <c r="G283" s="5" t="n"/>
     </row>
     <row r="284">
-      <c r="F284" s="4" t="n"/>
-      <c r="G284" s="4" t="n"/>
+      <c r="F284" s="5" t="n"/>
+      <c r="G284" s="5" t="n"/>
     </row>
     <row r="285">
-      <c r="F285" s="4" t="n"/>
-      <c r="G285" s="4" t="n"/>
+      <c r="F285" s="5" t="n"/>
+      <c r="G285" s="5" t="n"/>
     </row>
     <row r="286">
-      <c r="F286" s="4" t="n"/>
-      <c r="G286" s="4" t="n"/>
+      <c r="F286" s="5" t="n"/>
+      <c r="G286" s="5" t="n"/>
     </row>
     <row r="287">
-      <c r="F287" s="4" t="n"/>
-      <c r="G287" s="4" t="n"/>
+      <c r="F287" s="5" t="n"/>
+      <c r="G287" s="5" t="n"/>
     </row>
     <row r="288">
-      <c r="F288" s="4" t="n"/>
-      <c r="G288" s="4" t="n"/>
+      <c r="F288" s="5" t="n"/>
+      <c r="G288" s="5" t="n"/>
     </row>
     <row r="289">
-      <c r="F289" s="4" t="n"/>
-      <c r="G289" s="4" t="n"/>
+      <c r="F289" s="5" t="n"/>
+      <c r="G289" s="5" t="n"/>
     </row>
     <row r="290">
-      <c r="F290" s="4" t="n"/>
-      <c r="G290" s="4" t="n"/>
+      <c r="F290" s="5" t="n"/>
+      <c r="G290" s="5" t="n"/>
     </row>
     <row r="291">
-      <c r="F291" s="4" t="n"/>
-      <c r="G291" s="4" t="n"/>
+      <c r="F291" s="5" t="n"/>
+      <c r="G291" s="5" t="n"/>
     </row>
     <row r="292">
-      <c r="F292" s="4" t="n"/>
-      <c r="G292" s="4" t="n"/>
+      <c r="F292" s="5" t="n"/>
+      <c r="G292" s="5" t="n"/>
     </row>
     <row r="293">
-      <c r="F293" s="4" t="n"/>
-      <c r="G293" s="4" t="n"/>
+      <c r="F293" s="5" t="n"/>
+      <c r="G293" s="5" t="n"/>
     </row>
     <row r="294">
-      <c r="F294" s="4" t="n"/>
-      <c r="G294" s="4" t="n"/>
+      <c r="F294" s="5" t="n"/>
+      <c r="G294" s="5" t="n"/>
     </row>
     <row r="295">
-      <c r="F295" s="4" t="n"/>
-      <c r="G295" s="4" t="n"/>
+      <c r="F295" s="5" t="n"/>
+      <c r="G295" s="5" t="n"/>
     </row>
     <row r="296">
-      <c r="F296" s="4" t="n"/>
-      <c r="G296" s="4" t="n"/>
+      <c r="F296" s="5" t="n"/>
+      <c r="G296" s="5" t="n"/>
     </row>
     <row r="297">
-      <c r="F297" s="4" t="n"/>
-      <c r="G297" s="4" t="n"/>
+      <c r="F297" s="5" t="n"/>
+      <c r="G297" s="5" t="n"/>
     </row>
     <row r="298">
-      <c r="F298" s="4" t="n"/>
-      <c r="G298" s="4" t="n"/>
+      <c r="F298" s="5" t="n"/>
+      <c r="G298" s="5" t="n"/>
     </row>
     <row r="299">
-      <c r="F299" s="4" t="n"/>
-      <c r="G299" s="4" t="n"/>
+      <c r="F299" s="5" t="n"/>
+      <c r="G299" s="5" t="n"/>
     </row>
     <row r="300">
-      <c r="F300" s="4" t="n"/>
-      <c r="G300" s="4" t="n"/>
+      <c r="F300" s="5" t="n"/>
+      <c r="G300" s="5" t="n"/>
     </row>
     <row r="301">
-      <c r="F301" s="4" t="n"/>
-      <c r="G301" s="4" t="n"/>
+      <c r="F301" s="5" t="n"/>
+      <c r="G301" s="5" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -1785,6 +3536,90 @@
       <formula1>"yes,no,unsure"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D65" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D66" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D67" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D68" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D69" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D70" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D71" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D72" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D73" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D74" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D75" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D76" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D82" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D83" r:id="rId82"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
S6 final: adhoc_v5 (dev-only revisions) + evidence retry, enlarged sample, pre-registered threshold, single test run
- D41 pre-registered rule; D42 adhoc_v4/v5 from dev errors; D43 evidence retry (+store migration); D44 +600 negatives (v2 sample); D45 threshold 0.9 on dev; D46 result
- eval merges dev+test runs, test PR curve + baseline point in metrics.json; review sheet regenerated (90, blind)

Verification: make eval RUN=\"20261018T134630509400Z 20261018T134941952960Z\" -> test P_corr 69.5% (53.0-91.0), R 54.5% (44.8-63.8), F1 61.0%;
baselines CV area 40.9/80.2, keyword 41.3/56.4. Evidence failures 15.2% -> 4.3% after retry. make test: 62 passed.
</commit_message>
<xml_diff>
--- a/data/gold/for_partner/adjudication.xlsx
+++ b/data/gold/for_partner/adjudication.xlsx
@@ -594,11 +594,11 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>66198</v>
+        <v>67332</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Qu'entreprend le Conseil fédéral pour protéger et promouvoir la biodiversité?</t>
+          <t>Weg von Fast Fashion, aber wie?</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
@@ -608,7 +608,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Economiesuisse a souligné récemment l'énorme importance de la biodiversité pour la santé de l'économie et de la société. WSL et SCNAT viennent de publier un rapport concernant les subventions qui portent atteinte à la biodiversité et nuisent à long terme à l'économie du pays. Les associations environnementales ont déposé cette semaine une initiative en faveur de la biodiversité. Ces actions issues des milieux scientifiques, économiques et associatifs sont porteuses d'un message clair. Que fait le Conseil fédéral de son côté ?</t>
+          <t>TEXT: In den letzten 20 Jahren sind Textilien von einem Gebrauchsgegenstand zum Wegwerf-Artikel geworden. Die Tragedauer von Kleidern ist um 40 Prozent gesunken. Dafür hat sich die weltweite Produktion verdoppelt. Die billige und schnelllebige Fast-Fashion-Industrie hat immense Schattenseiten. Prekäre Arbeitsbedingungen und gesundheitsschädigende Umweltbelastungen prägen die globalen Lieferketten. 2018 haben deshalb das Bundesamt für Umwelt (BAFU) gemeinsam mit dem Staatssekretariat für Wirtschaft (SECO) sowie den Verbänden Swiss Textiles und amfori die Initiative "Nachhaltige Textilien Schweiz" als Multi-Stakeholder-Dialog gestartet. Daraus ist das Programm "Sustainable Textiles Switzerland 2030 (STS 2030)" entstanden, das einen wesentlichen Beitrag zur Erreichung der Nachhaltigen Entwicklungsziele (SDGs) im Schweizer Textil- und Bekleidungssektor entlang der gesamten Wertschöpfungskette leisten will. Die am Programm beteiligten Unternehmungen und Verbände setzen sich im Rahmen ihrer Eigenverantwortung in einem vorbildlichen Prozess für die Reduktion der Treibhausgasemissionen, die Förderung fairer Löhne und menschenwürdiger Arbeitsbedingungen, die Förderung innovativer Geschäftsm…</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr"/>
@@ -619,11 +619,11 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>155716</v>
+        <v>69244</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Coronavirus. Non scaricare i costi della pandemia sui premi di cassa malati</t>
+          <t>Nouvelles réglementations sur les dérives d’Internet</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
@@ -631,12 +631,7 @@
           <t>open</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>TEXT: Il Consiglio federale è incaricato di adottare le misure necessarie affinché negli anni 2021-2023 i premi dell'assicurazione malattie rimangano stabili e non siano innalzati in nessun caso.
-REASONING: La pandemia da coronavirus comporta un forte aumento dei costi della salute. Se da un lato dal 16 marzo al 27 aprile non sono stati eseguiti interventi elettivi, dall'altro non è dato sapere a quanto ne ammonteranno i costi effettivi sull'intero arco dell'anno né quanti di questi interventi, con i relativi costi, saranno rinviati ai prossimi anni. Gli assicuratori-malattie dispongono di riserve a cui possono attingere soltanto fino a un certo punto. Tuttavia i costi di una pandemia non devono sfociare in un aumento dei premi di cassa malati: vanno finanziati in maniera solidale e con un maggior coinvolgimento dei poteri pubblici (Confederazione e Cantoni). L'assicurazione malattie è finanziata con il sistema dei premi pro capite indipendenti dal reddito, che già oggi incidono in misura eccessiva sul budget di moltissime economie domestiche. L'incidenza media è del 14 per cento ed è destinata ad aumentare ulteriormente poiché durante la crisi del coronavirus i redditi sono dimin…</t>
-        </is>
-      </c>
+      <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="5" t="inlineStr"/>
       <c r="G3" s="5" t="inlineStr"/>
     </row>
@@ -645,11 +640,11 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>65463</v>
+        <v>287810</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Im Interesse der Rechtsstaatlichkeit, der Souveränität und der Neutralität der Schweiz die Crypto-Leaks-Affäre mit einer PUK umfassend aufklären</t>
+          <t>Contrôle étendu des données personnelles et des réseaux sociaux dans les procédures Esta. Conséquences pratiques et juridiques pour les citoyens suisses</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -659,8 +654,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Das Parlament setzt eine Parlamentarische Untersuchungskommission PUK ein zur Aufarbeitung der Spionage-Affäre um die Firma Crypto AG.
-REASONING: Im Interesse der Rechtsstaatlichkeit, der Souveränität und der Neutralität der Schweiz muss die Cryptoleaks-Affäre umfassend aufgeklärt werden. Eine PUK hat dazu die notwendigen Ressourcen und kann insbesondere auch Untersuchungsbeauftragte i.S. von Artikel 166 ParIG einsetzen.</t>
+          <t>TEXT: Le gouvernement américain (U.S. Customs and Border Protection) a annoncé le 10 décembre 2025 son intention d'imposer aux voyageurs en provenance des pays participant au programme Visa Waiver (dont la Suisse fait partie) qui demandent le visa ESTA (Electronic System for Travel Authorization) l'obligation de fournir, entre autres, l'historique de leurs activités sur les réseaux sociaux au cours des cinq dernières années, leurs adresses électroniques des dix dernières années et le lieu de naissance et de résidence de leurs parents, conjoints, frères et sœurs et enfants. Ce projet est actuellement en consultation. S’il devait se concrétiser, il aurait également des répercussions importantes pour les citoyens suisses qui voyagent aux États-Unis. À la lumière de ce qui précède, le Conseil fédéral est prié de répondre aux questions suivantes : Que pense-t-il des modifications annoncées (en particulier l'obligation de mettre à disposition les informations concernant les activités effectuées sur les réseaux sociaux au cours des cinq dernières années) au regard des droits civils et de la protection des données des citoyens suisses ? À quelles conséquences s’attend-il pour les touristes…</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr"/>
@@ -671,11 +665,11 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>66518</v>
+        <v>155776</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Rapporto sulla politica di sicurezza 2021</t>
+          <t>Covid-19. Eine Grundlage, um in der Bundesverwaltung die Verbreitung von Homeoffice zu beschleunigen?</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -683,7 +677,11 @@
           <t>open</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Der Umgang mit der Covid-19-Notlage hat allen Gesellschaftsschichten grosse Anpassungen abverlangt. Sehr deutlich zeigte sich dies bei der weit verbreiteten Nutzung des Homeoffice. Auch zahlreiche Bundesangestellte arbeiten zurzeit im Homeoffice. Diesbezüglich stellen die gegenwärtigen Umstände einen wichtigen Test dar, aus dem für die Zukunft Erfahrungen gesammelt werden können und der dazu genutzt werden kann, die Verbreitung des Homeoffice zu beschleunigen. Wie in anderen Bereichen könnte die Einführung von erleichterten Bedingungen für das Homeoffice auch in der Bundesverwaltung positive Auswirkungen auf verschiedene Bereiche haben, z. B. den Verkehr (weniger überfüllte öffentliche Verkehrsmittel und weniger Stau auf den Strassen), die Lebensqualität der Angestellten (bessere Vereinbarkeit von Berufs- und Familienleben, weniger Stress) und die Arbeitsleistung (grössere Flexibilität und Produktivität, geringeres Risiko eines Burnout). Weiter könnten solche Massnahme sich auch positiv auf die Bundesfinanzen auswirken dank einer effizienteren Verwaltung der gemieteten Räumlichkeiten und einem gezielteren Ressourceneinsatz. Unterstrichen werden muss zudem, dass eine flexibler…</t>
+        </is>
+      </c>
       <c r="F5" s="5" t="inlineStr"/>
       <c r="G5" s="5" t="inlineStr"/>
     </row>
@@ -692,11 +690,11 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>65226</v>
+        <v>159102</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Zugang zu unterstützter Kommunikation</t>
+          <t>Qual è il livello di sicurezza degli ambienti di lavoro nella Confederazione riguardo ad azioni di sabotaggio e/o di ascolto da parte di altri attori?</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -706,7 +704,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Kommunikation dient dem sozialen Austausch, ermöglicht gesellschaftliche Teilhabe und ist damit ein menschliches Grundbedürfnis. Mit der Ratifizierung der UNO-Behindertenrechtskonvention verpflichtete sich die Schweiz, auf individuelle Bedürfnisse abgestimmte Kommunikationsformen und Kommunikationsmittel zu fördern. Für Menschen mit eingeschränkter Lautsprache gibt es die Unterstützte Kommunikation (UK). Das Gelingen der UK hängt u.a. davon ab, ob die passenden Methoden und Hilfsmittel zum Einsatz kommen, ob genügend UK-Fachpersonal in den Institutionen arbeitet und ob das Umfeld UK täglich und in möglichst vielen Lebensbereichen nutzt. Ich bitte den Bundesrat um die Beantwortung folgender Fragen: 1. Wie viele Menschen sind in der Schweiz auf UK angewiesen? Wie sieht die Verteilung aus zwischen Menschen mit leichten und Menschen mit schweren Kommunikationsbeeinträchtigungen u.a. aufgrund von schweren sowie mehrfachen Behinderungen? 2. Was tun Bund und Kantone, um sicherzustellen, dass alle Personen, Kinder und Erwachsene, mit eingeschränkten lautsprachlichen Fähigkeiten während ihres gesamten Lebens in verschiedenen Lebensbereichen wie u.a. Frühbereich, Bildung, Wohnen, Arbei…</t>
+          <t>TEXT: L'incidente occorso in Germania alcune settimane fa suscita scalpore. Alcuni sabotatori hanno tagliato in diversi punti i cavi del sistema di comunicazione della Deutsche Bahn. Il traffico ferroviario è stato paralizzato e la comunicazione tra macchinisti e i posti di comando è stata interrotta. Uno scenario simile sarebbe ipotizzabile ovunque. In Svizzera, nel contesto della Confederazione, la sicurezza sul lavoro e un ambiente di lavoro basato sulla fiducia sono considerati elementi chiave. Tuttavia esistono sempre locali ed edifici in cui gli impiegati federali devono lavorare e tenere conversazioni confidenziali. Non sempre è possibile escludere che questi ambienti siano sicuri. Negli stessi edifici troviamo anche gli uffici di altre imprese, i cui cavi informatici vanno a finire negli stessi locali adibiti ai server, utilizzati dai servizi della Confederazione. Pertanto non si può escludere categoricamente un'azione di sabotaggio o l'ascolto mirato. In questo contesto invito il Consiglio federale a rispondere alle domande seguenti: 1. La Confederazione ha una visione d'insieme per verificare se tutti gli Uffici rilevanti per la sicurezza possano lavorare in modo "sicuro"…</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr"/>
@@ -717,11 +715,11 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>234936</v>
+        <v>67403</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Besteht die Gefahr, dass die Romandie bei den Offsets im Zusammenhang mit dem F-35A benachteiligt wird?</t>
+          <t>Wie geht es weiter mit der SwissCovid App?</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -731,7 +729,8 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Der Kauf der 36 Kampfflugzeuge des Typs F-35A bringt den Schweizer Unternehmen im Rahmen der Offsets rund 2,9 Milliarden Franken ein, wobei die Aufträge bis 2034 verteilt sein sollten. Dabei wurde vorgesehen, dass der Romandie 30 Prozent des Offsetvolumens zukommt, während 65 Prozent für die Deutschschweiz und 5 Prozent für das Tessin vorgesehen sind. Nun aber fürchten die Kantone der Romandie je länger je mehr, dass sie vergessen werden und dass die Zusagen, die beim Kauf der F-35A gemacht wurden, nicht eingehalten werden. Damit geht eine zunehmende Unzufriedenheit einher, sowohl in der Politik als auch in der Wirtschaft. Das Bundesunternehmen RUAG begehrt nämlich mehrere grosse Aufträge. Zur Instandhaltung der 36 Jets der Schweizer Armee sollen noch weitere Projekte dazukommen. Das Unternehmen ist jedoch vor allem in der Deutschschweiz angesiedelt, was nicht ohne Folgen für die Wirtschaft der Romandie bleiben würde, obwohl sie über zahlreiche Vorzüge verfügt. Insbesondere Genf, Freiburg und Neuenburg verfügen über viele Spezialistinnen und Spezialisten im Bereich der Luftfahrt. Mehr als siebzig grosse, mittlere und kleine Unternehmen der Romandie stellen der militärischen w…</t>
+          <t>TEXT: Gemäss den offiziellen Angaben des SwissCovid-App-Monitorings (vom 21. bis 27. Februar) haben in diesem Zeitraum 743 Nutzerinnen und Nutzer einen Covidcode eingegeben, bei 1 740 000 Downloads. In mehr als 13 Prozent der Fälle vergehen mindestens vier Tage zwischen dem Symptombeginn und der Zuweisung des Covidcodes. Sieht der Bundesrat in diesen Zahlen ein Zeichen des Erfolgs für die SwissCovid App in Bezug auf ihre Nützlichkeit im Kampf gegen die Ausbreitung des Virus?
+ANSWER: Die Antwort des Bundesrates existiert nur in französischer Sprache. (Bitte wechseln Sie auf der Homepage oben rechts die Sprache)</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr"/>
@@ -742,11 +741,11 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>156699</v>
+        <v>69934</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Kommunikation zur Mitwirkung der Schweiz in der Allianz für Multilateralismus</t>
+          <t>Personen mit Ausweis S: Wie viele haben zulasten der Schweizerinnen und Schweizer eine Arbeit gefunden?</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -756,7 +755,8 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Im letzten Herbst ist im Rahmen der UNO die Allianz für Multilateralismus als Netzwerk entstanden. - Ist die Schweiz in diesem Netzwerk auch engagiert? - Wann gedenkt der Bundesrat öffentlich über das Engagement und die Projekte des Netzwerkes zu orientieren?</t>
+          <t>TEXT: Bezüglich der Personen mit Ausweis S stelle ich folgende Fragen: 1. Wie viele von ihnen haben eine Arbeitsstelle gefunden? 2. Was für Verträge regeln ihr Arbeitsverhältnis zu den Unternehmen? 3. In welchen Sektoren sind sie tätig? 4. Haben diese Personen Stellen besetzt, die sonst von Schweizer Bürgerinnen und Bürgern eingenommen worden wären? Es wird darum gebeten, die Daten für die Schweiz insgesamt und nach Sprachregion darzustellen.
+ANSWER: Die Antwort des Bundesrates existiert nur in französischer Sprache. (Bitte wechseln Sie auf der Homepage oben rechts die Sprache)</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr"/>
@@ -767,11 +767,11 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>157177</v>
+        <v>71365</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Mestieri del futuro. Sostegno pubblico alla riconversione professionale</t>
+          <t>Selbstverteidigungsrecht der Staaten unter Beschuss?</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -781,8 +781,8 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Il Consiglio federale è incaricato di illustrare in un rapporto in che modo è possibile creare nuove prospettive professionali in settori in fase di cambiamento strutturale tramite un maggiore investimento pubblico nella formazione continua e professionale.
-REASONING: La transizione ecologica causa la perdita di posti di lavoro in alcuni settori dell'industria e dei servizi, ma allo stesso tempo permette lo sviluppo di nuove professioni legate a un'economia più sostenibile: questo è quanto emerge da un rapporto realizzato dall'Organizzazione Internazionale del Lavoro (OIL) nel 2018. Lo studio mostra un fattore essenziale affinché la transizione ecologica possa portare alla creazione di posti di lavoro: una riconversione professionale efficace e mirata. È dunque necessario disporre di un piano a lungo termine e di dati chiari per identificare le esigenze attuali e future dell'economia e fornire i mezzi per formare (nuovamente) milioni di persone. Tuttavia in Svizzera manca un piano di questo genere. Allo stesso tempo, la digitalizzazione sta allargando il divario tra l'economia di produzione di ieri e l'economia digitale di domani, lasciando indietro dei dipendenti a causa de…</t>
+          <t>TEXT: ICC-Chefankläger Karim Ahmat Khan hat im Zusammenhang mit dem Konflikt in Gaza einen Haftbefehl gegen Israels Regierungschef Benjamin Netanjahu beantragt und erhält Rückendeckung aus arabischen Staaten. Stellt der Bundesrat das Selbstverteidigungsrecht Israels ebenfalls infrage?
+ANSWER: La Suisse soutient la Cour pénale internationale (CPI) en tant qu'institution judiciaire indépendante et impartiale. La Suisse a toujours défendu l’indépendance de la CPI et continuera à le faire. La CPI a confirmé sa compétence pour la situation en Palestine en 2020 et autorisé l’ouverture d’une enquête. Des renvois supplémentaires n’étaient dès lors pas nécessaires pour accélérer la procédure comme c’était le cas pour la situation en Ukraine. Da es sich um ein laufendes Verfahren handelt, äussert sich der Bundesrat nicht zum Antrag des Anklägers auf Erlass von Haftbefehlen. Die zuständige Vorverfahrenskammer des IStGH wird diese Anträge nun zu prüfen haben. Die Unabhängigkeit des Gerichts muss respektiert werden. Als Mitglied des Römer Statuts ist die Schweiz grundsätzlich verpflichtet, Haftbefehle des IStGH zu vollstrecken. Über die Zulässigkeit und die Modalitäten der Zusammenarbeit mit d…</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr"/>
@@ -793,11 +793,11 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>62663</v>
+        <v>201902</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Quali rischi per la Confederazione comporta la strategia di convergenza di Swisscom?</t>
+          <t>Wissenschaftliche Studie zu allfällig übersetzten Mieten</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -807,7 +807,8 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Chiedo al Consiglio federale di rispondere alle seguenti domande: 1. Il Consiglio federale ritiene che la strategia di convergenza di Swisscom e la posizione dominante sul mercato che ne deriva comportino nuovi rischi per la Confederazione e/o l'economia pubblica (in particolare per quanto riguarda la problematica "too big to fail" e gli attacchi informatici)? 2. La Confederazione, in quanto azionista di maggioranza, segue attivamente la strategia e analizza gli eventuali rischi per la Confederazione e/o l'economia pubblica insiti nei nuovi settori di attività? In caso affermativo, come avviene ciò concretamente? In caso negativo, perché non lo ritiene necessario? 3. Il Consiglio federale ritiene che Swisscom, che è quotata in borsa, possa fallire senza che ciò causi enormi danni collaterali al bilancio della Confederazione e/o all'intera economia svizzera? Se la risposta è "no", quali conseguenze trae dal rischio legato alla problematica "too big to fail"? Se la risposta è "sì", da dove trae questa convinzione? 4. Il Consiglio federale è disposto a far verificare le questioni di cui sopra nel quadro dell'esame esterno del governo d'impresa delle aziende parastatali e a infor…</t>
+          <t>TEXT: Der Bundesrat wird beauftragt, umgehend eine wissenschaftliche Studie in Auftrag zu geben, die das Ausmass der übersetzten Mieten aufzeigt und die volkswirtschaftlichen Auswirkungen beleuchtet
+REASONING: Unser Mietrecht erlaubt mit der "Kostenmiete plus" eine Eigenkapitalrendite, welche den die Bindung an den hypothekarischen Referenzzinssatz (Kosten) um einen geringen Prozentsatz übersteigen darf. Lange Zeit setzte das Bundesgericht diesen auf 0,5 Prozent, seit 2 Jahren auf 2 Prozent über dem hypothekarischen Referenzzinssatz fest (auf Bauten, die nicht älter als 30 Jahre sind). In Realität betragen die effektiven Renditen aber nicht die maximal erlaubten, sondern oft werden betriebswirtschaftliche Renditen in zweistelliger Höhe erzielt. Die Mieten sind in den letzten 15 Jahren nur gestiegen, obwohl sie hätten wegen der tiefen Zinsen massiv sinken sollen. In einer Studie der Raiffeisen-Bank wurde die Abweichung der effektiven Mietzinse vom gesetzlichen Pfad auf 14 Milliarden Franken jährlich beziffert und die Mieten bis 40 Prozent zu hoch seien. In der neusten Studie des Büro Bass, werden die Mietpreise für das Jahr 2021 als mit 10,4 Milliarden Franken zu hoch berechnet und…</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr"/>
@@ -818,11 +819,11 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>154602</v>
+        <v>235223</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Foglio informativo dell'UFAM sulla ristorazione sostenibile. Non abbiamo altri problemi?</t>
+          <t>Le caratteristiche e i dispositivi di sicurezza del sistema svizzero di verifica dei medicamenti (SMVS) sono inadatti per il monitoraggio degli agenti terapeutici?</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -832,8 +833,8 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>TEXT: In un nuovo foglio informativo, l'UFAM fornisce raccomandazioni per una ristorazione gustosa e rispettosa dell'ambiente in occasione di eventi. Tra le altre cose si raccomanda che almeno due terzi del cibo a buffet siano composti da prodotti vegetariani e che il cibo vegetariano sia collocato in primo piano. In merito chiedo al Consiglio federale di rispondere alle seguenti domande: 1. Il Consiglio federale ritiene veramente che in questo ambito sussista una necessità di intervento da parte della Confederazione? 2. Il Consiglio federale concorda sul fatto che con questo genere di "raccomandazioni" a favore del cibo vegetariano si penalizza il settore della carne e delle macellerie? 3. Quanti collaboratori dell'UFAM hanno partecipato all'elaborazione di questo foglio informativo? 4. Quanto tempo è stato necessario e a quanto ammontano i relativi costi? 5. Il Consiglio federale ritiene veramente che sia compito dello Stato educare i cittadini e dire loro cosa mangiare e bere? 6. Il Consiglio federale può confermare esplicitamente che queste raccomandazioni di oggi non saranno i divieti di domani?
-ANSWER: 1. Il rapporto Ambiente Svizzera 2018 del Consiglio federale indica che i…</t>
+          <t>TEXT: Il Consiglio federale condivide l’opinione secondo cui non esiste una base legale che consenta di attuare mediante l’articolo 17a LATer, approvato ma non in vigore, la gestione digitale delle penurie di medicamenti per uso umano richiesta dalla mozione Ettlin e che è necessario elaborare una specifica base legale all’interno della LATer? L’introduzione del SMVS fa parte delle otto raccomandazioni proposte al Consiglio federale dalla task force per gli agenti terapeutici? Il monitoraggio necessita di un’ulteriore base legale o è sufficiente il sistema di preallarme dell’Ufficio federale dell’approvvigionamento economico del Paese (UFAE)? È vero che l’UFAE non intende servirsi del SMVS per la gestione digitale delle penurie di medicamenti per uso umano? Il Consiglio federale ritiene che esista un rischio significativo che in Svizzera entrino in commercio medicamenti contraffatti? Se sì, in quali casi? Il Consiglio federale condivide la posizione dei fornitori di servizi, secondo cui i costi di attuazione dei requisiti SMVS sono troppo elevati rispetto ai potenziali benefici?
+REASONING: Il 26 settembre 2023 il Parlamento ha approvato, con un adattamento del punto 2, la mozione …</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr"/>
@@ -844,11 +845,11 @@
         <v>11</v>
       </c>
       <c r="B12" t="n">
-        <v>235621</v>
+        <v>157707</v>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Réforme de la valeur locative. Montant des déductions concernées</t>
+          <t>Ordinanza sull’indicazione dei prezzi. Semplificare l’autocomparazione</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -858,8 +859,8 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Le 28 septembre 2025, la population se prononcera sur l'introduction d'un nouvel impôt immobilier cantonal sur les résidences secondaires. Ce projet est lié à la réforme fiscale qui supprime la valeur locative. Si la peuple se prononçait favorablement, la valeur locative ne serait plus imposée, mais un grand nombre de déductions aujourd'hui possibles, ne pourront plus être faites. En particulier, les intérêts hypothécaires (à part au tout début et de façon dégressive), les frais de rénovation y compris écologique, les frais d'entretien ne pourront plus être déduits du revenu. Le Conseil fédéral est prié de répondre aux questions suivantes: 1) Quel est le volume, en francs, des déductions octroyées au niveau fédéral qui sont aujourd'hui possible et qui ne seraient plus possibles si suppression de la valeur locative était acceptée 2) Quel est le montant d'impôt correspondant à ces déductions au niveau fédéral? 3) Si les cantons décident eux aussi de supprimer toutes les déductions qui ne sont plus possibles au niveau fédéral, quel serait le volume des déductions concernées, et le montant de l'impôt correspondant à ces déductions, cette fois-ci au niveau cantonal?
-ANSWER: Il es…</t>
+          <t>TEXT: Il Consiglio federale è incaricato di semplificare le disposizioni dell'ordinanza sull'indicazione dei prezzi (OIP; RS 942.211) riguardanti l'indicazione fallace dei prezzi (art. 16 cpv. 1 lett. a e cpv. 3 OIP) in modo da consentire l'autocomparazione senza che siano fissati limiti di tempo, in particolare per gli articoli di stagione come capi di abbigliamento, calzature, articoli sportivi, ecc., se la merce in questione è stata effettivamente proposta in precedenza, per almeno quattro settimane consecutive, al prezzo più alto indicato.
+REASONING: Le disposizioni piuttosto complesse dell'OIP sull'autocomparazione, che regolamentano le indicazioni di riduzione dei prezzi e le comparazioni con il prezzo di vendita iniziale, erano state introdotte per evitare che i consumatori fossero tratti in inganno, ma oggi sono superate. Più in particolare, la cosiddetta regola del dimezzamento secondo cui il "prezzo comparativo" può essere indicato solo per la metà del periodo durante il quale è stato o sarà praticato, e al massimo per due mesi, comporta per i venditori e per le autorità di controllo un onere sproporzionato rispetto al vantaggio che ne risulta per il cliente. Questa rego…</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr"/>
@@ -870,11 +871,11 @@
         <v>12</v>
       </c>
       <c r="B13" t="n">
-        <v>153348</v>
+        <v>337362</v>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Online-Handel prüfen, überwachen und einschränken?</t>
+          <t>Commissioni extraparlamentari. Riorganizzazione nel quadro della verifica 2025</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -882,12 +883,7 @@
           <t>open</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>TEXT: Immer häufiger werden Fälle bekannt, wo in der Schweiz verbotene Waffen und andere illegale Gegenstände auf ausländischen Online-Handelsplattformen gekauft und auf dem Paketweg in die Schweiz gesendet wurden. Dabei werden unter anderem Waffen in Folien eingeschweisst, um den Detektoren der Zollverwaltung eine Entdeckung zu erschweren, oder Gegenstände als Muster bezeichnet, um Zollgebühren zu vermeiden. Bislang können für solche illegalen Praktiken allerdings nur die Empfänger belangt werden. Der Bundesrat wird gebeten, folgende Fragen zu beantworten: 1. Beabsichtigt er, der Eidgenössischen Zollverwaltung die nötigen Mittel zur Verfügung zu stellen, damit die grosse Mehrheit dieser illegalen Pakete künftig aus dem Verkehr gezogen werden kann? 2. Besteht aus seiner Sicht auch die Notwendigkeit, die verantwortlichen Online-Portale und die Versender in die Verantwortung zu nehmen? 3. Kann im Rahmen von Freihandelsabkommen die beschriebene Problematik zusammen mit unseren Handelspartnern wirkungsvoll angegangen werden? 4. Welche weiteren Mittel sieht er, um den transnationalen Versand illegaler Pakete wirkungsvoll einzudämmen?
-REASONING: Die Digitalisierung ermöglicht einen imme…</t>
-        </is>
-      </c>
+      <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="5" t="inlineStr"/>
       <c r="G13" s="5" t="inlineStr"/>
     </row>
@@ -896,11 +892,11 @@
         <v>13</v>
       </c>
       <c r="B14" t="n">
-        <v>155827</v>
+        <v>63752</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Crisi dovuta al coronavirus. Soluzione globale per stabilizzare le finanze federali e le opere sociali</t>
+          <t>Dialog über die zentralen Werte unserer Gesellschaft</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -910,8 +906,8 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Il Consiglio federale è incaricato di presentare al Parlamento una soluzione globale che indichi come le prestazioni straordinarie fornite dalla Confederazione durante la crisi dovuta al coronavirus e le future perdite fiscali provocate dalla suddetta crisi debbano essere contabilizzate nei conti della Confederazione. Il Consiglio federale deve indicare in particolare come nei prossimi 6-8 anni dovrà essere coperto il disavanzo del fondo di compensazione stimato in 40 miliardi di franchi, come dovranno essere compensate le perdite fiscali stimate in cinque miliardi di franchi l'anno e quali misure dovranno essere adottate per consolidare le assicurazioni sociali del 1° e del 2° pilastro. Condizione: il freno all'indebitamento, che ha dato prova di efficacia, non deve essere allentato.
-REASONING: Il Consiglio federale ha espresso grande preoccupazione per le conseguenze economiche della crisi dovuta al coronavirus. Le prestazioni straordinarie graveranno le casse della Confederazione per un importo di circa 40 miliardi di franchi, che sarà trasferito a un fondo di compensazione. La base legale prevede che tale fondo sia riequilibrato entro 6-8 anni. Inoltre, a causa dell'immi…</t>
+          <t>TEXT: Der Bundesrat wird beauftragt, in einem Bericht aufzuzeigen, wie eine geeignete Plattform ausgestaltet sein sollte, welche die relevanten gesellschaftlichen Akteure und Organisationen zu einem offenen und gleichberechtigten Dialog vereinen könnte, um sich über die zentralen Werte unserer Gesellschaft auszutauschen.
+REASONING: Fundamentalistische Strömungen sind eine Bedrohung für unsere freie, demokratische Gesellschaft, welche durch unseren Rechtsstaat geschützt ist. Für ein friedliches Zusammenleben bedarf es gemeinsamer Werte, auf welche sich alle Mitglieder einer Gesellschaft einigen und berufen können. Gemeinsame Werte entstehen durch Diskussion, Austausch und Verständnis. Gemeinsame Werte benötigen jedoch auch eine breitabgestützte Legitimation in der Bevölkerung. Aus diesem Grund wäre ein offener und gleichberechtigter Dialog zwischen den unterschiedlichen relevanten gesellschaftlichen Akteuren und Organisationen eine ideale Plattform, um eine solche Wertediskussion zu führen. Ein solcher Dialog ist für die Schweiz nicht nur wünschenswert, sondern von elementarer Wichtigkeit. Wie die aktuellen Debatten zeigen, fehlt der Schweiz ein Verständnis für das gemeinsame gesel…</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr"/>
@@ -922,11 +918,11 @@
         <v>14</v>
       </c>
       <c r="B15" t="n">
-        <v>235813</v>
+        <v>64532</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Zentrales Informationssystem Digiflux. Was kostet die Umsetzung?</t>
+          <t>Allocation de maternité pour les femmes travaillant dans l'agriculture</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -936,8 +932,8 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Für die Verwendung von Pflanzenschutzmitteln und Nährstoffen wird ein zentrales Informationssystem (Digiflux) eingeführt. Der Bundesrat wird in diesem Zusammenhang gebeten, die folgenden Fragen zu beantworten: 1) Welche jährlichen Investitions-, Anwendungs- und Personalkosten sind mit dem Projekt verbunden? 2) Wie hoch ist der geschätzte zusätzliche administrative Aufwand für die Kantone, die Landwirtschaftsbetriebe und die anderen betroffenen Akteure? 3) Kann das Ziel der Transparenz auch erreicht werden, indem für die Landwirtschaftsbetriebe ein einfacheres System eingeführt wird, ein System, das beispielsweise auf Schätzungen und Befragungen beruht? 4) Ist der Bundesrat bereit, die Einführung der Digiflux-Anwendung zu verschieben, um den Anwenderinnen und Anwendern mehr Zeit für die Umsetzung zu gewähren?
-REASONING: Im Rahmen der parlamentarischen Initiative 19.475 wurden mehrere Gesetze geändert –dies mit dem Ziel, zur Verminderung der Risiken im Zusammenhang mit dem Einsatz von Pflanzenschutzmitteln und zur Reduktion der Nährstoffverluste Absenkpfade festzulegen. Das Landwirtschaftsgesetz wurde mit einer Mitteilungspflicht für Nährstofflieferungen, einschliesslich Kraft…</t>
+          <t>TEXT: En Suisse, les deux tiers des femmes travaillent dans l'entreprise ou l'exploitation agricole de leur mari ou compagnon sans être rémunérées. - Sachant que les étudiants ont droit aux allocations pour perte de gain sans avoir de revenus, le Conseil fédéral envisagerait-t-il de modifier l'art. 16b, al. 1, let. c, de la loi sur les allocations pour perte de gain, leur permettant de percevoir une allocation de maternité ? - Si non pourquoi ?
+ANSWER: Une telle modification n'est pas prévue par le Conseil fédéral. Aucune allocation de maternité minimale n'est versée, que ce soit pour les étudiantes ou pour toute autre personne, si aucun revenu n'est perçu avant l'accouchement. Cela résulte de la volonté du législateur et de compromis politiques qui ont fait suite aux longues négociations dans le cadre de l'introduction de l'allocation de maternité, le 1er juillet 2005.</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr"/>
@@ -948,11 +944,11 @@
         <v>15</v>
       </c>
       <c r="B16" t="n">
-        <v>330749</v>
+        <v>201868</v>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Intelligente Brillen: eine neue Dimension des Voyeurismus. Ist das Schweizer Recht den Anforderungen gewachsen?</t>
+          <t>Coopération internationale des autorités pénales dans la lutte contre la cybercriminalité</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -962,7 +958,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Intelligente Brillen vom Typ Ray-Ban Meta, von denen 2025 weltweit sieben Millionen Exemplare verkauft wurden und die nun bei Schweizer Optikern erhältlich sind, verfügen über einen Rahmen mit integrierter Kamera und integriertem Mikrofon, der von einer gewöhnlichen Brille nicht zu unterscheiden ist. Sie ermöglichen es, von anderen Personen unbemerkt und kontinuierlich Ton- und Bildaufnahmen zu machen. Jüngste Enthüllungen haben gezeigt, dass intime Bilder, die ohne Wissen der Betroffenen aufgenommen wurden – darunter Nacktszenen und besonders schützenswerte Personendaten –, für KI-Trainingszwecke an Subunternehmen weitergeleitet wurden. Der Hersteller plant zudem, die Gesichtserkennung zu integrieren. Eine neue Generation mit integriertem Bildschirm und Gestensteuerung ist in den Vereinigten Staaten bereits auf dem Markt und könnte bald auch in der Schweiz erhältlich sein. Das Schweizer Recht (Datenschutz, Schutz der Persönlichkeit, Strafbestimmungen zu Verletzungen der Privatsphäre) wurde mit Blick auf einen lokal begrenzten und wahrnehmbaren Voyeurismus konzipiert. Doch diese Technologien machen Voyeurismus allgegenwärtig, unsichtbar und sofort weltweit verbreitbar. Die Bü…</t>
+          <t>TEXT: Au vu de la forte hausse des cyberattaques d'origine étrangère contre des personnes physiques et morales en Suisse, je pose les questions suivantes au Conseil fédéral : 1. Y a-t-il une bonne coopération avec les autorités pénales étrangères lorsque les enquêtes de police sur des plaintes pénales déposées par des victimes suisses révèlent que les malfaiteurs opèrent de manière ciblée depuis l'étranger ? 2. Y a-t-il des pays qui ne coopèrent pas suffisamment avec la Suisse et qui sont donc souvent utilisés comme base par les cybercriminels ? 3. À combien le Conseil fédéral estime-t-il le nombre de cas où il est impossible de déterminer où se trouvent les auteurs ? 4. La présente interpellation fait écho aux cyberattaques menées depuis des mois contre des clients de PostFinance et d'autres entreprises suisses, qui, attirés par un site Internet falsifié (hameçonnage), permettent aux malfaiteurs d'accéder directement à leurs comptes et dépôts. Le Ministère public de la Confédération, chargé de l'enquête, a pu remonter la trace des auteurs jusqu'en Inde, à qui les cas traités ont été transmis pour qu'elle les poursuive. Le Conseil fédéral peut-il donner des informations plus détail…</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr"/>
@@ -973,11 +969,11 @@
         <v>16</v>
       </c>
       <c r="B17" t="n">
-        <v>156561</v>
+        <v>65590</v>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Verbot der Verwendung von Landessprachen bei nichtgewerbsmässigen Flügen. Warum lassen die vorübergehenden Ausnahmebestimmungen auf sich warten?</t>
+          <t>Velomitnahme im Zug, auch auf den Nachtzuglinien</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -987,8 +983,8 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Im Juni 2019 wurde das Monopol der englischen Sprache eingeführt, jedoch nicht für alle Flugplätze im Land, so etwa nicht für la Chaux-de-Fonds. Inzwischen wurde beschlossen, wieder zur Mehrsprachigkeit zurückzukehren. In seiner Antwort auf meine Frage 19.5691 sagte der Bundesrat, dass das BAZL neue Ausnahmen prüfe. Er will aber vorderhand nichts entscheiden und verweist auf hängige Rekurse. Sitten und Payerne sind in erster Linie betroffen. Was unternimmt der Bundesrat, damit alle Flugplätze gleich und gerecht behandelt werden und die verlangten Ausnahmen sofort gewährt werden können?
-ANSWER: Die Antwort des Bundesrates existiert nur in französischer Sprache. (Bitte wechseln Sie auf der Homepage oben rechts die Sprache)</t>
+          <t>TEXT: Der Bundesrat wird beauftragt, sicher zu stellen, dass 1. Velos auf jeder Zuglinie in der Schweiz und ohne Reservation mitgenommen werden können 2. Die Velomitnahme auch auf den geplanten Nachtzügen und auf den internationalen Linien möglich wird.
+REASONING: Auf den internationalen Zügen, die auch im Binnenverkehr der Schweiz Zugverbindungen sicherstellen, kann das Fahrrad nur noch mit Reservation mitgenommen werden. Die Reservation kann aber nicht in der SBB-App getätigt werden, sondern muss am Schalter gelöst werden und kostet 5 Franken. Ein Kauf im Zug ist manchmal möglich, der Preis dort 10 Franken. Dies ist nur die Reservation, das Veloticket kommt hinzu. Viele Personen möchten mit dem Velo reisen, sei es im Alltag oder auch in den Ferien. Gerade dieses Jahr haben wir gesehen, dass Ferien in der Schweiz für viele eine Option ist. Nachhaltiger Ferien machen und nachhaltiger Reisen ist die Zukunft. So sieht auch die Nachtzugnachfrage aus. Die Zahl der Fahrgäste in Nachtzügen ist im vergangenen Jahr um 25 Prozent gestiegen. Dies ist ein Trend, der der Notwendigkeit Rechnung trägt, die Auswirkungen unserer Mobilität auf die Umwelt und das Klima zu verringern. Die rasche Ent…</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr"/>
@@ -999,11 +995,11 @@
         <v>17</v>
       </c>
       <c r="B18" t="n">
-        <v>201868</v>
+        <v>67184</v>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Coopération internationale des autorités pénales dans la lutte contre la cybercriminalité</t>
+          <t>Dazit e controllo delle frontiere</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -1013,7 +1009,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Au vu de la forte hausse des cyberattaques d'origine étrangère contre des personnes physiques et morales en Suisse, je pose les questions suivantes au Conseil fédéral : 1. Y a-t-il une bonne coopération avec les autorités pénales étrangères lorsque les enquêtes de police sur des plaintes pénales déposées par des victimes suisses révèlent que les malfaiteurs opèrent de manière ciblée depuis l'étranger ? 2. Y a-t-il des pays qui ne coopèrent pas suffisamment avec la Suisse et qui sont donc souvent utilisés comme base par les cybercriminels ? 3. À combien le Conseil fédéral estime-t-il le nombre de cas où il est impossible de déterminer où se trouvent les auteurs ? 4. La présente interpellation fait écho aux cyberattaques menées depuis des mois contre des clients de PostFinance et d'autres entreprises suisses, qui, attirés par un site Internet falsifié (hameçonnage), permettent aux malfaiteurs d'accéder directement à leurs comptes et dépôts. Le Ministère public de la Confédération, chargé de l'enquête, a pu remonter la trace des auteurs jusqu'en Inde, à qui les cas traités ont été transmis pour qu'elle les poursuive. Le Conseil fédéral peut-il donner des informations plus détail…</t>
+          <t>TEXT: Nel quadro del Rapporto del Consiglio federale in adempimento del postulato 17.4177 del 14.12.2017, l'approccio risulta essere piuttosto teorico e poco orientato alla reale operatività quotidiana del personale che opera ai valichi ferroviari. In considerazione degli importanti cambiamenti previsti, è opportuno conoscere maggiori informazioni operative che toccano la quotidianità dei dipendenti e dei cittadini. 1. Sono previsti investimenti infrastrutturali utili alle attività di controllo, soprattutto merci, in tutte le stazioni di confine (Basilea, Buchs, Vallorbe, Ginevra, Domodossola, Luino, Chiasso)? Sono di competenza dell'AfD o direttamente delle FFS? Come è garantito il finanziamento e il coordinamento delle procedure? 2. Si prevede di installare scanner fissi per il traffico ferroviario merci? In quali stazioni? 3. La riforma in corso prevede un aggiornamento degli accordi internazionali vigenti per le stazioni di frontiera? Quali accordi si prevede di aggiornare con le rispettive controparti? 4. Il progetto Dazit prevede un coinvolgimento attivo - per ottimizzare i flussi di lavoro e i controlli - delle aziende ferroviarie svizzere leader nel traffico delle merci? Se…</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr"/>
@@ -1024,11 +1020,11 @@
         <v>18</v>
       </c>
       <c r="B19" t="n">
-        <v>66100</v>
+        <v>153337</v>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Vaterschaftsurlaub. Beeinflussung der Volksabstimmung durch den Bund?</t>
+          <t>Semplificare e velocizzare i mostri burocratici rappresentati dai permessi nel quadro dei contingenti per cittadini di Stati terzi e dai permessi di soggiorno di breve durata (permessi L) per cittadini UE/AELS</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -1038,8 +1034,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Anfang Mai 2020 wurde darüber berichtet, dass die Post, Postfinance und PostAuto Schweiz AG ab 2021 den Vätern neu 4 Wochen Vaterschaftsurlaub gewähren. In kürze nimmt das Volk in einer Referendumsabstimmung zum staatlichen Vaterschaftsurlaub von 2 Wochen Stellung. Wie beurteilt der Bundesrat seine Rolle und seine Wirkung im Abstimmungskampf, wenn ein Unternehmen des Bundes - der Bund ist alleiniger Aktionär der Schweizerischen Post AG - kurz vor dem Urnengang einen solchen Entscheid fällt?
-ANSWER: Die Post hat kürzlich den Abschluss der Verhandlungen mit syndicom und transfair zum neuen Dach-Gesamtarbeitsvertrag der Post bekanntgegeben. Dieser GAV tritt per 1. Januar 2021 in Kraft und beinhaltet neu einen Vaterschaftsurlaub von vier Wochen (bisher 2 Wochen). Die Personalpolitik liegt uneingeschränkt in der Verantwortung der bundesnahen Unternehmen. Dennoch formuliert der Bundesrat in seinen strategischen Zielvorgaben auch personalpolitische Ziele und trägt damit dem Umstand Rechnung, dass diese Unternehmen wichtige Arbeitgeber sind und eine Vorbildrolle einnehmen. Der Bundesrat mischt sich aber nicht in die Sozialpartnerschaft ein und beschränkt die personalpolitischen Ziel…</t>
+          <t>TEXT: Per le imprese che desiderano assumere lavoratori provenienti da Stati terzi, le procedure per ottenere i relativi permessi sono complesse e impegnative. La procedura stessa può facilmente richiedere sei mesi. Le grandi imprese dispongono di apposite divisioni o incaricano società di consulenza specializzate. Per ragioni di ordine finanziario, le PMI e le start-up non dispongono di questa possibilità. I tempi di trattamento per i permessi L per cittadini UE/AELS sono troppo lunghi e variano considerevolmente da un Cantone all'altro. In teoria il trattamento può essere eseguito in pochi secondi in quanto interamente standardizzato; eventuali eccezioni possono essere sottoposte a un responsabile cantonale. Uno sportello unico digitale nazionale per le PMI ridurrebbe notevolmente la complessità, abbreviando la durata delle procedure. Con EasyGov esiste già una piattaforma operativa approntata esattamente per procedure di questo tipo. Estendendo EasyGov ai permessi di lavoro si offrirebbe alle start-up e alle PMI una reale possibilità di presentare domande in maniera semplice e con procedure digitali ben condotte. Alla luce di quanto precede, invito il Consiglio federale a rispon…</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr"/>
@@ -1050,11 +1045,11 @@
         <v>19</v>
       </c>
       <c r="B20" t="n">
-        <v>155280</v>
+        <v>213693</v>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Rechtshilfe gegenüber Griechenland. Zu neuen Ersuchen ermuntern</t>
+          <t>Entreprises plates-formes et économie à la tâche ou "gig economy". Mieux protéger les travailleurs indépendants</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -1064,8 +1059,8 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Das Bundesstrafgericht und danach das Bundesgericht haben vorläufig die Herausgabe von Bankdaten an die griechischen Strafverfolgungsbehörden durch die Bundesanwaltschaft blockiert. Der Entscheid schockiert in einem krassen Korruptionsfall, der im Jahr 2013 bereits zur Verurteilung des ehemaligen Verteidigungsministers Tsochatzopoulos zu einer Freiheitsstrafe von 20 Jahren führte. Als Grund nannten die Gerichte den Verdacht, dass das Rechtshilfeersuchen auf den Bankdaten der Falciani-Liste beruhe. Wird das Bundesamt für Justiz den griechischen Behörden nahelegen, ihr Anliegen noch einmal vorzubringen und dabei zu belegen, dass das Ersuchen nicht auf den Daten der Falciani-Liste beruht?
-ANSWER: Die Antwort des Bundesrates existiert nur in französischer Sprache. (Bitte wechseln Sie auf der Homepage oben rechts die Sprache)</t>
+          <t>TEXT: Le Conseil fédéral est chargé d'élaborer un rapport dans lequel il propose des pistes pour améliorer la protection sociale des indépendants travaillant à la tâche. Il devra en particulier examiner comment les entreprises plateformes pourraient contribuer à assurer une meilleure couverture sociale aux personnes participant à cette économie dite collaborative ou de partage.
+REASONING: Déjà en plein essor, les modèles de travail flexible vont se développer encore sous l'effet d'une numérisation galopante. Ils consistent à proposer de brèves missions à des indépendants ou des personnes employées à temps très partiel. On peut s'attendre à ce que la tendance à l'ubérisation, dominée par les entreprises plateformes, prenne encore de l'ampleur. Cette évolution propose de nouveaux modèles d'entreprises mais elle ouvre aussi de nouvelles possibilités qui, à certaines conditions, peuvent tout à fait séduire les indépendants. Le problème est que ceux-ci se voient moins bien protégés contre les risques sociaux. Les acteurs politiques sont donc appelés à examiner les conditions de cette nouvelle économie et à les adapter si nécessaire afin qu'elle ne soit pas synonyme de réduction de la p…</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr"/>
@@ -1076,11 +1071,11 @@
         <v>20</v>
       </c>
       <c r="B21" t="n">
-        <v>69536</v>
+        <v>158836</v>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Nouvelle édition des Principes directeurs de l'OCDE à l'intention des entreprises multinationales</t>
+          <t>85 Prozent der cannabishaltigen Lebensmittel mit zu hohem THC-Gehalt</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -1090,7 +1085,8 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Le 8 juin, l'OCDE a, lors de sa conférence ministérielle (qui s'est tenue à Paris et à laquelle la Suisse participait), adopté une nouvelle édition de ses principes directeurs à l’intention des entreprises multinationales. La révision visait à intégrer dans les principes directeurs des précisions concernant le devoir de diligence, précisions qui avaient été élaborées dans le cadre de différents guides depuis la dernière révision (laquelle datait de 2011). 1. Les ministres de l'OCDE ont exigé, dans leurs précédentes recommandations relatives au rôle des États (OECD/LEGAL/0486), que les États membres édictent les lois nécessaires et vérifient régulièrement que celles-ci ne contiennent pas de lacunes, notamment en lien avec la mise en œuvre effective de ces lois et l'accès aux voies de recours. Ils recommandent aux États membres de combler les lacunes existantes en légiférant et de veiller à ce que les normes qu'ils édictent soient conformes aux nouveaux principes directeurs. Quelles mesures le Conseil fédéral a-t-il prises pour mettre en œuvre cette recommandation ? 2. La nouvelle édition des principes directeurs de l'OCDE prévoit un renforcement substantiel du devoir de dilige…</t>
+          <t>TEXT: Die Kantonschemiker der Schweiz haben 2021 in einer gemeinsamen Kampagne Lebensmittel, die Cannabis oder Cannabisextrakte mit zu hohem THC-Gehalt, sowie CBD (Cannabidiol) enthielten, kontrolliert. Von 100 untersuchten Produkten waren 85 zu beanstanden. Hier zeigen sich die Folgen der Gesetzeslücke, welche durch den legalen CBD-Hanfanbau im Jahr 2016 entstanden ist. Fragen: 1. Was waren die Folgen für Konsumentinnen und Konsumenten, welche Produkte mit zu hohem THC-Gehalte oder mit nicht bewilligten Hanfextrakte - die mit einem Abgabeverbot oder Rückruf belegt wurden - eingenommen oder geraucht hatten? 2. Was gedenkt der Bundesrat zum Schutz der Konsumentinnen und Konsumenten zu unternehmen? 3. Welche Gesetzesergänzungen sieht der Bundesrat vor, damit keine Produkte mit zu hohen THC-Werten verkauft werden können? 4. Welche Firmen und Verkaufsstellen wurden wie hoch gebüsst?
+ANSWER: Cannabis oder Hanf enthält natürlicherweise Cannabinoide; die bekanntesten sind THC (trans-delta-9-Tetrahydrocannabinol) und CBD (Cannabidiol). THC erzeugt im Gegensatz zu CBD psychotrope Wirkungen. 1. Der Bundesrat hat keine konkreten Informationen über mögliche Folgen für Konsumentinnen und Konsu…</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr"/>
@@ -1101,11 +1097,11 @@
         <v>21</v>
       </c>
       <c r="B22" t="n">
-        <v>65791</v>
+        <v>71058</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Conoscere meglio il bullismo in Svizzera per proteggere meglio i bambini</t>
+          <t>Kann die Post einen Beitrag zur digitalen Inklusion leisten?</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -1115,8 +1111,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Il Consiglio federale è incaricato di redigere un rapporto sul bullismo che permetta di ottenere i dati quantitativi e qualitativi necessari per mettere a punto misure contro la reiterazione delle violenze verbali, fisiche e piscologiche in ambito scolastico. Il rapporto conterrà in particolare: 1. alcune statistiche specifiche sul bullismo in Svizzera, 2. un bilancio degli attuali strumenti di sostegno della Confederazione, 3. un elenco esaustivo delle misure contro il bullismo messe in campo dalla Confederazione e dai Cantoni, 4. una valutazione della possibilità di predisporre degli aiuti per finanziare misure di prevenzione del bullismo, in analogia con le misure finanziarie varate per contrastare la violenza sulle donne e la violenza domestica.
-REASONING: Il bullismo nelle scuole è un problema sociale spesso banalizzato ma ampiamente diffuso e con risvolti molto pesanti. Le persone bullizzate, infatti, vengono minate nella loro autostima e corrono un rischio maggiore di cadere in depressione e sviluppare comportamenti antisociali, sintomi psicotici e persino idee suicidarie. Dall'altro lato le persone che commettono bullismo possono essere affette da disturbi psicologic…</t>
+          <t>TEXT: Verschiedene Studien wie beispielsweise der Digitalbarometer 2024 der Mobiliar haben festgestellt, dass fast ein Drittel der Bevölkerung nicht über grundlegende digitale Kompetenzen verfügt. Dabei gibt es signifikante Unterschiede nach Alter, Einkommen und Bildung. Auch wenn das Alter bei den digitalen Kompetenzen eine Rolle spielt, sind es beileibe nicht nur ältere Menschen, die Mühe haben, digitale Anwendungen wie beispielsweise E-Banking, Billetkäufe oder digitale Behördengänge zu nutzen. Dies ist oft auch mit Scham verbunden. Teilweise werden auch die eigenen Fähigkeiten überschätzt, gerade bei jüngeren Menschen. Da immer mehr Dinge des täglichen Lebens digitalisiert werden, stellt die mangelnde digitale Kompetenz ein zunehmendes Problem dar. In diesem Zusammenhang bitte ich den Bundesrat um die Beantwortung folgender Fragen: Wie schätzt der Bundesrat das Problem der fehlenden digitalen Kompetenzen ein und wie könnten diese verbessert werden? Auch Leistungen der öffentlichen Hand oder beispielsweise von bundesnahen Betrieben werden immer häufiger digitalisiert und teilweise nur noch digital angeboten. Wie kann sichergestellt werden, dass alle Personen Zugang zu diesen Lei…</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr"/>
@@ -1127,11 +1122,11 @@
         <v>22</v>
       </c>
       <c r="B23" t="n">
-        <v>214635</v>
+        <v>68353</v>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Transparence de la publicité politique diffusée sur les médias sociaux</t>
+          <t>Ablösung von Polycom durch ein mobiles Sicherheitsnetz. Wer übernimmt die Führung?</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
@@ -1141,8 +1136,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Le Conseil fédéral est chargé de présenter un projet de loi qui permettra aux utilisateurs de reconnaître en tant que telle la publicité politique dans les médias.
-REASONING: Dans sa réponse à l'ip. 21.4086, le Conseil fédéral déclare que " pour le moment, les éventuelles conséquences négatives [de la publicité politique numérique] sur la formation de l'opinion publique devraient être négligeables ". Simultanément, il reconnaît que les plateformes de communication numériques jouent " un rôle de plus en plus important " (71 % de la population suisse les ont utilisées en 2019) et " qu'elles revêtent une importance croissante pour la formation de l'opinion ". Le rapport du Conseil fédéral sur l'activité des opérateurs de plateformes numériques reconnaît en outre que le manque de transparence de la publicité politique sur ces plateformes est problématique. Il semble dès lors opportun de régler la publicité politique sur les plateformes numériques tant qu'elle n'est pas encore très répandue et avant qu'elle ne devienne effectivement problématique. Toute la publicité diffusée sur les médias sociaux devraient être signalée comme telle, afin que tous les utilisateurs comprennent qu'…</t>
+          <t>TEXT: Das Sicherheitsfunknetz Polycom ist am Ende seiner Lebensdauer und wird in den nächsten Jahren abgelöst werden müssen. Die Ablösung durch ein neues mobiles Sicherheitsnetz (MSK) ist einigermassen dringlich, da Polycom zunehmend instabil ist. Die Erstellung dieses neuen Mobilfunknetzes ist nötig, da insbesondere bei Grosseinsätzen eine breitbandige Kommunikation wichtig ist, die den Einsatzkräften vor Ort einen Zugriff auf einsatzrelevante Daten bietet; das muss auch bei einer Überlastung des privaten Mobilfunknetzes funktionieren. Ich bitte den Bundesrat in diesem Kontext um die Beantwortung folgender Fragen: 1. 2020 hat der Bundesrat ein Pilotprojekt ermöglicht. Was sind die Lehren aus dem Pilotprojekt? 2. Das Bundesamt für Bevölkerungsschutz (BABS) hat kommuniziert, dass die Auftragslage für die Durchführung des Projekts MSK unklar sei. Ist der Bundesrat der Ansicht, dass es eine Bundesaufgabe ist, die Erstellung des mobile Sicherheitsfunknetz anzuführen? Falls nicht, wer soll diese wichtige Aufgabe erfüllen? 3. Das BABS hat kommuniziert, dass die Ressourcen für ein solches Projekt nicht vorhanden seien. Wie viele Personen (%) sind zurzeit innerhalb des BABS mit der Vorbere…</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr"/>
@@ -1153,11 +1147,11 @@
         <v>23</v>
       </c>
       <c r="B24" t="n">
-        <v>64898</v>
+        <v>215214</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Modification de l'article 697l du code des obligations et accès à liste des ayants droit économiques</t>
+          <t>TVA. État des lieux de la nouvelle imposition des plateformes numériques</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -1167,7 +1161,8 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>TEXT: La loi fédérale du 21 juin 2019 sur la mise en oeuvre des recommandations du Forum mondial sur la transparence et l'échange de renseignements à des fins fiscales entraîne la disparition des actions au porteur. L'art. 697l du code des obligations (CO) est simplifié en conséquence et ne prévoit plus pour la société que l'obligation de tenir une liste des ayants droit économiques qui lui ont été annoncés. Conformément à la recommandation 24 du GAFI, l'art. 697l, al. 4, CO prévoit que la liste doit être tenue de manière à ce qu'il soit possible d'y accéder en tout temps en Suisse. La loi ne règle toutefois pas qui peut accéder à la liste. Le message concernant la mise en oeuvre des recommandations du GAFI révisées en 2012 n'imposait pas au conseil d'administration d'une société suisse de fournir de telles listes à l'autorité suisse compétente, sauf dans le cas de vérifications particulières dans le cadre d'une enquête du Ministère public, dans le domaine du droit pénal administratif ou en cas d'infraction fiscale (fraude fiscale). L'Administration fédérale des contributions (AFC) procède actuellement à la collecte systématique de ces listes par l'envoi d'une lettre-type aux contr…</t>
+          <t>TEXT: Depuis le 1er janvier 2025, les plateformes numériques sont assujetties à la TVA en Suisse. Comment le nombre d’inscriptions à la TVA et de taxations fiscales a-t-il évolué depuis l’instauration des nouvelles règles ? Comment l’augmentation des inscriptions à la TVA se répartit-elle entre les entreprises nationales et les entreprises étrangères ? Quelles mesures l’AFC prend-elle cette année pour s’assurer que toutes les entreprises disposant d’un IDE remplissent bel et bien leurs obligations en matière de TVA ?
+ANSWER: Questions 1 et 2 : les inscriptions à la TVA en tant que plateforme au sens de l’art. 20a, al. 1 de la loi fédérale du 12 juin 2009 sur la taxe sur la valeur ajoutée (LTVA ; RS 641.20) se répartissent à mi-mars entre vingt plateformes sises à l’étranger et quatre plateformes sises sur le territoire suisse. Toutefois, ces chiffres doivent être interprétés avec prudence pour les raisons suivantes : l’inscription en ligne en tant que plateforme pour les nouveaux assujettis n’est disponible que depuis novembre 2024 pour les plateformes étrangères et mars 2025 pour celles situées sur le territoire suisse ; par ailleurs, certaines entreprises ont pu omettre de décla…</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr"/>
@@ -1178,11 +1173,11 @@
         <v>24</v>
       </c>
       <c r="B25" t="n">
-        <v>235223</v>
+        <v>155052</v>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Le caratteristiche e i dispositivi di sicurezza del sistema svizzero di verifica dei medicamenti (SMVS) sono inadatti per il monitoraggio degli agenti terapeutici?</t>
+          <t>Contributi per procedimenti di spandimento a basse emissioni fino al 2021</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
@@ -1192,8 +1187,8 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Il Consiglio federale condivide l’opinione secondo cui non esiste una base legale che consenta di attuare mediante l’articolo 17a LATer, approvato ma non in vigore, la gestione digitale delle penurie di medicamenti per uso umano richiesta dalla mozione Ettlin e che è necessario elaborare una specifica base legale all’interno della LATer? L’introduzione del SMVS fa parte delle otto raccomandazioni proposte al Consiglio federale dalla task force per gli agenti terapeutici? Il monitoraggio necessita di un’ulteriore base legale o è sufficiente il sistema di preallarme dell’Ufficio federale dell’approvvigionamento economico del Paese (UFAE)? È vero che l’UFAE non intende servirsi del SMVS per la gestione digitale delle penurie di medicamenti per uso umano? Il Consiglio federale ritiene che esista un rischio significativo che in Svizzera entrino in commercio medicamenti contraffatti? Se sì, in quali casi? Il Consiglio federale condivide la posizione dei fornitori di servizi, secondo cui i costi di attuazione dei requisiti SMVS sono troppo elevati rispetto ai potenziali benefici?
-REASONING: Il 26 settembre 2023 il Parlamento ha approvato, con un adattamento del punto 2, la mozione …</t>
+          <t>TEXT: Il Consiglio federale è incaricato di modificare l'ordinanza concernente i pagamenti diretti nell'agricoltura (OPD; RS 910.13) in modo che i contributi per lo spandimento a basse emissioni di concimi liquidi aziendali e ottenuti dal riciclaggio siano versati fino al 2021 (invece del 2019). Una minoranza (Schneider Schüttel, Bendahan, Brélaz, Gmür Alois, Gschwind, Gysi, Hadorn, Kiener Nellen, Meyer Mattea) propone di respingere la mozione.
+ANSWER: A partire dal 2022 l'utilizzo di procedimenti di spandimento a basse emissioni sarà prescritto in virtù del diritto ambientale nell'ordinanza contro l'inquinamento atmosferico (OIAt) e, sempre dal 2022, diventerà parte integrante della prova che le esigenze ecologiche sono rispettate, la cui fornitura è indennizzata mediante pagamenti diretti. Non è quindi possibile mantenere i contributi oltre il 2021. Il Consiglio federale propone di accogliere la mozione.</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr"/>
@@ -1204,11 +1199,11 @@
         <v>25</v>
       </c>
       <c r="B26" t="n">
-        <v>337367</v>
+        <v>64903</v>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Legge sul sostegno alla banda larga (LSBL)</t>
+          <t>Si renda obbligatoria l'assicurazione malattia svizzera per i lavoratori frontalieri</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
@@ -1216,7 +1211,11 @@
           <t>open</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Secondo l'Ordinanza sull'assicurazione malattie 832.102 all'Art. 3 Frontalieri "1 A loro domanda vengono assoggettati all'assicurazione svizzera i frontalieri che esercitano un'attività lucrativa in Svizzera non soggetti all'obbligo d'assicurazione ai sensi dell'articolo 1 capoverso 2 lettera d ed e nonché i loro familiari, purché non esercitino all'estero un'attività lucrativa per cui siano tenuti ad assicurarsi contro le malattie." Nella pratica i lavoratori frontalieri possono esercitare il diritto di opzione, o vengono assoggettati all'assicurazione svizzera, o rimangono assicurati nel paese di residenza. È ipotizzabile che la maggior parte dei lavoratori frontalieri non sono assicurati in Svizzera per ragioni di costo e questo, a parità di salario, permette loro di avere un reddito disponibile molto più alto dei lavoratori svizzeri in quanto, ad esempio in Italia, l'assicurazione malattia è di fatto gratuita. Due operai, uno svizzero e l'altro frontaliere con residenza in Italia, entrambe con un salario lordo di 5000 franchi, per il frontaliere oltre al vantaggio economico di vivere in Italia - dove il costo della vita è di molto inferiore - ha pure il vantaggio di non d…</t>
+        </is>
+      </c>
       <c r="F26" s="5" t="inlineStr"/>
       <c r="G26" s="5" t="inlineStr"/>
     </row>
@@ -1225,11 +1224,11 @@
         <v>26</v>
       </c>
       <c r="B27" t="n">
-        <v>214312</v>
+        <v>204320</v>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Centovalliexpress. Quo vadis?</t>
+          <t>Quale impatto avrà la digitalizzazione sulla nostra salute?</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
@@ -1239,7 +1238,8 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Abbiamo recentemente potuto prendere atto con piacere dell'ordinazione da parte delle FART di nuovi elettrotreni per 94 mio a dimostrazione dell'impegno svizzero a voler mantenere viva la linea Locarno Domodossola anche per il traffico internazionale, sono anche previsti potenziamenti sul segmento svizzero finanziati nell'ambito Prossif 2035. Purtroppo questi investimenti non fanno da pari con il servizio offerto che è diventato negli anni sempre più scadente, oltretutto tassato extra sui convogli "panoramici" della SSIF . Tempi di percorrenza in crescita, infrastruttura ferroviaria sul segmento italiano con tratte percorse a passo d'uomo o quasi. Tempi di percorrenza attualmente attorno a 1h50' (erano a 1h45' nel 2010, stessi tempi negli anni 80 del secolo scorso prima dell'interramento a Locarno e con trasbordo per frana a Ré), in generale il Centovalliexpress percorre Locarno Domodossola a una velocità media inferiore a 30 km/h. Le ultime corse partono alle 17:45 da Locarno alle 19 da Domodossola! Nel 2010 l'Ata aveva presentato un progetto per la sistemazione della tratta che permetteva di ridurre i tempi fino a circa 1h30'. Questa linea rappresenterebbe un ideale collega…</t>
+          <t>TEXT: Il Consiglio federale è incaricato di presentare un rapporto allo scopo di analizzare l'impatto e gli effetti della digitalizzazione della nostra società sulla salute umana. Il rapporto dovrà contenere una serie di provvedimenti destinati a conciliare lo sviluppo della digitalizzazione con la tutela della salute e del benessere della popolazione, in particolar modo dei giovani in formazione.
+REASONING: Da parecchi anni, il Consiglio federale pubblica rapporti sulle opportunità offerte dalla digitalizzazione per il nostro sistema di formazione e la nostra società in generale. È assolutamente auspicabile trarre il massimo beneficio possibile dalla transizione digitale, ma non a scapito della salute della popolazione. Un rapporto di Educa del 2021 fa notare che l'impiego di risorse digitali ha conseguenze sulla salute o sul benessere soggettivo degli allievi o degli insegnanti. Il rapporto sottolinea inoltre che, secondo alcuni studi trasversali condotti nel Cantone di Vaud, i giovani che trascorrono più tempo davanti allo schermo accusano più spesso problemi di salute come mal di schiena, problemi posturali, sovrappeso e carenza di sonno. Inoltre, trascorrere molte ore davanti…</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr"/>
@@ -1250,11 +1250,11 @@
         <v>27</v>
       </c>
       <c r="B28" t="n">
-        <v>156261</v>
+        <v>155792</v>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Istituzione delle basi legali per un'attività parlamentare digitale e per la partecipazione digitale all'attività parlamentare fisica</t>
+          <t>Pour plus de force aux cantons</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
@@ -1264,8 +1264,8 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Occorre istituire le basi legali per un'attività parlamentare digitale e per la partecipazione digitale all'attività parlamentare fisica.
-REASONING: Con la crisi del Coronavirus l'attività parlamentare si è arrestata. La sessione primaverile è stata interrotta anzitempo e anche le Commissioni, su ordine degli Uffici delle rispettive Camere, non hanno più potuto riunirsi. Da molte parti ci si è chiesti come sarebbe stato possibile mantenere l'attività delle Camere in caso di crisi prolungata. La Costituzione prevede esplicitamente che i parlamentari siano presenti fisicamente e la legge sul Parlamento stabilisce che le Camere si riuniscono a Berna. Una perizia dell'Università di Zurigo giunge tuttavia alla conclusione che un funzionamento digitale del Parlamento sia del tutto possibile. I requisiti tecnici dovrebbero ovviamente essere elevati al fine di escludere qualsiasi abuso, fra cui la partecipazione di persone non autorizzate in vece dei membri preposti. Anche le condizioni per lo svolgimento dell'attività parlamentare dovranno essere definite severamente e valere solo in situazioni eccezionali, oltre ad essere assoggettate all'obbligo di autorizzazione (p. es. da parte…</t>
+          <t>TEXT: Les Autorités fédérales sont invitées à modifier l'article 16 al. 6 de la loi fédérale du 26 septembre 2014 concernant la surveillance de l'assurance-maladie sociale (LSAMal ; RS 832.12) comme il suit : Avant l'approbation des tarifs, les cantons peuvent donner leur avis aux assureurs et à l'autorité de surveillance sur l'évaluation des coûts et sur les tarifs de primes prévues pour leur territoire, à la condition que ces échanges ne prolongent pas la procédure d'approbation. Les cantons peuvent obtenir les informations nécessaires auprès des assureurs et de l'autorité de surveillance. Ces informations ne peuvent être ni rendues publiques ni transmises à des tiers.
+REASONING: 1. Introduction Le canton de Fribourg soumet à l'Assemblée fédérale trois initiatives autant de modifications de la loi fédérale sur la surveillance de l'assurance-maladie du 26 septembre 2014 (LSAMal). Les initiatives visent toutes trois à assurer une meilleure adéquation des primes d'assurance-maladie par rapport aux coûts des prestations qu'elles couvrent. Initiées par le canton du Tessin, plusieurs autres cantons ont adopté ou sont en train d'adopter le dépôt d'initiatives similaires. En résumé, la …</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr"/>
@@ -1276,11 +1276,11 @@
         <v>28</v>
       </c>
       <c r="B29" t="n">
-        <v>337362</v>
+        <v>235727</v>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Commissioni extraparlamentari. Riorganizzazione nel quadro della verifica 2025</t>
+          <t>Combien la Suisse a-t-elle dépensé pour aider l'Ukraine?</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
@@ -1288,7 +1288,12 @@
           <t>open</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr"/>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Le chef du DFAE Ignazio Cassis a récemment annoncé le versement de 1,8 milliard de francs d'aide supplémentaire à l'Ukraine d'ici à 2028, une somme énorme qu'il justifie par le fait que la Suisse doit " faire sa part ". Or, cet argument est des plus maladroits puisque la Suisse a déjà fait bien plus que sa part - et pas seulement du point de vue financier - depuis le début d'une guerre dont elle n'est pourtant aucunement responsable. L'ampleur des montants déboursés pour aider l'Ukraine appelle la plus grande transparence, laquelle n'est pour l'heure absolument pas garantie. Je prie dès lors le Conseil fédéral de répondre aux questions suivantes : - Combien la Suisse a-t-elle dépensé jusqu'ici pour l'accueil des réfugiés ukrainiens (en tenant compte des coûts liés à la couverture des soins médicaux) ? - À combien se monte l'aide versée par la Suisse à l'Ukraine sous différentes formes ? - À combien se monte l'aide versée par les autres pays en lien avec l'invasion de l'Ukraine ? - Le Conseil fédéral a-t-il l'intention de mettre à jour et de publier régulièrement (par ex. tous les six mois) les chiffres demandés ci-dessus ?
+ANSWER: L’aide versée par la Confédération depuis le…</t>
+        </is>
+      </c>
       <c r="F29" s="5" t="inlineStr"/>
       <c r="G29" s="5" t="inlineStr"/>
     </row>
@@ -1297,11 +1302,11 @@
         <v>29</v>
       </c>
       <c r="B30" t="n">
-        <v>153188</v>
+        <v>63574</v>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Stärkung der Volksrechte. Unterschriftensammlung für Initiativen und Referenden im Internet</t>
+          <t>Adeguamento del diritto federale agli sviluppi della tecnologia di registro distribuito. Legge federale</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
@@ -1309,12 +1314,7 @@
           <t>open</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>TEXT: Der Bundesrat wird aufgefordert, die gesetzlichen Grundlagen zu schaffen, um das elektronische Sammeln von Unterschriften für Initiativen und Referenden zu erlauben. Dazu zählt auch die Unterschrift über Touchscreens. Der Bund soll in diesem Zusammenhang die digitale Partizipation der stimmberechtigten Schweizerinnen und Schweizer im In- und Ausland stärken.
-REASONING: E-Collecting war ein fester Bestandteil der "Vote électronique"-Strategie des Bundesrates, um die Volksrechte der Schweiz zu modernisieren (vgl. BK, Strategische Planung Vote électronique, 18. März 2011). Im April 2015 kündigte der Bundesrat überraschend an, auf die Weiterführung im Bereich des E-Collectings zu verzichten. Die Folge davon ist eine Schwächung der direkten Demokratie, da wachsende Teile der Stimmberechtigten bei Unterschriftensammlungen ausgeschlossen und immer höhere finanzielle und personelle Ressourcen für die Komitees nötig werden. Eine Ergänzung des Bundesgesetzes über die politischen Rechte (BPR) soll daher digitale Unterschriften erlauben - etwa auf Touchscreens, so wie seit geraumer Zeit der Empfang von Paketen und Einschreiben bestätigt wird. Dies würde es einer breiteren Bevölkerungsgr…</t>
-        </is>
-      </c>
+      <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="5" t="inlineStr"/>
       <c r="G30" s="5" t="inlineStr"/>
     </row>
@@ -1323,11 +1323,11 @@
         <v>30</v>
       </c>
       <c r="B31" t="n">
-        <v>154613</v>
+        <v>71358</v>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Lancio del 5G in Svizzera. Onere supplementare per i cantoni. Quale compensazione da parte della Confederazione?</t>
+          <t>L’ex-ambassadeur Jean-Daniel Ruch dévoile des informations sensibles dans ses mémoires</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
@@ -1337,7 +1337,8 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Recentemente la Commissione federale delle comunicazioni (Comcom) ha attribuito nuove frequenze di radiocomunicazione a tre operatori svizzeri. I ricavi realizzati con questa operazione si aggirano sui 380 milioni di franchi e sono stati versati nelle casse federali a titolo di ricavi straordinari. Siccome le concessioni sono state attribuite per una durata di 15 anni, per i prossimi anni si prevede un numero significativo di domande di costruzione per nuove antenne. A titolo esemplificativo, nell'arco dei prossimi due a tre anni l'operatore Swisscom progetta di installare una ventina di piloni nel Cantone del Giura. Qualsiasi nuova costruzione o modifica di impianti preesistenti è sottoposta al rilascio di un'autorizzazione. L'introduzione del 5G in Svizzera implicherà pertanto inevitabilmente un incremento del carico di lavoro e costi supplementari per i Cantoni. Anche se le autorizzazioni rilasciate dalle amministrazioni cantonali sono soggette al versamento di tasse, altre prestazioni legate al trattamento di questi dossier (segnatamente i lavori generati dalle procedure di opposizione e di ricorso) sono particolarmente laboriose e non generano alcun introito. Le domande …</t>
+          <t>TEXT: Les mémoires de Jean-Daniel Ruch paraîtront le 12 juin. Il y dévoile des conversations confidentielles et secrètes (notamment des discussions menées avec des représentants turcs sur les efforts de paix concernant le conflit ukrainien). - Les (ex-)ambassadeurs ne sont-ils pas soumis au secret de fonction ? - Qui voudra encore mener des entretiens confidentiels avec la Suisse, si le contenu est ensuite dévoilé au public ? - Que fait le Conseil fédéral pour empêcher Jean-Daniel Ruch de continuer à violer son secret de fonction ?
+ANSWER: La réponse du Conseil fédéral n'existe qu'en allemand. (Veuillez changer la langue en haut à droite de la page d'accueil)</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr"/>
@@ -1348,11 +1349,11 @@
         <v>31</v>
       </c>
       <c r="B32" t="n">
-        <v>236031</v>
+        <v>297665</v>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Renvois vers l’Afghanistan. Un flop ?</t>
+          <t>Krieg im Nahen Osten (III)</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
@@ -1362,7 +1363,8 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Depuis l’automne 2024, les renvois de ressortissants afghans ont repris graduellement, mais ils se limitent pour l’instant aux personnes qui ont commis des crimes graves. En avril 2025, le Conseil fédéral a décidé d’ajuster sa pratique pour les hommes seuls qui ne présentent pas de vulnérabilités. Les conditions à remplir pour un renvoi sont les suivantes : ces hommes doivent séjourner en Suisse sans famille, être majeurs et en bonne santé et disposer en Afghanistan d’un réseau relationnel stable et solide qui leur permet de se réintégrer dans la société. On a pu lire dans la presse que cette nouvelle pratique n’avait conduit à aucun renvoi et qu’un migrant renvoyé en Afghanistan avait même dû être ramené en Suisse parce que les autorités afghanes avaient refusé de le réadmettre, à l’aéroport de Kaboul. On a appris dans le même temps que la Suisse versait à nouveau une aide au développement à l’Afghanistan, d’un montant annuel de 27 millions de francs. Je pose au Conseil fédéral les questions suivantes : Que pense-t-il des résultats de la nouvelle pratique appliquée pour le renvoi des migrants afghans qui n’ont pas le droit de rester en Suisse ? Ne considère-t-il pas que les …</t>
+          <t>TEXT: - Ist der Bundesrat inzwischen zum Schluss gekommen, dass sich die USA und Israel gemäss Art. 22a Abs. 2 Bst. a KMG in einem «internationalen bewaffneten Konflikt» befinden? - Wurde für Kriegsmaterial, dessen Ausfuhr in die betroffenen Länder bereits bewilligt wurde, eine Rücknahme und/oder Aussetzung der entsprechenden Bewilligungen verfügt? - Wird die Ausfuhr von Gütern gemäss GKG, insbesondere von besonderen militärischen Gütern, weiterhin bewilligt?
+ANSWER: Die Antwort des Bundesrates existiert nur in französischer Sprache. (Bitte wechseln Sie auf der Homepage oben rechts die Sprache)</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr"/>
@@ -1373,11 +1375,11 @@
         <v>32</v>
       </c>
       <c r="B33" t="n">
-        <v>159478</v>
+        <v>153348</v>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Étendre les compétences du SRC alors qu’il fiche les partis ?</t>
+          <t>Online-Handel prüfen, überwachen und einschränken?</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
@@ -1387,7 +1389,8 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Les médias ont révélé que le SRC continuait de collecter beaucoup trop de données et ne respectait pas les conditions de l'art. 5 LRens, qui lui interdit de rechercher et de traiter des informations relatives aux activités politiques. Cette pratique est extrêmement dommageable pour la démocratie et soulève des questions fondamentales en matière de gouvernance. - Dans ce contexte, est-il légitime de prévoir une extension des compétences du SRC ? - Le Conseil fédéral n'estimerait-il pas préférable de suspendre la révision de la LRens ?</t>
+          <t>TEXT: Immer häufiger werden Fälle bekannt, wo in der Schweiz verbotene Waffen und andere illegale Gegenstände auf ausländischen Online-Handelsplattformen gekauft und auf dem Paketweg in die Schweiz gesendet wurden. Dabei werden unter anderem Waffen in Folien eingeschweisst, um den Detektoren der Zollverwaltung eine Entdeckung zu erschweren, oder Gegenstände als Muster bezeichnet, um Zollgebühren zu vermeiden. Bislang können für solche illegalen Praktiken allerdings nur die Empfänger belangt werden. Der Bundesrat wird gebeten, folgende Fragen zu beantworten: 1. Beabsichtigt er, der Eidgenössischen Zollverwaltung die nötigen Mittel zur Verfügung zu stellen, damit die grosse Mehrheit dieser illegalen Pakete künftig aus dem Verkehr gezogen werden kann? 2. Besteht aus seiner Sicht auch die Notwendigkeit, die verantwortlichen Online-Portale und die Versender in die Verantwortung zu nehmen? 3. Kann im Rahmen von Freihandelsabkommen die beschriebene Problematik zusammen mit unseren Handelspartnern wirkungsvoll angegangen werden? 4. Welche weiteren Mittel sieht er, um den transnationalen Versand illegaler Pakete wirkungsvoll einzudämmen?
+REASONING: Die Digitalisierung ermöglicht einen imme…</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr"/>
@@ -1398,11 +1401,11 @@
         <v>33</v>
       </c>
       <c r="B34" t="n">
-        <v>67332</v>
+        <v>63757</v>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Weg von Fast Fashion, aber wie?</t>
+          <t>Revoca sistematica della cittadinanza ai "viaggiatori della jihad" con la doppia cittadinanza!</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
@@ -1412,7 +1415,8 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>TEXT: In den letzten 20 Jahren sind Textilien von einem Gebrauchsgegenstand zum Wegwerf-Artikel geworden. Die Tragedauer von Kleidern ist um 40 Prozent gesunken. Dafür hat sich die weltweite Produktion verdoppelt. Die billige und schnelllebige Fast-Fashion-Industrie hat immense Schattenseiten. Prekäre Arbeitsbedingungen und gesundheitsschädigende Umweltbelastungen prägen die globalen Lieferketten. 2018 haben deshalb das Bundesamt für Umwelt (BAFU) gemeinsam mit dem Staatssekretariat für Wirtschaft (SECO) sowie den Verbänden Swiss Textiles und amfori die Initiative "Nachhaltige Textilien Schweiz" als Multi-Stakeholder-Dialog gestartet. Daraus ist das Programm "Sustainable Textiles Switzerland 2030 (STS 2030)" entstanden, das einen wesentlichen Beitrag zur Erreichung der Nachhaltigen Entwicklungsziele (SDGs) im Schweizer Textil- und Bekleidungssektor entlang der gesamten Wertschöpfungskette leisten will. Die am Programm beteiligten Unternehmungen und Verbände setzen sich im Rahmen ihrer Eigenverantwortung in einem vorbildlichen Prozess für die Reduktion der Treibhausgasemissionen, die Förderung fairer Löhne und menschenwürdiger Arbeitsbedingungen, die Förderung innovativer Geschäftsm…</t>
+          <t>TEXT: Il Consiglio federale è incaricato di adottare le disposizioni necessarie per far applicare sistematicamente l'articolo 42 della legge sulla cittadinanza ai "viaggiatori della jihad" svizzeri con la doppia cittadinanza.
+REASONING: Sul sito della SEM https://www.sem.admin.ch/sem/it/home/themen/buergerrecht/schweizer_buergerrecht.html si legge che la revoca della cittadinanza in applicazione dell'articolo 42 LCit è concepibile solo in casi estremamente gravi, come quelli di criminali di guerra o terroristi. Nella sua risposta alla mia domanda 19.5162, il Consiglio federale ha precisato che una tale misura è possibile se la condotta della persona in questione è di grave pregiudizio agli interessi o alla buona reputazione della Svizzera. Si esige inoltre una condanna penale passata in giudicato, a meno che il perseguimento penale non possa essere portato a termine (p. es. in caso di malfunzionamento dell'apparato giudiziario). In questo contesto, il Governo ha evocato... una - sì, una sola! - procedura di revoca che, il 18 marzo 2019, era ancora soltanto avviata. Ha aggiunto che era al vaglio l'avvio di altre procedure, senza precisare quante né fornire alcuna cifra che permetta…</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr"/>
@@ -1423,11 +1427,11 @@
         <v>34</v>
       </c>
       <c r="B35" t="n">
-        <v>66800</v>
+        <v>331346</v>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Mesures contre l'immigration illégale (8/9). Systématiser l'échange des données concernant les immigrés illégaux</t>
+          <t>Reconnaissance intercantonale des attestations électroniques officielles</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -1437,8 +1441,7 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Afin de lutter durablement contre l'immigration illégale en Suisse et si possible d'y mettre un terme, il faut que l'échange des données sur les personnes concernées entre les cantons, les communes, les autorités sociales, les caisses-maladie, l'AVS, l'AI et d'autres assurances sociales devienne systématique. Il s'agit d'échanger et de comparer toutes les données relatives au statut de séjour, au lieu de domicile, à la couverture d'assurance, aux paiements des primes, aux réductions de primes, aux prestations des caisses-maladie, à l'AVS, à l'AI et à d'autres assurances sociales.
-REASONING: En fonction des estimations et des sources d'information, jusqu'à 100 000 immigrés illégaux - banalement appelés " sans-papiers " - seraient en Suisse. Afin de réduire l'attrait de notre pays à cet égard, il importe que ces personnes puissent être identifiées et renvoyées grâce à un échange systématique des données les concernant. Selon le rapport du Conseil fédéral " Pour un examen global de la problématique des sans-papiers " en réponse au postulat de la Commission des institutions politiques du Conseil national du 12 avril 2018 (18.3381), les assurances et les caisses-maladie surtout n…</t>
+          <t>TEXT: Dans le cadre du développement des services numériques cantonaux et communaux, certaines administrations délivrent désormais des attestations officielles sous forme électronique. Or, des cas concrets montrent que ces documents ne sont pas toujours reconnus par d’autres autorités. Ainsi, une attestation de domicile délivrée électroniquement par une commune valaisanne a été refusée par un état civil fribourgeois au motif que ce dernier doutait de son authenticité, faute de signature sur le document. Dans de tels cas, les autorités doivent établir a posteriori une version papier, ce qui annule les bénéfices de la démarche numérique. De telles situations nuisent à la crédibilité des services numériques, génèrent des coûts supplémentaires et freinent la transition vers une administration digitale efficace et harmonisée. Dans ce contexte, je prie le Conseil fédéral de répondre aux questions suivantes : Le Conseil fédéral a‑t‑il connaissance de cas dans lesquels des documents officiels électroniques émis par une autorité ne sont pas reconnus par une autre autorité, notamment dans un autre canton ? Quelles bases légales, quels standards ou quelles recommandations existent aujourd’hui…</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr"/>
@@ -1449,11 +1452,11 @@
         <v>35</v>
       </c>
       <c r="B36" t="n">
-        <v>331084</v>
+        <v>153262</v>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Finanzierung und Rüstungsplanung der Armee</t>
+          <t>Entità legale in Svizzera per i fornitori di servizi</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
@@ -1463,8 +1466,7 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Laut Vernehmlassungsunterlagen plant das VBS ab 2028 mit zusätzlichen jährlichen Ausgaben von 3,1 Milliarden Franken, die in den ersten Jahren durch Verschuldung des Rüstungsfonds finanziert werden sollen. 1. Finden diese zusätzlichen Milliardenausgaben Eingang in die Finanzplanung des Bundes? 2. Wie hoch ist der maximale «Bereinigungsbedarf» im Falle einer Ablehnung der Vorlage? 3. Welche Ausgaben wären von dieser «Bereinigung» betroffen? 4. Wären auch sicherheitsrelevante Ausgabenbereiche (FedPol, BACS, NDB, SEPOS usw.) von dieser «Bereinigung» betroffen? 5. In welchem Verhältnis steht die Höhe des maximalen «Bereinigungsbedarfs» zur Höhe der Ausgaben, die im Falle einer Ablehnung der Vorlage kurzfristig gekürzt werden müssen? Hat der Bundesrat das grösstmögliche Risiko berechnet und darf dieses wirklich eingegangen werden? 6. Welche Finanzmittel können für dringende Beschaffungen in den Jahren 2027, 2028 und 2029 freigespielt werden, wenn bereits bewilligte Beschaffungsvorhaben, die auf Bedrohungen mit einer geringen Eintretenswahrscheinlichkeit ausgerichtet sind, frühestens ab 2030 finanzwirksam würden?
-ANSWER: Der Bundesrat hat nach Abschluss der Vernehmlassung die Eckw…</t>
+          <t>TEXT: Le attuali mutazioni strutturali, in particolare la digitalizzazione, cambiano le carte in tavola nel settore delle telecomunicazioni. Occorre prevedere nuove misure legislative per adeguarsi a queste inevitabili evoluzioni. Le reti sociali, ad esempio Facebook o Twitter, fanno ormai parte integrante della vita quotidiana dei cittadini elvetici. Queste reti forniscono servizi al consumatore svizzero e sono pertanto presenti digitalmente sul nostro territorio. Non possiedono tuttavia necessariamente un'entità legale in Svizzera. Questa situazione è problematica. Quando si tratta di ottenere dati ai fini di un'indagine in caso di cybermobbing, diffamazione o altro la giustizia, infatti, si trova di fronte a un muro, come emerge dalla decisione del Tribunale federale 1B_185/2016, riguardante il Ministero pubblico vodese e Facebook Switzerland. I dati necessari all'inchieste possono infatti essere ottenuti soltanto con una procedura di assistenza giudiziaria internazionale, troppo lenta. Analogamente, di recente sono scoppiati casi di obsolescenza programmata. A titolo di esempio è possibile citare la situazione di Epson o di Apple. Tuttavia, per un consumatore o un gruppo di con…</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr"/>
@@ -1475,11 +1477,11 @@
         <v>36</v>
       </c>
       <c r="B37" t="n">
-        <v>62377</v>
+        <v>216073</v>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Rete nazionale di dati sicura. Credito d’impegno</t>
+          <t>Die Ausbeutung des Kongo, der Elfenbeinküste, Ecuadors oder Guineas darf keine Anpassungsvariable für Bundes- und Kantonsbudgets sein. Für eine Umverteilung von konfisziertem Eigentum und von Ersatzforderungen an die geschädigte Bevölkerung</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
@@ -1487,7 +1489,12 @@
           <t>open</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr"/>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Ich fordere den Bundesrat auf, Massnahmen zu prüfen, damit eingezogene Vermögenswerte und Ersatzforderungen, die in der Schweiz ansässigen multinationalen Unternehmen für im Ausland begangene Straftaten auferlegt werden, der Bevölkerung der Länder zugute kommen, in denen die Straftaten begangen wurden. Diese Rückzahlungen sollten nicht mehr davon abhängig gemacht werden, ob die Staaten beim Verfahren, das zu diesen Verurteilungen geführt hat, Unterstützung geleistet haben. Der Bundesrat soll zudem die Möglichkeit prüfen, diese Gelder für humanitäre Projekte oder Entwicklungs- oder Menschenrechtsprojekte zu verwenden, die von der Zivilgesellschaft dieser Länder - oder in Ermangelung solcher Programme oder ergänzend dazu - vom Bund (internationale Zusammenarbeit) oder von internationalen Regierungs- oder Nichtregierungsorganisationen durchgeführt werden.
+REASONING: In der Schweiz ansässige Unternehmen werden mit kriminellen Aktivitäten im Ausland in Verbindung gebracht. Vom Ausmass dieser Aktivitäten zeugen mehrere Strafverfahren, in die Gunvor und Glencore verwickelt sind. Das Strafrecht ermöglicht es den Justizbehörden, diese Unternehmen zusätzlich zu einer Geldstrafe zur Za…</t>
+        </is>
+      </c>
       <c r="F37" s="5" t="inlineStr"/>
       <c r="G37" s="5" t="inlineStr"/>
     </row>
@@ -1496,11 +1503,11 @@
         <v>37</v>
       </c>
       <c r="B38" t="n">
-        <v>65819</v>
+        <v>234999</v>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Chiusura dell'ultimo ufficio postale a Chêne-Bougeries</t>
+          <t>Promuovere una ricerca sostenibile grazie a un piano di abbandono degli esperimenti che causano sofferenza agli animali</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
@@ -1510,7 +1517,8 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>TEXT: La Posta sta valutando di chiudere l'ufficio postale del Comune di Chêne-Bougeries. Questo comune di oltre 11 000 abitanti perderebbe così il suo ultimo ufficio postale dopo la soppressione di quello di Conches nel 2015. Vi è una forte domanda e questa chiusura è incomprensibile. Infatti, in questo Comune nascono nuovi quartieri. Inoltre, un quarto della popolazione ha superato l'età di pensionamento e quasi il 10 per cento ha più di 80 anni. Queste persone fanno spesso capo agli uffici postali. In aggiunta questo ufficio postale è uno degli elementi strutturali preso in considerazione per lo sviluppo del Comune, in particolare per l'allestimento dell'infrastruttura dei trasporti pubblici. Una petizione era stata lanciata nel 2017 da un gruppo politico, sindacati e utenti; all'inizio del 2018 sono state raccolte 1251 firme, che sono state inviate alla direzione della Posta. Invito pertanto il Consiglio federale a rispondere alle seguenti domande: 1. Quante persone fanno capo all'ufficio postale di Chêne-Bougeries dal 2015? 2. Come intende garantire un servizio postale pubblico di qualità per gli abitanti di Chêne-Bougeries? 3. Se la Posta intende sostituire l'ufficio di Chêne…</t>
+          <t>TEXT: L’attuale legge federale sulla protezione degli animali deve prevedere un piano di abbandono graduale degli esperimenti che causano sofferenza agli animali, che stabilisca obiettivi, tappe e scadenze vincolanti. Tale piano dovrà essere elaborato coinvolgendo il mondo scientifico, le organizzazioni per la protezione degli animali e l’industria.
+REASONING: La legge federale sulla protezione degli animali stabilisce già oggi che gli esperimenti sugli animali devono essere limitati al minimo indispensabile (art. 17) e che infliggere sofferenze all’animale è lecito soltanto se inevitabile per lo scopo dell’esperimento (art. 20 cpv. 1). Già grazie all’aiuto di tecnologie odierne, molti degli obiettivi degli esperimenti possono essere raggiunti con metodi che non prevedono test sugli animali. È stato dimostrato che tali metodi sono chiaramente superiori alla sperimentazione animale in termini di trasferibilità, utilità e costi (1). Il loro sviluppo sta progredendo costantemente, ma può essere accelerato con misure appropriate, ad esempio grazie a maggiori finanziamenti. Se intensificherà gli sforzi per garantire lo sviluppo e l’applicazione di metodi senza sperimentazione animale s…</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr"/>
@@ -1521,11 +1529,11 @@
         <v>38</v>
       </c>
       <c r="B39" t="n">
-        <v>153731</v>
+        <v>67274</v>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Stromspeicher bezüglich Netznutzung technologieneutral und somit gleichbehandeln</t>
+          <t>Biodiversità e stabilità finanziaria. Rapporto del "Network for Greening the Financial System"</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
@@ -1535,8 +1543,7 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Ich bitte den Bundesrat, folgende Fragen zu beantworten: 1. Warum beabsichtigt der Bundesrat, Stromspeicher hinsichtlich der Verrechnung von Netznutzungsentgelten für den Bezug von Elektrizität aus dem Netz gegenüber Pumpspeicherkraftwerken zu diskriminieren - Regulierungsvorgaben sollten technologieneutral sein -? 2. Ist er sich bewusst, dass Stromspeicher beim Umbau des Energiesystems zukünftig eine wichtige Rolle für den Ausgleich zwischen stark fluktuierender und wetterabhängiger erneuerbarer Energie und dem Verbrauch übernehmen müssen? 3. Ist er nicht der Ansicht, dass mit der Belastung von Speichern mit Netznutzungsentgelten auch die Ausnahmeregelung für Pumpspeicherkraftwerke hinterfragt werden muss und gefährdet ist? 4. Ist er sich bewusst, dass er mit dem neuen Artikel 2 Absatz 3 der Stromversorgungsverordnung (StromVV; Speicher gelten für den Bezug als Endverbraucher) einen Widerspruch zu Artikel 4 Absatz 1 Litera b schafft, worin ein Endverbraucher definiert ist als Kunde, der Elektrizität für den eigenen Verbrauch kauft, und somit eine Rechtsunsicherheit?
-REASONING: In der Vernehmlassungsvorlage zu den Verordnungen der Strategie Stromnetze ist vorgesehen, dass, w…</t>
+          <t>TEXT: La Svizzera fa parte del "Network for Greening the Financial System" (NGFS), una rete che riunisce banche centrali e autorità di vigilanza e che si impegna a favore di un settore finanziario rispettoso del clima e della biodiversità. Nel rapporto "Biodiversity and Financial Stability" del 2021 sono state formulate quattro raccomandazioni per le banche centrali su ciò che possono già fare oggi a tale proposito. Chiedo pertanto al Consiglio federale di rispondere alle seguenti domande. 1. In che modo l'Esecutivo affronta i rischi economici e finanziari rilevanti per la biodiversità? (compito 1) 2. Il Consiglio federale analizza la dipendenza degli istituti finanziari svizzeri dagli ecosistemi e dalla biodiversità e l'impatto che tali istituti producono su di essi? (compito 2) 3. In caso contrario, per quale motivo? 4. Il Governo prevede di sviluppare metodi per comprendere meglio i rischi finanziari rilevanti per la biodiversità (escludendo lo strumento ENCORE)? (compito 3) 5. In che misura il Consiglio federale informa gli istituti finanziari in merito al loro impatto sulla biodiversità e alla loro dipendenza da quest'ultima? (compito 4) 6. Il Consiglio federale riceve regolar…</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr"/>
@@ -1547,11 +1554,11 @@
         <v>39</v>
       </c>
       <c r="B40" t="n">
-        <v>157707</v>
+        <v>154848</v>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Ordinanza sull’indicazione dei prezzi. Semplificare l’autocomparazione</t>
+          <t>Violence sexuelle à l'égard des enfants sur Internet. Que fait l'Office fédéral de la police?</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -1561,8 +1568,8 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Il Consiglio federale è incaricato di semplificare le disposizioni dell'ordinanza sull'indicazione dei prezzi (OIP; RS 942.211) riguardanti l'indicazione fallace dei prezzi (art. 16 cpv. 1 lett. a e cpv. 3 OIP) in modo da consentire l'autocomparazione senza che siano fissati limiti di tempo, in particolare per gli articoli di stagione come capi di abbigliamento, calzature, articoli sportivi, ecc., se la merce in questione è stata effettivamente proposta in precedenza, per almeno quattro settimane consecutive, al prezzo più alto indicato.
-REASONING: Le disposizioni piuttosto complesse dell'OIP sull'autocomparazione, che regolamentano le indicazioni di riduzione dei prezzi e le comparazioni con il prezzo di vendita iniziale, erano state introdotte per evitare che i consumatori fossero tratti in inganno, ma oggi sono superate. Più in particolare, la cosiddetta regola del dimezzamento secondo cui il "prezzo comparativo" può essere indicato solo per la metà del periodo durante il quale è stato o sarà praticato, e al massimo per due mesi, comporta per i venditori e per le autorità di controllo un onere sproporzionato rispetto al vantaggio che ne risulta per il cliente. Questa rego…</t>
+          <t>TEXT: Le Conseil fédéral est prié de répondre aux questions suivantes : 1. L'Office fédéral de la police (Fedpol) remplit-il bien la fonction d'interface entre les organes internationaux et les cantons dans le domaine de la pédocriminalité ? Quelles sont les ressources nécessaires à cette fin quant aux structures, au personnel et aux technologies ? 2. Comment sont traitées les dénonciations en nombre croissant qui arrivent de l'étranger, de manière à ce qu'elles soient examinées avec le soin requis et que les procédures pénales qui s'imposent puissent être menées dans les cantons ? 3. Comment sont gérées les dénonciations qui concernent la Suisse, tout en étant difficiles à attribuer à un canton précis ? 4. Quelle forme pourrait prendre un service national efficace centralisant les dénonciations portant sur des cas de violence sexuelle commise contre des enfants et mise en ligne ? 5. Quelles mesures faudrait-il prendre notamment sur les plans de la législation, des technologies et du personnel pour que la police fédérale joue efficacement son rôle dans la lutte contre la pédocriminalité ?
+REASONING: De plus en plus d'enfants sont victimes de harcèlement sexuel sur Internet (étude …</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr"/>
@@ -1573,11 +1580,11 @@
         <v>40</v>
       </c>
       <c r="B41" t="n">
-        <v>63936</v>
+        <v>202440</v>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Renforcement de la Division Sécurité humaine au niveau de la coopération internationale</t>
+          <t>Inkassounternehmen. Für eine bessere Information der Konsumentinnen und Konsumenten</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
@@ -1587,8 +1594,8 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Le Conseil fédéral est chargé de prendre des mesures afin de renforcer les moyens financiers de la Division sécurité humaine dans le cadre de nos actions de coopération internationale.
-REASONING: Au sein des activités de coopération internationale réalisées par notre pays, figure celles de la Division sécurité humaine. Pour leur réalisation, cette division dispose d'un budget de 2,3 % du crédit-cadre de la coopération internationale 2021-2024. Ce pourcentage m'apparaît nettement insuffisant. Dans la perspective "mieux vaut prévenir que guérir", il me semble plus logique de prendre toutes les mesures utiles avant l'éclatement de conflits, de tenter toutes les démarches visant à les désamorcer plutôt que de venir réparer les dégâts après. L'actualité et les échos que nous en donnent les médias montrent que de nombreuses populations et régions du globe souffrent de conflits qui auraient pu, et dû, être évités. Renforcer ce secteur de la sécurité humaine permettrait d'obtenir des "économies" en vies humaines et en catastrophes de tous genres. La Suisse est crédible dans les domaines des droits humains, du désarmement, du droit humanitaire. Son statut et sa réputation de pays neu…</t>
+          <t>TEXT: Der Bundesrat wird beauftragt, eine Einrichtung zur Entgegennahme von Beschwerden zu schaffen, damit Konsumentinnen und Konsumenten die Verarbeitung ihrer Daten durch private Inkassounternehmen und Kreditauskunfteien wenn nötig anfechten können. Die Einrichtung wäre dem Eidgenössischen Datenschutz- und Öffentlichkeitsbeauftragten (EDÖB) angegliedert, würde über ein eigenes Budget verfügen und auch Sensibilisierungs- und Informationsarbeit leisten.
+REASONING: Unternehmen, die im Bereich Inkasso tätig sind, geben Auskünfte über die Zahlungsfähigkeit der ihnen bekannten Debitorinnen und Debitoren, ohne dabei den gesetzlichen Rahmen immer einzuhalten. Die Art, wie die Daten gesammelt werden, ist undurchsichtig, insbesondere bei Online-Einkäufen oder wenn die Daten basierend auf Algorithmen gesammelt werden, die eine Person aufgrund von Verhaltensdaten bewerten. Die Konsumentinnen und Konsumenten haben so gut wie keine Kontrolle darüber, wie ihre persönlichen Daten und Informationen zu ihren Zahlungsgewohnheiten gesammelt und weitergegeben werden. Doch auf dieser Grundlage getroffene Entscheidungen können schwerwiegende Folgen haben: Es kann soweit kommen, dass Konsumentinnen und…</t>
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr"/>
@@ -1599,11 +1606,11 @@
         <v>41</v>
       </c>
       <c r="B42" t="n">
-        <v>340056</v>
+        <v>155280</v>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Jetzt handeln: Kriterien für Ausnahmebewilligungen nach Art. 5 WG überarbeiten</t>
+          <t>Rechtshilfe gegenüber Griechenland. Zu neuen Ersuchen ermuntern</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
@@ -1613,8 +1620,8 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Der Bundesrat wird beauftragt, die gesetzlichen Grundlagen so anzupassen, dass Ausnahmebewilligungen für verbotene Waffen nach Artikel 5 WG künftig restriktiver und nach einheitlichen, nachvollziehbaren Kriterien erteilt werden und der Ausnahmecharakter dieser Bewilligungen gewahrt bleibt.
-REASONING: Verbotene Waffen dürfen gemäss Waffengesetz nur ausnahmsweise und unter bestimmten Voraussetzungen erworben und besessen werden. Im Kanton Zürich wurden in den letzten sieben Jahren fast 20'000 verbotene Waffen mit einer Ausnahmebewilligung zugelassen, im Kanton Thurgau gut 5'300 und im Kanton Aargau mehr als 6'000. Im Kanton Basel-Landschaft wurden in dieser Zeit fast 1'900, in Genf knapp 1'300 Ausnahmebewilligungen ausgestellt und im Kanton Wallis sind es alleine dieses Jahr fast 400. Dies wirft die Frage auf, ob die heutige Bewilligungspraxis dem gesetzlich vorgesehenen Ausnahmecharakter noch ausreichend Rechnung trägt. Angesichts der Fälle, in denen Waffen zur Tötung oder schweren Gefährdung von Menschen eingesetzt werden, ist eine sorgfältige und restriktive Bewilligungspraxis von besonderer Bedeutung. Es muss gewährleistet sein, dass vor der Erteilung einer Ausnahmebewilli…</t>
+          <t>TEXT: Das Bundesstrafgericht und danach das Bundesgericht haben vorläufig die Herausgabe von Bankdaten an die griechischen Strafverfolgungsbehörden durch die Bundesanwaltschaft blockiert. Der Entscheid schockiert in einem krassen Korruptionsfall, der im Jahr 2013 bereits zur Verurteilung des ehemaligen Verteidigungsministers Tsochatzopoulos zu einer Freiheitsstrafe von 20 Jahren führte. Als Grund nannten die Gerichte den Verdacht, dass das Rechtshilfeersuchen auf den Bankdaten der Falciani-Liste beruhe. Wird das Bundesamt für Justiz den griechischen Behörden nahelegen, ihr Anliegen noch einmal vorzubringen und dabei zu belegen, dass das Ersuchen nicht auf den Daten der Falciani-Liste beruht?
+ANSWER: Die Antwort des Bundesrates existiert nur in französischer Sprache. (Bitte wechseln Sie auf der Homepage oben rechts die Sprache)</t>
         </is>
       </c>
       <c r="F42" s="5" t="inlineStr"/>
@@ -1625,11 +1632,11 @@
         <v>42</v>
       </c>
       <c r="B43" t="n">
-        <v>202440</v>
+        <v>201674</v>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Inkassounternehmen. Für eine bessere Information der Konsumentinnen und Konsumenten</t>
+          <t>Révision de la loi sur le renseignement. Le secret médical et professionnel en danger!</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
@@ -1639,8 +1646,7 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Der Bundesrat wird beauftragt, eine Einrichtung zur Entgegennahme von Beschwerden zu schaffen, damit Konsumentinnen und Konsumenten die Verarbeitung ihrer Daten durch private Inkassounternehmen und Kreditauskunfteien wenn nötig anfechten können. Die Einrichtung wäre dem Eidgenössischen Datenschutz- und Öffentlichkeitsbeauftragten (EDÖB) angegliedert, würde über ein eigenes Budget verfügen und auch Sensibilisierungs- und Informationsarbeit leisten.
-REASONING: Unternehmen, die im Bereich Inkasso tätig sind, geben Auskünfte über die Zahlungsfähigkeit der ihnen bekannten Debitorinnen und Debitoren, ohne dabei den gesetzlichen Rahmen immer einzuhalten. Die Art, wie die Daten gesammelt werden, ist undurchsichtig, insbesondere bei Online-Einkäufen oder wenn die Daten basierend auf Algorithmen gesammelt werden, die eine Person aufgrund von Verhaltensdaten bewerten. Die Konsumentinnen und Konsumenten haben so gut wie keine Kontrolle darüber, wie ihre persönlichen Daten und Informationen zu ihren Zahlungsgewohnheiten gesammelt und weitergegeben werden. Doch auf dieser Grundlage getroffene Entscheidungen können schwerwiegende Folgen haben: Es kann soweit kommen, dass Konsumentinnen und…</t>
+          <t>TEXT: Le conseil et le traitement des patients supposent que le corps médical prenne connaissance d'informations sensibles concernant la sphère privée et intime. Les personnes concernées communiquent de telles informations parce qu'elles sont sûres que la confidentialité est garantie. Cette obligation de confidentialité est la condition nécessaire à la réussite d'un diagnostic et d'un traitement. Sans aucune explication, le Conseil fédéral veut supprimer l'al. 2 de l'art. 28 LRens dans le projet de modification de la loi actuellement en consultation. Ce faisant, il affaiblit fortement la protection du secret professionnel. Selon le rapport explicatif, le SRC devrait désormais pouvoir ordonner des mesures soumises à autorisation (surveillance téléphonique et postale, intrusion dans des ordinateurs, etc.) également à l'encontre du personnel médical, des ecclésiastiques, des avocats et des journalistes. Il s'agirait d'une grave érosion des dispositions en matière de protection du secret, en particulier en ce qui concerne le secret médical, de l'avocat, de la confession et la protection des sources dans le journalisme, qui sont importants pour la confiance dans les relations et la démo…</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr"/>
@@ -1651,11 +1657,11 @@
         <v>43</v>
       </c>
       <c r="B44" t="n">
-        <v>213693</v>
+        <v>335116</v>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Entreprises plates-formes et économie à la tâche ou "gig economy". Mieux protéger les travailleurs indépendants</t>
+          <t>Förderprogramm für den bedarfsgerechten Ausbau von Tagesschulangeboten</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
@@ -1665,8 +1671,8 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Le Conseil fédéral est chargé d'élaborer un rapport dans lequel il propose des pistes pour améliorer la protection sociale des indépendants travaillant à la tâche. Il devra en particulier examiner comment les entreprises plateformes pourraient contribuer à assurer une meilleure couverture sociale aux personnes participant à cette économie dite collaborative ou de partage.
-REASONING: Déjà en plein essor, les modèles de travail flexible vont se développer encore sous l'effet d'une numérisation galopante. Ils consistent à proposer de brèves missions à des indépendants ou des personnes employées à temps très partiel. On peut s'attendre à ce que la tendance à l'ubérisation, dominée par les entreprises plateformes, prenne encore de l'ampleur. Cette évolution propose de nouveaux modèles d'entreprises mais elle ouvre aussi de nouvelles possibilités qui, à certaines conditions, peuvent tout à fait séduire les indépendants. Le problème est que ceux-ci se voient moins bien protégés contre les risques sociaux. Les acteurs politiques sont donc appelés à examiner les conditions de cette nouvelle économie et à les adapter si nécessaire afin qu'elle ne soit pas synonyme de réduction de la p…</t>
+          <t>TEXT: Der Bundesrat wird beauftragt, die gesetzlichen Grundlagen für ein zeitlich befristetes Förderprogramm zu schaffen, mit dem Kantone und Gemeinden beim Auf- und Ausbau von Tagesschulangeboten finanziell unterstützt werden können. Das Förderprogramm ist so auszugestalten, dass die Zuständigkeiten und die Autonomie der Kantone im Bildungsbereich uneingeschränkt gewahrt bleiben.
+REASONING: Tagesschulen leisten einen wichtigen Beitrag zur Chancengerechtigkeit, zur Vereinbarkeit von Familie und Beruf sowie zur besseren Nutzung des inländischen Arbeitskräftepotenzials. Sie verbinden Bildung, Förderung und Betreuung und schaffen verlässliche Strukturen für Kinder und Familien. Die Verfügbarkeit von Tagesschulangeboten ist in der Schweiz je nach Kanton und Gemeinde sehr unterschiedlich. Dadurch entstehen Ungleichheiten sowohl für Familien als auch für Kinder. Mit der unbefristeten Unterstützung der familien- und schulergänzenden Kinderbetreuung auf Bundesebene hat das Parlament die Bedeutung einer guten Betreuungsinfrastruktur anerkannt. Der Ausbau von Tagesschulangeboten stellt eine sinnvolle Ergänzung dieser Politik dar. Tagesschulen erleichtern Eltern die Vereinbarkeit von Familie…</t>
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr"/>
@@ -1677,11 +1683,11 @@
         <v>44</v>
       </c>
       <c r="B45" t="n">
-        <v>71679</v>
+        <v>213749</v>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Jeu vidéo à caractère islamiste vendu sur « Steam » : le Conseil fédéral va-t-il réagir en conséquence ?</t>
+          <t>Explosion des coûts de la santé. A quand des mesures efficaces contre le gaspillage de l'argent des primes et pour freiner la hausse des coûts?</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
@@ -1691,8 +1697,7 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Nous avons appris avec stupeur qu’un jeu vidéo est en vente sur la très populaire plateforme « Steam », intitulé « Fursan al-Aqsa: The Knights of the Al-Aqsa Mosque », glorifiant explicitement les abominables attaques terroristes du 7 octobre 2023 en Israël lors desquelles plus de 1000 personnes, principalement des civils sans défense, ont été massacrées. Ce jeu est une promotion explicite de l’idéologie islamiste et des crimes contre l’humanité commis lors de l’attaque du Hamas contre Israël en 2023. Le 29 novembre dernier, nous apprenions par voie de presse que le Royaume-Uni a interdit et banni ce « jeu » de la plateforme « Steam » et de tout support officiel permettant de se le procurer. L’apologie du terrorisme islamiste, de la haine et des crimes de guerre et crimes contre l’humanité n’étant pas tolérable dans notre pays, la Confédération compte-t-elle aussi intervenir afin d’interdire ce « jeu » vidéo abjecte ?
-ANSWER: L'incitation à la violence ou la discrimination envers une personne ou un groupe de personnes en raison de leur appartenance religieuse ou ethnique ainsi que la négation d'un génocide sont largement couverts par le Code pénal. La répression pénale de ce…</t>
+          <t>TEXT: Comme chaque année à cette même période, le jeu des caisses-maladie bat son plein. Les assureurs font parvenir de la publicité aux ménages par les canaux les plus divers : certaines caisses-maladie proposent des rabais et d'autres promettent des baisses de primes pour l'année prochaine, alors que l'association des assureurs-maladie Santésuisse a annoncé cet été une hausse générale des primes de l'ordre de 3 %. 1. Tout laisse à penser dans ce contexte que, comme lors des précédentes années électorales, les caisses-maladie puisent plus profondément dans leurs réserves qu'à l'ordinaire pour réduire au maximum la hausse des primes. Que pense l'Office fédéral de la santé publique de ce soupçon en sa qualité d'autorité d'approbation des primes ? Des réserves ont-elles dû ou devraient-elles être réduites pour obtenir des primes plus basses ? 2. La numérisation doit profiter au système de santé : elle améliore l'efficacité et la qualité des soins ainsi que l'information des assurés et des patients. Il y a un an, le Conseil fédéral a proposé le rejet d'une intervention qui visait à créer une base légale garantissant que la documentation médicale du patient soit tenue de manière struct…</t>
         </is>
       </c>
       <c r="F45" s="5" t="inlineStr"/>
@@ -1703,11 +1708,11 @@
         <v>45</v>
       </c>
       <c r="B46" t="n">
-        <v>155922</v>
+        <v>235214</v>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Atténuer la crise du coronavirus pour les personnes à faibles revenus</t>
+          <t>Woran orientiert sich die Finma bei ihrer Regulierungstätigkeit?</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
@@ -1717,8 +1722,7 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Le Conseil fédéral est chargé avec les cantons d'augmenter le montant des subsides aux primes d'assurance-maladie de 50 % pendant deux ans pour les personnes ayant de faibles revenus afin d'éviter que davantage de personnes en Suisse ne sombrent dans la précarité.
-REASONING: Dans notre pays, près d'un million de personnes vivent dans la précarité ou juste au-dessus du seuil de pauvreté selon les derniers chiffres de l'Office fédéral de la statistique, soit une personne sur sept. La situation s'est considérablement aggravée depuis avec la pandémie, qui a privé de nombreux ménages de leur revenu principal. Un nombre croissant de personnes ne peuvent plus payer leurs primes d'assurance-maladie, qui déjà avant la crise représentaient une charge très importante pour les familles. Dans cette situation extraordinaire, la Confédération et les cantons doivent augmenter de 50 %, pour une durée de deux ans le montant des subsides aux primes d'assurance-maladie. Les finances fédérales et cantonales permettent de supporter cette charge supplémentaire. Elle permettra d'éviter la précarisation d'une partie de la population, qui coûterait très cher à l'État à long terme. Agir maintenant, po…</t>
+          <t>TEXT: Im Schweizer Finanzmarkt spielt wie weltweit üblich international ausgearbeitetes Soft Law eine zentrale Rolle. Dieses wird in Behördennetzwerken ausgearbeitet, in denen Zentralbanken bzw. Finanzmarktaufsichtbehörden zusammenarbeiten und internationale Standards setzen. So ist die schweizerische Finanzmarktaufsicht FINMA in verschiedenen internationalen Gremien vertreten. In diesen Gremien wird internationales Soft Law im Bereich Finanzmarktregulierung mit Spillover-Effekt auf nationaler Ebene entwickelt. Dieses Soft Law in Form von (Mindest-)Standards hat zwar keine Bindungswirkung, muss aber von der FINMA bei ihrer Regulierungstätigkeit berücksichtigt werden. Aktuelle Beispiele aus der Regulierungstätigkeit der FINMA bezeugen die Einhaltung dieses Grundsatzes: Geplantes Rundschreiben Naturbezogene Finanzrisiken (Rundschreiben basiert u.a. auf Soft Law des Basler Ausschusses für Bankenaufsicht) Totalrevision Rundschreiben 13/5 Liquidität – Versicherer (Revision erfolgt u.a. im Hinblick auf Soft Law der internationalen Vereinigung der Versicherungsaufsichtsbehörden) Gleichzeitig muss festgestellt werden, dass die Beachtung internationaler (Mindest-)Standards unweigerlich zu Z…</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr"/>
@@ -1729,11 +1733,11 @@
         <v>46</v>
       </c>
       <c r="B47" t="n">
-        <v>288093</v>
+        <v>65002</v>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Sicurezza dei prodotti: rafforzare la libera concorrenza tra attori svizzeri e stranieri del commercio online</t>
+          <t>Coronavirus. Un Parlement virtuel serait-il une solution?</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
@@ -1743,7 +1747,8 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>TEXT: I recenti avvenimenti che hanno coinvolto la piattaforma di e-commerce cinese Shein nella vicina Francia sollevano interrogativi legittimi anche in Svizzera. Se si considera che ogni giorno arrivano a Zurigo circa 500 000 pacchi dalla Cina, risulta difficile stabilire se i controlli di qualità imposti ai prodotti svizzeri siano applicati nella stessa misura anche ai prodotti cinesi. Alcuni degli articoli in vendita sulle piattaforme cinesi stanno suscitando un certo scalpore. Su Temu, ad esempio, è possibile trovare puntatori laser il cui uso è severamente vietato in Svizzera a causa dei possibili rischi per la vista associati. Inoltre, un recente studio dimostra che l'86 per cento dei giocattoli disponibili sulle principali piattaforme di commercio online straniere (Temu, Shein, Amazon) sono considerati pericolosi per la salute dei bambini. Come giustifica il Consiglio federale il fatto che i prodotti in vendita sulle piattaforme cinesi non soddisfino gli stessi requisiti di qualità dei prodotti svizzeri, soprattutto in termini di sicurezza? Come intende obbligare le piattaforme straniere a rispettare le stesse regole imposte ai loro concorrenti svizzeri? Quali misure intend…</t>
+          <t>TEXT: Alors que la Suisse risque elle aussi de se retrouver dans une situation de crise en raison de la propagation du coronavirus, je prie le Bureau de répondre aux questions suivantes : 1. Comment le bon fonctionnement des institutions peut-il être garanti en période de crise ? 2. Le Parlement aurait-il la possibilité à l'heure actuelle de prendre des décisions dans une situation de crise sans avoir à se réunir physiquement ? 3. Dans la négative, quelles bases légales ou constitutionnelles faudrait-il créer pour que le travail parlementaire puisse avoir lieu en situation de crise sans que le Parlement ait à se réunir physiquement ? 4. Quelles mesures techniques y aurait-il lieu de prendre (identités électroniques, logiciels permettant de conduire de bout en bout les processus politiques, etc.) pour que le travail parlementaire puisse être effectué en ligne avec toute l'efficacité et toute la sécurité requises ?
+REASONING: Les défis que les parlementaires de milice doivent relever dans leur quotidien parlementaire sont déjà nombreux. Mais dans des situations de crise telles que celle qui s'annonce avec l'épidémie de coronavirus, il est encore plus difficile de garantir le bon dér…</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr"/>
@@ -1754,11 +1759,11 @@
         <v>47</v>
       </c>
       <c r="B48" t="n">
-        <v>63574</v>
+        <v>155568</v>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Adeguamento del diritto federale agli sviluppi della tecnologia di registro distribuito. Legge federale</t>
+          <t>Servizio d'appoggio dell'esercito a favore delle autorità civili nell'ambito dei provvedimenti per combattere la pandemia di Covid-19</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
@@ -1775,11 +1780,11 @@
         <v>48</v>
       </c>
       <c r="B49" t="n">
-        <v>65002</v>
+        <v>161710</v>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Coronavirus. Un Parlement virtuel serait-il une solution?</t>
+          <t>Lancement de DigiFLUX - Comment le point 5.4 sur la surface traitée de l'annexe 3b de l'OSIAgr va-t-il être mis en œuvre concrètement ?</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
@@ -1789,8 +1794,8 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Alors que la Suisse risque elle aussi de se retrouver dans une situation de crise en raison de la propagation du coronavirus, je prie le Bureau de répondre aux questions suivantes : 1. Comment le bon fonctionnement des institutions peut-il être garanti en période de crise ? 2. Le Parlement aurait-il la possibilité à l'heure actuelle de prendre des décisions dans une situation de crise sans avoir à se réunir physiquement ? 3. Dans la négative, quelles bases légales ou constitutionnelles faudrait-il créer pour que le travail parlementaire puisse avoir lieu en situation de crise sans que le Parlement ait à se réunir physiquement ? 4. Quelles mesures techniques y aurait-il lieu de prendre (identités électroniques, logiciels permettant de conduire de bout en bout les processus politiques, etc.) pour que le travail parlementaire puisse être effectué en ligne avec toute l'efficacité et toute la sécurité requises ?
-REASONING: Les défis que les parlementaires de milice doivent relever dans leur quotidien parlementaire sont déjà nombreux. Mais dans des situations de crise telles que celle qui s'annonce avec l'épidémie de coronavirus, il est encore plus difficile de garantir le bon dér…</t>
+          <t>TEXT: Conformément à l'annexe 3b, point 5.4, de l'ordonnance sur les systèmes d'information dans le domaine de l'agriculture (OSIAgr), seule la surface traitée doit être indiquée dans le cadre des recensements sur l'utilisation des produits phytosanitaires. Or, cette surface devra apparemment être géoréférencée à la parcelle près sur la plateforme DigiFLUX. Que prévoit-on concrètement pour la mise en œuvre ?
+ANSWER: La déclaration de l’utilisation de produits phytosanitaires concerne les données relatives à toute utilisation professionnelle, donc les données de chaque cas concret de traitement (art. 16a, al. 1, let. e, OSIAgr). Toute application de produits phytosanitaires doit ainsi faire l’objet d’une saisie, incluant les données suivantes : désignation du produit phytosanitaire, date de l’utilisation, quantité utilisée, surface traitée, plante cultivée ou objet traité (art. 16a, al. 2, et annexe 3b, OSIAgr, ainsi qu’art. 62, al. 1bis, OPPh). L’obligation légale d’informer porte sur le lieu et le type de culture où des produits phytosanitaires ont été utilisés. Dans le cadre du relevé des données pertinentes pour les paiements directs, les exploitations sont déjà tenues, dans le…</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr"/>
@@ -1801,11 +1806,11 @@
         <v>49</v>
       </c>
       <c r="B50" t="n">
-        <v>340378</v>
+        <v>68419</v>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Weiteres IT - Experimentierfeld beim Bund mit Microsoft 365?</t>
+          <t>Förderung von Audiowerken als Schweizer Kulturgut</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
@@ -1815,7 +1820,7 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Kaum ist die Einführung von Microsoft 365 in der Bundesverwaltung abgeschlossen, wird bereits an einer Open-Source-Alternative gearbeitet. Grundsätzlich ist es richtig, Abhängigkeiten zu prüfen. Es stellt sich jedoch die Frage, ob der Bund hier erneut Gefahr läuft, ein funktionierendes System zum kostspieligen IT-Experimentierfeld zu machen. Microsoft 365 ist etabliert und wird in der Bundesverwaltung breit eingesetzt. Microsoft verfügt zudem über Rechenzentrumsregionen in der Schweiz und arbeitet eng mit Schweizer Partnern zusammen. Für besonders schützenswerte Daten hat der Bund zusätzliche Vorgaben und eigene Infrastrukturen. Vor diesem Hintergrund muss nachvollziehbar dargelegt werden, welchen konkreten Mehrwert ein paralleles oder neues System tatsächlich bringt. Die Vergangenheit zeigt, dass IT-Projekte des Bundes immer wieder durch Verzögerungen, Kostenüberschreitungen, Schnittstellenprobleme oder mangelnde Praxistauglichkeit aufgefallen sind. Umso weniger verständlich wäre es, ein funktionierendes und erst kürzlich eingeführtes System aus politischen Überlegungen abzustellen, ohne Kosten, Risiken und Nutzen vollständig offenzulegen. Der Bundesrat wird gebeten, folgend…</t>
+          <t>TEXT: Audiowerke sind Hörspiele, Reportagen, Doku-Serien und hochwertige Talks, die als Podcasts oder über das lineare Radio veröffentlicht werden. Das Angebot und die Nachfrage des Publikums nach hochwertigen Schweizer Produktionen ist stark gestiegen. Die Digitalisierung vereinfacht zwar die Realisierung von unabhängigen Produktionen und Online-Distributionsplattformen ermöglichen deren Verbreitung. Doch die Finanzierungsmöglichkeiten sind prekär. Aufwändige Audioformate geraten zudem auch im linearen Radio zunehmend unter Spardruck. Audiowerke leisten einen wichtigen Beitrag zur kulturellen Vielfalt und zur gesellschaftlichen Verständigung in der Schweiz. Sie fördern die Auseinandersetzung mit relevanten gesellschaftlichen und politischen Themen und die Kultur des aktiven Zuhörens, was wichtige Grundlagen einer funktionierenden Demokratie sind. Schweizer Audioschaffende realisieren ihre preisgekrönten Podcasts vermehrt ausserhalb von gebührenfinanzierten Radiostationen. In der Vielfalt von Berufsbildern, Themen und Methoden ist die wachsende Schweizer Audiobranche mit der Schweizer Filmindustrie vergleichbar. Während der Bund jedoch das Schweizer Filmschaffen als eigene kulturel…</t>
         </is>
       </c>
       <c r="F50" s="5" t="inlineStr"/>
@@ -1826,11 +1831,11 @@
         <v>50</v>
       </c>
       <c r="B51" t="n">
-        <v>68304</v>
+        <v>340891</v>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Les règles sur la transparence du financement de la vie politique doivent être mises en oeuvre de manière conforme à la volonté du Parlement</t>
+          <t>Lettre d’EMS-Chemie Holding AG au conseiller national Fabian Molina. Protéger la liberté d’expression des élus fédéraux</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
@@ -1840,7 +1845,7 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>TEXT: 1. Que pense le Conseil fédéral des critiques émises au sujet de l'ordonnance par plusieurs participants à la procédure de consultation, et de quelle manière entend-il en tenir compte dans la version définitive de l'ordonnance ? 2. Est-il problématique selon lui de vouloir contraindre le Contrôle fédéral des finances (CDF), contre la volonté de son directeur, à contrôler si les règles sur la transparence du financement des partis sont respectées ? 3. En adoptant le contre-projet, le Parlement a montré clairement qu'il souhaitait la plus grande transparence possible dans le financement de la vie politique et la mise en place de règles uniformes et contrôlables applicables à tous, afin de favoriser la libre formation de l'opinion des citoyens avant les votations et les élections. Quelle serait la réglementation nécessaire, selon le Conseil fédéral, pour que la loi et l'ordonnance garantissent la transparence du financement des partis ? 4. La mesure prévoyant que l'autorité compétente effectue des contrôles par échantillonnage pour vérifier si les règles sur la transparence sont mises en oeuvre correctement a été ajoutée par les Chambres lors des délibérations parlementaires, et…</t>
+          <t>TEXT: Le conseiller national Fabian Molina a reçu le 24 septembre 2026 une lettre recommandée d’EMS-Chemie Holding AG se référant expressément à sa question 26.7751, adressée au Conseil fédéral durant l’heure des questions. L'entreprise lui reproche d’avoir sciemment diffusé, avec sa question consultable publiquement au Conseil fédéral, des allégations fausses, dénigrantes et diffamatoires et le somme de s’abstenir à l’avenir de faire de telles déclarations, sous peine de poursuites dans le cas contraire. Ce ne sont donc pas des propos qui auraient été tenus en dehors des séances des Chambres fédérales qui sont ici attaqués, mais bien le droit de poser des questions dont jouissent les conseillers nationaux. Dans sa question, le conseiller Fabian Molina mentionne une enquête du journal en ligne « Republik » et demande au Conseil fédéral de procéder à des vérifications. Or c’est précisément la fonction de l’heure des questions. Je prie donc le Bureau de bien vouloir répondre aux questions suivantes : Le Bureau confirme-t-il que la question 26.7751, en tant que déclaration faite devant un conseil, jouit de l’immunité absolue en vertu de l’art. 162, al. 1, de la Constitution fédérale e…</t>
         </is>
       </c>
       <c r="F51" s="5" t="inlineStr"/>
@@ -1851,11 +1856,11 @@
         <v>51</v>
       </c>
       <c r="B52" t="n">
-        <v>331167</v>
+        <v>66518</v>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>G7-Gipfel: Vom 10. bis 19. Juni 2026 lässt der Bundesrat an der Grenze zu Frankreich verstärkte Grenzkontrollen durchführen. Was macht er bei grenzüberschreitender Kriminalität?</t>
+          <t>Rapporto sulla politica di sicurezza 2021</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
@@ -1863,12 +1868,7 @@
           <t>open</t>
         </is>
       </c>
-      <c r="E52" s="2" t="inlineStr">
-        <is>
-          <t>TEXT: Polizeimeldungen bestätigen, dass Tätergruppen aus Frankreich wiederholt Fahrzeugdiebstähle und weitere Delikte in der Schweiz begehen. - Ist der Bundesrat der Ansicht, dass verstärkte Grenzkontrollen nicht nur zum Schutz des G7-Gipfels, sondern auch zur Bekämpfung der grenzüberschreitenden Kriminalität beitragen können? - Bestehen die notwendigen rechtlichen und operativen Möglichkeiten, um die Kontrolldichte an der Grenze zu Frankreich (analog zu den Massnahmen zum G7-Gipfel) zu erhöhen?
-ANSWER: Bei früheren G8-Treffen ist es zu gewaltsamen Auseinandersetzungen, Stör- und Sabotageaktionen sowie zu Sachbeschädigungen gekommen. Vor diesem Hintergrund hat der Kanton Genf beim Bundesrat für die Dauer des G7-Gipfels ein Gesuch um temporäre Wiedereinführung von Binnengrenzkontrollen an den Land- und Seegrenze eingereicht. Dieses hat der Bundesrat gutgeheissen. Für die Bekämpfung von grenzüberschreitender Kriminalität setzen Bund und Kantone aber grundsätzlich auf andere Instrumente: Das Bundesamt für Zoll und Grenzsicherheit (BAZG) ist an der Grenze und im Grenzraum präsent und kontrolliert im Rahmen seines Auftrages lage- und risikobasiert den grenzüberschreitenden Waren- und P…</t>
-        </is>
-      </c>
+      <c r="E52" s="2" t="inlineStr"/>
       <c r="F52" s="5" t="inlineStr"/>
       <c r="G52" s="5" t="inlineStr"/>
     </row>
@@ -1877,11 +1877,11 @@
         <v>52</v>
       </c>
       <c r="B53" t="n">
-        <v>159482</v>
+        <v>71811</v>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Steigende Heizkosten: Wie rasch kann der Bundesrat handeln?</t>
+          <t>Proteggere la nostra democrazia dalle influenze estere</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
@@ -1891,7 +1891,8 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Gemäss Antwort auf 22.7358 hat der Bundesrat Massnahmen betreffend steigende Heizkosten geprüft, die rasch umsetzbar sein sollen und an die Ergänzungsleistungen oder Prämienverbilligung anknüpfen. Er hat aber keine Entscheide getroffen. - Mit welchen Fristen rechnet der Bundesrat für die Umsetzung dieser Massnahmen nach einem Entscheid? - Können diese spätestens auf den Zeitpunkt der Abrechnung Heizkostenperiode Juni 2023 in Kraft treten?</t>
+          <t>TEXT: La legge sui diritti politici è modificata di modo che le liberalità monetarie e non monetarie provenienti dall’estero comportino sanzioni penali dissuasive (in particolare sotto forma di multe) nei confronti degli attori politici che le accettano intenzionalmente.
+REASONING: I nostri diritti popolari (iniziativa, referendum, petizione) e le nostre elezioni sono un punto di forza del nostro sistema politico. La democrazia semi-diretta rende la Svizzera un luogo di dibattito in cui il Popolo dispone di ampi poteri, una caratteristica di cui essere orgogliosi. La Svizzera è uno Stato sovrano e indipendente. La formazione dell’opinione dell’elettorato non deve essere influenzata da finanziamenti esteri che seguono altre agende politiche. Attualmente la legge federale sui diritti politici (LDP) impedisce agli attori politici (partiti, persone fisiche o giuridiche e società di persone che conducono una campagna in vista di un’elezione nelle Camere federali o di una votazione federale) di accettare finanziamenti provenienti dall’estero. Una liberalità (non) monetaria deve essere restituita a chi l’ha versata. Se la restituzione non è possibile o non è ragionevolmente esigibile, la…</t>
         </is>
       </c>
       <c r="F53" s="5" t="inlineStr"/>
@@ -1902,11 +1903,11 @@
         <v>53</v>
       </c>
       <c r="B54" t="n">
-        <v>235974</v>
+        <v>288093</v>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Le prospettive dell'AVS erano errate. Lo sono anche quelle dell'AI?</t>
+          <t>Sicurezza dei prodotti: rafforzare la libera concorrenza tra attori svizzeri e stranieri del commercio online</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
@@ -1916,8 +1917,7 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Chiedo al Consiglio federale di rispondere alle seguenti domande: È noto che sono stati commessi errori nelle previsioni dell’AVS. Sono stati commessi gli stessi errori anche per quanto riguarda le cifre dell’AI? I debiti dell’AI gravano l’AVS. L’Amministrazione federale ha ripetutamente comunicato a partire da quando l’AI potrà ridurre il debito nel bilancio dell’AVS. Quali dati sono stati comunicati dal 2012? Quali motivazioni sono state addotte dal 2012 per la costante posticipazione di questo momento? Quando saranno presentate al Parlamento nuove basi di dati che contengano anche la crescita delle nuove rendite e la diminuzione dei tassi di uscita, fattori menzionati da Compenswiss? Il Consiglio federale come garantisce una maggiore attendibilità delle previsioni dell’AI affinché si disponga di basi sicure per una prossima revisione dell’AI?
-REASONING: Il 18 febbraio 2025 il Consiglio di amministrazione di Compenswiss ha comunicato che «[a]nche per il fondo AI le prospettive finanziarie sono peggiorate a causa dell’aumento delle nuove rendite e della diminuzione dei tassi di uscita» e avvertito che «[d]ata la sua situazione finanziaria, è improbabile che l’AI possa ridur…</t>
+          <t>TEXT: I recenti avvenimenti che hanno coinvolto la piattaforma di e-commerce cinese Shein nella vicina Francia sollevano interrogativi legittimi anche in Svizzera. Se si considera che ogni giorno arrivano a Zurigo circa 500 000 pacchi dalla Cina, risulta difficile stabilire se i controlli di qualità imposti ai prodotti svizzeri siano applicati nella stessa misura anche ai prodotti cinesi. Alcuni degli articoli in vendita sulle piattaforme cinesi stanno suscitando un certo scalpore. Su Temu, ad esempio, è possibile trovare puntatori laser il cui uso è severamente vietato in Svizzera a causa dei possibili rischi per la vista associati. Inoltre, un recente studio dimostra che l'86 per cento dei giocattoli disponibili sulle principali piattaforme di commercio online straniere (Temu, Shein, Amazon) sono considerati pericolosi per la salute dei bambini. Come giustifica il Consiglio federale il fatto che i prodotti in vendita sulle piattaforme cinesi non soddisfino gli stessi requisiti di qualità dei prodotti svizzeri, soprattutto in termini di sicurezza? Come intende obbligare le piattaforme straniere a rispettare le stesse regole imposte ai loro concorrenti svizzeri? Quali misure intend…</t>
         </is>
       </c>
       <c r="F54" s="5" t="inlineStr"/>
@@ -1928,11 +1928,11 @@
         <v>54</v>
       </c>
       <c r="B55" t="n">
-        <v>153874</v>
+        <v>69534</v>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Vorstösse verbindlich behandeln</t>
+          <t>Una strategia svizzera per i semiconduttori (Swiss Chip Strategy)</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
@@ -1942,8 +1942,8 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Gestützt auf Artikel 160 Absatz 1 der Bundesverfassung und Artikel 107 des Parlamentsgesetzes reiche ich folgende parlamentarische Initiative ein: Im Bundesgesetz über die Bundesversammlung (Parlamentsgesetz, ParlG) ist eine Frist zur Behandlung von Motionen und Postulaten vorzusehen ähnlich wie für parlamentarische Initiativen. Motionen und Postulate dürfen nicht mehr unbehandelt abgeschrieben werden. Es darf jedoch keine Einschränkung der Anzahl eingereichter Vorstösse geben. Stattdessen könnte das Büro beispielsweise verpflichtet werden, ältere Vorstösse prioritär zu behandeln.
-REASONING: Motionen und Postulate sind wichtige Instrumente der Parlamentsarbeit. Wir als gewählte Vertreterinnen und Vertreter des Volkes können über diese Instrumente unsere politischen Anliegen zielgerichtet einbringen und nehmen so auch massgeblich unseren Wählerauftrag wahr. Nur leider geht es im Schnitt über ein Jahr, bis die Vorstösse überhaupt im Rat behandelt werden. Dies führt dazu, dass wichtige Anliegen verschleppt werden oder sogar verloren gehen. Dies zeugt nicht von einem effizienten Ratsbetrieb. Das entspricht auch nicht dem Tempo, in dem unsere Welt funktioniert oder unsere Wirtsch…</t>
+          <t>TEXT: Il settore dei semiconduttori riveste un ruolo strategico ed è sempre più importante nelle filiere produttive mondiali e svizzere, in un contesto sociale che si sta digitalizzando rapidamente. In Svizzera operano aziende strategiche a livello mondiale: forniscono tecnologie per la fabbricazione di semiconduttori. Il rischio di concorrenza sleale – soprattutto da parte dell’UE e degli USA – mediante programmi di sovvenzione per diverse decine di miliardi, che prevedono condizioni relative alla localizzazione produttiva, è elevato. Sono aspetti che mettono a rischio il sistema d’innovazione e produzione svizzero e le nostre industrie. Invito il Consiglio federale ad analizzare la situazione, in particolare sotto il profilo dei rischi e delle opportunità legati agli sviluppi più recenti, valutando anche i rischi dovuti al decoupling delle filiere produttive. Chiedo al Consiglio federale di riferire al Parlamento mediante un rapporto con proposte finalizzate in particolare a migliorare le condizioni quadro per le imprese interessate e favorire l’innovazione (Swiss Chip Strategy).
+REASONING: In una società digitalizzata come la nostra, i componenti al silicio sono onnipresenti: c…</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr"/>
@@ -1954,11 +1954,11 @@
         <v>55</v>
       </c>
       <c r="B56" t="n">
-        <v>71286</v>
+        <v>65463</v>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Opposition locale contre les centres fédéraux pour requérants d’asile</t>
+          <t>Im Interesse der Rechtsstaatlichkeit, der Souveränität und der Neutralität der Schweiz die Crypto-Leaks-Affäre mit einer PUK umfassend aufklären</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
@@ -1968,8 +1968,8 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>TEXT: - Lorsqu’un centre fédéral pour requérants d’asile est prévu, l’opposition de la population locale a-t-elle une influence sur sa réalisation et son exploitation ? - La Confédération pense-t-elle que cette opposition disparaîtra d’elle-même avec le temps ?
-ANSWER: La réponse du Conseil fédéral n'existe qu'en allemand. (Veuillez changer la langue en haut à droite de la page d'accueil)</t>
+          <t>TEXT: Das Parlament setzt eine Parlamentarische Untersuchungskommission PUK ein zur Aufarbeitung der Spionage-Affäre um die Firma Crypto AG.
+REASONING: Im Interesse der Rechtsstaatlichkeit, der Souveränität und der Neutralität der Schweiz muss die Cryptoleaks-Affäre umfassend aufgeklärt werden. Eine PUK hat dazu die notwendigen Ressourcen und kann insbesondere auch Untersuchungsbeauftragte i.S. von Artikel 166 ParIG einsetzen.</t>
         </is>
       </c>
       <c r="F56" s="5" t="inlineStr"/>
@@ -1980,11 +1980,11 @@
         <v>56</v>
       </c>
       <c r="B57" t="n">
-        <v>251354</v>
+        <v>215066</v>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Sanzioni contro le opposizioni abusive nel settore edilizio</t>
+          <t>Pour une meilleure reconnaissance des cancers professionnels</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
@@ -1994,8 +1994,8 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Il Consiglio federale è incaricato di creare una base legale che permetta di sanzionare le opposizioni abusive. In futuro, coloro che presenteranno opposizione senza un interesse da proteggere o con intenzioni palesemente abusive dovranno poter essere obbligati ad assumere i costi ed eventualmente a risarcire i danni. Il Consiglio federale è tenuto a illustrare come disposizioni in tal senso possano essere disciplinate nella legge sulla pianificazione del territorio (LPT) o in altre leggi federali pertinenti senza compromettere i legittimi diritti di partecipazione della popolazione.
-REASONING: La situazione giuridica attuale consente di protrarre per anni o addirittura di impedire del tutto progetti di costruzione e sviluppo presentando opposizioni di modesta entità o pretestuose. Uno studio recentemente pubblicato dall’Ufficio federale delle abitazioni (UFAB) e dall’Ufficio federale dello sviluppo territoriale (ARE) dimostra chiaramente che le opposizioni sono il motivo più frequente alla base di ritardi e annullamenti di progetti di costruzione di abitazioni. Ne conseguono un aumento dei costi di costruzione, un calo dell’attività edilizia e un’accentuazione della penuria…</t>
+          <t>TEXT: Je prie le Conseil fédéral de répondre aux questions suivantes : - Quel est le coût économique des cancers professionnels en Suisse ? - Quelles mesures prévoit le Conseil fédéral pour lutter contre la sous-reconnaissance de cancers professionnels ? - Quelles mesures prévoit le Conseil fédéral pour clarifier les critères de reconnaissance des cancers professionnels ? - Quelles mesures prévoit le Conseil fédéral pour inciter les soignants à mieux s'impliquer dans les démarches de déclaration des cancers professionnels ? - Quels moyens la SUVA prévoit-elle d'utiliser pour rechercher activement une composante professionnelle chez les patients suisses atteints de cancers professionnels ?
+REASONING: En Suisse, entre 350 à 1850 cancers professionnels ne seraient pas reconnus par l'assurance accident comme maladie professionnelle (Krief et al 2022). Selon les auteurs de l'étude, le problème ne réside pas tant dans la reconnaissance du cancer comme maladie professionnelle par l'assureur accident mais d'avantage dans l'identification des cas potentiels par les soignants et le déclenchement du processus de déclaration. En effet, les cancers professionnels présentant une longe latence d…</t>
         </is>
       </c>
       <c r="F57" s="5" t="inlineStr"/>
@@ -2006,11 +2006,11 @@
         <v>57</v>
       </c>
       <c r="B58" t="n">
-        <v>334999</v>
+        <v>70197</v>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Proteggere i minori dalle immagini intime generate con l'intelligenza artificiale</t>
+          <t>Comment faire face à la pénurie de médicaments?</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
@@ -2020,8 +2020,7 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Il Consiglio federale è incaricato di presentare, nell’ambito dei progetti legislativi in corso, modifiche giuridiche e misure concrete di attuazione per proteggere i minori dalle immagini sintetiche non consensuali (deepfake sessuali e «nudificazione»), assicurarne la rapida rimozione, permettere un perseguimento penale efficace e garantire un sostegno coordinato alle scuole. Si tratta di adeguare il diritto penale e la legge sulle piattaforme nonché d’instaurare un coordinamento federale con i Cantoni per prevenire e reprimere efficacemente la creazione, la diffusione e lo sfruttamento di immagini intime sintetiche non consensuali che coinvolgono minori, con meccanismi rapidi di segnalazione, conservazione delle prove e sostegno alle vittime.
-REASONING: Le prove si moltiplicano: i deepfake sessuali sono utilizzati prevalentemente a fini pornografici o degradanti, e i minori sono esposti a rischi maggiori rispetto agli adulti. L’UNICEF ha di recente affermato che l’abuso tramite deepfake è un abuso, e ha esortato i governi e l’industria a intervenire per contrastare le immagini sessualizzate generate con l’intelligenza artificiale che coinvolgono minori. Anche le politiche …</t>
+          <t>TEXT: Depuis plusieurs mois, certains médicaments d’usage courant ne sont plus disponibles dans nos pharmacies (pansements gastriques, comprimés contre les refroidissements, sprays nasaux, sirops contre la toux,...). Certains de ces médicaments ont des alternatives qui ne sont parfois pas remboursées par l’AOS. Quelles mesures le Conseil fédéral développe-t-il en ce moment face à cette pénurie? Compte-t-il notamment élargir la liste des spécialités?</t>
         </is>
       </c>
       <c r="F58" s="5" t="inlineStr"/>
@@ -2032,11 +2031,11 @@
         <v>58</v>
       </c>
       <c r="B59" t="n">
-        <v>65774</v>
+        <v>157177</v>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Utiliser "Government Technology" dans l'administration</t>
+          <t>Mestieri del futuro. Sostegno pubblico alla riconversione professionale</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
@@ -2046,7 +2045,8 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Lors de la session d'automne 2020, le Conseil national a suivi la proposition du Conseil fédéral d'adopter le postulat 20.3240 " Création d'un centre d'innovation dans l'administration fédérale ". Le progrès technologique, la numérisation et les nouveaux processus qui y sont associés se sont déjà implantés dans la plupart des secteurs de l'économie privée et ont entraîné de nombreux changements. La plateforme Government Technology (GovTech) élargit la palette numérique pour y inclure la collaboration du secteur public avec des entreprises innovantes du secteur privé, y compris des jeunes pousses technologiques. Dans ce contexte, je prie le Conseil fédéral de répondre aux questions suivantes. 1. Le rapport qui sera établi en réponse au postulat 20.3240 pourra-t-il aussi mettre en évidence des aspects qui pourraient être favorisés par l'utilisation ciblée de GovTech dans la coopération avec des jeunes pousses technologiques ? 2. Quels sont les domaines d'application dans lesquels le Conseil fédéral voit des possibilités de tester et d'appliquer les solutions de ces jeunes pousses ? 3. Peut-il envisager d'impliquer spécifiquement ces jeunes pousses dans l'administration ? Si oui…</t>
+          <t>TEXT: Il Consiglio federale è incaricato di illustrare in un rapporto in che modo è possibile creare nuove prospettive professionali in settori in fase di cambiamento strutturale tramite un maggiore investimento pubblico nella formazione continua e professionale.
+REASONING: La transizione ecologica causa la perdita di posti di lavoro in alcuni settori dell'industria e dei servizi, ma allo stesso tempo permette lo sviluppo di nuove professioni legate a un'economia più sostenibile: questo è quanto emerge da un rapporto realizzato dall'Organizzazione Internazionale del Lavoro (OIL) nel 2018. Lo studio mostra un fattore essenziale affinché la transizione ecologica possa portare alla creazione di posti di lavoro: una riconversione professionale efficace e mirata. È dunque necessario disporre di un piano a lungo termine e di dati chiari per identificare le esigenze attuali e future dell'economia e fornire i mezzi per formare (nuovamente) milioni di persone. Tuttavia in Svizzera manca un piano di questo genere. Allo stesso tempo, la digitalizzazione sta allargando il divario tra l'economia di produzione di ieri e l'economia digitale di domani, lasciando indietro dei dipendenti a causa de…</t>
         </is>
       </c>
       <c r="F59" s="5" t="inlineStr"/>
@@ -2057,11 +2057,11 @@
         <v>59</v>
       </c>
       <c r="B60" t="n">
-        <v>67123</v>
+        <v>251354</v>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Zugang zu Angeboten der Kinder- und Jugendarbeit für bis 25-Jährige und kinder- und jugendgerechte Informationen in der Corona-Krise</t>
+          <t>Sanzioni contro le opposizioni abusive nel settore edilizio</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
@@ -2071,7 +2071,8 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Seit dem 13. September 2021 gilt für weite Bereiche des öffentlichen Lebens für Personen ab 16 Jahren die Pflicht, ein Covid-Zertifikat vorzuweisen. Diese Neuerung bringt für Jugendliche ab 16 Jahren erneut eine deutliche Einschränkung ihres Lebens. Ausserschulische Angebote bieten Lernorte, die für umfassende Bildung, physisches und psychisches Wohlbefinden sowie gesunde Entwicklung zentral sind. Die Angebote der Offenen Kinder- und Jugendarbeit (OKJA) gehören zum Grundangebot für Kinder und Jugendliche. Um ihre zentralen Funktionen der Früherkennung und -intervention sowie der Förderung der gesunden Entwicklung leisten zu können, müssen die Einrichtungen einen niederschwelligen Zugang gewährleisten können. Die Zertifikatspflicht ab 16 Jahren führt zu einer unangemessenen Hürde bei diesem Zugang. Erste Rückmeldungen aus der Praxis zeigen, dass ein Teil der Jugendlichen und Familien die Angebote gar nicht mehr besuchen - obwohl gerade unter ihnen viele die Freiräume und Unterstützung dringend nötig hätten. In Zusammenhang mit der Coronakrise und der damit verbundenen, zum Teil widersprüchlichen und nicht kinder- und jugendgerechten Kommunikation, ist das Recht auf Information…</t>
+          <t>TEXT: Il Consiglio federale è incaricato di creare una base legale che permetta di sanzionare le opposizioni abusive. In futuro, coloro che presenteranno opposizione senza un interesse da proteggere o con intenzioni palesemente abusive dovranno poter essere obbligati ad assumere i costi ed eventualmente a risarcire i danni. Il Consiglio federale è tenuto a illustrare come disposizioni in tal senso possano essere disciplinate nella legge sulla pianificazione del territorio (LPT) o in altre leggi federali pertinenti senza compromettere i legittimi diritti di partecipazione della popolazione.
+REASONING: La situazione giuridica attuale consente di protrarre per anni o addirittura di impedire del tutto progetti di costruzione e sviluppo presentando opposizioni di modesta entità o pretestuose. Uno studio recentemente pubblicato dall’Ufficio federale delle abitazioni (UFAB) e dall’Ufficio federale dello sviluppo territoriale (ARE) dimostra chiaramente che le opposizioni sono il motivo più frequente alla base di ritardi e annullamenti di progetti di costruzione di abitazioni. Ne conseguono un aumento dei costi di costruzione, un calo dell’attività edilizia e un’accentuazione della penuria…</t>
         </is>
       </c>
       <c r="F60" s="5" t="inlineStr"/>
@@ -2082,11 +2083,11 @@
         <v>60</v>
       </c>
       <c r="B61" t="n">
-        <v>70545</v>
+        <v>339430</v>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Deklaration von Werbung bei Influencern in der Schweiz</t>
+          <t>Technologies quantiques : pour une stratégie nationale d’anticipation</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
@@ -2096,8 +2097,8 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Der Bundesrat wird beauftragt eine gesetzliche Grundlage zu schaffen, welche die Transparenz und Fairness im Bereich der Influencer-Werbung in der Schweiz fördert. Angesichts der aktuellen Situation, ist nur eine Minderheit der kommerziellen Partnerschaften von Influencer:innen transparent deklariert. Deshalb ist es von entscheidender Bedeutung, klare und verbindliche Regeln zu etablieren.
-REASONING: Mit der Verbreitung sozialer Medien wie Instagram kam auch der Aufstieg der Influencer:innen (Deutsch: Beeinflusser:innen). Solche Influencer:innen sind für ihre Fans Vorbilder in Sachen Mode, Fitness, Entschlackungstees, Nahrungsergänzungsmittel, Schönheit bzw. Schönheitsprodukte, Kochen etc. Deren Empfehlungen gelten viel und sind der Werbeindustrie darum viel Geld wert. Gemäss einer EU-Untersuchung veröffentlichen 97 Prozent der Influencer:innen kommerzielle Inhalte, jedoch deklarieren nur 20 Prozent diese Partnerschaften transparent. Konsumenten dürfen nicht durch versteckte Werbung getäuscht werden. Umso mehr, wenn die Zielgruppe sehr jung und leicht beeinflussbar ist. Die fehlende Deklaration von Werbung zeigt auf, dass in der aktuellen Situation Handlungsbedarf besteht. D…</t>
+          <t>OTHER (Texte déposé): Le Conseil fédéral est chargé de présenter un rapport analysant : a) les principaux impacts prévisibles de la révolution quantique sur les grands domaines de l'action publique, ainsi que les principales mesures à envisager ; b) le positionnement stratégique de la Suisse pour saisir les opportunités et limiter les risques ; c) les conditions-cadres nécessaires pour développer, attirer et retenir en Suisse les entreprises et les talents à la pointe de ces technologies. Il formulera des propositions pour atteindre ces objectifs et posera les bases d'une stratégie nationale quantique.
+OTHER (Développement): La révolution quantique n'est plus une hypothèse de long terme. En 2026, les ordinateurs quantiques sortent des laboratoires et commencent à surpasser les systèmes classiques dans des domaines stratégiques. Leur convergence avec l'intelligence artificielle ouvre une ère de puissance de calcul sans précédent, avec des implications majeures, notamment pour la sécurité, la santé, la finance, la formation et la souveraineté numérique. La Suisse a eu la sagesse d'anticiper ces ruptures. La Swiss Quantum Initiative, dotée de 82,1 millions de francs pour la période F…</t>
         </is>
       </c>
       <c r="F61" s="5" t="inlineStr"/>
@@ -2108,11 +2109,11 @@
         <v>61</v>
       </c>
       <c r="B62" t="n">
-        <v>65119</v>
+        <v>158650</v>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Chasser sans preuve de la sûreté du tir est-il sûr, respectueux des animaux et efficace?</t>
+          <t>Protezione contro le molestie sessuali nelle commesse pubbliche</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
@@ -2122,7 +2123,8 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Depuis le 1er janvier 2017, fournir la preuve de la sûreté du tir est obligatoire dans toute la Suisse pour pouvoir s'adonner à la chasse. La conférence des services de la faune, de la chasse et de la pêche de la Suisse et de la Principauté de Liechtenstein a présenté le principe applicable : " La sécurité de la manipulation de l'arme de chasse et la précision du tir sont des éléments indispensables pour une chasse responsable et respectueuse envers la protection des animaux. Pour des raisons de protection des animaux, de sécurité, de valorisation du gibier mais aussi pour une chasse efficace, l'artisanat de base des chasseurs, la sûreté du tir revêt une importance capitale. Un entraînement régulier de tir et une attestation valable sur la sûreté du tir devraient être évidents pour chaque chasseur ". En raison du coronavirus, les stands de tir sont fermés dans toute la Suisse jusqu'à nouvel ordre. Les services cantonaux de la chasse réagissent manifestement de façon très différente. Certains prolongent automatiquement jusqu'au 30 septembre 2020 les permis de tir échus, d'autres exigent un renouvellement de la preuve de la sûreté du tir dans les deux mois à compter de la levée…</t>
+          <t>TEXT: Il Consiglio federale è incaricato di modificare l'articolo 4 capoverso 1 dell'ordinanza sugli appalti pubblici (OAPub) come segue: Art. 4 Condizioni di partecipazione e criteri di idoneità 1 Il committente può delegare l'esecuzione dei controlli relativi alla parità salariale e a una protezione efficace contro il mobbing e le molestie sessuali segnatamente all'Ufficio federale per l'uguaglianza fra donna e uomo (UFU). L'UFU definisce i dettagli dei controlli in una direttiva. Il committente può trasmettere all'UFU l'autodichiarazione degli offerenti relativa all'osservanza della parità salariale. Una minoranza della Commissione (Friedli Esther, Aeschi Thomas, Amaudruz, Burgherr, Dettling, Feller, Gössi, Regazzi, Ritter, Schneeberger, Steinemann, Tuena) propone di respingere la mozione.
+REASONING: Attualmente la legislazione sugli appalti pubblici prevede che le commesse siano aggiudicate soltanto alle imprese che osservano le "disposizioni in materia di tutela dei lavoratori e delle condizioni di lavoro". Ciò presuppone anche il rispetto della legge sul lavoro, in particolare la tutela dell'integrità personale dei lavoratori che vi è disciplinata e che si riferisce anche ai…</t>
         </is>
       </c>
       <c r="F62" s="5" t="inlineStr"/>
@@ -2133,11 +2135,11 @@
         <v>62</v>
       </c>
       <c r="B63" t="n">
-        <v>159211</v>
+        <v>337367</v>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Soumettre la Société suisse de radiodiffusion et télévision au Contrôle fédéral des finances</t>
+          <t>Legge sul sostegno alla banda larga (LSBL)</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
@@ -2145,12 +2147,7 @@
           <t>open</t>
         </is>
       </c>
-      <c r="E63" s="2" t="inlineStr">
-        <is>
-          <t>TEXT: La loi fédérale sur la radio et la télévision est modifiée de sorte que la Société suisse de radiodiffusion et télévision (SSR) soit soumise au Contrôle fédéral des finances (CDF) en tant qu'autorité de surveillance financière.
-REASONING: La SSR remplit un mandat de prestations global au niveau national et au niveau des régions linguistiques. Elle est principalement financée par la redevance, dont le montant total s'élève à plus d'un milliard de francs. Compte tenu de cette somme, du volume important des activités, du très grand intérêt public et des discussions politiques en cours, la SSR devrait être soumise à la surveillance financière du CDF, comme les autres organisations auxquelles la Confédération confie l'exécution de tâches publiques (voir art. 8, al. 1, let. d, LCF). En tant qu'organe indépendant, le CDF devrait pouvoir examiner les finances de la SSR du point de vue des risques et de la gestion des activités, en étroite collaboration avec les autres autorités et organes chargés de contrôler la société. L'autonomie dans la conception et la gestion des programmes de radio et de télévision, garantie par l'art. 93, al. 3, Cst., resterait opposable au CDF. D'autres org…</t>
-        </is>
-      </c>
+      <c r="E63" s="2" t="inlineStr"/>
       <c r="F63" s="5" t="inlineStr"/>
       <c r="G63" s="5" t="inlineStr"/>
     </row>
@@ -2159,11 +2156,11 @@
         <v>63</v>
       </c>
       <c r="B64" t="n">
-        <v>64883</v>
+        <v>63751</v>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Luftfahrtgesetz. Änderung</t>
+          <t>Der Bundesrat soll den falsch eingeschlagenen Weg zur Flugsicherheit korrigieren</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
@@ -2171,7 +2168,12 @@
           <t>open</t>
         </is>
       </c>
-      <c r="E64" s="2" t="inlineStr"/>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Der Bundesrat wird beauftragt, dafür zu sorgen, dass die am 1. Januar 2019 in Kraft getretene Änderung des Luftfahrtgesetzes (LFG) - insbesondere Artikel 10a - so umgesetzt wird, dass sie dem Willen des Gesetzgebers entspricht und für alle Stakeholder eine praxistaugliche Lösung ermöglicht.
+REASONING: Gemäss Schreiben vom Bazl vom 4. März 2019 sei es der Wille des Gesetzgebers, dass die Radiotelefonie mit dem Flugsicherungsdienst im Luftraum über der Schweiz auf Englisch stattfindet. Bei der Beratung der Teilrevision 1 plus des LFG (16.062) in den Räten war die Standardsprache für den Funkverkehr (Art. 10a) umstritten gewesen. Schliesslich einigten sich die Räte darauf, dass der Funkverkehr grundsätzlich in Englisch zu erfolgen hat, der Bundesrat aber Ausnahmen definieren soll. Im Hinblick auf die Umsetzung mit Definition der Ausnahmen ging der Gesetzgeber davon aus, dass diese vom internationalen Rahmen fraglich abweichende Regelung nur die Landesflughäfen und den kommerziellen internationalen Linienluftverkehr betreffen soll. Bei den unteren Lufträumen, für die allgemeine Luftfahrt, die Militärflugplätze und die Regionalflugplätze soll mittels Ausnahmeregelung wie bis anhi…</t>
+        </is>
+      </c>
       <c r="F64" s="5" t="inlineStr"/>
       <c r="G64" s="5" t="inlineStr"/>
     </row>
@@ -2180,11 +2182,11 @@
         <v>64</v>
       </c>
       <c r="B65" t="n">
-        <v>297761</v>
+        <v>214539</v>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Chiarimenti giuridici e potenzialità dell'impiego dell'intelligenza artificiale nei settori della polizia e della sicurezza interna</t>
+          <t>Promuovere e non ostacolare la ricerca e la sperimentazione clinica con dispositivi medici non commerciali. Gli emolumenti e gli oneri vanno urgentemente adeguati</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
@@ -2194,7 +2196,8 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Il Consiglio federale è incaricato di presentare un rapporto sull’impiego dell’intelligenza artificiale (IA) nei settori della polizia, della sicurezza interna e del perseguimento penale, illustrandone il potenziale, le basi legali e i limiti costituzionali, in particolare per la protezione della vita privata. Sulla base di queste conclusioni, dovrà sottoporre al Parlamento linee guida per un utilizzo dell’IA coerente e conforme ai diritti fondamentali nei settori della polizia, della sicurezza interna e del perseguimento penale, che tenga conto della sovranità digitale della Svizzera. Il rapporto dovrà in particolare: 1. illustrare il potenziale e gli ambiti d’applicazione delle tecnologie di IA per rendere più efficace la lotta alla criminalità e contribuire alla salvaguardia della sicurezza interna; 2. analizzare il quadro giuridico esistente per l’utilizzo delle tecnologie di IA nel settore della sicurezza e identificare le eventuali lacune; 3. esporre i limiti costituzionali all’impiego delle tecnologie di IA nei settori della polizia e della sicurezza, e definire le condizioni quadro e le linee guida per l’utilizzo di queste tecnologie; 4. mostrare come i requisiti in m…</t>
+          <t>TEXT: Il Consiglio federale è incaricato di adeguare le disposizioni di esecuzione della legge sugli agenti terapeutici (in particolare gli art. 4-9), al fine di consentire lo sviluppo della ricerca clinica non commerciale. I gravosi oneri previsti da tali disposizioni e le tariffe fissate per la sperimentazione clinica devono essere oggetto di un adeguamento in modo da non ostacolare l'avvio di importanti progetti di ricerca.
+REASONING: La ricerca clinica non commerciale è importante per l'innovazione. Dall'introduzione della nuova ordinanza sugli emolumenti essa ne è risultata fortemente ostacolata o resa quasi impossibile. Soprattutto in ambito universitario i progetti condotti da giovani ricercatori non sono quasi più possibili in quanto non finanziabili. Il diritto vigente e l'ordinanza sugli emolumenti ostacolano fortemente la ricerca non operando alcuna distinzione tra ricerca commerciale e non commerciale. Tutto ciò non è nell'interesse né della ricerca di base, né delle istituzioni, né dei pazienti e rappresenta un ostacolo in particolare per i giovani ricercatori. L'equiparazione della ricerca non commerciale a quella delle imprese commerciali private non è nel nostro in…</t>
         </is>
       </c>
       <c r="F65" s="5" t="inlineStr"/>
@@ -2205,11 +2208,11 @@
         <v>65</v>
       </c>
       <c r="B66" t="n">
-        <v>153475</v>
+        <v>159211</v>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Web 3.0 - Quelle place pour la Suisse dans un web décentralisé?</t>
+          <t>Soumettre la Société suisse de radiodiffusion et télévision au Contrôle fédéral des finances</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
@@ -2219,8 +2222,8 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Le Conseil fédéral est prié d'étudier les perspectives du Web 3.0, les opportunités économiques pour la Suisse et les possibilités d'y promouvoir nos valeurs. Le Web actuel est très centralisé. L'essor de la technologie "blockchain" pourrait remettre en cause la suprématie des GAFA et permettre une redistribution du pouvoir vers les internautes et de nouveaux acteurs. Le potentiel de la "blockchain" est tel que l'Europe et la Suisse pourraient retrouver une capacité d'influence sur Internet. Nous sommes à un moment charnière : c'est maintenant qu'il faut agir. Cette étude précisera les enjeux du Web 3.0 ; définira notre stratégie en matière de Web 3.0 et de "blockchain" (puisque la Suisse est dans le top 3 mondial); déterminera les talents nécessaires ; se demandera s'il faudrait créer des "blockchain" publiques ; évaluera ce que nous sommes prêts à faire pour protéger la sphère privée, favoriser une concurrence plus juste, répartir le pouvoir de manière plus équilibrée : trois promesses du Web 3.0.
-REASONING: La technologie "blockchain" pourrait bouleverser la structure sous-jacente d'Internet. La sécurité quasiment inviolable qu'elle apporte transformerait profondément la …</t>
+          <t>TEXT: La loi fédérale sur la radio et la télévision est modifiée de sorte que la Société suisse de radiodiffusion et télévision (SSR) soit soumise au Contrôle fédéral des finances (CDF) en tant qu'autorité de surveillance financière.
+REASONING: La SSR remplit un mandat de prestations global au niveau national et au niveau des régions linguistiques. Elle est principalement financée par la redevance, dont le montant total s'élève à plus d'un milliard de francs. Compte tenu de cette somme, du volume important des activités, du très grand intérêt public et des discussions politiques en cours, la SSR devrait être soumise à la surveillance financière du CDF, comme les autres organisations auxquelles la Confédération confie l'exécution de tâches publiques (voir art. 8, al. 1, let. d, LCF). En tant qu'organe indépendant, le CDF devrait pouvoir examiner les finances de la SSR du point de vue des risques et de la gestion des activités, en étroite collaboration avec les autres autorités et organes chargés de contrôler la société. L'autonomie dans la conception et la gestion des programmes de radio et de télévision, garantie par l'art. 93, al. 3, Cst., resterait opposable au CDF. D'autres org…</t>
         </is>
       </c>
       <c r="F66" s="5" t="inlineStr"/>
@@ -2231,11 +2234,11 @@
         <v>66</v>
       </c>
       <c r="B67" t="n">
-        <v>64326</v>
+        <v>156064</v>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Stopp der Datensammelwut in der Armee!</t>
+          <t>Promozione dell'home office e libertà imprenditoriale</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
@@ -2245,8 +2248,7 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Der Bundesrat wird beauftragt das Bundesgesetz über die Archivierung (BGA) so abzuändern, dass die Armee nicht mehr gegenüber dem Bundesarchiv angebotspflichtig ist.
-REASONING: Das Bundesarchiv sieht in einer Vielzahl von Daten der Armeeformationen eine wichtige Quellengrundlage für die Militär-, Sozial-, und Kulturgeschichte der Schweiz. Deshalb ist die Armee gemäss dem Bundesgesetz über die Archivierung Artikel 1 Absatz 1 litera b gegenüber dem Bundesarchiv angebotspflichtig. Dies bedeutet, dass Einheiten und Truppenkörper heikle Personendaten, welche nicht anonymisiert werden (z. Bsp. Disziplinarstrafdossiers) via das Bundesarchiv nach Ablauf einer Schutzfrist der Öffentlichkeit zugänglich machen muss. Im Falle der Überweisung der Disziplinarstrafdossiers bedeutet dies einen Verstoss gegen Artikel 205 des Militärstrafgesetzes, welches die Vernichtung der Unterlagen nach 5 Jahren vorschreibt. Angehörige der Armee können mit der Datenübermittlung an das Bundesarchiv, ohne ihr Wissen und ohne ihr ausdrückliches Einverständnis, zu Personen des öffentlichen Interesses werden. Kein Angehöriger der Armee kann deshalb kontrollieren, welche Daten an das Bundesarchiv gesendet werde…</t>
+          <t>TEXT: In seguito alla crisi del coronavirus si sono nuovamente levate delle voci in campo politico che auspicano una maggiore promozione dell'home office (lavoro a domicilio, telelavoro ecc.). A questo proposito, chiedo al Consiglio federale di rispondere alle seguenti domande: 1. Quale promozione diretta e indiretta dell'home office esiste da parte della Confederazione? 2. Quali sono le basi legali di questa promozione? 3. Su quali disposizioni di diritto del lavoro si basa in generale l'home office? 4. Cosa pensa il Consiglio federale del fatto che il sostegno statale dell'home office influenza in modo molto forte la cultura d'impresa? 5. Quali effetti produce la sentenza del Tribunale federale che impone al datore di lavoro di farsi carico di parte della pigione in caso di home office? 6. Come si pone tale promozione rispetto alla libertà economica e imprenditoriale? C'è un possibile conflitto con la libertà economica sancita dalla Costituzione? 7. Come giudica il Consiglio federale il fatto che nel caso dell'home office gli scambi e le relazioni personali e sociali diventano meno importanti? 8. Esistono studi o indizi riscontrati nella prassi, soprattutto relativi al periodo de…</t>
         </is>
       </c>
       <c r="F67" s="5" t="inlineStr"/>
@@ -2257,11 +2259,11 @@
         <v>67</v>
       </c>
       <c r="B68" t="n">
-        <v>67184</v>
+        <v>235974</v>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Dazit e controllo delle frontiere</t>
+          <t>Le prospettive dell'AVS erano errate. Lo sono anche quelle dell'AI?</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
@@ -2271,7 +2273,8 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Nel quadro del Rapporto del Consiglio federale in adempimento del postulato 17.4177 del 14.12.2017, l'approccio risulta essere piuttosto teorico e poco orientato alla reale operatività quotidiana del personale che opera ai valichi ferroviari. In considerazione degli importanti cambiamenti previsti, è opportuno conoscere maggiori informazioni operative che toccano la quotidianità dei dipendenti e dei cittadini. 1. Sono previsti investimenti infrastrutturali utili alle attività di controllo, soprattutto merci, in tutte le stazioni di confine (Basilea, Buchs, Vallorbe, Ginevra, Domodossola, Luino, Chiasso)? Sono di competenza dell'AfD o direttamente delle FFS? Come è garantito il finanziamento e il coordinamento delle procedure? 2. Si prevede di installare scanner fissi per il traffico ferroviario merci? In quali stazioni? 3. La riforma in corso prevede un aggiornamento degli accordi internazionali vigenti per le stazioni di frontiera? Quali accordi si prevede di aggiornare con le rispettive controparti? 4. Il progetto Dazit prevede un coinvolgimento attivo - per ottimizzare i flussi di lavoro e i controlli - delle aziende ferroviarie svizzere leader nel traffico delle merci? Se…</t>
+          <t>TEXT: Chiedo al Consiglio federale di rispondere alle seguenti domande: È noto che sono stati commessi errori nelle previsioni dell’AVS. Sono stati commessi gli stessi errori anche per quanto riguarda le cifre dell’AI? I debiti dell’AI gravano l’AVS. L’Amministrazione federale ha ripetutamente comunicato a partire da quando l’AI potrà ridurre il debito nel bilancio dell’AVS. Quali dati sono stati comunicati dal 2012? Quali motivazioni sono state addotte dal 2012 per la costante posticipazione di questo momento? Quando saranno presentate al Parlamento nuove basi di dati che contengano anche la crescita delle nuove rendite e la diminuzione dei tassi di uscita, fattori menzionati da Compenswiss? Il Consiglio federale come garantisce una maggiore attendibilità delle previsioni dell’AI affinché si disponga di basi sicure per una prossima revisione dell’AI?
+REASONING: Il 18 febbraio 2025 il Consiglio di amministrazione di Compenswiss ha comunicato che «[a]nche per il fondo AI le prospettive finanziarie sono peggiorate a causa dell’aumento delle nuove rendite e della diminuzione dei tassi di uscita» e avvertito che «[d]ata la sua situazione finanziaria, è improbabile che l’AI possa ridur…</t>
         </is>
       </c>
       <c r="F68" s="5" t="inlineStr"/>
@@ -2282,11 +2285,11 @@
         <v>68</v>
       </c>
       <c r="B69" t="n">
-        <v>339430</v>
+        <v>214819</v>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Technologies quantiques : pour une stratégie nationale d’anticipation</t>
+          <t>Bundesgericht. Wahl von zwei ordentlichen Richtern/Richterinnen</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
@@ -2294,12 +2297,7 @@
           <t>open</t>
         </is>
       </c>
-      <c r="E69" s="2" t="inlineStr">
-        <is>
-          <t>OTHER (Texte déposé): Le Conseil fédéral est chargé de présenter un rapport analysant : a) les principaux impacts prévisibles de la révolution quantique sur les grands domaines de l'action publique, ainsi que les principales mesures à envisager ; b) le positionnement stratégique de la Suisse pour saisir les opportunités et limiter les risques ; c) les conditions-cadres nécessaires pour développer, attirer et retenir en Suisse les entreprises et les talents à la pointe de ces technologies. Il formulera des propositions pour atteindre ces objectifs et posera les bases d'une stratégie nationale quantique.
-OTHER (Développement): La révolution quantique n'est plus une hypothèse de long terme. En 2026, les ordinateurs quantiques sortent des laboratoires et commencent à surpasser les systèmes classiques dans des domaines stratégiques. Leur convergence avec l'intelligence artificielle ouvre une ère de puissance de calcul sans précédent, avec des implications majeures, notamment pour la sécurité, la santé, la finance, la formation et la souveraineté numérique. La Suisse a eu la sagesse d'anticiper ces ruptures. La Swiss Quantum Initiative, dotée de 82,1 millions de francs pour la période F…</t>
-        </is>
-      </c>
+      <c r="E69" s="2" t="inlineStr"/>
       <c r="F69" s="5" t="inlineStr"/>
       <c r="G69" s="5" t="inlineStr"/>
     </row>
@@ -2308,11 +2306,11 @@
         <v>69</v>
       </c>
       <c r="B70" t="n">
-        <v>339887</v>
+        <v>161893</v>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Datencenter und Energiespeicher in militärischen Bunkern und Kavernen ermöglichen!</t>
+          <t>Excursions en famille dans le jet du Conseil fédéral</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
@@ -2322,8 +2320,8 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Der Bundesrat wird beauftragt, die notwendigen gesetzlichen und organisatorischen Voraussetzungen zu schaffen, damit geeignete, militärisch nicht oder nur teilweise genutzte Bunker, Kavernen und andere geschützte Untertageanlagen für sicherheitsrelevante zivile und kommerzielle Zwecke genutzt werden können. Insbesondere sollen folgende Nutzungen ermöglicht werden: – geschützte Rechen- und Datencenter – Batterie- und Energiespeicher – kritische Kommunikations- und Versorgungsinfrastrukturen; – weitere Nutzungen, welche gleichzeitig die Resilienz und Versorgungssicherheit der Schweiz stärken. Die militärischen und sicherheitspolitischen Interessen haben jederzeit Vorrang. Strategisch wichtige Anlagen sollen im Eigentum des Bundes verbleiben und bei Bedarf wieder vollständig für militärische Zwecke zur Verfügung stehen. Dazu sind geeignete Vermietungs-, Nutzungs- und Zusammenarbeitsmodelle mit öffentlichen und privaten Partnern zu schaffen sowie bestehende rechtliche Hindernisse für eine solche Doppelnutzung soweit möglich zu beseitigen.
-REASONING: Die Armee verfügt über zahlreiche Bunker, Kavernen und andere hochwertige geschützte Untertageanlagen. Ein Teil davon wird heute ni…</t>
+          <t>TEXT: Début mai, le CN Nussbaumer et le CE Herzog se sont rendus à Rome avec le Service de transport aérien de la Confédération (STAC). Selon les médias, les fils de Mme Herzog ont voyagé avec eux dans le jet du Conseil fédéral. - Quelle était leur fonction dans la délégation officielle pour la prestation de serment de la Garde suisse ? - Si les fils ne faisaient pas partie de la délégation officielle, depuis quand le LTDB peut-il être réservé pour des "excursions familiales" ?
+ANSWER: Selon le ch. 2.10 de la Directive de la Délégation administrative du 13 mai 2022 concernant les activités internationales des délégations parlementaires permanentes et des délégations parlementaires non permanentes, l’Assemblée fédérale peut, une fois par année, prendre en charge les frais d’une personne accompagnante dans le cadre d’un voyage officiel des présidents ou présidentes des conseils à l’étranger. Par le passé, une personne accompagnait les présidents ou présidentes des conseils lors d’un « voyage présidentiel » officiel à l’étranger, qui avait lieu une fois par année, sans délégation du Parlement, généralement dans une destination lointaine. Cette forme de « voyage présidentiel » a été a…</t>
         </is>
       </c>
       <c r="F70" s="5" t="inlineStr"/>
@@ -2334,11 +2332,11 @@
         <v>70</v>
       </c>
       <c r="B71" t="n">
-        <v>70317</v>
+        <v>64434</v>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Doppelbesteuerung. Abkommen mit Serbien</t>
+          <t>Garantire il diritto alle prestazioni complementari alle persone che nell'infanzia hanno subito collocamenti coatti e alle persone internate sulla base di una decisione amministrativa</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
@@ -2346,7 +2344,11 @@
           <t>open</t>
         </is>
       </c>
-      <c r="E71" s="2" t="inlineStr"/>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: La Commissione della sicurezza sociale e della sanità del Consiglio degli Stati decide di elaborare un progetto volto a garantire che la riparazione morale dovuta alle persone che nell'infanzia hanno subito collocamenti coatti e alle persone internate sulla base di una decisione amministrativa non pregiudichi il loro diritto alle prestazioni complementari. A tale scopo occorre stralciare la parte finale della lettera c dell'articolo 4 capoverso 6 della legge federale sulle misure coercitive a scopo assistenziale e i collocamenti extrafamiliari prima del 1981 (LMCCE).</t>
+        </is>
+      </c>
       <c r="F71" s="5" t="inlineStr"/>
       <c r="G71" s="5" t="inlineStr"/>
     </row>
@@ -2355,11 +2357,11 @@
         <v>71</v>
       </c>
       <c r="B72" t="n">
-        <v>154501</v>
+        <v>155827</v>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Come incoraggiare lo spirito pionieristico svizzero?</t>
+          <t>Crisi dovuta al coronavirus. Soluzione globale per stabilizzare le finanze federali e le opere sociali</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
@@ -2369,8 +2371,8 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Le buone condizioni quadro per la ricerca presto non saranno più sufficienti a garantire alla Svizzera il suo posto di leader mondiale nel campo dell'innovazione, dei brevetti e delle blockchain. I nuovi giganti del digitale stanno nascendo altrove. In 18 mesi, l'utile della piattaforma cinese blockchain Binance è passato da zero a un miliardo di fanchi e l'impresa sta sviluppando un intero ecosistema a tempo di record: Binance Labs, Binance Info, Binance Chian, Binance Uganda ecc. Quella delle blockchain è una "tecnologia di frontiera" che permette di superare i limiti conosciuti della tecnologia. La padronanza tecnologica non basta più per essere concorrenziale in questo settore: è necessario sviluppare in Svizzera uno spirito pionieristico paragonabile a quello della Silicon Valley. Qual è la posizione del Consiglio federale al riguardo?
-REASONING: La Svizzera sostiene attivamente l'innovazione con l'agenzia Innosuisse, i suoi cinque parchi dell'innovazione, gli intensi scambi tra economia e formazione superiore, il dinamismo delle sue università e numerose start-up. Ma il nostro deve diventare un vero Paese delle opportunità. Trovare un finanziamento per un prototipo è r…</t>
+          <t>TEXT: Il Consiglio federale è incaricato di presentare al Parlamento una soluzione globale che indichi come le prestazioni straordinarie fornite dalla Confederazione durante la crisi dovuta al coronavirus e le future perdite fiscali provocate dalla suddetta crisi debbano essere contabilizzate nei conti della Confederazione. Il Consiglio federale deve indicare in particolare come nei prossimi 6-8 anni dovrà essere coperto il disavanzo del fondo di compensazione stimato in 40 miliardi di franchi, come dovranno essere compensate le perdite fiscali stimate in cinque miliardi di franchi l'anno e quali misure dovranno essere adottate per consolidare le assicurazioni sociali del 1° e del 2° pilastro. Condizione: il freno all'indebitamento, che ha dato prova di efficacia, non deve essere allentato.
+REASONING: Il Consiglio federale ha espresso grande preoccupazione per le conseguenze economiche della crisi dovuta al coronavirus. Le prestazioni straordinarie graveranno le casse della Confederazione per un importo di circa 40 miliardi di franchi, che sarà trasferito a un fondo di compensazione. La base legale prevede che tale fondo sia riequilibrato entro 6-8 anni. Inoltre, a causa dell'immi…</t>
         </is>
       </c>
       <c r="F72" s="5" t="inlineStr"/>
@@ -2381,11 +2383,11 @@
         <v>72</v>
       </c>
       <c r="B73" t="n">
-        <v>156405</v>
+        <v>339511</v>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>Misure per potenziare l'agricoltura alpestre e di montagna</t>
+          <t>TARDOC : Où est passée l’amélioration annoncée pour nos médecins de famille ?</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
@@ -2395,8 +2397,8 @@
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Il Consiglio federale è incaricato di valutare quali misure possono essere adottate nell'ambito della politica agricola al fine di potenziare l'agricoltura alpestre e di montagna in seguito all'affossamento della revisione della legge sulla caccia
-REASONING: La popolazione di lupi in rapida crescita nelle aree di montagna aumenta ulteriormente la pressione sull'agricoltura e sull'economia alpestre nonché sul turismo alpino. La situazione è già oggi talmente precaria che alcuni alpi non vengono più caricati o viene anticipata la discesa dall'alpe. Il rigetto della revisione della legge sulla caccia in occasione della votazione popolare di settembre 2020 ha inasprito ulteriormente la situazione. È elevato il rischio che venga abbandonata la gestione di numerose aziende dedite all'agricoltura di montagna. Senza contromisure incombe la minaccia di un'accelerazione dell'esodo e dell'abbandono di intere vallate. Inoltre, sono da attendersi sempre più conflitti con le attività turistiche, da un lato a causa delle misure per la protezione delle greggi, dall'altro perché i bovini dopo gli attacchi dei lupi diventano paurosi e aggressivi. Entrambe le situazioni causano già grandi prob…</t>
+          <t>OTHER (Texte déposé): Le Conseil fédéral est prié de répondre aux questions suivantes : - Le Conseil fédéral dispose-t-il d'éléments concrets démontrant que la mise en œuvre de TARDOC améliore la situation des médecins de premier recours ? - Dans le cas contraire, quelles sont les raisons pour lesquelles les promesses de revalorisation ne se concrétisent pas ? - Quelles mesures concrètes le Conseil fédéral compte-t-il prendre pour mettre en œuvre ma motion 22.4357, validée par les Chambres fédérales et visant à revaloriser la médecine de premier recours, en respectant la neutralité des coûts ? - Quand soumettra-t-il au Parlement des propositions concrètes en la matière ?
+OTHER (Développement): Depuis des années, le Conseil fédéral et le Parlement entendent revaloriser la médecine de premier recours, notamment en rééquilibrant les tarifs par rapport à ceux de la médecine à forte composante médico-technique. Les acteurs du TARDOC avaient annoncé que le nouveau tarif contribuerait à cet objectif, ce que prévoyait aussi le Conseil fédéral. Or, les promesses des acteurs du TARDOC semblent aujourd'hui s’évanouir : les données provisoires ne laissent pas entrevoir de réelle amélioration …</t>
         </is>
       </c>
       <c r="F73" s="5" t="inlineStr"/>
@@ -2407,11 +2409,11 @@
         <v>73</v>
       </c>
       <c r="B74" t="n">
-        <v>155864</v>
+        <v>70545</v>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Modification de la loi sur l'assurance-chômage</t>
+          <t>Deklaration von Werbung bei Influencern in der Schweiz</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
@@ -2421,8 +2423,8 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Le Conseil fédéral est chargé de revoir certaines dispositions de la loi sur l'assurance chômage, en particulier l'art. 31, al. 3, let. b, afin que dans une PME familiale le conjoint de l'employeur, occupé dans l'entreprise de celui-ci, puisse bénéficier d'une indemnité plafonnée en cas de réduction de l'horaire de travail (RHT) consécutive à des circonstances non imputables à l'employeur (cas de rigueur selon l'art. 32, al. 3). Une minorité de la commission (Aeschi Thomas, Amaudruz, de Courten, Dobler, Glarner, Herzog Verena, Riniker, Rösti, Sauter, Schläpfer) propose de rejeter la motion.
-REASONING: La crise Covid-19 a démontré la précarité des petites entreprises familiales, notamment celles où le conjoint est exclu du droit à l'indemnité en cas de réduction de l'horaire de travail (RHT), au même titre qu'une personne exerçant une influence sur l'entreprise (art. 31 ch. 3 al b et c). L'ordonnance 2 Covid-19 a corrigé pour la durée de la crise cette lacune de la loi sur l'assurance chômage en octroyant à ces personnes des mesures RHT. Il s'agit de prolonger cette mesure par une modification de la loi afin que le Conseil fédéral n'ait pas à édicter de nouvelles règles pour …</t>
+          <t>TEXT: Der Bundesrat wird beauftragt eine gesetzliche Grundlage zu schaffen, welche die Transparenz und Fairness im Bereich der Influencer-Werbung in der Schweiz fördert. Angesichts der aktuellen Situation, ist nur eine Minderheit der kommerziellen Partnerschaften von Influencer:innen transparent deklariert. Deshalb ist es von entscheidender Bedeutung, klare und verbindliche Regeln zu etablieren.
+REASONING: Mit der Verbreitung sozialer Medien wie Instagram kam auch der Aufstieg der Influencer:innen (Deutsch: Beeinflusser:innen). Solche Influencer:innen sind für ihre Fans Vorbilder in Sachen Mode, Fitness, Entschlackungstees, Nahrungsergänzungsmittel, Schönheit bzw. Schönheitsprodukte, Kochen etc. Deren Empfehlungen gelten viel und sind der Werbeindustrie darum viel Geld wert. Gemäss einer EU-Untersuchung veröffentlichen 97 Prozent der Influencer:innen kommerzielle Inhalte, jedoch deklarieren nur 20 Prozent diese Partnerschaften transparent. Konsumenten dürfen nicht durch versteckte Werbung getäuscht werden. Umso mehr, wenn die Zielgruppe sehr jung und leicht beeinflussbar ist. Die fehlende Deklaration von Werbung zeigt auf, dass in der aktuellen Situation Handlungsbedarf besteht. D…</t>
         </is>
       </c>
       <c r="F74" s="5" t="inlineStr"/>
@@ -2433,11 +2435,11 @@
         <v>74</v>
       </c>
       <c r="B75" t="n">
-        <v>214904</v>
+        <v>201807</v>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>Abbau von Handelshemmnissen beim Import von Gebrauchtwagen</t>
+          <t>Rapporto sulle condizioni di lavoro e gli infortuni nel settore delle economie di piattaforma</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
@@ -2447,8 +2449,8 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Der Bundesrat wird beauftragt, auf Verordnungsstufe rechtliche Grundlagen für den weltweiten Import von Gebrauchtwagen zu schaffen. Heute können insbesondere amerikanische Fahrzeuge, die als Gebrauchtwagen in die Schweiz importiert werden, in der Schweiz nicht zugelassen werden, weil das Datum der 1. Inverkehrsetzung (1. Inv.) in den amerikanischen Fahrzeugpapieren nicht immer vermerkt ist. Nordamerika registriert primär den Modelljahrgang eines Personenwagens oder eines Nutzfahrzeuges. Dennoch verlangen die Schweizer Behörden von der amerikanischen Verkehrsbehörde einen Nachweis über die 1. Inv., was in der Praxis nahezu unmöglich ist. Der Handel mit Gebrauchtwagen ist aufgrund dieses Handelshemmnisses praktisch inexistent, was der Volkswirtschaft schadet. Die Motion bezweckt nur den Abbau einer bürokratischen Formalität, Lärm-, Abgas- und Sicherheitsvorschriften sind davon nicht betroffen.
-REASONING: Amerikanische Fahrzeuge erhalten bei der 1. Inv. in den USA als Zulassungsdokument ein sogenanntes "Certificate of Title", welches vom National Motor Vehicle Title Informations System (NMVTIS) ausgestellt wird. In diesem offiziellen Dokument wird ausschliesslich das Modell-Jah…</t>
+          <t>TEXT: Il Consiglio federale è incaricato di redigere un rapporto sulle condizioni di lavoro e gli infortuni nel settore dell'economia di piattaforma che includa in particolare le statistiche sul numero e il tipo di infortuni nonché le relative cause.
+REASONING: Da vari anni diverse società di piattaforma hanno stabilito le loro attività in Svizzera e altre sono state fondate nel nostro Paese. Negli ultimi anni sono stati presentati anche vari interventi parlamentari riguardanti lo status da accordare ad autisti, fattorini e corrieri che lavorano per queste piattaforme. Vi sono però pochi studi o statistiche sulle condizioni di lavoro e, in particolare, sul numero e il tipo di infortuni del personale impiegato in questo settore in Svizzera. Il Consiglio federale è pertanto incaricato di redigere un rapporto su questa categoria di dipendenti, dato che è in questo modo che vanno ormai definiti. Il rapporto deve in particolare indicare il numero e il tipo di infortuni che riguardano i lavoratori di queste piattaforme e, per quanto possibile, le relative cause. Una ricerca francese del 2021 ha dimostrato che il 25 per cento delle 517 persone interpellate aveva già subito un infortunio …</t>
         </is>
       </c>
       <c r="F75" s="5" t="inlineStr"/>
@@ -2459,11 +2461,11 @@
         <v>75</v>
       </c>
       <c r="B76" t="n">
-        <v>155776</v>
+        <v>251317</v>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Covid-19. Eine Grundlage, um in der Bundesverwaltung die Verbreitung von Homeoffice zu beschleunigen?</t>
+          <t>Réglementation des plateformes numériques</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
@@ -2473,7 +2475,7 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Der Umgang mit der Covid-19-Notlage hat allen Gesellschaftsschichten grosse Anpassungen abverlangt. Sehr deutlich zeigte sich dies bei der weit verbreiteten Nutzung des Homeoffice. Auch zahlreiche Bundesangestellte arbeiten zurzeit im Homeoffice. Diesbezüglich stellen die gegenwärtigen Umstände einen wichtigen Test dar, aus dem für die Zukunft Erfahrungen gesammelt werden können und der dazu genutzt werden kann, die Verbreitung des Homeoffice zu beschleunigen. Wie in anderen Bereichen könnte die Einführung von erleichterten Bedingungen für das Homeoffice auch in der Bundesverwaltung positive Auswirkungen auf verschiedene Bereiche haben, z. B. den Verkehr (weniger überfüllte öffentliche Verkehrsmittel und weniger Stau auf den Strassen), die Lebensqualität der Angestellten (bessere Vereinbarkeit von Berufs- und Familienleben, weniger Stress) und die Arbeitsleistung (grössere Flexibilität und Produktivität, geringeres Risiko eines Burnout). Weiter könnten solche Massnahme sich auch positiv auf die Bundesfinanzen auswirken dank einer effizienteren Verwaltung der gemieteten Räumlichkeiten und einem gezielteren Ressourceneinsatz. Unterstrichen werden muss zudem, dass eine flexibler…</t>
+          <t>TEXT: Le 16 avril 2025, le Conseil fédéral a annoncé qu’il repoussait la publication du message relatif à la réglementation des plateformes numériques. Depuis, presque six mois se sont écoulés et, apparemment, ce report n’a eu aucun effet positif sur le montant des droits de douane imposés sur les produits suisses par les États-Unis. Quand le Conseil fédéral prévoit-il de transmettre le message au Parlement ?</t>
         </is>
       </c>
       <c r="F76" s="5" t="inlineStr"/>
@@ -2484,11 +2486,11 @@
         <v>76</v>
       </c>
       <c r="B77" t="n">
-        <v>215214</v>
+        <v>66348</v>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>TVA. État des lieux de la nouvelle imposition des plateformes numériques</t>
+          <t>Covid-19. Cherche-t-on à justifier des restrictions drastiques au moyen d'arguments infondés?</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
@@ -2498,8 +2500,8 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Depuis le 1er janvier 2025, les plateformes numériques sont assujetties à la TVA en Suisse. Comment le nombre d’inscriptions à la TVA et de taxations fiscales a-t-il évolué depuis l’instauration des nouvelles règles ? Comment l’augmentation des inscriptions à la TVA se répartit-elle entre les entreprises nationales et les entreprises étrangères ? Quelles mesures l’AFC prend-elle cette année pour s’assurer que toutes les entreprises disposant d’un IDE remplissent bel et bien leurs obligations en matière de TVA ?
-ANSWER: Questions 1 et 2 : les inscriptions à la TVA en tant que plateforme au sens de l’art. 20a, al. 1 de la loi fédérale du 12 juin 2009 sur la taxe sur la valeur ajoutée (LTVA ; RS 641.20) se répartissent à mi-mars entre vingt plateformes sises à l’étranger et quatre plateformes sises sur le territoire suisse. Toutefois, ces chiffres doivent être interprétés avec prudence pour les raisons suivantes : l’inscription en ligne en tant que plateforme pour les nouveaux assujettis n’est disponible que depuis novembre 2024 pour les plateformes étrangères et mars 2025 pour celles situées sur le territoire suisse ; par ailleurs, certaines entreprises ont pu omettre de décla…</t>
+          <t>TEXT: Au motif que des mesures très restrictives auraient permis d'éviter le pire en Suisse romande, campagne est faite en vue d'un confinement partiel. N'est-il pas malhonnête, d'un point de vue scientifique, d'affirmer qu'un effet épidémiologique peut être attribué au confinement, alors que - selon la Task Force COVID-19 de la Confédération - les différences de taux de contamination entre la Suisse alémanique et la Suisse romande ne s'expliquent pas ?
+ANSWER: La réponse du Conseil fédéral n'existe qu'en allemand. (Veuillez changer la langue en haut à droite de la page d'accueil)</t>
         </is>
       </c>
       <c r="F77" s="5" t="inlineStr"/>
@@ -2510,11 +2512,11 @@
         <v>77</v>
       </c>
       <c r="B78" t="n">
-        <v>280488</v>
+        <v>68517</v>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Combler les lacunes en matière de capacité de défense</t>
+          <t>Per una stampa scritta indipendente è necessario adeguare gli importi del sostegno indiretto</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
@@ -2524,8 +2526,7 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Le Conseil fédéral est chargé de montrer sans attendre au Parlement comment l’armée peut – compte tenu de la dégradation croissante de la situation sécuritaire en Europe – combler le plus rapidement possible les plus grandes lacunes en matière de capacité de défense et quels sont les moyens financiers nécessaires à cet effet. Une minorité de la commission (Roth Franziska, Zopfi) propose de rejeter la motion.
-ANSWER: Compte tenu de la détérioration de la situation en matière de politique de sécurité, le Conseil fédéral a décidé, le 28 janvier 2026, de renforcer de manière substantielle la sécurité et la défense de la Suisse. Les moyens supplémentaires nécessaires, d’un montant d’environ 31 milliards de francs, doivent être couverts par une augmentation temporaire et affectée de la taxe sur la valeur ajoutée de 0,8 point de pourcentage à partir de 2028, pour une durée de dix ans. Ces recettes supplémentaires seront versées dans un fonds pour l’armement ayant une capacité d’endettement, qui doit permettre de couvrir de manière flexible les concentrations de paiements et le versement rapide des acomptes nécessaires dans le cadre des acquisitions d’armement. Afin de combler plus …</t>
+          <t>TEXT: La legge sulle poste (LPO) e le altre pertinenti disposizioni legali devono essere modificate in modo tale da permettere uno sviluppo del sostegno indiretto alla stampa. Si tratta in particolare di modificare l'articolo 16 capoverso 7 LPO affinché il sostegno indiretto alla stampa destinato ai giornali e ai periodici (...) sia aumentato di 15 milioni di franchi all'anno, così da garantire delle riduzioni per la distribuzione postale per un periodo transitorio di sette anni. Parallelamente, il sostegno alla stampa associativa e delle fondazioni deve essere aumentato di 10 milioni di franchi all'anno, pure per una durata limitata. Occorre inoltre introdurre, mediante una modifica della legge sulle poste, un sostegno alla distribuzione mattutina esclusivamente nei giorni feriali, di cui potranno beneficiare i titoli della stampa locale e regionale che hanno una tiratura media, autenticata da un organo di controllo indipendente e riconosciuto, compresa tra i 1000 e i 40 000 esemplari per edizione e che non appartengono a una rete di edizioni locali con propria testata la cui tiratura media complessiva supera i 100 000 esemplari per edizione. Per questa seconda parte, la Confedera…</t>
         </is>
       </c>
       <c r="F78" s="5" t="inlineStr"/>
@@ -2536,11 +2537,11 @@
         <v>78</v>
       </c>
       <c r="B79" t="n">
-        <v>161136</v>
+        <v>287659</v>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>EU-Richtlinie über Plattformarbeit. Will sich die Schweiz daran orientieren?</t>
+          <t>Was unternimmt der Bund gegen illegale Online-Spiele?</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
@@ -2550,7 +2551,7 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Kürzlich hat die EU eine Richtlinie über die Plattformarbeit angenommen. Diese Richtlinie ist ein wichtiger Fortschritt für Arbeitnehmerinnen und Arbeitnehmer, die in der Plattformwirtschaft tätig sind. Damit werden zwei wichtige Prinzipien eingeführt: 1. Plattformunternehmen gelten automatisch als Arbeitgeber. 2. Bei der Verwendung von Algorithmen in der Arbeitsplanung wird mehr Transparenz verlangt. Aufgrund der Annahme der EU-Richtlinie über Plattformarbeit bitten wir den Bundesrat, die folgenden Fragen zu beantworten: Welche Anpassungen wären nötig und wie könnte die Beweislastumkehr gesetzlich verankert werden? Gibt es Überlegungen in diese Richtung? Welche Massnahmen haben Bund und Kantone ergriffen, um Gerichtsurteile durchzusetzen, die Plattformen wie Uber oder Uber Eats als Arbeitgeber qualifizieren, um diese Unternehmen dem Arbeitsgesetz zu unterstellen und um sicherzustellen, dass Uber oder Uber Eats den Verpflichtungen als Arbeitgeber nachkommt? Wie viel Aufwand haben die Sozialversicherungen bisher betrieben, um die neuen Verträge der Plattformen, die eine selbstständige Tätigkeit vorsehen, zu bearbeiten und gerichtlich vorzugehen? Wie beurteilt der Bund die Rich…</t>
+          <t>TEXT: Trotz gesetzlicher Zugangssperren können illegale Online-Geldspiele weiterhin relativ einfach umgangen werden. - Was unternimmt der Bundesrat, um die Wirksamkeit dieser Sperren zu erhöhen? - Wie hoch schätzt er die jährlichen Einnahmeverluste für den Bund durch nicht bewilligte Online-Geldspielangebote? - Welche Erkenntnisse liefert die ESBK hierzu?</t>
         </is>
       </c>
       <c r="F79" s="5" t="inlineStr"/>
@@ -2561,11 +2562,11 @@
         <v>79</v>
       </c>
       <c r="B80" t="n">
-        <v>253526</v>
+        <v>62377</v>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Unabhängigere Regulierungskostenschätzung</t>
+          <t>Rete nazionale di dati sicura. Credito d’impegno</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
@@ -2573,12 +2574,7 @@
           <t>open</t>
         </is>
       </c>
-      <c r="E80" s="2" t="inlineStr">
-        <is>
-          <t>TEXT: Der Bundesrat wird beauftragt, das Bundesgesetz über die Entlastung der Unternehmen von Regulierungskosten (Unternehmensentlastungsgesetz, UEG) zu ändern, sodass die Federführung bei den nach Artikel 5 UEG sowie nach Artikel 111 Absatz 4 des Bundesgesetzes über die Bundesversammlung zu erstellenden Regulierungskostenschätzungen künftig beim Eidgenössischen Departement für Wirtschaft, Bildung und Forschung liegt.
-REASONING: Gemäss Artikel 5 Absatz 1 UEG schätzen die verantwortlichen Einheiten der Bundesverwaltung bei der Ausarbeitung von rechtsetzenden Erlassen des Bundes die einmaligen und wiederkehrenden Kosten, die den Unternehmen als Folge der Auferlegung von Handlungs-, Duldungs- oder Unterlassungspflichten entstehen. Das Eidgenössische Departement für Wirtschaft, Bildung und Forschung WBF stellt dazu die methodischen Grundlagen zur Verfügung. In der Praxis zeigt sich aber folgendes Problem: Die Regulierungskosten werden in den Verlautbarungen der für den jeweiligen Erlass zuständigen Verwaltungseinheit oft kleingeredet. Das Beispiel der vom Bundesamt für Lebensmittelsicherheit und Veterinärwesen (BLV) in Auftrag gegebenen Regulierungsfolgenabschätzung (RFA) zu einer Wer…</t>
-        </is>
-      </c>
+      <c r="E80" s="2" t="inlineStr"/>
       <c r="F80" s="5" t="inlineStr"/>
       <c r="G80" s="5" t="inlineStr"/>
     </row>
@@ -2587,11 +2583,11 @@
         <v>80</v>
       </c>
       <c r="B81" t="n">
-        <v>213749</v>
+        <v>65226</v>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>Explosion des coûts de la santé. A quand des mesures efficaces contre le gaspillage de l'argent des primes et pour freiner la hausse des coûts?</t>
+          <t>Zugang zu unterstützter Kommunikation</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
@@ -2601,7 +2597,7 @@
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Comme chaque année à cette même période, le jeu des caisses-maladie bat son plein. Les assureurs font parvenir de la publicité aux ménages par les canaux les plus divers : certaines caisses-maladie proposent des rabais et d'autres promettent des baisses de primes pour l'année prochaine, alors que l'association des assureurs-maladie Santésuisse a annoncé cet été une hausse générale des primes de l'ordre de 3 %. 1. Tout laisse à penser dans ce contexte que, comme lors des précédentes années électorales, les caisses-maladie puisent plus profondément dans leurs réserves qu'à l'ordinaire pour réduire au maximum la hausse des primes. Que pense l'Office fédéral de la santé publique de ce soupçon en sa qualité d'autorité d'approbation des primes ? Des réserves ont-elles dû ou devraient-elles être réduites pour obtenir des primes plus basses ? 2. La numérisation doit profiter au système de santé : elle améliore l'efficacité et la qualité des soins ainsi que l'information des assurés et des patients. Il y a un an, le Conseil fédéral a proposé le rejet d'une intervention qui visait à créer une base légale garantissant que la documentation médicale du patient soit tenue de manière struct…</t>
+          <t>TEXT: Kommunikation dient dem sozialen Austausch, ermöglicht gesellschaftliche Teilhabe und ist damit ein menschliches Grundbedürfnis. Mit der Ratifizierung der UNO-Behindertenrechtskonvention verpflichtete sich die Schweiz, auf individuelle Bedürfnisse abgestimmte Kommunikationsformen und Kommunikationsmittel zu fördern. Für Menschen mit eingeschränkter Lautsprache gibt es die Unterstützte Kommunikation (UK). Das Gelingen der UK hängt u.a. davon ab, ob die passenden Methoden und Hilfsmittel zum Einsatz kommen, ob genügend UK-Fachpersonal in den Institutionen arbeitet und ob das Umfeld UK täglich und in möglichst vielen Lebensbereichen nutzt. Ich bitte den Bundesrat um die Beantwortung folgender Fragen: 1. Wie viele Menschen sind in der Schweiz auf UK angewiesen? Wie sieht die Verteilung aus zwischen Menschen mit leichten und Menschen mit schweren Kommunikationsbeeinträchtigungen u.a. aufgrund von schweren sowie mehrfachen Behinderungen? 2. Was tun Bund und Kantone, um sicherzustellen, dass alle Personen, Kinder und Erwachsene, mit eingeschränkten lautsprachlichen Fähigkeiten während ihres gesamten Lebens in verschiedenen Lebensbereichen wie u.a. Frühbereich, Bildung, Wohnen, Arbei…</t>
         </is>
       </c>
       <c r="F81" s="5" t="inlineStr"/>
@@ -2612,11 +2608,11 @@
         <v>81</v>
       </c>
       <c r="B82" t="n">
-        <v>154878</v>
+        <v>66800</v>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Ist die Zukunft einer vielfältigen und qualitativ hochstehenden Kulturberichterstattung gefährdet?</t>
+          <t>Mesures contre l'immigration illégale (8/9). Systématiser l'échange des données concernant les immigrés illégaux</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
@@ -2626,7 +2622,8 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Sowohl das Informations- und Kommunikationsverhalten der Bevölkerung als auch die Medienlandschaft wandeln sich stark und rasch. Dies wirkt sich insbesondere auch auf die mediale Kulturberichterstattung aus. Es gibt immer weniger selbstständige Kulturredaktionen, sowohl in den Printmedien wie in den elektronischen Medien nimmt der Raum, der der Kultur zur Verfügung steht, ab. Mediale Kulturinformation konzentriert sich zunehmend entweder auf Grossereignisse wie Premieren auf grossen Bühnen oder Neuerscheinungen prominenter Autorinnen und Autoren oder auf kulturelle Anlässe von lokaler oder regionaler Bedeutung. So verliert die Schweiz an Vielfalt der Themen und der kritischen Stimmen und an überregionalen Kulturinformationen insbesondere über die Sprachregionen hinaus. So verliert immer mehr wertvolles Kulturschaffen an Aufmerksamkeit. Denn das Kulturschaffen ist auf eine kompetente, rege und vielfältige öffentliche Kulturkritik angewiesen. Sie ist es auch, die in der Bevölkerung das Interesse am kulturellen Schaffen und Darbieten des ganzen Landes weckt und wachhält. Wenn Kultur gefördert wird, ist es auch im Interesse der Förderung, dass sie auch Beachtung findet. In diesem…</t>
+          <t>TEXT: Afin de lutter durablement contre l'immigration illégale en Suisse et si possible d'y mettre un terme, il faut que l'échange des données sur les personnes concernées entre les cantons, les communes, les autorités sociales, les caisses-maladie, l'AVS, l'AI et d'autres assurances sociales devienne systématique. Il s'agit d'échanger et de comparer toutes les données relatives au statut de séjour, au lieu de domicile, à la couverture d'assurance, aux paiements des primes, aux réductions de primes, aux prestations des caisses-maladie, à l'AVS, à l'AI et à d'autres assurances sociales.
+REASONING: En fonction des estimations et des sources d'information, jusqu'à 100 000 immigrés illégaux - banalement appelés " sans-papiers " - seraient en Suisse. Afin de réduire l'attrait de notre pays à cet égard, il importe que ces personnes puissent être identifiées et renvoyées grâce à un échange systématique des données les concernant. Selon le rapport du Conseil fédéral " Pour un examen global de la problématique des sans-papiers " en réponse au postulat de la Commission des institutions politiques du Conseil national du 12 avril 2018 (18.3381), les assurances et les caisses-maladie surtout n…</t>
         </is>
       </c>
       <c r="F82" s="5" t="inlineStr"/>
@@ -2637,11 +2634,11 @@
         <v>82</v>
       </c>
       <c r="B83" t="n">
-        <v>153461</v>
+        <v>339163</v>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>Jeux vidéo. Prévenir les abus des microtransactions apparentées aux jeux d'argent</t>
+          <t>Gesetzliche Grundlagen für einen transparenten und sparsamen Ressourcenverbrauch von Rechenzentren</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
@@ -2651,44 +2648,208 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Le Conseil fédéral est chargé de proposer un système pour réguler l'emploi des microtransactions avec de l'argent réel dans les jeux vidéos, quelle que soit la plateforme. En particulier, le Conseil fédéral est chargé de déterminer quels types de microtransactions sont apparentées à des jeux d'argent et doivent être régulées comme telles, et de garantir la protection des joueurs, en particulier mineurs. Les pratiques posant le plus de problèmes et devant faire appel à régulation sont : 1. les microtransactions avec de l'argent réel donnant un avantage aux joueurs, mais où la récompense est aléatoire ; 2. les systèmes de microtransactions particulièrement conçus pour générer de l'addiction chez les joueurs ; 3. les microtransactions ciblant en particulier les mineurs.
-REASONING: De nombreux jeux vidéos pour appareils mobiles, consoles de jeux ou sur PC comportent, parfois au delà d'un prix d'achat élevé, un système de microtransaction. Dans des modèles "free to play", ce système peut être le seul moyen de rentabiliser le jeu, mais dans d'autres cas, il s'agit de sources de recettes supplémentaires. Ces microtransactions permettent aux joueurs qui dépensent de l'argent réel, d…</t>
+          <t>TEXT: Der Bundesrat wird beauftragt, auf Grundlage von Art. 89 BV, die gesetzlichen Grundlagen für einen transparenten und sparsamen Verbrauch von Ressourcen von grösseren Rechenzentren zu schaffen. Die gesetzlichen Grundlagen sollen folgende Elemente umfassen: Die jährliche Offenlegung von Strom- und Wasserverbrauch Vorgaben zum (schrittweisen) Bezug von Energie aus erneuerbaren Quellen Effizienzstandards, um das ungenutzte Effizienzpotenzial zu realisieren Die Regelung der Nutzung der anfallenden Abwärme
+REASONING: Rechenzentren verbrauchten in der Schweiz schon im Jahr 2024 rund 2,1 Terawattstunden Strom, das entspricht 3,6 Prozent des gesamtschweizerischen Stromverbrauchs. Bis 2030 wird laut dem Kurzbericht des Bundesamts für Energie (EnergieSchweiz / TEP Energy, Mai 2026) ein Anstieg auf 2,5 bis 3,2 Terawattstunden erwartet; in einem Hochszenario sogar auf 3,5 Terawattstunden, was einem Plus von 70 Prozent gegenüber heute entspräche. Dieselbe Studie zeigt: Das ungenutzte Energieeffizienzpotenzial in Schweizer Rechenzentren beträgt rund 38 Prozent des aktuellen Verbrauchs. Dieses Potenzial wird durch den Markt bisher nicht ausgeschöpft. Namentlich bei unternehmensinternen Rech…</t>
         </is>
       </c>
       <c r="F83" s="5" t="inlineStr"/>
       <c r="G83" s="5" t="inlineStr"/>
     </row>
     <row r="84">
-      <c r="F84" s="5" t="n"/>
-      <c r="G84" s="5" t="n"/>
+      <c r="A84" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" t="n">
+        <v>65483</v>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>Transport pour handicapés. Un chaînon manquant dans l'offre de mobilité</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Le Conseil fédéral est chargé de produire un rapport, en complément de celui demandé par le postulat 20.3874, sur la manière dont les lacunes de l'offre en transport pour handicapés devraient être comblées de sorte que le droit à la mobilité personnelle inscrit dans la Convention relative aux droits des personnes handicapées soit honoré et mis en oeuvre dans le droit suisse (" Les États Parties prennent des mesures efficaces pour assurer la mobilité personnelle des personnes handicapées, dans la plus grande autonomie possible "). Il ciblera en particulier le cas des personnes qui, en raison de leur handicap, ne peuvent pas, ou que de manière limitée, utiliser les transports publics. L'avis et les expériences des handicapés qui doivent recourir à ces transports seront pris en compte.
+REASONING: Pour s'intégrer à la société de manière autonome et en bénéficiant des mêmes droits que les autres personnes, les handicapés doivent pouvoir se déplacer. En raison de leur handicap, certaines personnes ne peuvent pas, ou que de manière limitée, utiliser les transports publics. Une offre adaptée est donc nécessaire si elles veulent effectuer leurs tâches quotidiennes, avoir accès aux lo…</t>
+        </is>
+      </c>
+      <c r="F84" s="5" t="inlineStr"/>
+      <c r="G84" s="5" t="inlineStr"/>
     </row>
     <row r="85">
-      <c r="F85" s="5" t="n"/>
-      <c r="G85" s="5" t="n"/>
+      <c r="A85" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" t="n">
+        <v>68999</v>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>Prix des médicaments : à quand la transparence sur les investissements des entreprises pharmaceutiques ?</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Les coûts de recherche et de développement sont un argument principal de l'industrie pharmaceutique pour justifier les prix élevés des médicaments, mais l'investissement réel n'est pas transmis aux autorités. Une nouvelle étude calcule des marges de profit de 40 à 90 %. Le Conseil fédéral prévoit-il des mesures pour que les entreprises pharmaceutiques soient enfin obligées de publier leurs investissements, comme c'est déjà le cas dans les pays voisins, par exemple en Italie ?</t>
+        </is>
+      </c>
+      <c r="F85" s="5" t="inlineStr"/>
+      <c r="G85" s="5" t="inlineStr"/>
     </row>
     <row r="86">
-      <c r="F86" s="5" t="n"/>
-      <c r="G86" s="5" t="n"/>
+      <c r="A86" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" t="n">
+        <v>64898</v>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>Modification de l'article 697l du code des obligations et accès à liste des ayants droit économiques</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: La loi fédérale du 21 juin 2019 sur la mise en oeuvre des recommandations du Forum mondial sur la transparence et l'échange de renseignements à des fins fiscales entraîne la disparition des actions au porteur. L'art. 697l du code des obligations (CO) est simplifié en conséquence et ne prévoit plus pour la société que l'obligation de tenir une liste des ayants droit économiques qui lui ont été annoncés. Conformément à la recommandation 24 du GAFI, l'art. 697l, al. 4, CO prévoit que la liste doit être tenue de manière à ce qu'il soit possible d'y accéder en tout temps en Suisse. La loi ne règle toutefois pas qui peut accéder à la liste. Le message concernant la mise en oeuvre des recommandations du GAFI révisées en 2012 n'imposait pas au conseil d'administration d'une société suisse de fournir de telles listes à l'autorité suisse compétente, sauf dans le cas de vérifications particulières dans le cadre d'une enquête du Ministère public, dans le domaine du droit pénal administratif ou en cas d'infraction fiscale (fraude fiscale). L'Administration fédérale des contributions (AFC) procède actuellement à la collecte systématique de ces listes par l'envoi d'une lettre-type aux contr…</t>
+        </is>
+      </c>
+      <c r="F86" s="5" t="inlineStr"/>
+      <c r="G86" s="5" t="inlineStr"/>
     </row>
     <row r="87">
-      <c r="F87" s="5" t="n"/>
-      <c r="G87" s="5" t="n"/>
+      <c r="A87" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" t="n">
+        <v>280490</v>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>Budget 2026. Supplément II</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr"/>
+      <c r="F87" s="5" t="inlineStr"/>
+      <c r="G87" s="5" t="inlineStr"/>
     </row>
     <row r="88">
-      <c r="F88" s="5" t="n"/>
-      <c r="G88" s="5" t="n"/>
+      <c r="A88" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" t="n">
+        <v>155207</v>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>Pour le versement mensuel de l'allocation pour perte de gain revenant aux personnes servant dans l'armée suisse</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: L'allocation pour perte de gain qui revient aux personnes sans activité lucrative, aux indépendants et aux personnes en formation qui effectuent une école de recrues, un service sans interruption ou un service de changement de grade n'est versée pour la première fois qu'au terme de plus d'un mois, parfois même après deux mois, voire trois. Cette situation peut plonger les personnes concernées ou leurs parents dans des difficultés financières. - Le Conseil fédéral est-il disposé à faire en sorte que les allocations pour perte de gain soient versées ponctuellement, à savoir le 25 de chaque mois, comme c'est le cas pour le salaire des employés de la Confédération ? - Dans la négative, quelles sont les raisons qui s'y opposent ?
+ANSWER: La réponse du Conseil fédéral n'existe qu'en allemand. (Veuillez changer la langue en haut à droite de la page d'accueil)</t>
+        </is>
+      </c>
+      <c r="F88" s="5" t="inlineStr"/>
+      <c r="G88" s="5" t="inlineStr"/>
     </row>
     <row r="89">
-      <c r="F89" s="5" t="n"/>
-      <c r="G89" s="5" t="n"/>
+      <c r="A89" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" t="n">
+        <v>153731</v>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>Stromspeicher bezüglich Netznutzung technologieneutral und somit gleichbehandeln</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Ich bitte den Bundesrat, folgende Fragen zu beantworten: 1. Warum beabsichtigt der Bundesrat, Stromspeicher hinsichtlich der Verrechnung von Netznutzungsentgelten für den Bezug von Elektrizität aus dem Netz gegenüber Pumpspeicherkraftwerken zu diskriminieren - Regulierungsvorgaben sollten technologieneutral sein -? 2. Ist er sich bewusst, dass Stromspeicher beim Umbau des Energiesystems zukünftig eine wichtige Rolle für den Ausgleich zwischen stark fluktuierender und wetterabhängiger erneuerbarer Energie und dem Verbrauch übernehmen müssen? 3. Ist er nicht der Ansicht, dass mit der Belastung von Speichern mit Netznutzungsentgelten auch die Ausnahmeregelung für Pumpspeicherkraftwerke hinterfragt werden muss und gefährdet ist? 4. Ist er sich bewusst, dass er mit dem neuen Artikel 2 Absatz 3 der Stromversorgungsverordnung (StromVV; Speicher gelten für den Bezug als Endverbraucher) einen Widerspruch zu Artikel 4 Absatz 1 Litera b schafft, worin ein Endverbraucher definiert ist als Kunde, der Elektrizität für den eigenen Verbrauch kauft, und somit eine Rechtsunsicherheit?
+REASONING: In der Vernehmlassungsvorlage zu den Verordnungen der Strategie Stromnetze ist vorgesehen, dass, w…</t>
+        </is>
+      </c>
+      <c r="F89" s="5" t="inlineStr"/>
+      <c r="G89" s="5" t="inlineStr"/>
     </row>
     <row r="90">
-      <c r="F90" s="5" t="n"/>
-      <c r="G90" s="5" t="n"/>
+      <c r="A90" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" t="n">
+        <v>155593</v>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>Système satellite Composante Spatiale Optique. Arrangement cadre avec la France</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr"/>
+      <c r="F90" s="5" t="inlineStr"/>
+      <c r="G90" s="5" t="inlineStr"/>
     </row>
     <row r="91">
-      <c r="F91" s="5" t="n"/>
-      <c r="G91" s="5" t="n"/>
+      <c r="A91" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" t="n">
+        <v>153295</v>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>Augmenter les places d'accueil extrafamilial par un financement partagé afin que les parents puissent mieux concilier vie familiale et vie professionnelle</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>TEXT: Le Conseil fédéral est chargé d'examiner la possibilité d'élaborer un modèle permettant d'assurer le financement durable d'une offre adaptée de places d'accueil extrafamilial et extrascolaire. Ce modèle répondra aux exigences suivantes : tout enfant dont les parents ne peuvent assurer eux-mêmes la garde parce qu'ils exercent une activité professionnelle ou sont engagés dans une activité bénévole, une formation ou une formation continue attestées a droit à un bon de garde jusqu'à la fin de la scolarité obligatoire. Ce bon couvrira au moins les deux tiers du coût total d'une place d'accueil reconnue par le canton. Les communes, les cantons, la Confédération et les entreprises de plus de 250 employés veilleront conjointement à ce qu'un nombre suffisant de places d'accueil soient proposées et financées.
+REASONING: De nombreux parents ne peuvent pas se permettre de faire garder leur enfant par des professionnels. Les garderies, les groupes de jeux et l'accueil familial de jour sont financés en grande partie par les contributions parentales. Le montant payé par les parents pour la garderie représente environ deux tiers du coût total en moyenne, selon le canton et la commune. Cette…</t>
+        </is>
+      </c>
+      <c r="F91" s="5" t="inlineStr"/>
+      <c r="G91" s="5" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="F92" s="5" t="n"/>
@@ -3619,6 +3780,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId80"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D82" r:id="rId81"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D83" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D84" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D85" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D86" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D87" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D88" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D90" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D91" r:id="rId90"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
S8 follow-up: visible review state, German reading aid (official / unofficial Apertus 8B), review sheet in official DE
- detail panel: Confirmed/Rejected by reviewer state, pressed buttons, saved line (D51)
- REVIEW_LANG reading aid: official version for federal affairs, unofficial Apertus translation otherwise (TRANSLATE_MODEL=8B: 4.5s vs 166s) (D52)
- adjudication.xlsx: 88/90 rows in official German, same selection (D53)
- partner's 5 cases vs model and PolitMonitor (D54); .impeccable config (Inter ok)

Verification: browser check — confirm feedback visible, federal official DE shown, cantonal FR translated in 3.9s; make test: 63 passed; metrics.json unchanged.
</commit_message>
<xml_diff>
--- a/data/gold/for_partner/adjudication.xlsx
+++ b/data/gold/for_partner/adjudication.xlsx
@@ -623,7 +623,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Nouvelles réglementations sur les dérives d’Internet</t>
+          <t>Neue Regelungen zu Auswüchsen im Internet</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
@@ -631,7 +631,11 @@
           <t>open</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Official DE version; original is FR] </t>
+        </is>
+      </c>
       <c r="F3" s="5" t="inlineStr"/>
       <c r="G3" s="5" t="inlineStr"/>
     </row>
@@ -644,7 +648,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Contrôle étendu des données personnelles et des réseaux sociaux dans les procédures Esta. Conséquences pratiques et juridiques pour les citoyens suisses</t>
+          <t>Erweiterte Kontrolle personenbezogener Daten und sozialer Medien im Esta-Verfahren. Praktische und rechtliche Konsequenzen für Schweizer Staatsangehörige</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -654,7 +658,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Le gouvernement américain (U.S. Customs and Border Protection) a annoncé le 10 décembre 2025 son intention d'imposer aux voyageurs en provenance des pays participant au programme Visa Waiver (dont la Suisse fait partie) qui demandent le visa ESTA (Electronic System for Travel Authorization) l'obligation de fournir, entre autres, l'historique de leurs activités sur les réseaux sociaux au cours des cinq dernières années, leurs adresses électroniques des dix dernières années et le lieu de naissance et de résidence de leurs parents, conjoints, frères et sœurs et enfants. Ce projet est actuellement en consultation. S’il devait se concrétiser, il aurait également des répercussions importantes pour les citoyens suisses qui voyagent aux États-Unis. À la lumière de ce qui précède, le Conseil fédéral est prié de répondre aux questions suivantes : Que pense-t-il des modifications annoncées (en particulier l'obligation de mettre à disposition les informations concernant les activités effectuées sur les réseaux sociaux au cours des cinq dernières années) au regard des droits civils et de la protection des données des citoyens suisses ? À quelles conséquences s’attend-il pour les touristes…</t>
+          <t>[Official DE version; original is FR] TEXT: Die US-Regierung (U.S. Customs and Border Protection) hat am 10. Dezember 2025 angekündigt, dass Reisende aus Ländern, die am Visa Waiver Program teilnehmen (darunter auch die Schweiz) und ein sogenanntes ESTA-Visum (Electronic System for Travel Authorization) beantragen, künftig unter anderem folgende Angaben machen müssen: die Social-Media-Historie der letzten 5 Jahre, ihre E-Mail-Adressen der letzten 10 Jahre sowie den Geburtsort und Wohnort ihrer Eltern, ihrer Ehepartnerin oder ihres Ehepartners, ihrer Geschwister und Kinder. Der Vorschlag befindet sich derzeit in der Beratung und hätte, falls er umgesetzt wird, auch erhebliche Auswirkungen auf Schweizer Staatsangehörige, die in die Vereinigten Staaten reisen. In diesem Zusammenhang bitte ich den Bundesrat, folgende Fragen zu beantworten: Wie beurteilt er die angekündigten Änderungen (insbesondere die Pflicht, Informationen über die Aktivitäten in den sozialen Medien der letzten fünf Jahre zur Verfügung zu stellen) im Hinblick auf die Bürgerrechte und den Datenschutz der Schweizer Bürgerinnen und Bürger? Welche konkreten Auswirkungen erwartet er für Schweizer Touristinnen und Touristen, für Geschäftsreisende (einschliessl…</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr"/>
@@ -694,7 +698,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Qual è il livello di sicurezza degli ambienti di lavoro nella Confederazione riguardo ad azioni di sabotaggio e/o di ascolto da parte di altri attori?</t>
+          <t>Wie sicher sind die Arbeitsumgebungen beim Bund vor Sabotage und/oder Abhöraktionen durch andere Akteure?</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -704,7 +708,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>TEXT: L'incidente occorso in Germania alcune settimane fa suscita scalpore. Alcuni sabotatori hanno tagliato in diversi punti i cavi del sistema di comunicazione della Deutsche Bahn. Il traffico ferroviario è stato paralizzato e la comunicazione tra macchinisti e i posti di comando è stata interrotta. Uno scenario simile sarebbe ipotizzabile ovunque. In Svizzera, nel contesto della Confederazione, la sicurezza sul lavoro e un ambiente di lavoro basato sulla fiducia sono considerati elementi chiave. Tuttavia esistono sempre locali ed edifici in cui gli impiegati federali devono lavorare e tenere conversazioni confidenziali. Non sempre è possibile escludere che questi ambienti siano sicuri. Negli stessi edifici troviamo anche gli uffici di altre imprese, i cui cavi informatici vanno a finire negli stessi locali adibiti ai server, utilizzati dai servizi della Confederazione. Pertanto non si può escludere categoricamente un'azione di sabotaggio o l'ascolto mirato. In questo contesto invito il Consiglio federale a rispondere alle domande seguenti: 1. La Confederazione ha una visione d'insieme per verificare se tutti gli Uffici rilevanti per la sicurezza possano lavorare in modo "sicuro"…</t>
+          <t>[Official DE version; original is IT] TEXT: Ein Vorfall, der sich vor wenigen Wochen in Deutschland zugetragen hat, lässt aufhorchen. Saboteure durchtrennten an verschieden Stellen Leitungen für das Funknetz der Bahn. Der Verkehr war stillgelegt und die Kommunikation zwischen den Lokomotivführern und den Leitstellen unterbrochen. Ein ähnliches Szenario könnte sich an jedem anderen Ort abspielen. Bei uns in der Schweiz im Bundesumfeld wird die Arbeitssicherheit und auch das vertrauensvolle Arbeiten als zentraler Schlüssel angesehen. Es gibt aber noch immer Räume und Gebäude in welchen Bundesangestellte arbeiten und vertrauliche Gespräche führen müssen, in welchen nicht in jedem Fall ausgeschlossen werden kann, dass diese Umgebung gesichert ist. Im gleichen Gebäude arbeiten andere Unternehmen und die Informatikleitungen dieser unterschiedlichen Unternehmen, auch unserer Bundesstellen, münden im gleichen Serverraum. Ein Sabotageakt oder auch das gezielte Abhören kann nicht in jedem Fall ausgeschlossen werden. In diesem Zusammenhang bitte ich den Bundesrat, die nachfolgenden Fragen zu beantworten: 1. Hat der Bund eine Übersicht, ob alle sicherheitsrelevanten Ämter 'sicher' arbeiten können? 2. Gibt es Hinweise auf verdeckte…</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr"/>
@@ -823,7 +827,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Le caratteristiche e i dispositivi di sicurezza del sistema svizzero di verifica dei medicamenti (SMVS) sono inadatti per il monitoraggio degli agenti terapeutici?</t>
+          <t>Sind Sicherheitsmerkmale und -vorrichtungen nach dem SMVS für das Monitoring von Arzneimitteln ungeeignet?</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -833,8 +837,8 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Il Consiglio federale condivide l’opinione secondo cui non esiste una base legale che consenta di attuare mediante l’articolo 17a LATer, approvato ma non in vigore, la gestione digitale delle penurie di medicamenti per uso umano richiesta dalla mozione Ettlin e che è necessario elaborare una specifica base legale all’interno della LATer? L’introduzione del SMVS fa parte delle otto raccomandazioni proposte al Consiglio federale dalla task force per gli agenti terapeutici? Il monitoraggio necessita di un’ulteriore base legale o è sufficiente il sistema di preallarme dell’Ufficio federale dell’approvvigionamento economico del Paese (UFAE)? È vero che l’UFAE non intende servirsi del SMVS per la gestione digitale delle penurie di medicamenti per uso umano? Il Consiglio federale ritiene che esista un rischio significativo che in Svizzera entrino in commercio medicamenti contraffatti? Se sì, in quali casi? Il Consiglio federale condivide la posizione dei fornitori di servizi, secondo cui i costi di attuazione dei requisiti SMVS sono troppo elevati rispetto ai potenziali benefici?
-REASONING: Il 26 settembre 2023 il Parlamento ha approvato, con un adattamento del punto 2, la mozione …</t>
+          <t>[Official DE version; original is IT] TEXT: Teilt der Bundesrat die Einschätzung, dass die gesetzliche Grundlage fehlt, um mit dem verabschiedeten Art. 17a HMG das digitale Management von Versorgungsengpässen bei Humanarzneimitteln gemäss der Motion Ettlin umzusetzen und dass eine entsprechende Rechtsgrundlage im HMG erst zu schaffen ist? Gehört die Einführung des SMVS zu den acht Empfehlungen, welche die «Taskforce Engpass Medikamente» zuhanden des Bundesrats vorschlägt? Braucht es überhaupt eine zusätzliche Rechtsgrundlage für das Monitoring oder reicht das System der Frühwarnung beim BWL? Trifft es zu, dass das BWL gar nicht plant, das SMVS für das digitale Management von Versorgungsengpässen bei Humanarzneimitteln zu nutzen? Geht der Bundesrat von einer signifikanten Gefahr von Fälschungen für die in der Schweiz gehandelten Medikamente aus und wenn ja, bei welchen? Teilt der Bundesrat die Position von Leistungserbringenden, dass der Aufwand zur Implementierung der SMVS-Vorgaben unverhältnismässig hoch sei im Vergleich zum erzielbaren Nutzen?
+REASONING: Das Parlament hat am 26. September 2023 die Motion Ettlin 22.3859 «Masterplan zur digitalen Transformation im Gesundheitswesen. Nutzung von gesetzlichen Standards u…</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr"/>
@@ -849,7 +853,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Ordinanza sull’indicazione dei prezzi. Semplificare l’autocomparazione</t>
+          <t>Preisbekanntgabeverordnung. Selbstvergleich vereinfachen</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -859,8 +863,8 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Il Consiglio federale è incaricato di semplificare le disposizioni dell'ordinanza sull'indicazione dei prezzi (OIP; RS 942.211) riguardanti l'indicazione fallace dei prezzi (art. 16 cpv. 1 lett. a e cpv. 3 OIP) in modo da consentire l'autocomparazione senza che siano fissati limiti di tempo, in particolare per gli articoli di stagione come capi di abbigliamento, calzature, articoli sportivi, ecc., se la merce in questione è stata effettivamente proposta in precedenza, per almeno quattro settimane consecutive, al prezzo più alto indicato.
-REASONING: Le disposizioni piuttosto complesse dell'OIP sull'autocomparazione, che regolamentano le indicazioni di riduzione dei prezzi e le comparazioni con il prezzo di vendita iniziale, erano state introdotte per evitare che i consumatori fossero tratti in inganno, ma oggi sono superate. Più in particolare, la cosiddetta regola del dimezzamento secondo cui il "prezzo comparativo" può essere indicato solo per la metà del periodo durante il quale è stato o sarà praticato, e al massimo per due mesi, comporta per i venditori e per le autorità di controllo un onere sproporzionato rispetto al vantaggio che ne risulta per il cliente. Questa rego…</t>
+          <t>[Official DE version; original is IT] TEXT: Der Bundesrat wird beauftragt, die Preisbekanntgabeverordnung (PBV; SR 942.211) wie folgt zu ändern: Die Vorschriften über die irreführende Preisbekanntgabe (Art. 16 Abs. 1 Bst. a und Abs. 3 PBV) sind so zu vereinfachen, dass der Selbstvergleich insbesondere bei Saisonware wie Bekleidung, Schuhe, Sportartikel usw. zeitlich uneingeschränkt praktiziert werden kann, wenn die Ware unmittelbar vorher mindestens während vier Wochen zum höheren Preis tatsächlich angeboten wurde.
+REASONING: In der Preisbekanntgabeverordnung geht es beim Selbstvergleich darum, die Irreführung der Konsumentenschaft zu verhindern, indem recht komplexe Regeln für die Bekanntgabe von Preisreduktionen und Vergleiche zum ursprünglichen Verkaufspreis gelten. Diese Regeln sind nicht mehr zeitgemäss. Die sog. Halbierungsregel verursacht unverhältnismässigen Aufwand für die Anbieter und die Kontrollbehörden, ohne den Kunden einen echten Nutzen zu stiften. Die Halbierungsregel bestimmt, dass die Ware nur halb so lange mit Angabe der Preisreduktion angeboten werden darf, wie sie vorher zum vollen Preis angeboten wurde. Zudem gilt eine Maximaldauer von zwei Monaten. Die Regelung mag früher einmal sinnvoll gewesen…</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr"/>
@@ -875,7 +879,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Commissioni extraparlamentari. Riorganizzazione nel quadro della verifica 2025</t>
+          <t>Ausserparlamentarische Kommissionen. Gesetzliche Neuordnung im Rahmen der Überprüfung 2025</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -883,7 +887,11 @@
           <t>open</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Official DE version; original is IT] </t>
+        </is>
+      </c>
       <c r="F13" s="5" t="inlineStr"/>
       <c r="G13" s="5" t="inlineStr"/>
     </row>
@@ -922,7 +930,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Allocation de maternité pour les femmes travaillant dans l'agriculture</t>
+          <t>Mutterschaftsentschädigung für in der Landwirtschaft tätige Frauen</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -932,8 +940,8 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>TEXT: En Suisse, les deux tiers des femmes travaillent dans l'entreprise ou l'exploitation agricole de leur mari ou compagnon sans être rémunérées. - Sachant que les étudiants ont droit aux allocations pour perte de gain sans avoir de revenus, le Conseil fédéral envisagerait-t-il de modifier l'art. 16b, al. 1, let. c, de la loi sur les allocations pour perte de gain, leur permettant de percevoir une allocation de maternité ? - Si non pourquoi ?
-ANSWER: Une telle modification n'est pas prévue par le Conseil fédéral. Aucune allocation de maternité minimale n'est versée, que ce soit pour les étudiantes ou pour toute autre personne, si aucun revenu n'est perçu avant l'accouchement. Cela résulte de la volonté du législateur et de compromis politiques qui ont fait suite aux longues négociations dans le cadre de l'introduction de l'allocation de maternité, le 1er juillet 2005.</t>
+          <t>[Official DE version; original is FR] TEXT: In der Schweiz arbeiten zwei Drittel aller Frauen, die im Landwirtschaftsbetrieb oder -unternehmen ihres Ehemanns oder Lebenspartners tätig sind, unentgeltlich. Studierende haben Anrecht auf Erwerbsersatz, ohne über ein Einkommen zu verfügen. - Beabsichtigt der Bundesrat vor diesem Hintergrund, Artikel 16b Absatz 1 Buchstabe c EOG anzupassen, damit diese Frauen eine Mutterschaftsentschädigung beanspruchen können? - Wenn nicht, warum nicht?
+ANSWER: Die Antwort des Bundesrates existiert nur in französischer Sprache. (Bitte wechseln Sie auf der Homepage oben rechts die Sprache)</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr"/>
@@ -948,7 +956,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Coopération internationale des autorités pénales dans la lutte contre la cybercriminalité</t>
+          <t>Internationale Zusammenarbeit von Strafbehörden im Kampf gegen Cyberkriminalität</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -958,7 +966,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Au vu de la forte hausse des cyberattaques d'origine étrangère contre des personnes physiques et morales en Suisse, je pose les questions suivantes au Conseil fédéral : 1. Y a-t-il une bonne coopération avec les autorités pénales étrangères lorsque les enquêtes de police sur des plaintes pénales déposées par des victimes suisses révèlent que les malfaiteurs opèrent de manière ciblée depuis l'étranger ? 2. Y a-t-il des pays qui ne coopèrent pas suffisamment avec la Suisse et qui sont donc souvent utilisés comme base par les cybercriminels ? 3. À combien le Conseil fédéral estime-t-il le nombre de cas où il est impossible de déterminer où se trouvent les auteurs ? 4. La présente interpellation fait écho aux cyberattaques menées depuis des mois contre des clients de PostFinance et d'autres entreprises suisses, qui, attirés par un site Internet falsifié (hameçonnage), permettent aux malfaiteurs d'accéder directement à leurs comptes et dépôts. Le Ministère public de la Confédération, chargé de l'enquête, a pu remonter la trace des auteurs jusqu'en Inde, à qui les cas traités ont été transmis pour qu'elle les poursuive. Le Conseil fédéral peut-il donner des informations plus détail…</t>
+          <t>[Official DE version; original is FR] TEXT: Angesichts der stark zunehmenden Cyberattacken ausländischer Herkunft gegen natürliche und juristische Personen in der Schweiz frage ich den Bundesrat an: 1. Wie gut funktioniert die Zusammenarbeit mit ausländischen Strafbehörden, wenn die polizeilichen Abklärungen über Strafanträge schweizerischer Geschädigter ergeben, dass die Täterschaft gezielt aus dem Ausland operiert? 2. Gibt es Staaten, die diesbezüglich ungenügend mit der Schweiz kooperieren und deshalb von cyberkrimineller Täterschaft besonders als Ausgangsbasis genutzt werden? 3. Wie hoch schätzt der Bundesrat die Fälle, wo der Standort der Täterschaft überhaupt nicht eruiert werden kann? 4. Vorliegende Interpellation basiert auf monatelangen Cyberattacken auf Kunden der PostFinance und weiterer Schweizer Unternehmen, die über eine gefälschte Webseite ("Phishing") angelockt wurden, mit dem Ziel, der Täterschaft direkten Zugriff auf ihre Konti und Depots zu ermöglichen. Als Ursprungland konnte die mit der Abklärung beauftragte Bundesanwaltschaft Indien eruieren. In der Folge wurden die aufgearbeiteten Fälle an die indischen Strafbehörden zur Weiterverfolgung übergeben. Kann der Bundesrat nähere Angaben zum aktuellen …</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr"/>
@@ -999,7 +1007,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Dazit e controllo delle frontiere</t>
+          <t>Dazit und Grenzkontrollen</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -1009,7 +1017,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Nel quadro del Rapporto del Consiglio federale in adempimento del postulato 17.4177 del 14.12.2017, l'approccio risulta essere piuttosto teorico e poco orientato alla reale operatività quotidiana del personale che opera ai valichi ferroviari. In considerazione degli importanti cambiamenti previsti, è opportuno conoscere maggiori informazioni operative che toccano la quotidianità dei dipendenti e dei cittadini. 1. Sono previsti investimenti infrastrutturali utili alle attività di controllo, soprattutto merci, in tutte le stazioni di confine (Basilea, Buchs, Vallorbe, Ginevra, Domodossola, Luino, Chiasso)? Sono di competenza dell'AfD o direttamente delle FFS? Come è garantito il finanziamento e il coordinamento delle procedure? 2. Si prevede di installare scanner fissi per il traffico ferroviario merci? In quali stazioni? 3. La riforma in corso prevede un aggiornamento degli accordi internazionali vigenti per le stazioni di frontiera? Quali accordi si prevede di aggiornare con le rispettive controparti? 4. Il progetto Dazit prevede un coinvolgimento attivo - per ottimizzare i flussi di lavoro e i controlli - delle aziende ferroviarie svizzere leader nel traffico delle merci? Se…</t>
+          <t>[Official DE version; original is IT] TEXT: Gemäss dem Bericht des Bundesrates in Erfüllung des Postulats 17.4177 vom 14. Dezember 2017 wird ein eher theoretischer Ansatz verfolgt, der wenig auf den tatsächlichen Berufsalltag des Personals, das an den Eisenbahngrenzübergängen arbeitet, ausgerichtet ist. In Anbetracht der bedeutenden geplanten Änderungen ist es angezeigt, dass mehr Informationen über das Operative und über die Auswirkungen auf den Alltag der Angestellten und der Bevölkerung bekannt werden. 1. Sind Investitionen in die Infrastruktur geplant zur Verbesserung der Kontrollen, insbesondere des Güterverkehrs, an allen Grenzbahnhöfen (Basel, Buchs, Vallorbe, Genf, Domodossola, Luino, Chiasso)? Ist dafür die Eidgenössische Zollverwaltung (EZV) oder direkt die SBB zuständig? Wie werden die Finanzierung und die Koordination der Verfahren sichergestellt? 2. Sind für den Bahngüterverkehr festinstallierte Scanner vorgesehen? An welchen Bahnhöfen? 3. Ist im Rahmen der laufenden Reform vorgesehen, die internationalen Abkommen, die für die Grenzbahnhöfe gelten, an die heutige Situation anzupassen? Welche Abkommen sollen mit den jeweiligen Vertragspartnern angepasst werden? 4. Sieht das Projekt DaziT - zur Optimierung d…</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr"/>
@@ -1024,7 +1032,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Semplificare e velocizzare i mostri burocratici rappresentati dai permessi nel quadro dei contingenti per cittadini di Stati terzi e dai permessi di soggiorno di breve durata (permessi L) per cittadini UE/AELS</t>
+          <t>Die Bürokratiemonster "Bewilligungen von Drittstaatenkontingenten" und "Kurzaufenthaltsbewilligungen (L-Bewilligungen) für EU-/Efta-Bürger" müssen vereinfacht und beschleunigt werden</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -1034,7 +1042,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Per le imprese che desiderano assumere lavoratori provenienti da Stati terzi, le procedure per ottenere i relativi permessi sono complesse e impegnative. La procedura stessa può facilmente richiedere sei mesi. Le grandi imprese dispongono di apposite divisioni o incaricano società di consulenza specializzate. Per ragioni di ordine finanziario, le PMI e le start-up non dispongono di questa possibilità. I tempi di trattamento per i permessi L per cittadini UE/AELS sono troppo lunghi e variano considerevolmente da un Cantone all'altro. In teoria il trattamento può essere eseguito in pochi secondi in quanto interamente standardizzato; eventuali eccezioni possono essere sottoposte a un responsabile cantonale. Uno sportello unico digitale nazionale per le PMI ridurrebbe notevolmente la complessità, abbreviando la durata delle procedure. Con EasyGov esiste già una piattaforma operativa approntata esattamente per procedure di questo tipo. Estendendo EasyGov ai permessi di lavoro si offrirebbe alle start-up e alle PMI una reale possibilità di presentare domande in maniera semplice e con procedure digitali ben condotte. Alla luce di quanto precede, invito il Consiglio federale a rispon…</t>
+          <t>[Official DE version; original is IT] TEXT: Die mit der Bewilligung von Drittstaatenkontingenten verbundenen Prozesse sind für Unternehmen komplex und anspruchsvoll. Der Prozess selbst dauert gut und gerne ein halbes Jahr. Grossunternehmen haben dafür eigene Abteilungen oder beauftragen spezialisierte Beratungsunternehmen. Für KMU und Start-ups besteht diese Möglichkeit aus finanziellen Gründen nicht. Die Bearbeitungszeiten bei den L-Bewilligungen für EU-/Efta-Bürger sind zu lange und von Kanton zu Kanton sehr unterschiedlich. Die Bearbeitung kann theoretisch in Sekunden erledigt werden, da voll regelbasiert, allfällige Ausnahmen können einem Sachbearbeiter im Kanton zugewiesen werden. Ein digitaler, nationaler One-Stop-Shop für KMU würde die Komplexität deutlich senken und die Länge des Prozesses verkürzen. Mit EasyGov besteht bereits eine Plattform, die für genau solche Prozesse gebaut wurde und bereits in Betrieb ist. Eine Erweiterung von EasyGov um Arbeitsbewilligungen würde für Start-ups und KMU eine echte Chance bieten, einfach und mit gut geführten digitalen Prozessen Anträge zu stellen. Vor diesem Hintergrund wird der Bundesrat gebeten, folgende Fragen zu beantworten: 1. Teilt er die Ansicht, dass die Antragste…</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr"/>
@@ -1049,7 +1057,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Entreprises plates-formes et économie à la tâche ou "gig economy". Mieux protéger les travailleurs indépendants</t>
+          <t>Plattformunternehmen und Gig Economy. Bessere Absicherung von selbstständig Erwerbstätigen</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -1059,8 +1067,8 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Le Conseil fédéral est chargé d'élaborer un rapport dans lequel il propose des pistes pour améliorer la protection sociale des indépendants travaillant à la tâche. Il devra en particulier examiner comment les entreprises plateformes pourraient contribuer à assurer une meilleure couverture sociale aux personnes participant à cette économie dite collaborative ou de partage.
-REASONING: Déjà en plein essor, les modèles de travail flexible vont se développer encore sous l'effet d'une numérisation galopante. Ils consistent à proposer de brèves missions à des indépendants ou des personnes employées à temps très partiel. On peut s'attendre à ce que la tendance à l'ubérisation, dominée par les entreprises plateformes, prenne encore de l'ampleur. Cette évolution propose de nouveaux modèles d'entreprises mais elle ouvre aussi de nouvelles possibilités qui, à certaines conditions, peuvent tout à fait séduire les indépendants. Le problème est que ceux-ci se voient moins bien protégés contre les risques sociaux. Les acteurs politiques sont donc appelés à examiner les conditions de cette nouvelle économie et à les adapter si nécessaire afin qu'elle ne soit pas synonyme de réduction de la p…</t>
+          <t>[Official DE version; original is FR] TEXT: Der Bundesrat wird beauftragt, in einem Bericht darzulegen, wie die soziale Absicherung von selbstständig Erwerbstätigen der sogenannten Gig Economy gestärkt werden kann. Dabei ist auch und insbesondere zu prüfen, wie Plattformunternehmen zur Verbesserung der sozialen Absicherung beitragen können.
+REASONING: Das schon heute verbreitete Bedürfnis nach flexiblen Arbeitsmodellen wird im Zuge der fortschreitenden digitalen Transformation weiter zunehmen. Es ist davon auszugehen, dass der Trend "Gig Economy" - jenes Teils der Arbeitswelt, der von Plattformunternehmen dominiert wird und/oder in welchem kleine Aufträge kurzfristig an unabhängige Selbstständigerwerbende oder Beschäftigte mit Kleinstpensen vergeben werden - weiter an Bedeutung gewinnen wird. Diese Entwicklung eröffnet nicht nur Unternehmen neue Geschäftsmodelle, sondern auch den einzelnen Erwerbstätigen erweiterte und unter gewissen Umständen durchaus attraktive Arbeitsmodelle. Problematisch ist hingegen, dass die betroffenen selbstständig Erwerbstätigen über einen schlechteren Schutz gegen soziale Risiken verfügen. Die Politik ist aufgerufen, die bestehenden Rahmenbedingungen zu überprüfen und gegebenenfalls anzupas…</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr"/>
@@ -1151,7 +1159,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>TVA. État des lieux de la nouvelle imposition des plateformes numériques</t>
+          <t>Bestandsaufnahme der neuen MWST-Plattformbesteuerung</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -1161,8 +1169,8 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Depuis le 1er janvier 2025, les plateformes numériques sont assujetties à la TVA en Suisse. Comment le nombre d’inscriptions à la TVA et de taxations fiscales a-t-il évolué depuis l’instauration des nouvelles règles ? Comment l’augmentation des inscriptions à la TVA se répartit-elle entre les entreprises nationales et les entreprises étrangères ? Quelles mesures l’AFC prend-elle cette année pour s’assurer que toutes les entreprises disposant d’un IDE remplissent bel et bien leurs obligations en matière de TVA ?
-ANSWER: Questions 1 et 2 : les inscriptions à la TVA en tant que plateforme au sens de l’art. 20a, al. 1 de la loi fédérale du 12 juin 2009 sur la taxe sur la valeur ajoutée (LTVA ; RS 641.20) se répartissent à mi-mars entre vingt plateformes sises à l’étranger et quatre plateformes sises sur le territoire suisse. Toutefois, ces chiffres doivent être interprétés avec prudence pour les raisons suivantes : l’inscription en ligne en tant que plateforme pour les nouveaux assujettis n’est disponible que depuis novembre 2024 pour les plateformes étrangères et mars 2025 pour celles situées sur le territoire suisse ; par ailleurs, certaines entreprises ont pu omettre de décla…</t>
+          <t>[Official DE version; original is FR] TEXT: Seit dem 1. 1. 2025 gilt in der Schweiz eine neue Mehrwertsteuerregelung für elektronische Plattformen. Wie haben sich die Anzahl der MWST-Anmeldungen und die Steuerveranlagungen seit der Einführung der neuen Regelung entwickelt? Wie verteilt sich der Anstieg der MWST-Anmeldungen auf inländische und ausländische Unternehmen? Welche Massnahmen ergreift die ESTV konkret in diesem Jahr, um sicherzustellen, dass alle Unternehmen mit einer UID ihre Mehrwertsteuerpflicht tatsächlich erfüllen?
+ANSWER: Zu 1 und 2: Die MWST-Anmeldungen als Plattform im Sinne von Artikel 20a Absatz 1 des Bundesgesetzes vom 12. Juni 2009 über die Mehrwertsteuer (MWSTG; SR 641.20) verteilen sich auf zwanzig Plattformen mit Sitz im Ausland und vier Plattformen mit Sitz im Inland (Stand: Mitte März 2025). Diese Zahlen sind jedoch namentlich aus folgenden Gründen mit Vorsicht zu interpretieren: Die Online-Anmeldung als Plattform für neue Steuerpflichtige ist für im Ausland ansässige Plattformen erst seit November 2024 und für Plattformen mit Sitz im Inland erst seit März 2025 verfügbar; darüber hinaus haben es einige Unternehmen möglicherweise versäumt, bei der Anmeldung ihren Status als Plattform anzugebe…</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr"/>
@@ -1177,7 +1185,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Contributi per procedimenti di spandimento a basse emissioni fino al 2021</t>
+          <t>Beiträge für emissionsmindernde Ausbringverfahren bis 2021</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
@@ -1187,8 +1195,8 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Il Consiglio federale è incaricato di modificare l'ordinanza concernente i pagamenti diretti nell'agricoltura (OPD; RS 910.13) in modo che i contributi per lo spandimento a basse emissioni di concimi liquidi aziendali e ottenuti dal riciclaggio siano versati fino al 2021 (invece del 2019). Una minoranza (Schneider Schüttel, Bendahan, Brélaz, Gmür Alois, Gschwind, Gysi, Hadorn, Kiener Nellen, Meyer Mattea) propone di respingere la mozione.
-ANSWER: A partire dal 2022 l'utilizzo di procedimenti di spandimento a basse emissioni sarà prescritto in virtù del diritto ambientale nell'ordinanza contro l'inquinamento atmosferico (OIAt) e, sempre dal 2022, diventerà parte integrante della prova che le esigenze ecologiche sono rispettate, la cui fornitura è indennizzata mediante pagamenti diretti. Non è quindi possibile mantenere i contributi oltre il 2021. Il Consiglio federale propone di accogliere la mozione.</t>
+          <t>[Official DE version; original is IT] TEXT: Der Bundesrat wird beauftragt, die Verordnung über die Direktzahlungen an die Landwirtschaft (SR 910.13) dahingehend zu ändern, dass die Beiträge für die emissionsmindernde Ausbringung von flüssigen Hof- und Recyclingdüngern bis 2021 (anstelle 2019) ausgerichtet werden. Eine Minderheit (Schneider Schüttel, Bendahan, Brélaz, Gmür Alois, Gschwind, Gysi, Hadorn, Kiener Nellen, Meyer Mattea) beantragt die Ablehnung der Motion.
+ANSWER: Ab 2022 soll der Einsatz von emissionsmindernden Ausbringungsverfahren in der Luftreinhalteverordnung (LRV) umweltrechtlich vorgeschrieben werden und wird, ebenfalls ab 2022, Bestandteil des ökologischen Leistungsnachweises, dessen Einhaltung mit Direktzahlungen abgegolten wird. Eine Weiterführung der Beiträge über 2021 hinaus ist folglich nicht möglich. Der Bundesrat beantragt die Annahme der Motion.</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr"/>
@@ -1203,7 +1211,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Si renda obbligatoria l'assicurazione malattia svizzera per i lavoratori frontalieri</t>
+          <t>Die schweizerische Krankenversicherung soll für Grenzgängerinnen und Grenzgänger obligatorisch werden</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
@@ -1213,7 +1221,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Secondo l'Ordinanza sull'assicurazione malattie 832.102 all'Art. 3 Frontalieri "1 A loro domanda vengono assoggettati all'assicurazione svizzera i frontalieri che esercitano un'attività lucrativa in Svizzera non soggetti all'obbligo d'assicurazione ai sensi dell'articolo 1 capoverso 2 lettera d ed e nonché i loro familiari, purché non esercitino all'estero un'attività lucrativa per cui siano tenuti ad assicurarsi contro le malattie." Nella pratica i lavoratori frontalieri possono esercitare il diritto di opzione, o vengono assoggettati all'assicurazione svizzera, o rimangono assicurati nel paese di residenza. È ipotizzabile che la maggior parte dei lavoratori frontalieri non sono assicurati in Svizzera per ragioni di costo e questo, a parità di salario, permette loro di avere un reddito disponibile molto più alto dei lavoratori svizzeri in quanto, ad esempio in Italia, l'assicurazione malattia è di fatto gratuita. Due operai, uno svizzero e l'altro frontaliere con residenza in Italia, entrambe con un salario lordo di 5000 franchi, per il frontaliere oltre al vantaggio economico di vivere in Italia - dove il costo della vita è di molto inferiore - ha pure il vantaggio di non d…</t>
+          <t>[Official DE version; original is IT] TEXT: Artikel 3 Absatz 1 der Verordnung über die Krankenversicherung (SR 832.102) (Grenzgänger und Grenzgängerinnen) lautet wie folgt: "Nicht der Versicherungspflicht nach Artikel 1 Absatz 2 Buchstaben d und e unterstellte Grenzgänger und Grenzgängerinnen, die in der Schweiz eine Erwerbstätigkeit ausüben, sowie ihre Familienangehörigen, sofern diese im Ausland nicht eine krankenversicherungspflichtige Erwerbstätigkeit ausüben, werden auf eigenes Gesuch hin der schweizerischen Versicherung unterstellt." In der Praxis können die Grenzgängerinnen und Grenzgänger von ihrem Optionsrecht Gebrauch machen; sie werden also entweder der schweizerischen Versicherung unterstellt oder sie bleiben in ihrem Wohnland versichert. Es kann davon ausgegangen werden, dass sich die meisten Grenzgängerinnen und Grenzgänger aus Kostengründen nicht in der Schweiz versichern lassen. Da beispielsweise in Italien die Krankenversicherung praktisch gratis ist, haben sie bei gleichem Lohn deshalb ein viel höheres Einkommen als Schweizer Arbeitnehmerinnen und Arbeitnehmer. Nehmen wir als Beispiel zwei Arbeiter, einer Schweizer, der andere Grenzgänger aus Italien, beide mit einem Bruttoeinkommen von 5000 Franken: …</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr"/>
@@ -1228,7 +1236,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Quale impatto avrà la digitalizzazione sulla nostra salute?</t>
+          <t>Welche Auswirkungen hat die Digitalisierung auf unsere Gesundheit?</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
@@ -1238,8 +1246,8 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Il Consiglio federale è incaricato di presentare un rapporto allo scopo di analizzare l'impatto e gli effetti della digitalizzazione della nostra società sulla salute umana. Il rapporto dovrà contenere una serie di provvedimenti destinati a conciliare lo sviluppo della digitalizzazione con la tutela della salute e del benessere della popolazione, in particolar modo dei giovani in formazione.
-REASONING: Da parecchi anni, il Consiglio federale pubblica rapporti sulle opportunità offerte dalla digitalizzazione per il nostro sistema di formazione e la nostra società in generale. È assolutamente auspicabile trarre il massimo beneficio possibile dalla transizione digitale, ma non a scapito della salute della popolazione. Un rapporto di Educa del 2021 fa notare che l'impiego di risorse digitali ha conseguenze sulla salute o sul benessere soggettivo degli allievi o degli insegnanti. Il rapporto sottolinea inoltre che, secondo alcuni studi trasversali condotti nel Cantone di Vaud, i giovani che trascorrono più tempo davanti allo schermo accusano più spesso problemi di salute come mal di schiena, problemi posturali, sovrappeso e carenza di sonno. Inoltre, trascorrere molte ore davanti…</t>
+          <t>[Official DE version; original is IT] TEXT: Der Bundesrat wird beauftragt, einen Bericht zur Analyse der Auswirkungen der Digitalisierung unserer Gesellschaft auf die menschliche Gesundheit vorzulegen. Der Bericht soll eine Reihe von Massnahmen enthalten, welche die Entwicklung der Digitalisierung mit der Erhaltung der Gesundheit und des Wohlbefindens der Bevölkerung, insbesondere der Schülerinnen und Schüler, in Einklang bringen.
+REASONING: Seit mehreren Jahren veröffentlicht der Bundesrat Berichte, in denen er die Chancen der Digitalisierung für unser Bildungssystem und unsere Gesellschaft im Allgemeinen aufzeigt. Es ist durchaus sinnvoll, den digitalen Wandel bestmöglich zu nutzen, aber dies darf nicht auf Kosten der Gesundheit der Bevölkerung geschehen. Denn wie ein Bericht von Educa 2021 feststellt, hat "die Nutzung digitaler Ressourcen Konsequenzen für Gesundheit oder subjektives Wohlbefinden von Schülerinnen und Schülern oder Lehrpersonen". In diesem Bericht heisst es weiter: "Querschnittsstudien aus dem Kanton Waadt zeigen ebenfalls, dass Jugendliche, die mehr Zeit vor dem Bildschirm verbringen, häufiger über gesundheitliche Störungen wie Rückenschmerzen, Haltungsschäden, Übergewicht und Schlafmangel berichten…</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr"/>
@@ -1254,7 +1262,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Pour plus de force aux cantons</t>
+          <t>Den Kantonen mehr Mitspracherecht</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
@@ -1264,8 +1272,8 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Les Autorités fédérales sont invitées à modifier l'article 16 al. 6 de la loi fédérale du 26 septembre 2014 concernant la surveillance de l'assurance-maladie sociale (LSAMal ; RS 832.12) comme il suit : Avant l'approbation des tarifs, les cantons peuvent donner leur avis aux assureurs et à l'autorité de surveillance sur l'évaluation des coûts et sur les tarifs de primes prévues pour leur territoire, à la condition que ces échanges ne prolongent pas la procédure d'approbation. Les cantons peuvent obtenir les informations nécessaires auprès des assureurs et de l'autorité de surveillance. Ces informations ne peuvent être ni rendues publiques ni transmises à des tiers.
-REASONING: 1. Introduction Le canton de Fribourg soumet à l'Assemblée fédérale trois initiatives autant de modifications de la loi fédérale sur la surveillance de l'assurance-maladie du 26 septembre 2014 (LSAMal). Les initiatives visent toutes trois à assurer une meilleure adéquation des primes d'assurance-maladie par rapport aux coûts des prestations qu'elles couvrent. Initiées par le canton du Tessin, plusieurs autres cantons ont adopté ou sont en train d'adopter le dépôt d'initiatives similaires. En résumé, la …</t>
+          <t>[Official DE version; original is FR] TEXT: Die Bundesbehörden werden eingeladen, Artikel 16 Abs. 6 des Bundesgesetzes betreffend die Aufsicht über die soziale Krankenversicherung vom 26. September 2014 (KVAG; SR 832.12) wie folgt zu ändern: Vor der Genehmigung des Prämientarifs können die Kantone zu den für ihren Kanton geschätzten Kosten und den vorgesehenen Prämientarifen gegenüber den Versicherern und der Aufsichtsbehörde Stellung nehmen; das Genehmigungsverfahren darf dadurch nicht verzögert werden. Die Kantone können bei den Versicherern und der Aufsichtsbehörde die dazu benötigten Informationen einholen. Diese Informationen dürfen weder veröffentlicht noch weitergeleitet werden.
+REASONING: 1. Einleitung Der Kanton Freiburg unterbreitet der Bundesversammlung drei Standesinitiativen zu Änderungen des Bundesgesetzes betreffend die Aufsicht über die soziale Krankenversicherung vom 26. September 2014 (KVAG). Alle drei Initiativen zielen auf angemessenere Krankenversicherungsprämien im Vergleich zu den Kosten der Leistungen ab, die sie abdecken. Ausgehend vom Kanton Tessin haben mehrere andere Kantone beschlossen oder sind daran zu beschliessen, gleichlautende Initiativen einzureichen. Zusammengefasst will die erste …</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr"/>
@@ -1280,7 +1288,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Combien la Suisse a-t-elle dépensé pour aider l'Ukraine?</t>
+          <t>Wie viel hat die Schweiz ausgegeben, um der Ukraine zu helfen?</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
@@ -1290,8 +1298,7 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Le chef du DFAE Ignazio Cassis a récemment annoncé le versement de 1,8 milliard de francs d'aide supplémentaire à l'Ukraine d'ici à 2028, une somme énorme qu'il justifie par le fait que la Suisse doit " faire sa part ". Or, cet argument est des plus maladroits puisque la Suisse a déjà fait bien plus que sa part - et pas seulement du point de vue financier - depuis le début d'une guerre dont elle n'est pourtant aucunement responsable. L'ampleur des montants déboursés pour aider l'Ukraine appelle la plus grande transparence, laquelle n'est pour l'heure absolument pas garantie. Je prie dès lors le Conseil fédéral de répondre aux questions suivantes : - Combien la Suisse a-t-elle dépensé jusqu'ici pour l'accueil des réfugiés ukrainiens (en tenant compte des coûts liés à la couverture des soins médicaux) ? - À combien se monte l'aide versée par la Suisse à l'Ukraine sous différentes formes ? - À combien se monte l'aide versée par les autres pays en lien avec l'invasion de l'Ukraine ? - Le Conseil fédéral a-t-il l'intention de mettre à jour et de publier régulièrement (par ex. tous les six mois) les chiffres demandés ci-dessus ?
-ANSWER: L’aide versée par la Confédération depuis le…</t>
+          <t>[Official DE version; original is FR] TEXT: Ignazio Cassis, der Vorsteher des EDA, hat kürzlich angekündigt, die Schweiz werde der Ukraine bis 2028 weitere 1,8 Milliarden Franken an Hilfsgeldern zukommen lassen. Das ist natürlich eine enorme Summe. Bundesrat Cassis rechtfertigte sie in der Öffentlichkeit mit der Begründung, auch die Schweiz müsse ihren Beitrag leisten. Diese Argumentation vermag nicht zu überzeugen, da die Schweiz im Zusammenhang mit dem Krieg in der Ukraine - für den sie logischerweise keine Verantwortung trägt - schon jetzt viel mehr als ihren Beitrag geleistet hat, und zwar nicht nur aus finanzieller Sicht. In Bezug auf die beträchtlichen Summen, die wegen des Kriegs in der Ukraine ausgegeben wurden, braucht es mehr Transparenz - eine Transparenz, an der es zum aktuellen Zeitpunkt mangelt. Ich frage den Bundesrat: - Wie viel hat die Schweiz bis heute für die aufgenommenen ukrainischen Flüchtlinge ausgegeben (einschliesslich der Kosten für die Krankenversicherung)? - Wie viele Hilfsgelder hat sie, in verschiedenen Formen, an die Ukraine ausbezahlt? - Wie viele Hilfsgelder hat sie im Zusammenhang mit dem Angriff auf die Ukraine an andere Länder ausbezahlt? - Hat der Bundesrat die Absicht, die entsprec…</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr"/>
@@ -1306,7 +1313,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Adeguamento del diritto federale agli sviluppi della tecnologia di registro distribuito. Legge federale</t>
+          <t>Anpassung des Bundesrechts an Entwicklungen der Technik verteilter elektronischer Register. Bundesgesetz</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
@@ -1314,7 +1321,11 @@
           <t>open</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Official DE version; original is IT] </t>
+        </is>
+      </c>
       <c r="F30" s="5" t="inlineStr"/>
       <c r="G30" s="5" t="inlineStr"/>
     </row>
@@ -1327,7 +1338,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>L’ex-ambassadeur Jean-Daniel Ruch dévoile des informations sensibles dans ses mémoires</t>
+          <t>Alt-Botschafter Jean Daniel Ruch veröffentlicht am 12. Juni seine Memoiren und damit brisante Informationen</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
@@ -1337,8 +1348,8 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Les mémoires de Jean-Daniel Ruch paraîtront le 12 juin. Il y dévoile des conversations confidentielles et secrètes (notamment des discussions menées avec des représentants turcs sur les efforts de paix concernant le conflit ukrainien). - Les (ex-)ambassadeurs ne sont-ils pas soumis au secret de fonction ? - Qui voudra encore mener des entretiens confidentiels avec la Suisse, si le contenu est ensuite dévoilé au public ? - Que fait le Conseil fédéral pour empêcher Jean-Daniel Ruch de continuer à violer son secret de fonction ?
-ANSWER: La réponse du Conseil fédéral n'existe qu'en allemand. (Veuillez changer la langue en haut à droite de la page d'accueil)</t>
+          <t>[Official DE version; original is FR] TEXT: Jean Daniel Ruch veröffentlicht am 12. Juni seine Memoiren. In diesen legt er vertrauliche und geheime Gespräche offen (u.a. mit türkischen Vertretern über die Friedensbemühungen im Ukraine Konflikt). - Sind (Alt-) Botschafter an keine Schweigepflicht gebunden? - Wer will mit der Schweiz noch vertraulich sprechen, wenn nachher alles in der Öffentlichkeit ausgebreitet wird? - Was unternimmt der Bundesrat gegen Alt-Botschafter Jean Daniel Ruch, damit er seine Geheimnisverletzungen nicht weiterverbreitet?
+ANSWER: Das Personal des EDA untersteht den Pflichten gemäss Bundespersonalgesetzgebung. Neben der Pflicht zur Wahrung der Interessen des Arbeitgebers und des Bundes gelten für die Angestellten unter anderem auch das Berufs-, Geschäfts und Amtsgeheimnis. Mit der Beendigung des Arbeitsverhältnisses erlischt die Treuepflicht der Bundesangestellten. Die Pflicht zur Wahrung des Amts- und Berufsgeheimnisses bleibt auch nach Beendigung des Arbeitsverhältnisses bestehen. Herr Jean-Daniel Ruch hat den Entwurf seiner Memoiren den zuständigen Stellen im EDA vorgelegt und die notwendigen Anpassungen zur Erfüllung der gesetzlichen Pflichten akzeptiert.</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr"/>
@@ -1405,7 +1416,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Revoca sistematica della cittadinanza ai "viaggiatori della jihad" con la doppia cittadinanza!</t>
+          <t>Systematische Ausbürgerung von "Dschihad-Touristen" mit doppelter Staatsbürgerschaft</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
@@ -1415,8 +1426,8 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Il Consiglio federale è incaricato di adottare le disposizioni necessarie per far applicare sistematicamente l'articolo 42 della legge sulla cittadinanza ai "viaggiatori della jihad" svizzeri con la doppia cittadinanza.
-REASONING: Sul sito della SEM https://www.sem.admin.ch/sem/it/home/themen/buergerrecht/schweizer_buergerrecht.html si legge che la revoca della cittadinanza in applicazione dell'articolo 42 LCit è concepibile solo in casi estremamente gravi, come quelli di criminali di guerra o terroristi. Nella sua risposta alla mia domanda 19.5162, il Consiglio federale ha precisato che una tale misura è possibile se la condotta della persona in questione è di grave pregiudizio agli interessi o alla buona reputazione della Svizzera. Si esige inoltre una condanna penale passata in giudicato, a meno che il perseguimento penale non possa essere portato a termine (p. es. in caso di malfunzionamento dell'apparato giudiziario). In questo contesto, il Governo ha evocato... una - sì, una sola! - procedura di revoca che, il 18 marzo 2019, era ancora soltanto avviata. Ha aggiunto che era al vaglio l'avvio di altre procedure, senza precisare quante né fornire alcuna cifra che permetta…</t>
+          <t>[Official DE version; original is IT] TEXT: Der Bundesrat wird beauftragt, dafür zu sorgen, dass Artikel 42 BüG systematisch bei Schweizer "Dschihad-Touristen" mit doppelter Staatsbürgerschaft angewendet wird.
+REASONING: Auf der Website des Staatssekretariats für Migration (SEM) (https://www.sem.admin.ch/sem/de/home/themen/buergerrecht/schweizer_buergerrecht.html) steht, dass der Entzug des Schweizer Bürgerrechtes gemäss Artikel 42 BüG nur in einem gravierenden Fall denkbar sei. Als Beispiele werden verurteilte Kriegsverbrecher oder Terroristen genannt. In seiner Antwort auf meine Frage 19.5162 hat der Bundesrat erklärt, dass eine solche Massnahme möglich sei, wenn das Verhalten der Person den Interessen oder dem Ansehen der Schweiz erheblich nachteilig ist, und darüber hinaus eine strafrechtliche Verurteilung rechtskräftig ist, ausser wenn die Strafverfolgung nicht stattfinden kann (z. B. aufgrund eines nicht funktionierenden Justizwesens). In diesem Zusammenhang erwähnte der Bundesrat am 18. März 2019 ein einziges Ausbürgerungsverfahren, das bisher lediglich eingeleitet wurde. Er fügte hinzu, dass die Eröffnung weiterer Verfahren geprüft würde, wobei der Bundesrat keine genauen Angaben machte, mit denen sich einschä…</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr"/>
@@ -1431,7 +1442,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Reconnaissance intercantonale des attestations électroniques officielles</t>
+          <t>Interkantonale Anerkennung von amtlichen Bescheinigungen in elektronischer Form</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -1441,7 +1452,7 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Dans le cadre du développement des services numériques cantonaux et communaux, certaines administrations délivrent désormais des attestations officielles sous forme électronique. Or, des cas concrets montrent que ces documents ne sont pas toujours reconnus par d’autres autorités. Ainsi, une attestation de domicile délivrée électroniquement par une commune valaisanne a été refusée par un état civil fribourgeois au motif que ce dernier doutait de son authenticité, faute de signature sur le document. Dans de tels cas, les autorités doivent établir a posteriori une version papier, ce qui annule les bénéfices de la démarche numérique. De telles situations nuisent à la crédibilité des services numériques, génèrent des coûts supplémentaires et freinent la transition vers une administration digitale efficace et harmonisée. Dans ce contexte, je prie le Conseil fédéral de répondre aux questions suivantes : Le Conseil fédéral a‑t‑il connaissance de cas dans lesquels des documents officiels électroniques émis par une autorité ne sont pas reconnus par une autre autorité, notamment dans un autre canton ? Quelles bases légales, quels standards ou quelles recommandations existent aujourd’hui…</t>
+          <t>[Official DE version; original is FR] TEXT: Im Rahmen des Ausbaus der digitalen Dienste auf kantonaler und kommunaler Ebene stellen einige Behörden nun amtliche Bescheinigungen in elektronischer Form aus. Konkrete Fälle zeigen jedoch, dass diese Dokumente von anderen Behörden nicht immer anerkannt werden. So wurde eine von einer Walliser Gemeinde elektronisch ausgestellte Wohnsitzbestätigung von einem Freiburger Zivilstandsamt abgelehnt mit der Begründung, dass dieses aufgrund der fehlenden Unterschrift an der Echtheit des Dokuments zweifelte. In solchen Fällen müssen die Behörden nachträglich ein Dokument in Papierform erstellen, wodurch der Nutzen des digitalen Verfahrens verloren geht. Solche Situationen untergraben die Glaubwürdigkeit digitaler Dienste, verursachen Mehrkosten und behindern den Übergang zu einer effizienten und einheitlichen digitalen Verwaltung. Ich bitte deshalb den Bundesrat, folgende Fragen zu beantworten: Sind dem Bundesrat Fälle bekannt, in denen von einer Behörde ausgestellte amtliche Dokumente in elektronischer Form von einer anderen Behörde, insbesondere in einem anderen Kanton, nicht anerkannt werden? Welche rechtlichen Grundlagen, Standards oder Empfehlungen gibt es derzeit auf Bundeseben…</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr"/>
@@ -1456,7 +1467,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Entità legale in Svizzera per i fornitori di servizi</t>
+          <t>Gesetzliche Vertretung von Dienstleistern in der Schweiz</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
@@ -1466,7 +1477,7 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Le attuali mutazioni strutturali, in particolare la digitalizzazione, cambiano le carte in tavola nel settore delle telecomunicazioni. Occorre prevedere nuove misure legislative per adeguarsi a queste inevitabili evoluzioni. Le reti sociali, ad esempio Facebook o Twitter, fanno ormai parte integrante della vita quotidiana dei cittadini elvetici. Queste reti forniscono servizi al consumatore svizzero e sono pertanto presenti digitalmente sul nostro territorio. Non possiedono tuttavia necessariamente un'entità legale in Svizzera. Questa situazione è problematica. Quando si tratta di ottenere dati ai fini di un'indagine in caso di cybermobbing, diffamazione o altro la giustizia, infatti, si trova di fronte a un muro, come emerge dalla decisione del Tribunale federale 1B_185/2016, riguardante il Ministero pubblico vodese e Facebook Switzerland. I dati necessari all'inchieste possono infatti essere ottenuti soltanto con una procedura di assistenza giudiziaria internazionale, troppo lenta. Analogamente, di recente sono scoppiati casi di obsolescenza programmata. A titolo di esempio è possibile citare la situazione di Epson o di Apple. Tuttavia, per un consumatore o un gruppo di con…</t>
+          <t>[Official DE version; original is IT] TEXT: Mit den gegenwärtigen strukturellen Veränderungen, namentlich der Digitalisierung, ändern die Gegebenheiten im Bereich der Telekommunikation. Daher müssen neue gesetzgeberische Massnahmen vorgesehen werden, um sich an diese unaufhaltsamen Entwicklungen anzupassen. Die sozialen Netzwerke wie Facebook und Twitter sind fester Bestandteil des Alltags der Schweizerinnen und Schweizer. Die Netzwerke erbringen Dienste für die Schweizer Konsumentinnen und Konsumenten und befinden sich daher digital auf unserem Staatsgebiet. Dennoch haben sie nicht zwangsläufig einen eigenständigen rechtlichen Status in der Schweiz. Diese Situation ist problematisch. In Fällen von Cybermobbing, übler Nachrede oder bei anderen Ermittlungen stösst die Justiz nämlich an Grenzen, wenn es darum geht, für ein Verfahren Daten zu erlangen. Davon zeugt der Bundesgerichtsentscheid 1B_185/2016 in einer Rechtssache zwischen der waadtländischen Staatsanwaltschaft und Facebook Switzerland. Demnach braucht es ein - allzu langsames - Verfahren internationaler Rechtshilfe in Strafsachen, um an die für die Ermittlung nötigen Daten zu gelangen. Hinzu kommt, dass kürzlich Fälle von geplanter Obsoleszenz Aufsehen erregt h…</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr"/>
@@ -1507,7 +1518,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Promuovere una ricerca sostenibile grazie a un piano di abbandono degli esperimenti che causano sofferenza agli animali</t>
+          <t>Zukunftsfähige Forschung mit einem Plan für den Ausstieg aus belastenden Tierversuchen fördern</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
@@ -1517,8 +1528,8 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>TEXT: L’attuale legge federale sulla protezione degli animali deve prevedere un piano di abbandono graduale degli esperimenti che causano sofferenza agli animali, che stabilisca obiettivi, tappe e scadenze vincolanti. Tale piano dovrà essere elaborato coinvolgendo il mondo scientifico, le organizzazioni per la protezione degli animali e l’industria.
-REASONING: La legge federale sulla protezione degli animali stabilisce già oggi che gli esperimenti sugli animali devono essere limitati al minimo indispensabile (art. 17) e che infliggere sofferenze all’animale è lecito soltanto se inevitabile per lo scopo dell’esperimento (art. 20 cpv. 1). Già grazie all’aiuto di tecnologie odierne, molti degli obiettivi degli esperimenti possono essere raggiunti con metodi che non prevedono test sugli animali. È stato dimostrato che tali metodi sono chiaramente superiori alla sperimentazione animale in termini di trasferibilità, utilità e costi (1). Il loro sviluppo sta progredendo costantemente, ma può essere accelerato con misure appropriate, ad esempio grazie a maggiori finanziamenti. Se intensificherà gli sforzi per garantire lo sviluppo e l’applicazione di metodi senza sperimentazione animale s…</t>
+          <t>[Official DE version; original is IT] TEXT: Das bestehende Tierschutzgesetz soll mit einem stufenweisen Ausstiegsplan aus belastenden Tierversuchen ergänzt werden. Der Ausstiegsplan legt verbindliche Ziele, Meilensteine und Fristen fest. Die Ausarbeitung des Ausstiegsplans soll unter Einbezug von Wissenschaft, Tierschutz und Industrie erfolgen.
+REASONING: Das Tierschutzgesetz legt bereits heute fest, dass Tierversuche auf das unerlässliche Mass zu beschränken sind (Art. 17) und Belastungen nur zugelassen sind, soweit diese für den Zweck des Versuchs unvermeidlich sind (Art. 20 Abs. 1). Bereits mit heutigen Technologien können eine Vielzahl der Ziele der Versuche mit Methoden ohne Tierversuche erreicht werden. Dabei zeigt sich, dass diese tierversuchsfreien Methoden in punkto Übertragbarkeit, Nutzen und Kosten dem Tierversuch deutlich überlegen sind (1). Die Entwicklung dieser Methoden schreitet kontinuierlich voran: Mit entsprechenden Massnahmen wie bspw. eine stärkere Finanzierung kann sie aber auch beschleunigt werden. Wenn die Schweiz sich vermehrt dafür einsetzt, dass tierversuchsfreie Methoden in unserem Forschungsplatz entwickelt und angewendet werden, kann sie sich auf lange Sicht als wichtige, internationale I…</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr"/>
@@ -1533,7 +1544,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Biodiversità e stabilità finanziaria. Rapporto del "Network for Greening the Financial System"</t>
+          <t>Biodiversität und Finanzstabilität. Bericht des Network for Greening the Financial System</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
@@ -1543,7 +1554,7 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>TEXT: La Svizzera fa parte del "Network for Greening the Financial System" (NGFS), una rete che riunisce banche centrali e autorità di vigilanza e che si impegna a favore di un settore finanziario rispettoso del clima e della biodiversità. Nel rapporto "Biodiversity and Financial Stability" del 2021 sono state formulate quattro raccomandazioni per le banche centrali su ciò che possono già fare oggi a tale proposito. Chiedo pertanto al Consiglio federale di rispondere alle seguenti domande. 1. In che modo l'Esecutivo affronta i rischi economici e finanziari rilevanti per la biodiversità? (compito 1) 2. Il Consiglio federale analizza la dipendenza degli istituti finanziari svizzeri dagli ecosistemi e dalla biodiversità e l'impatto che tali istituti producono su di essi? (compito 2) 3. In caso contrario, per quale motivo? 4. Il Governo prevede di sviluppare metodi per comprendere meglio i rischi finanziari rilevanti per la biodiversità (escludendo lo strumento ENCORE)? (compito 3) 5. In che misura il Consiglio federale informa gli istituti finanziari in merito al loro impatto sulla biodiversità e alla loro dipendenza da quest'ultima? (compito 4) 6. Il Consiglio federale riceve regolar…</t>
+          <t>[Official DE version; original is IT] TEXT: Die Schweiz ist beim Network for Greening the Financial System (NGFS) engagiert, einem Zusammenschluss der Zentralbanken und Aufsichtsbehörden, die sich für einen klima- und biodiversitätsfreundlichen Finanzsektor einsetzen. 2021 wurde im Bericht "Biodiversity and Financial Stability" vier Empfehlungen abgegeben, was Zentralbanken schon heute unternehmen können. Deshalb ersuche ich den Bundesrat zur Beantwortung folgender Fragen: 1. Was tut der Bundesrat um die biodiversitätsrelevanten ökonomischen und finanziellen Risiken zu adressieren? (Task 1) 2. Analysiert der Bundesrat die Abhängigkeit und die Wirkung Schweizer Finanzinstitute auf Ökosysteme und Biodiversität? (Task 2) 3. Wenn nein, warum nicht? 4. Plant der Bundesrat Methoden aufzubauen, um biodiversitätsrelevante Finanzrisiken besser zu verstehen (abgesehen vom ENCORE Tool)? (Task 3) 5. Inwiefern informiert der Bundesrat Finanzinstitute über Abhängigkeiten und Wirkungen der Finanzinstitute auf die Biodiversität? (Task 4) 6. Lässt sich der Bundesrat über die entsprechenden Arbeiten bei der SNB und der FINMA regelmässig informieren? 7. Erfolgt eine externe Überprüfung, ob die SNB und die FINMA diese neuen Risiken richti…</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr"/>
@@ -1558,7 +1569,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Violence sexuelle à l'égard des enfants sur Internet. Que fait l'Office fédéral de la police?</t>
+          <t>Sexuelle Gewalt an Kindern im Internet. Was macht das Bundesamt für Polizei?</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -1568,8 +1579,8 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Le Conseil fédéral est prié de répondre aux questions suivantes : 1. L'Office fédéral de la police (Fedpol) remplit-il bien la fonction d'interface entre les organes internationaux et les cantons dans le domaine de la pédocriminalité ? Quelles sont les ressources nécessaires à cette fin quant aux structures, au personnel et aux technologies ? 2. Comment sont traitées les dénonciations en nombre croissant qui arrivent de l'étranger, de manière à ce qu'elles soient examinées avec le soin requis et que les procédures pénales qui s'imposent puissent être menées dans les cantons ? 3. Comment sont gérées les dénonciations qui concernent la Suisse, tout en étant difficiles à attribuer à un canton précis ? 4. Quelle forme pourrait prendre un service national efficace centralisant les dénonciations portant sur des cas de violence sexuelle commise contre des enfants et mise en ligne ? 5. Quelles mesures faudrait-il prendre notamment sur les plans de la législation, des technologies et du personnel pour que la police fédérale joue efficacement son rôle dans la lutte contre la pédocriminalité ?
-REASONING: De plus en plus d'enfants sont victimes de harcèlement sexuel sur Internet (étude …</t>
+          <t>[Official DE version; original is FR] TEXT: Der Bundesrat wird beauftragt zu prüfen: 1. wie das Fedpol zielführend die Schnittstelle zwischen internationaler Ebene und Kantonen im Bereich der Pädokriminalität wahrnimmt sowie welche strukturellen, personellen und technischen Mittel dazu nötig sind; 2. wie mit den ständig ansteigenden Verdachtsmeldungen aus dem Ausland umgegangen wird, damit diese ebenso sorgfältig geprüft werden können und zu den nötigen Strafverfahren in den Kantonen führen; 3. wie mit Verdachtsmeldungen umgegangen wird, welche zwar die Schweiz betreffen, jedoch nicht eindeutig einem Kanton zugeordnet werden können; 4. wie eine wirksame nationale Meldestelle für Verdachtsmeldungen auf sexuelle Gewalt an Kindern online konzipiert sein sollte; 5. welche gesetzlichen, technischen, personellen und sonstigen Massnahmen nötig sind, damit die Bundespolizei ihre Aufgabe der Bekämpfung der Pädokriminalität wirksam wahrnehmen kann.
+REASONING: Immer mehr Kinder werden via Internet sexuell belästigt ("EU Kids online"-Studie). Die an die Schweiz übermittelten Verdachtsmeldungen auf Kinderpornografie steigen exponentiell (Pressemitteilung Fedpol). Es werden immer mehr Fälle von Schweizern bekannt, welche sich einen…</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr"/>
@@ -1636,7 +1647,7 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Révision de la loi sur le renseignement. Le secret médical et professionnel en danger!</t>
+          <t>Revision des Nachrichtendienstgesetzes. Arztgeheimnis und Berufsgeheimnis sind in Gefahr!</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
@@ -1646,7 +1657,7 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Le conseil et le traitement des patients supposent que le corps médical prenne connaissance d'informations sensibles concernant la sphère privée et intime. Les personnes concernées communiquent de telles informations parce qu'elles sont sûres que la confidentialité est garantie. Cette obligation de confidentialité est la condition nécessaire à la réussite d'un diagnostic et d'un traitement. Sans aucune explication, le Conseil fédéral veut supprimer l'al. 2 de l'art. 28 LRens dans le projet de modification de la loi actuellement en consultation. Ce faisant, il affaiblit fortement la protection du secret professionnel. Selon le rapport explicatif, le SRC devrait désormais pouvoir ordonner des mesures soumises à autorisation (surveillance téléphonique et postale, intrusion dans des ordinateurs, etc.) également à l'encontre du personnel médical, des ecclésiastiques, des avocats et des journalistes. Il s'agirait d'une grave érosion des dispositions en matière de protection du secret, en particulier en ce qui concerne le secret médical, de l'avocat, de la confession et la protection des sources dans le journalisme, qui sont importants pour la confiance dans les relations et la démo…</t>
+          <t>[Official DE version; original is FR] TEXT: Die Beratung und Behandlung von Patientinnen und Patienten haben zur Folge, dass das medizinische Personal sensible Informationen erhält, die deren Privat- und Intimsphäre betreffen. Die betroffenen Personen geben solche Informationen preis, weil sie sich sicher sind, dass diese vertraulich behandelt werden. Diese Pflicht zur Gewährleistung der Vertraulichkeit ist eine zwingende Voraussetzung für den Erfolg einer Diagnose und einer Behandlung. Der Bundesrat will im Entwurf, der zurzeit in Vernehmlassung ist, Artikel 28 Absatz 2 NDG ohne Angabe einer Begründung streichen. Dadurch schwächt er den Schutz des Berufsgeheimnisses deutlich. Laut dem erläuternden Bericht soll der NDB genehmigungspflichtige Massnahmen (Überwachung des Post- und Fernmeldeverkehrs, Eindringen in Computer usw.) neu auch für medizinisches Personal, Geistliche, Anwältinnen und Anwälte und Journalistinnen und Journalisten anordnen können. Das wäre eine gravierende Aufweichung der Bestimmungen zum Schutz des Berufsgeheimnisses, insbesondere des Arztgeheimnisses, des Anwaltsgeheimnisses, des Beichtgeheimnisses und des Quellenschutzes im Journalismus, die für das Vertrauen in Beziehungen und in die Demokratie …</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr"/>
@@ -1687,7 +1698,7 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Explosion des coûts de la santé. A quand des mesures efficaces contre le gaspillage de l'argent des primes et pour freiner la hausse des coûts?</t>
+          <t>Explosion der Gesundheitskosten. Wann kommen endlich wirksame Massnahmen gegen die Verschwendung von Prämiengeldern und zur Dämpfung der Kosten?</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
@@ -1697,7 +1708,7 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Comme chaque année à cette même période, le jeu des caisses-maladie bat son plein. Les assureurs font parvenir de la publicité aux ménages par les canaux les plus divers : certaines caisses-maladie proposent des rabais et d'autres promettent des baisses de primes pour l'année prochaine, alors que l'association des assureurs-maladie Santésuisse a annoncé cet été une hausse générale des primes de l'ordre de 3 %. 1. Tout laisse à penser dans ce contexte que, comme lors des précédentes années électorales, les caisses-maladie puisent plus profondément dans leurs réserves qu'à l'ordinaire pour réduire au maximum la hausse des primes. Que pense l'Office fédéral de la santé publique de ce soupçon en sa qualité d'autorité d'approbation des primes ? Des réserves ont-elles dû ou devraient-elles être réduites pour obtenir des primes plus basses ? 2. La numérisation doit profiter au système de santé : elle améliore l'efficacité et la qualité des soins ainsi que l'information des assurés et des patients. Il y a un an, le Conseil fédéral a proposé le rejet d'une intervention qui visait à créer une base légale garantissant que la documentation médicale du patient soit tenue de manière struct…</t>
+          <t>[Official DE version; original is FR] TEXT: Wie jedes Jahr zur gleichen Zeit ist das Spiel der Krankenkassen in vollem Gange. Die Werbung der Versicherer erreicht die Haushalte auf den verschiedensten Kanälen. Einige Krankenkassen informieren über Rabatte, andere versprechen Prämienreduktionen für das nächste Jahr, während Santésuisse im Sommer einen allgemeinen Anstieg der Krankenkassenprämien von 3 Prozent ankündigte. 1. Das legt den Verdacht, dass die Krankenkassen - wie in früheren Wahljahren - stärker als üblich auf die Reserven zurückgreifen müssen, um den Prämienanstieg zu minimieren. Wie stellt sich das Bundesamt für Gesundheit (BAG) als zuständige Prämiengenehmigungsbehörde zu diesem Verdacht? Mussten und müssten Reserven für günstigere Prämien abgebaut werden? 2. Die Digitalisierung muss auch im Gesundheitswesen positiv genutzt werden. Sie bringt Effizienzsteigerungen, mehr Qualität und mehr Informationen für Versicherte und Patienten. Vor einem Jahr hat der Bundesrat einen Vorstoss abgelehnt, der eine gesetzliche Grundlage verlangte, um sicherzustellen, dass sowohl die medizinischen Patientendokumentationen elektronisch strukturiert geführt wie auch für die Behandlung relevante Dokumente wie Rezepte, Überwei…</t>
         </is>
       </c>
       <c r="F45" s="5" t="inlineStr"/>
@@ -1737,7 +1748,7 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Coronavirus. Un Parlement virtuel serait-il une solution?</t>
+          <t>E-Parlament als eine mögliche Antwort auf Notsituationen wie infolge des Coronavirus</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
@@ -1747,8 +1758,9 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Alors que la Suisse risque elle aussi de se retrouver dans une situation de crise en raison de la propagation du coronavirus, je prie le Bureau de répondre aux questions suivantes : 1. Comment le bon fonctionnement des institutions peut-il être garanti en période de crise ? 2. Le Parlement aurait-il la possibilité à l'heure actuelle de prendre des décisions dans une situation de crise sans avoir à se réunir physiquement ? 3. Dans la négative, quelles bases légales ou constitutionnelles faudrait-il créer pour que le travail parlementaire puisse avoir lieu en situation de crise sans que le Parlement ait à se réunir physiquement ? 4. Quelles mesures techniques y aurait-il lieu de prendre (identités électroniques, logiciels permettant de conduire de bout en bout les processus politiques, etc.) pour que le travail parlementaire puisse être effectué en ligne avec toute l'efficacité et toute la sécurité requises ?
-REASONING: Les défis que les parlementaires de milice doivent relever dans leur quotidien parlementaire sont déjà nombreux. Mais dans des situations de crise telles que celle qui s'annonce avec l'épidémie de coronavirus, il est encore plus difficile de garantir le bon dér…</t>
+          <t>[Official DE version; original is FR] TEXT: Vor dem Hintergrund einer drohenden Notstandssituation aufgrund des Coronavirus, auch in der Schweiz, bitte ich das Büro um Beantwortung nachstehender Fragen: 1. Wie kann das gute Funktionieren der Institutionen in Notsituationen aufrechterhalten werden? 2. Wäre es im Grundsatz möglich, in Notsituationen parlamentarische Entscheide zu fällen, ohne dass das Parlament sich physisch im Parlament versammelt? 3. Falls das heute nicht möglich ist, welche verfassungsrechtlichen/gesetzgeberischen Grundlagen müssen geschaffen werden, damit der Ratsbetrieb in Krisensituationen auch ohne physische Anwesenheit aufrechterhalten werden kann? 4. Welche technischen Voraussetzungen (elektronische Identitäten, Programme zur Abwicklung von politischen Prozessen etc.) wären erforderlich, um den Ratsbetrieb online sicher und effizient zu gestalten?
+REASONING: Die Herausforderungen, die der Ratsbetrieb an die Parlamentarierinnen und Parlamentarier im Milizsystem im Alltag stellen, sind bereits gross. Im Zuge von Notsituationen wie z.B. in der aktuellen Ausgangslage mit dem Coronavirus, ist die Sicherstellung des formalen Ratsbetriebs und der materiellen Ratsarbeit zusätzlich erschwert.
+ANSWER: 1…</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr"/>
@@ -1763,7 +1775,7 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Servizio d'appoggio dell'esercito a favore delle autorità civili nell'ambito dei provvedimenti per combattere la pandemia di Covid-19</t>
+          <t>Assistenzdienst der Armee zugunsten der zivilen Behörden im Rahmen der Massnahmen zur Bekämpfung der Covid-19-Pandemie</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
@@ -1771,7 +1783,11 @@
           <t>open</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr"/>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Official DE version; original is IT] </t>
+        </is>
+      </c>
       <c r="F48" s="5" t="inlineStr"/>
       <c r="G48" s="5" t="inlineStr"/>
     </row>
@@ -1784,7 +1800,7 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Lancement de DigiFLUX - Comment le point 5.4 sur la surface traitée de l'annexe 3b de l'OSIAgr va-t-il être mis en œuvre concrètement ?</t>
+          <t>Einführung DigiFLUX - Wie wird die Verordnung (SR 919.117.71) bezüglich Flächenangabe (Anhang 3b - 5.4) genau umgesetzt?</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
@@ -1794,8 +1810,8 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Conformément à l'annexe 3b, point 5.4, de l'ordonnance sur les systèmes d'information dans le domaine de l'agriculture (OSIAgr), seule la surface traitée doit être indiquée dans le cadre des recensements sur l'utilisation des produits phytosanitaires. Or, cette surface devra apparemment être géoréférencée à la parcelle près sur la plateforme DigiFLUX. Que prévoit-on concrètement pour la mise en œuvre ?
-ANSWER: La déclaration de l’utilisation de produits phytosanitaires concerne les données relatives à toute utilisation professionnelle, donc les données de chaque cas concret de traitement (art. 16a, al. 1, let. e, OSIAgr). Toute application de produits phytosanitaires doit ainsi faire l’objet d’une saisie, incluant les données suivantes : désignation du produit phytosanitaire, date de l’utilisation, quantité utilisée, surface traitée, plante cultivée ou objet traité (art. 16a, al. 2, et annexe 3b, OSIAgr, ainsi qu’art. 62, al. 1bis, OPPh). L’obligation légale d’informer porte sur le lieu et le type de culture où des produits phytosanitaires ont été utilisés. Dans le cadre du relevé des données pertinentes pour les paiements directs, les exploitations sont déjà tenues, dans le…</t>
+          <t>[Official DE version; original is FR] TEXT: Die Verordnung über Informationssysteme im Bereich der Landwirtschaft erklärt im Anhang 3b Absatz 5.4, dass für die Erhebungen im Bereich Verwendung vom Pflanzenschutzmitteln allein die behandelte Fläche angegeben werden muss. Nun soll diese jedoch auf der Plattform DigiFLUX georeferenziert/parzellengenau erfasst werden. Wie genau ist hierbei die Umsetzung geplant?
+ANSWER: Die Antwort des Bundesrates existiert nur in französischer Sprache. (Bitte wechseln Sie auf der Homepage oben rechts die Sprache)</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr"/>
@@ -1835,7 +1851,7 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Lettre d’EMS-Chemie Holding AG au conseiller national Fabian Molina. Protéger la liberté d’expression des élus fédéraux</t>
+          <t>Schutz der parlamentarischen Redefreiheit – Schreiben der EMS-Chemie Holding AG an Nationalrat Fabian Molina</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
@@ -1845,7 +1861,7 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Le conseiller national Fabian Molina a reçu le 24 septembre 2026 une lettre recommandée d’EMS-Chemie Holding AG se référant expressément à sa question 26.7751, adressée au Conseil fédéral durant l’heure des questions. L'entreprise lui reproche d’avoir sciemment diffusé, avec sa question consultable publiquement au Conseil fédéral, des allégations fausses, dénigrantes et diffamatoires et le somme de s’abstenir à l’avenir de faire de telles déclarations, sous peine de poursuites dans le cas contraire. Ce ne sont donc pas des propos qui auraient été tenus en dehors des séances des Chambres fédérales qui sont ici attaqués, mais bien le droit de poser des questions dont jouissent les conseillers nationaux. Dans sa question, le conseiller Fabian Molina mentionne une enquête du journal en ligne « Republik » et demande au Conseil fédéral de procéder à des vérifications. Or c’est précisément la fonction de l’heure des questions. Je prie donc le Bureau de bien vouloir répondre aux questions suivantes : Le Bureau confirme-t-il que la question 26.7751, en tant que déclaration faite devant un conseil, jouit de l’immunité absolue en vertu de l’art. 162, al. 1, de la Constitution fédérale e…</t>
+          <t>[Official DE version; original is FR] TEXT: Am 24. September 2026 hat die EMS-Chemie Holding AG Nationalrat Fabian Molina ein eingeschriebenes Schreiben zukommen lassen, das sich ausdrücklich auf dessen Frage 26.7751 an den Bundesrat in der Fragestunde bezieht. Das Unternehmen wirft ihm darin vor, mittels seiner «öffentlich einsehbaren Frage an den Bundesrat» wissentlich falsche, verunglimpfende und rufschädigende Behauptungen zu verbreiten, fordert ihn auf, «derartige Aussagen künftig zu unterlassen», und droht andernfalls damit, ihn «hierfür haftbar zu machen». Gegenstand der Beanstandung ist damit nicht eine Äusserung ausserhalb des Ratsbetriebs, sondern die Ausübung des parlamentarischen Fragerechts selbst. Nationalrat Molina hat in seiner Frage eine publizierte Recherche des Onlinemagazins «Republik» referiert und den Bundesrat um Prüfung gebeten. Genau dafür ist das Instrument der Fragestunde da. Ich bitte das Büro deshalb, um die Beantwortung folgender Fragen: Bestätigt das Büro, dass die Frage 26.7751 als Äusserung in einem Rat unter die absolute Immunität gemäss Art. 162 Abs. 1 BV und Art. 16 ParlG fällt und Nationalrat Molina dafür weder straf- noch zivilrechtlich belangt werden kann? Und teilt das Büro die A…</t>
         </is>
       </c>
       <c r="F51" s="5" t="inlineStr"/>
@@ -1860,7 +1876,7 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Rapporto sulla politica di sicurezza 2021</t>
+          <t>Sicherheitspolitischer Bericht 2021</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
@@ -1868,7 +1884,11 @@
           <t>open</t>
         </is>
       </c>
-      <c r="E52" s="2" t="inlineStr"/>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Official DE version; original is IT] </t>
+        </is>
+      </c>
       <c r="F52" s="5" t="inlineStr"/>
       <c r="G52" s="5" t="inlineStr"/>
     </row>
@@ -1881,7 +1901,7 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Proteggere la nostra democrazia dalle influenze estere</t>
+          <t>Unsere Demokratie vor ausländischen Einflüssen schützen</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
@@ -1891,8 +1911,8 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>TEXT: La legge sui diritti politici è modificata di modo che le liberalità monetarie e non monetarie provenienti dall’estero comportino sanzioni penali dissuasive (in particolare sotto forma di multe) nei confronti degli attori politici che le accettano intenzionalmente.
-REASONING: I nostri diritti popolari (iniziativa, referendum, petizione) e le nostre elezioni sono un punto di forza del nostro sistema politico. La democrazia semi-diretta rende la Svizzera un luogo di dibattito in cui il Popolo dispone di ampi poteri, una caratteristica di cui essere orgogliosi. La Svizzera è uno Stato sovrano e indipendente. La formazione dell’opinione dell’elettorato non deve essere influenzata da finanziamenti esteri che seguono altre agende politiche. Attualmente la legge federale sui diritti politici (LDP) impedisce agli attori politici (partiti, persone fisiche o giuridiche e società di persone che conducono una campagna in vista di un’elezione nelle Camere federali o di una votazione federale) di accettare finanziamenti provenienti dall’estero. Una liberalità (non) monetaria deve essere restituita a chi l’ha versata. Se la restituzione non è possibile o non è ragionevolmente esigibile, la…</t>
+          <t>[Official DE version; original is IT] TEXT: Der Bundesrat wird beauftragt, das Bundesgesetz über die politischen Rechte (BPR) dahingehend zu ändern, dass die vorsätzliche Annahme monetärer und nichtmonetärer Zuwendungen aus dem Ausland durch politische Akteurinnen und Akteure abschreckende strafrechtliche Sanktionen nach sich zieht (namentlich in Form von Bussen).
+REASONING: Unsere Volksrechte (Initiative, Referendum, Petition) und auch unsere Wahlen sind eine Stärke unseres politischen Systems. Die halbdirekte Demokratie macht unser Land zu einem Ort der Debatte, an dem das Volk weitgehend mitbestimmen kann. Darauf können wir stolz sein. Die Schweiz ist ein souveräner und unabhängiger Staat. Die Meinungsbildung der Wählerschaft darf nicht von Finanzierungen ausländischer Akteure beeinflusst werden, die andere politische Agenden verfolgen. Das geltende BPR verbietet politischen Akteurinnen und Akteuren (Parteien, natürliche und juristische Personen sowie Personengesellschaften, die im Hinblick auf eine Wahl in die eidgenössischen Räte oder auf eine eidgenössische Abstimmung Kampagnen führen), Geld aus dem Ausland anzunehmen. Wer eine (nicht-)monetäre Zuwendung erhält, muss diese zurückerstatten. Ist eine Rückerstattun…</t>
         </is>
       </c>
       <c r="F53" s="5" t="inlineStr"/>
@@ -1907,7 +1927,7 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Sicurezza dei prodotti: rafforzare la libera concorrenza tra attori svizzeri e stranieri del commercio online</t>
+          <t>Produktesicherheit. Förderung eines freien Wettbewerbs zwischen schweizerischen und ausländischen Online-Händlern</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
@@ -1917,7 +1937,7 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>TEXT: I recenti avvenimenti che hanno coinvolto la piattaforma di e-commerce cinese Shein nella vicina Francia sollevano interrogativi legittimi anche in Svizzera. Se si considera che ogni giorno arrivano a Zurigo circa 500 000 pacchi dalla Cina, risulta difficile stabilire se i controlli di qualità imposti ai prodotti svizzeri siano applicati nella stessa misura anche ai prodotti cinesi. Alcuni degli articoli in vendita sulle piattaforme cinesi stanno suscitando un certo scalpore. Su Temu, ad esempio, è possibile trovare puntatori laser il cui uso è severamente vietato in Svizzera a causa dei possibili rischi per la vista associati. Inoltre, un recente studio dimostra che l'86 per cento dei giocattoli disponibili sulle principali piattaforme di commercio online straniere (Temu, Shein, Amazon) sono considerati pericolosi per la salute dei bambini. Come giustifica il Consiglio federale il fatto che i prodotti in vendita sulle piattaforme cinesi non soddisfino gli stessi requisiti di qualità dei prodotti svizzeri, soprattutto in termini di sicurezza? Come intende obbligare le piattaforme straniere a rispettare le stesse regole imposte ai loro concorrenti svizzeri? Quali misure intend…</t>
+          <t>[Official DE version; original is IT] TEXT: Die jüngsten Vorfälle rund um den chinesischen Online-Händler Shein in Frankreich werfen auch in der Schweiz berechtigte Fragen auf. Angesichts der Tatsache, dass täglich rund 500 000 Pakete aus China in Zürich eintreffen, ist es fraglich, ob die Qualitätskontrollen, die für schweizerische Produkte durchgeführt werden, in gleichem Umfang auch für chinesische Produkte durchgeführt werden. Einige Produkte, die im chinesischen Online-Handel erhältlich sind, erfordern ein Eingreifen. So sind bei Temu beispielsweise Laserpointer erhältlich, deren Nutzung in der Schweiz aufgrund der damit verbundenen Gefahr für die Augen strikt verboten ist. Zudem zeigt eine aktuelle Studie, dass 86 Prozent der Kinderspielzeuge, die bei grossen ausländischen Online-Händlern (Temu, Shein, Amazon) erhältlich sind, als gesundheitsgefährdend für Kinder eingestuft werden. Wie rechtfertigt der Bundesrat, dass Produkte aus dem chinesischen Online-Handel nicht denselben Qualitätsanforderungen unterliegen wie schweizerische Produkte, insbesondere in Bezug auf die Sicherheit? Mit welchen Mitteln will der Bundesrat ausländische Online-Händler dazu bringen, die gleichen Vorschriften wie ihre schweizerischen Ko…</t>
         </is>
       </c>
       <c r="F54" s="5" t="inlineStr"/>
@@ -1932,7 +1952,7 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Una strategia svizzera per i semiconduttori (Swiss Chip Strategy)</t>
+          <t>Eine schweizerische Halbleiterstrategie (Swiss Chip Strategy)</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
@@ -1942,8 +1962,8 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Il settore dei semiconduttori riveste un ruolo strategico ed è sempre più importante nelle filiere produttive mondiali e svizzere, in un contesto sociale che si sta digitalizzando rapidamente. In Svizzera operano aziende strategiche a livello mondiale: forniscono tecnologie per la fabbricazione di semiconduttori. Il rischio di concorrenza sleale – soprattutto da parte dell’UE e degli USA – mediante programmi di sovvenzione per diverse decine di miliardi, che prevedono condizioni relative alla localizzazione produttiva, è elevato. Sono aspetti che mettono a rischio il sistema d’innovazione e produzione svizzero e le nostre industrie. Invito il Consiglio federale ad analizzare la situazione, in particolare sotto il profilo dei rischi e delle opportunità legati agli sviluppi più recenti, valutando anche i rischi dovuti al decoupling delle filiere produttive. Chiedo al Consiglio federale di riferire al Parlamento mediante un rapporto con proposte finalizzate in particolare a migliorare le condizioni quadro per le imprese interessate e favorire l’innovazione (Swiss Chip Strategy).
-REASONING: In una società digitalizzata come la nostra, i componenti al silicio sono onnipresenti: c…</t>
+          <t>[Official DE version; original is IT] TEXT: Die Halbleiterindustrie ist von strategischer Bedeutung und wird in einer sich schnell digitalisierenden Gesellschaft in den globalen und nationalen Produktionsketten immer wichtiger. Die Schweiz verfügt über weltweit tätige Schlüsselunternehmen, die Technologie für die Herstellung von Halbleitern liefern. Die Gefahr eines unfairen Wettbewerbs ist hoch, insbesondere weil die EU und die USA Subventionsprogramme in zweistelliger Milliardenhöhe vorsehen, die Auflagen für die lokale Produktion enthalten. Dies gefährdet den Innovations- und Produktionsstandort Schweiz und seine Industrie. Ich ersuche den Bundesrat, die Situation zu analysieren, insbesondere die Risiken und Chancen der jüngsten Entwicklungen. Zudem soll er das Risiko analysieren, das mit dem «Decoupling» der Produktionsketten verbunden ist. Es soll dem Parlament einen Bericht vorgelegt werden, der Vorschläge enthält, insbesondere zur Verbesserung der Rahmenbedingungen für die betroffenen Unternehmen und zur Förderung der Innovation (Swiss Chip Strategy).
+REASONING: In unserer digitalisierten Gesellschaft sind Siliziumkomponenten allgegenwärtig: Computer, Telefone, Sensoren, Autos, Maschinen, Energie, Raumfahrt, Rü…</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr"/>
@@ -1984,7 +2004,7 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Pour une meilleure reconnaissance des cancers professionnels</t>
+          <t>Mehr Anerkennung für berufsbedingte Krebserkrankungen</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
@@ -1994,8 +2014,8 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Je prie le Conseil fédéral de répondre aux questions suivantes : - Quel est le coût économique des cancers professionnels en Suisse ? - Quelles mesures prévoit le Conseil fédéral pour lutter contre la sous-reconnaissance de cancers professionnels ? - Quelles mesures prévoit le Conseil fédéral pour clarifier les critères de reconnaissance des cancers professionnels ? - Quelles mesures prévoit le Conseil fédéral pour inciter les soignants à mieux s'impliquer dans les démarches de déclaration des cancers professionnels ? - Quels moyens la SUVA prévoit-elle d'utiliser pour rechercher activement une composante professionnelle chez les patients suisses atteints de cancers professionnels ?
-REASONING: En Suisse, entre 350 à 1850 cancers professionnels ne seraient pas reconnus par l'assurance accident comme maladie professionnelle (Krief et al 2022). Selon les auteurs de l'étude, le problème ne réside pas tant dans la reconnaissance du cancer comme maladie professionnelle par l'assureur accident mais d'avantage dans l'identification des cas potentiels par les soignants et le déclenchement du processus de déclaration. En effet, les cancers professionnels présentant une longe latence d…</t>
+          <t>[Official DE version; original is FR] TEXT: Ich bitte den Bundesrat um Antwort auf folgende Fragen: - Wie hoch sind die Kosten, die der Wirtschaft in der Schweiz durch berufsbedingte Krebserkrankungen entstehen? - Welche Massnahmen plant der Bundesrat zur Bekämpfung der mangelhaften Anerkennung berufsbedingter Krebserkrankungen? - Welche Massnahmen plant der Bundesrat, um die Kriterien für die Anerkennung berufsbedingter Krebserkrankungen zu klären? - Welche Massnahmen sieht der Bundesrat vor, um die Pflegekräfte zu motivieren, sich besser an der Meldung berufsbedingter Krebserkrankungen zu beteiligen? - Welche Mittel will die Suva einsetzen, um bei Schweizer Patientinnen und Patienten, die berufsbedingt an Krebs erkrankt sind, nach einer beruflichen Komponente zu suchen?
+REASONING: In der Schweiz werden offenbar zwischen 350 und 1850 Fälle berufsbedingter Krebserkrankungen von der Unfallversicherung nicht als Berufskrankheit anerkannt (Krief et al. 2022). Den Autorinnen und Autoren der Studie zufolge liegt das Problem nicht so sehr in der Anerkennung von Krebs als Berufskrankheit durch den Unfallversicherer, sondern vielmehr in der Identifizierung potenzieller Fälle durch das Pflegepersonal und der Auslösung des Meld…</t>
         </is>
       </c>
       <c r="F57" s="5" t="inlineStr"/>
@@ -2010,7 +2030,7 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Comment faire face à la pénurie de médicaments?</t>
+          <t>Wie kann der Medikamentenknappheit begegnet werden?</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
@@ -2020,7 +2040,7 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Depuis plusieurs mois, certains médicaments d’usage courant ne sont plus disponibles dans nos pharmacies (pansements gastriques, comprimés contre les refroidissements, sprays nasaux, sirops contre la toux,...). Certains de ces médicaments ont des alternatives qui ne sont parfois pas remboursées par l’AOS. Quelles mesures le Conseil fédéral développe-t-il en ce moment face à cette pénurie? Compte-t-il notamment élargir la liste des spécialités?</t>
+          <t>[Official DE version; original is FR] TEXT: Seit mehreren Monaten sind einige gebräuchliche Medikamente in unseren Apotheken nicht mehr erhältlich (Medikamente gegen Magenbeschwerden, Tabletten gegen Erkältungen, Nasensprays, Hustensirup usw.). Für einige dieser Medikamente gibt es Alternativen, die jedoch nicht immer von der Krankenversicherung bezahlt werden. Welche Massnahmen arbeitet der Bundesrat momentan aus, um der Knappheit zu begegnen? Beabsichtigt er namentlich auch, die Spezialitätenliste zu erweitern?</t>
         </is>
       </c>
       <c r="F58" s="5" t="inlineStr"/>
@@ -2035,7 +2055,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Mestieri del futuro. Sostegno pubblico alla riconversione professionale</t>
+          <t>Berufe der Zukunft. Öffentliche Unterstützung für die berufliche Umschulung</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
@@ -2045,8 +2065,8 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Il Consiglio federale è incaricato di illustrare in un rapporto in che modo è possibile creare nuove prospettive professionali in settori in fase di cambiamento strutturale tramite un maggiore investimento pubblico nella formazione continua e professionale.
-REASONING: La transizione ecologica causa la perdita di posti di lavoro in alcuni settori dell'industria e dei servizi, ma allo stesso tempo permette lo sviluppo di nuove professioni legate a un'economia più sostenibile: questo è quanto emerge da un rapporto realizzato dall'Organizzazione Internazionale del Lavoro (OIL) nel 2018. Lo studio mostra un fattore essenziale affinché la transizione ecologica possa portare alla creazione di posti di lavoro: una riconversione professionale efficace e mirata. È dunque necessario disporre di un piano a lungo termine e di dati chiari per identificare le esigenze attuali e future dell'economia e fornire i mezzi per formare (nuovamente) milioni di persone. Tuttavia in Svizzera manca un piano di questo genere. Allo stesso tempo, la digitalizzazione sta allargando il divario tra l'economia di produzione di ieri e l'economia digitale di domani, lasciando indietro dei dipendenti a causa de…</t>
+          <t>[Official DE version; original is IT] TEXT: Der Bundesrat wird beauftragt, in einem Bericht aufzuzeigen, wie mithilfe eines verstärkten Engagements der öffentlichen Hand zugunsten der Weiterbildung und der Berufsbildung neue berufliche Perspektiven in Brachen, die einen Strukturwandel durchlaufen, geschaffen werden können.
+REASONING: Der ökologische Wandel bringt Arbeitsplätze in bestimmten Industrie- und Dienstleistungssektoren zum Verschwinden, ermöglicht aber gleichzeitig auch den Aufschwung neuer Berufe in Zusammenhang mit einer nachhaltigeren Wirtschaft. Dies geht aus dem Bericht der Internationalen Arbeitsorganisation (IAO) aus dem Jahr 2018 hervor. Diese Studie zeigt einen Faktor auf, der sehr wichtig ist, damit der ökologische Wandel zur Schaffung von Arbeitsplätzen führt: eine wirksame und gezielte berufliche Umschulung. Dazu sind ein langfristiger Plan und eindeutige Zahlen notwendig, um so die aktuellen und künftigen Bedürfnisse der Wirtschaft zu bestimmen und die Mittel für die (Um-)Schulung von Tausenden von Arbeitnehmerinnen und Arbeitnehmern zu planen. In der Schweiz besteht kein solcher Plan. Gleichzeitig vertieft die Digitalisierung den Graben zwischen der alten Produktionswirtschaft und der neuen dig…</t>
         </is>
       </c>
       <c r="F59" s="5" t="inlineStr"/>
@@ -2061,7 +2081,7 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Sanzioni contro le opposizioni abusive nel settore edilizio</t>
+          <t>Missbräuchliche Baueinsprachen sanktionieren</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
@@ -2071,8 +2091,8 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Il Consiglio federale è incaricato di creare una base legale che permetta di sanzionare le opposizioni abusive. In futuro, coloro che presenteranno opposizione senza un interesse da proteggere o con intenzioni palesemente abusive dovranno poter essere obbligati ad assumere i costi ed eventualmente a risarcire i danni. Il Consiglio federale è tenuto a illustrare come disposizioni in tal senso possano essere disciplinate nella legge sulla pianificazione del territorio (LPT) o in altre leggi federali pertinenti senza compromettere i legittimi diritti di partecipazione della popolazione.
-REASONING: La situazione giuridica attuale consente di protrarre per anni o addirittura di impedire del tutto progetti di costruzione e sviluppo presentando opposizioni di modesta entità o pretestuose. Uno studio recentemente pubblicato dall’Ufficio federale delle abitazioni (UFAB) e dall’Ufficio federale dello sviluppo territoriale (ARE) dimostra chiaramente che le opposizioni sono il motivo più frequente alla base di ritardi e annullamenti di progetti di costruzione di abitazioni. Ne conseguono un aumento dei costi di costruzione, un calo dell’attività edilizia e un’accentuazione della penuria…</t>
+          <t>[Official DE version; original is IT] TEXT: Der Bundesrat wird beauftragt, eine gesetzliche Grundlage zu schaffen, um missbräuchliche Einsprachen zu sanktionieren. Einsprecherinnen und Einsprecher, die ohne schutzwürdiges Interesse oder in erkennbar rechtsmissbräuchlicher Absicht handeln, sollen künftig zu einer Kostenübernahme und gegebenenfalls zu Schadenersatzleistungen verpflichtet werden können. Der Bundesrat soll darlegen, wie entsprechende Regelungen im Raumplanungsgesetz (RPG) oder in anderen einschlägigen Bundesgesetzen verankert werden können, ohne die legitimen Mitwirkungsrechte der Bevölkerung zu beeinträchtigen.
+REASONING: Die heutige Rechtslage ermöglicht es, Bau- und Entwicklungsprojekte bereits durch geringfügige oder vorgeschobene Einsprachen über Jahre hinweg zu verzögern oder gänzlich zu verhindern. Eine kürzlich veröffentlichte Studie des Bundesamts für Wohnungswesen (BWO) und des Bundesamts für Raumentwicklung (ARE) zeigt deutlich, dass Einsprachen der häufigste Grund für Verzögerungen und Projektabbrüchen im Wohnungsbau sind. Die Folgen sind höhere Baukosten, eine abnehmende Bautätigkeit und eine Verschärfung der Wohnungsknappheit. Besonders problematisch ist, dass Einsprachen nicht selten wenige…</t>
         </is>
       </c>
       <c r="F60" s="5" t="inlineStr"/>
@@ -2097,7 +2117,7 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>OTHER (Texte déposé): Le Conseil fédéral est chargé de présenter un rapport analysant : a) les principaux impacts prévisibles de la révolution quantique sur les grands domaines de l'action publique, ainsi que les principales mesures à envisager ; b) le positionnement stratégique de la Suisse pour saisir les opportunités et limiter les risques ; c) les conditions-cadres nécessaires pour développer, attirer et retenir en Suisse les entreprises et les talents à la pointe de ces technologies. Il formulera des propositions pour atteindre ces objectifs et posera les bases d'une stratégie nationale quantique.
+          <t>[Original FR; no official DE version] OTHER (Texte déposé): Le Conseil fédéral est chargé de présenter un rapport analysant : a) les principaux impacts prévisibles de la révolution quantique sur les grands domaines de l'action publique, ainsi que les principales mesures à envisager ; b) le positionnement stratégique de la Suisse pour saisir les opportunités et limiter les risques ; c) les conditions-cadres nécessaires pour développer, attirer et retenir en Suisse les entreprises et les talents à la pointe de ces technologies. Il formulera des propositions pour atteindre ces objectifs et posera les bases d'une stratégie nationale quantique.
 OTHER (Développement): La révolution quantique n'est plus une hypothèse de long terme. En 2026, les ordinateurs quantiques sortent des laboratoires et commencent à surpasser les systèmes classiques dans des domaines stratégiques. Leur convergence avec l'intelligence artificielle ouvre une ère de puissance de calcul sans précédent, avec des implications majeures, notamment pour la sécurité, la santé, la finance, la formation et la souveraineté numérique. La Suisse a eu la sagesse d'anticiper ces ruptures. La Swiss Quantum Initiative, dotée de 82,1 millions de francs pour la période F…</t>
         </is>
       </c>
@@ -2113,7 +2133,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Protezione contro le molestie sessuali nelle commesse pubbliche</t>
+          <t>Schutz vor sexueller Belästigung bei öffentlichen Aufträgen</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
@@ -2123,8 +2143,8 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Il Consiglio federale è incaricato di modificare l'articolo 4 capoverso 1 dell'ordinanza sugli appalti pubblici (OAPub) come segue: Art. 4 Condizioni di partecipazione e criteri di idoneità 1 Il committente può delegare l'esecuzione dei controlli relativi alla parità salariale e a una protezione efficace contro il mobbing e le molestie sessuali segnatamente all'Ufficio federale per l'uguaglianza fra donna e uomo (UFU). L'UFU definisce i dettagli dei controlli in una direttiva. Il committente può trasmettere all'UFU l'autodichiarazione degli offerenti relativa all'osservanza della parità salariale. Una minoranza della Commissione (Friedli Esther, Aeschi Thomas, Amaudruz, Burgherr, Dettling, Feller, Gössi, Regazzi, Ritter, Schneeberger, Steinemann, Tuena) propone di respingere la mozione.
-REASONING: Attualmente la legislazione sugli appalti pubblici prevede che le commesse siano aggiudicate soltanto alle imprese che osservano le "disposizioni in materia di tutela dei lavoratori e delle condizioni di lavoro". Ciò presuppone anche il rispetto della legge sul lavoro, in particolare la tutela dell'integrità personale dei lavoratori che vi è disciplinata e che si riferisce anche ai…</t>
+          <t>[Official DE version; original is IT] TEXT: Der Bundesrat wird beauftragt, Artikel 4 Absatz 1 der Verordnung über das öffentliche Beschaffungswesen wie folgt anzupassen: Art. 4 Teilnahmebedingungen und Eignungskriterien 1 Die Auftraggeberin kann die Durchführung der Kontrollen in Bezug auf die Lohngleichheit sowie einen wirksamen Schutz vor Mobbing und sexueller Belästigung insbesondere dem Eidgenössischen Büro für die Gleichstellung von Frau und Mann (EBG) übertragen. Das EBG bestimmt die Einzelheiten seiner Kontrollen in einer Richtlinie. Die Auftraggeberin kann die Selbstdeklarationen der Anbieterinnen über die Einhaltung der Lohngleichheit dem EBG weiterleiten. Eine Minderheit der Kommission (Friedli Esther, Aeschi Thomas, Amaudruz, Burgherr, Dettling, Feller, Gössi, Regazzi, Ritter, Schneeberger, Steinemann, Tuena) beantragt, die Motion abzulehnen.
+REASONING: Heute ist im öffentlichen Beschaffungswesen geregelt, dass Aufträge nur an Unternehmen vergeben werden, die die "massgeblichen Arbeitsschutzbestimmungen und Arbeitsbedingungen" einhalten. Das beinhaltet auch die Erfüllung des Arbeitsgesetzes, insbesondere dem darin geregelten Schutz der persönlichen Integrität der Arbeitnehmenden. Damit sind auch Fälle von M…</t>
         </is>
       </c>
       <c r="F62" s="5" t="inlineStr"/>
@@ -2139,7 +2159,7 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Legge sul sostegno alla banda larga (LSBL)</t>
+          <t>Breitbandfördergesetz (BBFG)</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
@@ -2147,7 +2167,11 @@
           <t>open</t>
         </is>
       </c>
-      <c r="E63" s="2" t="inlineStr"/>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Official DE version; original is IT] </t>
+        </is>
+      </c>
       <c r="F63" s="5" t="inlineStr"/>
       <c r="G63" s="5" t="inlineStr"/>
     </row>
@@ -2186,7 +2210,7 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Promuovere e non ostacolare la ricerca e la sperimentazione clinica con dispositivi medici non commerciali. Gli emolumenti e gli oneri vanno urgentemente adeguati</t>
+          <t>Forschung und klinische Versuche mit nichtkommerziellen Medizinprodukten fördern und nicht behindern. Anpassung von Gebühren und Auflagen ist dringend</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
@@ -2196,8 +2220,8 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Il Consiglio federale è incaricato di adeguare le disposizioni di esecuzione della legge sugli agenti terapeutici (in particolare gli art. 4-9), al fine di consentire lo sviluppo della ricerca clinica non commerciale. I gravosi oneri previsti da tali disposizioni e le tariffe fissate per la sperimentazione clinica devono essere oggetto di un adeguamento in modo da non ostacolare l'avvio di importanti progetti di ricerca.
-REASONING: La ricerca clinica non commerciale è importante per l'innovazione. Dall'introduzione della nuova ordinanza sugli emolumenti essa ne è risultata fortemente ostacolata o resa quasi impossibile. Soprattutto in ambito universitario i progetti condotti da giovani ricercatori non sono quasi più possibili in quanto non finanziabili. Il diritto vigente e l'ordinanza sugli emolumenti ostacolano fortemente la ricerca non operando alcuna distinzione tra ricerca commerciale e non commerciale. Tutto ciò non è nell'interesse né della ricerca di base, né delle istituzioni, né dei pazienti e rappresenta un ostacolo in particolare per i giovani ricercatori. L'equiparazione della ricerca non commerciale a quella delle imprese commerciali private non è nel nostro in…</t>
+          <t>[Official DE version; original is IT] TEXT: Der Bundesrat wird beauftragt, das Ausführungsrecht zum Heilmittelgesetz, insbesondere zu den Artikeln 4 bis 9, anzupassen, damit die nicht-kommerzielle klinische Forschung gefördert wird. Die aufwändigen Auflagen und die Tarife für die nicht-kommerziellen Versuche sind anzupassen, damit sie nicht weiter dazu führen, dass wichtige Forschungsvorhaben gar nicht erst gestartet werden können.
+REASONING: Die nicht-kommerzielle klinische Forschung ist wichtig für die Innovation. Seit der Einführung der neuen Gebührenverordnung wird sie stark behindert resp. fast verunmöglicht. Gerade im universitären Umfeld sind Forschungsprojekte junger Forschender kaum mehr möglich, weil sie schlicht nicht finanzierbar sind. Das geltende Recht und die Gebührenverordnung unterscheiden nicht zwischen kommerzieller und nicht-kommerzieller Forschung und schränken die Forschung wesentlich ein. Das ist nicht im Sinne der Grundlagenforschung, der Institutionen und der Patientinnen und Patienten, denn dadurch werden insbesondere junge Forschende eingeschränkt. Die Gleichbehandlung nicht-kommerzieller Forschung mit der Forschung privater kommerzieller Unternehmen ist nicht in unserem Interesse. Bereits d…</t>
         </is>
       </c>
       <c r="F65" s="5" t="inlineStr"/>
@@ -2212,7 +2236,7 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Soumettre la Société suisse de radiodiffusion et télévision au Contrôle fédéral des finances</t>
+          <t>Die Schweizerische Radio- und Fernsehgesellschaft der Eidgenössischen Finanzkontrolle unterstellen</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
@@ -2222,8 +2246,8 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>TEXT: La loi fédérale sur la radio et la télévision est modifiée de sorte que la Société suisse de radiodiffusion et télévision (SSR) soit soumise au Contrôle fédéral des finances (CDF) en tant qu'autorité de surveillance financière.
-REASONING: La SSR remplit un mandat de prestations global au niveau national et au niveau des régions linguistiques. Elle est principalement financée par la redevance, dont le montant total s'élève à plus d'un milliard de francs. Compte tenu de cette somme, du volume important des activités, du très grand intérêt public et des discussions politiques en cours, la SSR devrait être soumise à la surveillance financière du CDF, comme les autres organisations auxquelles la Confédération confie l'exécution de tâches publiques (voir art. 8, al. 1, let. d, LCF). En tant qu'organe indépendant, le CDF devrait pouvoir examiner les finances de la SSR du point de vue des risques et de la gestion des activités, en étroite collaboration avec les autres autorités et organes chargés de contrôler la société. L'autonomie dans la conception et la gestion des programmes de radio et de télévision, garantie par l'art. 93, al. 3, Cst., resterait opposable au CDF. D'autres org…</t>
+          <t>[Official DE version; original is FR] TEXT: Das Bundesgesetz über Radio und Fernsehen wird dahingehend geändert, dass die Schweizerische Radio- und Fernsehgesellschaft (SRG) der Finanzaufsicht durch die Eidgenössische Finanzkontrolle (EFK) unterstellt wird.
+REASONING: Die SRG hat auf nationaler und sprachregionaler Ebene einen grundlegenden Leistungsauftrag zu erfüllen. Sie wird grösstenteils über die Abgabe für Radio und Fernsehen in der Höhe von über 1 Milliarde Franken finanziert. Angesichts dieser finanziellen Bedeutung, der umfangreichen Tätigkeiten, des grossen öffentlichen Interesses und der aktuellen politischen Diskussionen sollte auch die SRG der Finanzaufsicht durch die EFK unterstellt werden, wie andere Organisationen auch, denen der Bund die Erfüllung einer öffentlichen Aufgabe übertragen hat (vgl. Art. 8 Abs. 1 Bst. d des Finanzkontrollgesetzes, FKG). Die EFK hätte als unabhängige Stelle die Möglichkeit, bei der SRG risikobasierte und mit der Geschäftsführung zusammenhängende Finanzaufsichtsprüfungen durchzuführen, dies in enger Abstimmung mit Kontrolltätigkeiten anderer Behörden und Organe. Die Autonomie von Radio und Fernsehen in der Programmplanung und -gestaltung, wie sie von Artikel 93 Absatz 3 der …</t>
         </is>
       </c>
       <c r="F66" s="5" t="inlineStr"/>
@@ -2238,7 +2262,7 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Promozione dell'home office e libertà imprenditoriale</t>
+          <t>Förderung von Homeoffice und unternehmerische Freiheit</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
@@ -2248,7 +2272,7 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>TEXT: In seguito alla crisi del coronavirus si sono nuovamente levate delle voci in campo politico che auspicano una maggiore promozione dell'home office (lavoro a domicilio, telelavoro ecc.). A questo proposito, chiedo al Consiglio federale di rispondere alle seguenti domande: 1. Quale promozione diretta e indiretta dell'home office esiste da parte della Confederazione? 2. Quali sono le basi legali di questa promozione? 3. Su quali disposizioni di diritto del lavoro si basa in generale l'home office? 4. Cosa pensa il Consiglio federale del fatto che il sostegno statale dell'home office influenza in modo molto forte la cultura d'impresa? 5. Quali effetti produce la sentenza del Tribunale federale che impone al datore di lavoro di farsi carico di parte della pigione in caso di home office? 6. Come si pone tale promozione rispetto alla libertà economica e imprenditoriale? C'è un possibile conflitto con la libertà economica sancita dalla Costituzione? 7. Come giudica il Consiglio federale il fatto che nel caso dell'home office gli scambi e le relazioni personali e sociali diventano meno importanti? 8. Esistono studi o indizi riscontrati nella prassi, soprattutto relativi al periodo de…</t>
+          <t>[Official DE version; original is IT] TEXT: Infolge der Corona-Krise werden politisch wieder Stimmen laut, die eine verstärkte Förderung des Homeoffice (Heimarbeit, Telearbeit, etc.) installieren möchten. Ich bitte den Bundesrat diesbezüglich folgende Fragen zu beantworten: 1. Welche direkte und indirekte Förderung gibt es von Seiten des Bundes für Homeoffice? 2. Welches sind die gesetzlichen Grundlagen für diese Förderung? 3. Welches sind generell die arbeitsrechtlichen Grundlagen von Homeoffice? 4. Wie stellt sich der Bundesrat zur Tatsache, dass eine staatliche Förderung von Homeoffice eine sehr starke Einflussnahme auf die Unternehmenskultur darstellt? 5. Welche Auswirkungen hat das Bundesgerichtsurteil, welches verlangt, dass der Arbeitgeber einen Teil der Wohnungsmiete bei Homeoffice übernehmen muss, auf das Thema? 6. Wie steht eine diesbezügliche Förderung zur wirtschaftlichen und unternehmerischen Freiheit? Gibt es einen möglichen Konflikt mit der in der Verfassung verbrieften Wirtschaftsfreiheit? 7. Wie gewichtet der Bundesrat den Umstand, dass bei Homeoffice der persönliche und soziale Austausch und Beziehungen weniger wichtig werden? 8. Gibt es Studien oder Hinweise aus der Praxis, insbesondere aus der Coron…</t>
         </is>
       </c>
       <c r="F67" s="5" t="inlineStr"/>
@@ -2263,7 +2287,7 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Le prospettive dell'AVS erano errate. Lo sono anche quelle dell'AI?</t>
+          <t>Die AHV-Perspektiven waren falsch. Stimmen auch die IV-Zahlen nicht?</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
@@ -2273,8 +2297,8 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Chiedo al Consiglio federale di rispondere alle seguenti domande: È noto che sono stati commessi errori nelle previsioni dell’AVS. Sono stati commessi gli stessi errori anche per quanto riguarda le cifre dell’AI? I debiti dell’AI gravano l’AVS. L’Amministrazione federale ha ripetutamente comunicato a partire da quando l’AI potrà ridurre il debito nel bilancio dell’AVS. Quali dati sono stati comunicati dal 2012? Quali motivazioni sono state addotte dal 2012 per la costante posticipazione di questo momento? Quando saranno presentate al Parlamento nuove basi di dati che contengano anche la crescita delle nuove rendite e la diminuzione dei tassi di uscita, fattori menzionati da Compenswiss? Il Consiglio federale come garantisce una maggiore attendibilità delle previsioni dell’AI affinché si disponga di basi sicure per una prossima revisione dell’AI?
-REASONING: Il 18 febbraio 2025 il Consiglio di amministrazione di Compenswiss ha comunicato che «[a]nche per il fondo AI le prospettive finanziarie sono peggiorate a causa dell’aumento delle nuove rendite e della diminuzione dei tassi di uscita» e avvertito che «[d]ata la sua situazione finanziaria, è improbabile che l’AI possa ridur…</t>
+          <t>[Official DE version; original is IT] TEXT: Ich ersuche den Bundesrat um die Beantwortung folgender Fragen: Die Fehler bei den AHV-Prognosen sind bekannt. Sind auch bei den IV-Zahlen die gleichen Fehler gemacht worden? Die IV-Schulden belasten die AHV. Es wurde von der Bundesverwaltung immer wieder mitgeteilt, ab wann die IV die Schulden in der Bilanz der AHV abbauen kann. Welche Daten wurden seit dem Jahr 2012 kommuniziert? Welche Begründungen wurden seit 2012 für den ständig nach hinten verschobenen 'Turnaround' genannt? Wann werden dem Parlament neue Datengrundlagen vorgelegt, welche auch die von Compenswiss erwähnten Faktoren Neurentenzuwachs und geringere Abgangsquoten beinhalten? Wie sichert der Bundesrat eine erhöhte Verlässlichkeit der IV-Prognosen, damit für eine kommende IV-Revision gesicherte Grundlagen bestehen?
+REASONING: Am 18. Februar 2025 hat der Verwaltungsrat von Compenswiss informiert: "Auch für den IV-Fonds haben sich die finanziellen Perspektiven aufgrund des Anstiegs der Neurenten sowie geringerer Abgangsquoten verschlechtert." Zudem warnt Compenswiss: "Aufgrund ihrer finanziellen Lage ist es eher unwahrscheinlich, dass die IV in absehbarer Zeit in der Lage sein wird, diese Schuld aus eigener Kra…</t>
         </is>
       </c>
       <c r="F68" s="5" t="inlineStr"/>
@@ -2310,7 +2334,7 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Excursions en famille dans le jet du Conseil fédéral</t>
+          <t>Familienausflüge mit dem Bundesratsjet</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
@@ -2320,8 +2344,8 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Début mai, le CN Nussbaumer et le CE Herzog se sont rendus à Rome avec le Service de transport aérien de la Confédération (STAC). Selon les médias, les fils de Mme Herzog ont voyagé avec eux dans le jet du Conseil fédéral. - Quelle était leur fonction dans la délégation officielle pour la prestation de serment de la Garde suisse ? - Si les fils ne faisaient pas partie de la délégation officielle, depuis quand le LTDB peut-il être réservé pour des "excursions familiales" ?
-ANSWER: Selon le ch. 2.10 de la Directive de la Délégation administrative du 13 mai 2022 concernant les activités internationales des délégations parlementaires permanentes et des délégations parlementaires non permanentes, l’Assemblée fédérale peut, une fois par année, prendre en charge les frais d’une personne accompagnante dans le cadre d’un voyage officiel des présidents ou présidentes des conseils à l’étranger. Par le passé, une personne accompagnait les présidents ou présidentes des conseils lors d’un « voyage présidentiel » officiel à l’étranger, qui avait lieu une fois par année, sans délégation du Parlement, généralement dans une destination lointaine. Cette forme de « voyage présidentiel » a été a…</t>
+          <t>[Official DE version; original is FR] TEXT: Anfang Mai reisten NR Nussbaumer und SR Herzog mit dem Lufttransportdienst des Bundes (LTDB) nach Rom. Medienberichten zufolge reisten auch die Söhne von Frau Herzog im Bundesratsjet mit. - Welche Aufgabe hatten sie in der offiziellen Delegation zur Vereidigung der Schweizergarde? - Wenn die Söhne nicht zur offiziellen Delegation gehörten: Seit wann kann der LTDB für «Familienausflüge» genutzt werden?
+ANSWER: Gemäss Punkt 2.10. der Weisung der Verwaltungsdelegation vom 13. Mai 2022 betreffend internationale Aktivitäten von ständigen und nicht ständigen parlamentarischen Delegationen kann die Bundesversammlung einmal pro Jahr bei einer offiziellen Auslandreise einer Ratspräsidentin oder eines Ratspräsidenten die Reisekosten einer privaten Begleitperson übernehmen. Früher wurden Ratspräsidentinnen und Ratspräsidenten bei den einmal jährlich stattfindenden offiziellen «Präsidialreisen» ohne Parlamentsdelegation von einer privaten Begleitperson ins Ausland begleitet, meistens zu einer fernen Destination. Die Präsidialreisen wurden in diesem Format abgeschafft. Seit einigen Jahren hat es sich etabliert, dass Privatpersonen Ratspräsidentinnen und Ratspräsidenten begleiten, die an …</t>
         </is>
       </c>
       <c r="F70" s="5" t="inlineStr"/>
@@ -2336,7 +2360,7 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Garantire il diritto alle prestazioni complementari alle persone che nell'infanzia hanno subito collocamenti coatti e alle persone internate sulla base di una decisione amministrativa</t>
+          <t>Gewährleistung der Ergänzungsleistungen ehemaliger Verdingkinder und Administrativversorgter</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
@@ -2346,7 +2370,7 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>TEXT: La Commissione della sicurezza sociale e della sanità del Consiglio degli Stati decide di elaborare un progetto volto a garantire che la riparazione morale dovuta alle persone che nell'infanzia hanno subito collocamenti coatti e alle persone internate sulla base di una decisione amministrativa non pregiudichi il loro diritto alle prestazioni complementari. A tale scopo occorre stralciare la parte finale della lettera c dell'articolo 4 capoverso 6 della legge federale sulle misure coercitive a scopo assistenziale e i collocamenti extrafamiliari prima del 1981 (LMCCE).</t>
+          <t>[Official DE version; original is IT] TEXT: Die Kommission für soziale Sicherheit und Gesundheit des Ständerates beschliesst, eine Vorlage auszuarbeiten, um sicherzustellen, dass die Genugtuung für ehemalige Verdingkinder und Administrativversorgte den Anspruch auf Ergänzungsleistungen nicht beeinträchtigt. Dafür ist die Streichung des letzten Satzteils von Artikel 4 Absatz 6 Buchstabe c des Bundesgesetzes über die Aufarbeitung der fürsorgerischen Zwangsmassnahmen und Fremdplatzierungen vor 1981 (AFZFG) erforderlich.</t>
         </is>
       </c>
       <c r="F71" s="5" t="inlineStr"/>
@@ -2361,7 +2385,7 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Crisi dovuta al coronavirus. Soluzione globale per stabilizzare le finanze federali e le opere sociali</t>
+          <t>Umfassende Lösung zur Bewältigung der Corona-Krise. Stabilisierung des Bundeshaushaltes und der Sozialwerke</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
@@ -2371,8 +2395,8 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Il Consiglio federale è incaricato di presentare al Parlamento una soluzione globale che indichi come le prestazioni straordinarie fornite dalla Confederazione durante la crisi dovuta al coronavirus e le future perdite fiscali provocate dalla suddetta crisi debbano essere contabilizzate nei conti della Confederazione. Il Consiglio federale deve indicare in particolare come nei prossimi 6-8 anni dovrà essere coperto il disavanzo del fondo di compensazione stimato in 40 miliardi di franchi, come dovranno essere compensate le perdite fiscali stimate in cinque miliardi di franchi l'anno e quali misure dovranno essere adottate per consolidare le assicurazioni sociali del 1° e del 2° pilastro. Condizione: il freno all'indebitamento, che ha dato prova di efficacia, non deve essere allentato.
-REASONING: Il Consiglio federale ha espresso grande preoccupazione per le conseguenze economiche della crisi dovuta al coronavirus. Le prestazioni straordinarie graveranno le casse della Confederazione per un importo di circa 40 miliardi di franchi, che sarà trasferito a un fondo di compensazione. La base legale prevede che tale fondo sia riequilibrato entro 6-8 anni. Inoltre, a causa dell'immi…</t>
+          <t>[Official DE version; original is IT] TEXT: Der Bundesrat wird beauftragt, dem Parlament eine umfassende Lösung zu präsentieren, wie die ausserordentlichen Leistungen des Bundes während der Coronakrise und die kommenden Steuerausfälle durch die Coronakrise in den Rechnungen des Bundes behandelt werden sollen. Insbesondere muss der Bundesrat aufzuzeigen, wie das geschätzte 40 Milliarden Franken-Loch im Ausgleichfonds in den kommenden 6-8 Jahren abgebaut, wie die Steuerausfälle von geschätzt 5 Milliarden Franken pro Jahr aufgefangen und welche Massnahmen für die Sicherung der Sozialwerke 1. und 2. Säule gesichert werden sollen. Auflage: Die erfolgreiche Schuldenbremse darf nicht ausgeschalten werden.
+REASONING: Der Bundesrat hat sich zu den wirtschaftlichen Folgen aufgrund der Coronakrise sehr besorgt geäussert. So soll die Bundeskasse durch ausserordentliche Leistungen mit rund 40 Milliarden Franken belastet werden, welche in einen Ausgleichsfond transferiert werden. Dieser Ausgleichfond ist gemäss gesetzlichen Grundlagen in 6- 8 Jahren wieder auszugleichen. Zudem erwartet der Bundesrat aufgrund der bevorstehenden Rezession Steuerausfälle von rund 5 Milliarden Franken pro Jahr. Der Ausgleichsbeitrag sowie die Steueraus…</t>
         </is>
       </c>
       <c r="F72" s="5" t="inlineStr"/>
@@ -2397,7 +2421,7 @@
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>OTHER (Texte déposé): Le Conseil fédéral est prié de répondre aux questions suivantes : - Le Conseil fédéral dispose-t-il d'éléments concrets démontrant que la mise en œuvre de TARDOC améliore la situation des médecins de premier recours ? - Dans le cas contraire, quelles sont les raisons pour lesquelles les promesses de revalorisation ne se concrétisent pas ? - Quelles mesures concrètes le Conseil fédéral compte-t-il prendre pour mettre en œuvre ma motion 22.4357, validée par les Chambres fédérales et visant à revaloriser la médecine de premier recours, en respectant la neutralité des coûts ? - Quand soumettra-t-il au Parlement des propositions concrètes en la matière ?
+          <t>[Original FR; no official DE version] OTHER (Texte déposé): Le Conseil fédéral est prié de répondre aux questions suivantes : - Le Conseil fédéral dispose-t-il d'éléments concrets démontrant que la mise en œuvre de TARDOC améliore la situation des médecins de premier recours ? - Dans le cas contraire, quelles sont les raisons pour lesquelles les promesses de revalorisation ne se concrétisent pas ? - Quelles mesures concrètes le Conseil fédéral compte-t-il prendre pour mettre en œuvre ma motion 22.4357, validée par les Chambres fédérales et visant à revaloriser la médecine de premier recours, en respectant la neutralité des coûts ? - Quand soumettra-t-il au Parlement des propositions concrètes en la matière ?
 OTHER (Développement): Depuis des années, le Conseil fédéral et le Parlement entendent revaloriser la médecine de premier recours, notamment en rééquilibrant les tarifs par rapport à ceux de la médecine à forte composante médico-technique. Les acteurs du TARDOC avaient annoncé que le nouveau tarif contribuerait à cet objectif, ce que prévoyait aussi le Conseil fédéral. Or, les promesses des acteurs du TARDOC semblent aujourd'hui s’évanouir : les données provisoires ne laissent pas entrevoir de réelle amélioration …</t>
         </is>
       </c>
@@ -2439,7 +2463,7 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>Rapporto sulle condizioni di lavoro e gli infortuni nel settore delle economie di piattaforma</t>
+          <t>Bericht über Arbeitsbedingungen und Arbeitsunfälle in der Plattformwirtschaft</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
@@ -2449,8 +2473,8 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Il Consiglio federale è incaricato di redigere un rapporto sulle condizioni di lavoro e gli infortuni nel settore dell'economia di piattaforma che includa in particolare le statistiche sul numero e il tipo di infortuni nonché le relative cause.
-REASONING: Da vari anni diverse società di piattaforma hanno stabilito le loro attività in Svizzera e altre sono state fondate nel nostro Paese. Negli ultimi anni sono stati presentati anche vari interventi parlamentari riguardanti lo status da accordare ad autisti, fattorini e corrieri che lavorano per queste piattaforme. Vi sono però pochi studi o statistiche sulle condizioni di lavoro e, in particolare, sul numero e il tipo di infortuni del personale impiegato in questo settore in Svizzera. Il Consiglio federale è pertanto incaricato di redigere un rapporto su questa categoria di dipendenti, dato che è in questo modo che vanno ormai definiti. Il rapporto deve in particolare indicare il numero e il tipo di infortuni che riguardano i lavoratori di queste piattaforme e, per quanto possibile, le relative cause. Una ricerca francese del 2021 ha dimostrato che il 25 per cento delle 517 persone interpellate aveva già subito un infortunio …</t>
+          <t>[Official DE version; original is IT] TEXT: Der Bundesrat wird beauftragt, einen Bericht über die Arbeitsbedingungen und Arbeitsunfälle in der Plattformwirtschaft zu erstellen. Der Bericht muss insbesondere Auskunft über die Anzahl und die Art der Arbeitsunfälle sowie über deren Ursachen geben.
+REASONING: Seit einigen Jahren sind verschiedene Firmen der Plattformwirtschaft auch in der Schweiz aktiv; andere solche Firmen wurden hier gegründet. Zur Frage, welchen Status die Personen haben, die für diese Plattformen als Fahrerin oder als Kurier arbeiten, wurden mehrere parlamentarische Vorstösse eingereicht. Es gibt jedoch nur wenige Studien und Statistiken zu den Arbeitsbedingungen der Arbeitnehmenden in diesem Sektor in der Schweiz, insbesondere zur Anzahl und zur Art der Arbeitsunfälle. Ich beauftrage den Bundesrat, einen Bericht über diese Kategorie von Arbeitnehmenden, als die sie neu gelten, zu erstellen. Der Bericht muss Angaben enthalten über die Anzahl und die Art der Arbeitsunfälle, zu denen es in diesem Sektor kommt, und soweit möglich über deren Ursachen. Eine französische Studie aus dem Jahr 2021 ergab, dass 25 Prozent der 517 Befragten bereits einen Unfall erlitten hatten und dass diese Unfälle in den meist…</t>
         </is>
       </c>
       <c r="F75" s="5" t="inlineStr"/>
@@ -2465,7 +2489,7 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Réglementation des plateformes numériques</t>
+          <t>Regulierung der Plattformen</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
@@ -2475,7 +2499,7 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Le 16 avril 2025, le Conseil fédéral a annoncé qu’il repoussait la publication du message relatif à la réglementation des plateformes numériques. Depuis, presque six mois se sont écoulés et, apparemment, ce report n’a eu aucun effet positif sur le montant des droits de douane imposés sur les produits suisses par les États-Unis. Quand le Conseil fédéral prévoit-il de transmettre le message au Parlement ?</t>
+          <t>[Official DE version; original is FR] TEXT: Am 16. April 2025 beschloss der Bundesrat, die Botschaft zur Regulierung der Plattformen zu verschieben. In der Zwischenzeit ist fast ein halbes Jahr vergangen, offensichtlich hatte die Verschiebung keine positiven Auswirkungen auf die Höhe der Zölle in den USA für Schweizer Produkte. Wann wird der Bundesrat die Botschaft zu Handen des Parlaments verabschieden?</t>
         </is>
       </c>
       <c r="F76" s="5" t="inlineStr"/>
@@ -2490,7 +2514,7 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>Covid-19. Cherche-t-on à justifier des restrictions drastiques au moyen d'arguments infondés?</t>
+          <t>Covid-19. Harte Einschränkungen mit Kaffeesatzlesen rechtfertigen?</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
@@ -2500,8 +2524,8 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Au motif que des mesures très restrictives auraient permis d'éviter le pire en Suisse romande, campagne est faite en vue d'un confinement partiel. N'est-il pas malhonnête, d'un point de vue scientifique, d'affirmer qu'un effet épidémiologique peut être attribué au confinement, alors que - selon la Task Force COVID-19 de la Confédération - les différences de taux de contamination entre la Suisse alémanique et la Suisse romande ne s'expliquent pas ?
-ANSWER: La réponse du Conseil fédéral n'existe qu'en allemand. (Veuillez changer la langue en haut à droite de la page d'accueil)</t>
+          <t>[Official DE version; original is FR] TEXT: Mit dem Argument, harte Massnahmen hätten in der Westschweiz Schlimmeres verhindert, wird nun Werbung für den Teil-Lockdown gemacht. Ist es aus wissenschaftlicher Sicht nicht unredlich zu behaupten, man könne einem Lockdown eine epidemiologische Wirkung zuschreiben, obwohl gemäss COVID Taskforce des Bundes die unterschiedlichen Infektionszahlen der Deutsch- und Westschweiz gar nicht erklärbar sind?
+ANSWER: Die Westschweizer Kantone haben früher als die restliche Schweiz einen raschen Anstieg der Fallzahlen erlebt. In der Folge haben viele von ihnen einschränkende Massnahmen eingeführt. In den letzten Wochen verzeichnete die gesamte Westschweiz stark sinkende Fallzahlen. Diese Tendenz ist in den Deutschschweizer Kantonen mit wenig restriktiven Massnahmen nicht festzustellen. Im Gegenteil ist in einigen Regionen sogar ein beunruhigender Wiederanstieg der Infektionszahlen festzustellen. Das Bild ist klar: Die von den stark betroffenen Kantonen ergriffenen Massnahmen haben gewirkt und dort zu einer Trendwende geführt. Kantone mit steigenden oder über längere Zeit auf hohem Niveau stagnierenden Fallzahlen sind deshalb angehalten, ebenfalls weitergehende Massnahmen zu ergreifen.</t>
         </is>
       </c>
       <c r="F77" s="5" t="inlineStr"/>
@@ -2516,7 +2540,7 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Per una stampa scritta indipendente è necessario adeguare gli importi del sostegno indiretto</t>
+          <t>Für eine unabhängige Presse sind die Beträge zur indirekten Förderung anzupassen</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
@@ -2526,7 +2550,7 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>TEXT: La legge sulle poste (LPO) e le altre pertinenti disposizioni legali devono essere modificate in modo tale da permettere uno sviluppo del sostegno indiretto alla stampa. Si tratta in particolare di modificare l'articolo 16 capoverso 7 LPO affinché il sostegno indiretto alla stampa destinato ai giornali e ai periodici (...) sia aumentato di 15 milioni di franchi all'anno, così da garantire delle riduzioni per la distribuzione postale per un periodo transitorio di sette anni. Parallelamente, il sostegno alla stampa associativa e delle fondazioni deve essere aumentato di 10 milioni di franchi all'anno, pure per una durata limitata. Occorre inoltre introdurre, mediante una modifica della legge sulle poste, un sostegno alla distribuzione mattutina esclusivamente nei giorni feriali, di cui potranno beneficiare i titoli della stampa locale e regionale che hanno una tiratura media, autenticata da un organo di controllo indipendente e riconosciuto, compresa tra i 1000 e i 40 000 esemplari per edizione e che non appartengono a una rete di edizioni locali con propria testata la cui tiratura media complessiva supera i 100 000 esemplari per edizione. Per questa seconda parte, la Confedera…</t>
+          <t>[Official DE version; original is IT] TEXT: Das Postgesetz und die anderen einschlägigen Bestimmungen werden so geändert, dass die indirekte Presseförderung ausgebaut werden kann. Zu ändern ist insbesondere Artikel 16 Absatz 7, und zwar so, dass die indirekte Presseförderung für Zeitungen und Zeitschriften um jährlich 15 Millionen erhöht wird, damit die Ermässigung für deren Zustellung während einer Übergangsphase von sieben Jahren garantiert ist. Gleichzeitig und ebenfalls für einen befristeten Zeitraum ist der Beitrag an die Ermässigung der Zustellung von Mitgliedschafts- und Stiftungspresse um jährlich 10 Millionen zu erhöhen. Zudem soll im Postgesetz neu ein Beitrag an die Frühzustellung während der Woche eingeführt werden. Davon profitieren sollen die Lokal- und Regionalzeitungen mit einer von einem anerkannten unabhängigen Kontrollorgan bestätigten Auflage von zwischen 1000 und 40 000 Exemplaren. Wenn sie zu einem Kopfblatt gehören, darf dessen mittlere Auflage nicht über 100 000 Exemplaren liegen. Dafür stellt der Bund jährlich 30 Millionen Franken bereit. Für die Umsetzung dieser Massnahme sind der Artikel 19a der Fassung des Postgesetzes nach Bundesgesetz vom 18. Juli 2021 über ein Massnahmenpaket zugunsten de…</t>
         </is>
       </c>
       <c r="F78" s="5" t="inlineStr"/>
@@ -2566,7 +2590,7 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Rete nazionale di dati sicura. Credito d’impegno</t>
+          <t>Nationales sicheres Datenverbundsystem. Verpflichtungskredit</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
@@ -2574,7 +2598,11 @@
           <t>open</t>
         </is>
       </c>
-      <c r="E80" s="2" t="inlineStr"/>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Official DE version; original is IT] </t>
+        </is>
+      </c>
       <c r="F80" s="5" t="inlineStr"/>
       <c r="G80" s="5" t="inlineStr"/>
     </row>
@@ -2612,7 +2640,7 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Mesures contre l'immigration illégale (8/9). Systématiser l'échange des données concernant les immigrés illégaux</t>
+          <t>Massnahmen gegen die illegale Migration (8/9). Datenaustausch bei illegalen Migranten systematisieren</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
@@ -2622,8 +2650,8 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Afin de lutter durablement contre l'immigration illégale en Suisse et si possible d'y mettre un terme, il faut que l'échange des données sur les personnes concernées entre les cantons, les communes, les autorités sociales, les caisses-maladie, l'AVS, l'AI et d'autres assurances sociales devienne systématique. Il s'agit d'échanger et de comparer toutes les données relatives au statut de séjour, au lieu de domicile, à la couverture d'assurance, aux paiements des primes, aux réductions de primes, aux prestations des caisses-maladie, à l'AVS, à l'AI et à d'autres assurances sociales.
-REASONING: En fonction des estimations et des sources d'information, jusqu'à 100 000 immigrés illégaux - banalement appelés " sans-papiers " - seraient en Suisse. Afin de réduire l'attrait de notre pays à cet égard, il importe que ces personnes puissent être identifiées et renvoyées grâce à un échange systématique des données les concernant. Selon le rapport du Conseil fédéral " Pour un examen global de la problématique des sans-papiers " en réponse au postulat de la Commission des institutions politiques du Conseil national du 12 avril 2018 (18.3381), les assurances et les caisses-maladie surtout n…</t>
+          <t>[Official DE version; original is FR] TEXT: Um die Anwesenheit von illegalen Migranten in der Schweiz dauerhaft zu bekämpfen und wenn immer möglich dauerhaft zu unterbinden, muss der Datenaustausch zwischen Kantonen, Gemeinden, Sozialbehörden, Krankenkassen, AHV, IV und weiteren Sozialversicherungen bezogen auf diese Personen systematisiert werden. So sind sämtliche relevanten Daten von illegalen Migranten betreffend Aufenthaltsstatus, Wohnort, Versicherungsstatus, Prämienzahlungen, Prämienvergünstigungen, Versicherungsleistungen von Krankenkassen, AHV, IV und weiteren Sozialversicherungen auszutauschen und abzugleichen.
+REASONING: Je nach Schätzung und Quelle halten sich in der Schweiz bis zu hunderttausend illegale Migranten auf - verharmlosend auch "Sans-Papiers" genannt. Um die Attraktivität der Schweiz für illegale Migranten zu reduzieren, ist es wichtig, dass diese durch einen systematischen Austausch ermittelt und ausgeschafft werden. Gemäss dem Bericht "Gesamthafte Prüfung der Problematik der Sans-Papiers" des Bundesrats, in Erfüllung des Postulats der Staatspolitischen Kommission des Nationalrats vom 12. April 2018 (18.3381), sind heute vor allem Versicherungen und Krankenkassen nicht in der Lage, den Aufenth…</t>
         </is>
       </c>
       <c r="F82" s="5" t="inlineStr"/>
@@ -2664,7 +2692,7 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>Transport pour handicapés. Un chaînon manquant dans l'offre de mobilité</t>
+          <t>Behindertenfahrdienste. Ein fehlendes Glied in der Mobilitätskette</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
@@ -2674,8 +2702,8 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Le Conseil fédéral est chargé de produire un rapport, en complément de celui demandé par le postulat 20.3874, sur la manière dont les lacunes de l'offre en transport pour handicapés devraient être comblées de sorte que le droit à la mobilité personnelle inscrit dans la Convention relative aux droits des personnes handicapées soit honoré et mis en oeuvre dans le droit suisse (" Les États Parties prennent des mesures efficaces pour assurer la mobilité personnelle des personnes handicapées, dans la plus grande autonomie possible "). Il ciblera en particulier le cas des personnes qui, en raison de leur handicap, ne peuvent pas, ou que de manière limitée, utiliser les transports publics. L'avis et les expériences des handicapés qui doivent recourir à ces transports seront pris en compte.
-REASONING: Pour s'intégrer à la société de manière autonome et en bénéficiant des mêmes droits que les autres personnes, les handicapés doivent pouvoir se déplacer. En raison de leur handicap, certaines personnes ne peuvent pas, ou que de manière limitée, utiliser les transports publics. Une offre adaptée est donc nécessaire si elles veulent effectuer leurs tâches quotidiennes, avoir accès aux lo…</t>
+          <t>[Official DE version; original is FR] TEXT: Der Bundesrat wird beauftragt, in einem Bericht in Ergänzung zum Postulat 20.3874 aufzuzeigen, wie die Angebotslücken der Behindertenfahrdienste ergänzt werden müssen, damit das in der UNO-Behindertenrechtskonvention (UNO-BRK) verankerte Recht von Menschen mit Behinderungen auf persönliche Mobilität mit grösstmöglicher Unabhängigkeit gesetzgeberisch umgesetzt und praktisch eingelöst werden kann. Dabei ist der Fokus auf Menschen zu richten, die öffentliche Verkehrsmittel behinderungsbedingt nicht oder nur eingeschränkt nutzen können. Bei der Erstellung des Berichtes sollen die Perspektiven und Erfahrungen von Menschen mit Behinderungen, die auf Behindertenfahrdienste angewiesen sind, berücksichtigt werden.
+REASONING: Mobilität ist eine Grundvoraussetzung für die selbstbestimmte und gleichberechtigte Teilhabe von Menschen mit Behinderungen am gesellschaftlichen Leben. Menschen, die öffentliche Verkehrsmittel behinderungsbedingt nicht oder nur eingeschränkt nutzen können, sind u.a. für Besorgungen des täglichen Lebens, für die Freizeitgestaltung, für die Arbeitstätigkeit und für die medizinische Versorgung auf Behindertentransportdienste angewiesen. Das Behindertengleichstellun…</t>
         </is>
       </c>
       <c r="F84" s="5" t="inlineStr"/>
@@ -2690,7 +2718,7 @@
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>Prix des médicaments : à quand la transparence sur les investissements des entreprises pharmaceutiques ?</t>
+          <t>Medikamentenpreise: Wann herrscht endlich Klarheit über die Investitionen der Pharmaunternehmen?</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
@@ -2700,7 +2728,7 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Les coûts de recherche et de développement sont un argument principal de l'industrie pharmaceutique pour justifier les prix élevés des médicaments, mais l'investissement réel n'est pas transmis aux autorités. Une nouvelle étude calcule des marges de profit de 40 à 90 %. Le Conseil fédéral prévoit-il des mesures pour que les entreprises pharmaceutiques soient enfin obligées de publier leurs investissements, comme c'est déjà le cas dans les pays voisins, par exemple en Italie ?</t>
+          <t>[Official DE version; original is FR] TEXT: Die Pharmaindustrie führt ihre Forschungs- und Entwicklungskosten als wichtiges Argument an, um ihre hohen Medikamentenpreise zu rechtfertigen. Ihre tatsächlichen Investitionen gibt sie den Behörden aber nicht bekannt. Eine neuere Studie geht von Gewinnmargen zwischen 40 und 90 Prozent aus. Sieht der Bundesrat Massnahmen vor, um die Pharmaunternehmen endlich zu verpflichten, nach dem Beispiel unserer Nachbarländer wie etwa Italien ihre Investitionen zu veröffentlichen?</t>
         </is>
       </c>
       <c r="F85" s="5" t="inlineStr"/>
@@ -2715,7 +2743,7 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Modification de l'article 697l du code des obligations et accès à liste des ayants droit économiques</t>
+          <t>Änderung von Artikel 697l des Obligationenrechts und Zugriff auf das Verzeichnis der wirtschaftlich berechtigten Personen</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
@@ -2725,7 +2753,7 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>TEXT: La loi fédérale du 21 juin 2019 sur la mise en oeuvre des recommandations du Forum mondial sur la transparence et l'échange de renseignements à des fins fiscales entraîne la disparition des actions au porteur. L'art. 697l du code des obligations (CO) est simplifié en conséquence et ne prévoit plus pour la société que l'obligation de tenir une liste des ayants droit économiques qui lui ont été annoncés. Conformément à la recommandation 24 du GAFI, l'art. 697l, al. 4, CO prévoit que la liste doit être tenue de manière à ce qu'il soit possible d'y accéder en tout temps en Suisse. La loi ne règle toutefois pas qui peut accéder à la liste. Le message concernant la mise en oeuvre des recommandations du GAFI révisées en 2012 n'imposait pas au conseil d'administration d'une société suisse de fournir de telles listes à l'autorité suisse compétente, sauf dans le cas de vérifications particulières dans le cadre d'une enquête du Ministère public, dans le domaine du droit pénal administratif ou en cas d'infraction fiscale (fraude fiscale). L'Administration fédérale des contributions (AFC) procède actuellement à la collecte systématique de ces listes par l'envoi d'une lettre-type aux contr…</t>
+          <t>[Official DE version; original is FR] TEXT: Das Bundesgesetz vom 21. Juni 2019 zur Umsetzung von Empfehlungen des Global Forum über Transparenz und Informationsaustausch für Steuerzwecke auferlegt die Abschaffung der Inhaberaktien. Darum wird Artikel 697l des Obligationenrechts (OR) weiter vereinfacht: Die Gesellschaft ist nur noch verpflichtet, ein Verzeichnis über die ihr gemeldeten wirtschaftlich berechtigten Personen zu führen. Dieses Verzeichnis bleibt aber sowohl für Aktionärinnen und Aktionäre als auch für Dritte unzugänglich. Um die Einhaltung der GAFI-Empfehlung Nr. 24 sicherzustellen, legt Artikel 697l Absatz 4 OR fest, dass das Verzeichnis so geführt werden muss, dass in der Schweiz jederzeit darauf zugegriffen werden kann. Das Gesetz schweigt sich aber darüber aus, wer das Recht auf Zugriff hat. In der Botschaft zum Bundesgesetz zur Umsetzung der 2012 revidierten GAFI-Empfehlungen war keine Verpflichtung des Verwaltungsrats schweizerischer Gesellschaften, den Behörden solche Verzeichnisse zu liefern, vorgesehen. Eine Ausnahme wurde gemacht für besondere Abklärungen der Staatsanwaltschaft im Zusammenhang mit einem verwaltungsstrafrechtlichen oder einem steuerrechtlichen Verfahren (Steuerhinterziehung). Die E…</t>
         </is>
       </c>
       <c r="F86" s="5" t="inlineStr"/>
@@ -2740,7 +2768,7 @@
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>Budget 2026. Supplément II</t>
+          <t>Voranschlag 2026. Nachtrag II</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
@@ -2748,7 +2776,11 @@
           <t>open</t>
         </is>
       </c>
-      <c r="E87" s="2" t="inlineStr"/>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Official DE version; original is FR] </t>
+        </is>
+      </c>
       <c r="F87" s="5" t="inlineStr"/>
       <c r="G87" s="5" t="inlineStr"/>
     </row>
@@ -2761,7 +2793,7 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Pour le versement mensuel de l'allocation pour perte de gain revenant aux personnes servant dans l'armée suisse</t>
+          <t>Monatliche Auszahlung der Erwerbsausfallentschädigung für Dienstleistende in der Schweizer Armee</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
@@ -2771,8 +2803,8 @@
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>TEXT: L'allocation pour perte de gain qui revient aux personnes sans activité lucrative, aux indépendants et aux personnes en formation qui effectuent une école de recrues, un service sans interruption ou un service de changement de grade n'est versée pour la première fois qu'au terme de plus d'un mois, parfois même après deux mois, voire trois. Cette situation peut plonger les personnes concernées ou leurs parents dans des difficultés financières. - Le Conseil fédéral est-il disposé à faire en sorte que les allocations pour perte de gain soient versées ponctuellement, à savoir le 25 de chaque mois, comme c'est le cas pour le salaire des employés de la Confédération ? - Dans la négative, quelles sont les raisons qui s'y opposent ?
-ANSWER: La réponse du Conseil fédéral n'existe qu'en allemand. (Veuillez changer la langue en haut à droite de la page d'accueil)</t>
+          <t>[Official DE version; original is FR] TEXT: Die Erwerbsausfallentschädigung (EO) für nichterwerbstätige, selbstständigerwerbende oder in Ausbildung befindliche Dienstleistende in Rekrutenschulen, Durchdiener-Dienstleistungen oder Gradänderungsdiensten wird erstmals erst nach Ablauf von mehr als einem Monat ausbezahlt, teilweise sogar erst nach Ablauf von zwei oder gar drei Monaten. Dies kann die betroffenen Dienstleistenden beziehungsweise deren Eltern in finanzielle Schwierigkeiten bringen. - Ist der Bundesrat bereit, die EO jeweils pünktlich (wie den Lohn für die Angestellten des Bundes) auf den 25. des Monats auszuzahlen? - Falls nein, welche Gründe sprechen dagegen?
+ANSWER: Die EO-Entschädigung wird nach Erhalt der vollständigen EO-Anmeldung ausbezahlt. Die Ausgleichskassen sind angewiesen, zeitnah die eingehenden Anmeldungen zu bearbeiten und die Auszahlungen vorzunehmen. Sie haben zu diesem Zweck mehrere Zahlungsläufe im Monat. Verzögerungen können sich durch unvollständig respektive verspätet eingereichte Formulare oder allfällige Abklärungen ergeben. Nach vorliegenden Informationen handelt es sich nur um sehr vereinzelte Fälle. Der Bundesrat erachtet es daher nicht als notwendig, die Bestimmungen anzupassen.</t>
         </is>
       </c>
       <c r="F88" s="5" t="inlineStr"/>
@@ -2813,7 +2845,7 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Système satellite Composante Spatiale Optique. Arrangement cadre avec la France</t>
+          <t>Satellitensystem Composante Spatiale Optique. Rahmenvereinbarung mit Frankreich</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
@@ -2821,7 +2853,11 @@
           <t>open</t>
         </is>
       </c>
-      <c r="E90" s="2" t="inlineStr"/>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Official DE version; original is FR] </t>
+        </is>
+      </c>
       <c r="F90" s="5" t="inlineStr"/>
       <c r="G90" s="5" t="inlineStr"/>
     </row>
@@ -2834,7 +2870,7 @@
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>Augmenter les places d'accueil extrafamilial par un financement partagé afin que les parents puissent mieux concilier vie familiale et vie professionnelle</t>
+          <t>Vereinbarkeit von Familie und Beruf stärken. Mehr familienergänzende Betreuungsplätze dank geteilter Finanzierung</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
@@ -2844,8 +2880,8 @@
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>TEXT: Le Conseil fédéral est chargé d'examiner la possibilité d'élaborer un modèle permettant d'assurer le financement durable d'une offre adaptée de places d'accueil extrafamilial et extrascolaire. Ce modèle répondra aux exigences suivantes : tout enfant dont les parents ne peuvent assurer eux-mêmes la garde parce qu'ils exercent une activité professionnelle ou sont engagés dans une activité bénévole, une formation ou une formation continue attestées a droit à un bon de garde jusqu'à la fin de la scolarité obligatoire. Ce bon couvrira au moins les deux tiers du coût total d'une place d'accueil reconnue par le canton. Les communes, les cantons, la Confédération et les entreprises de plus de 250 employés veilleront conjointement à ce qu'un nombre suffisant de places d'accueil soient proposées et financées.
-REASONING: De nombreux parents ne peuvent pas se permettre de faire garder leur enfant par des professionnels. Les garderies, les groupes de jeux et l'accueil familial de jour sont financés en grande partie par les contributions parentales. Le montant payé par les parents pour la garderie représente environ deux tiers du coût total en moyenne, selon le canton et la commune. Cette…</t>
+          <t>[Official DE version; original is FR] TEXT: Der Bundesrat wird aufgefordert zu prüfen, ob zur dauerhaften Finanzierung eines bedarfsgerechten Angebotes an familien- und schulergänzenden Betreuungsplätzen ein Modell mit folgenden Eckpfeilern ausgearbeitet werden kann: Jedes Kind, dessen Eltern aufgrund von Erwerbsarbeit, ausgewiesener Freiwilligenarbeit oder Ausbildung/Weiterbildung die Betreuung nicht selber sicherstellen können, hat bis zum Ende der obligatorischen Schulzeit Anrecht auf einen Betreuungsgutschein. Dieser deckt mindestens zwei Drittel der Vollkosten eines vom Kanton anerkannten Betreuungsplatzes. Gemeinden, Kantone, Bund und Unternehmen mit mehr als 250 Angestellten sind gemeinsam verantwortlich, dass genügend Betreuungsplätze zur Verfügung stehen und finanziert werden.
+REASONING: Für viele Eltern ist es heute schlicht zu teuer, ihre Kinder professionell betreuen zu lassen. Kitas, Spielgruppen und Tagesfamilien werden mehrheitlich über Elternbeiträge finanziert - im Durchschnitt beträgt der Elternanteil bei den Kitas je nach Kanton und Gemeinde rund zwei Drittel der Vollkosten; bei den Spielgruppen sind es sogar bis zu drei Viertel. Eltern in der Schweiz zahlen deutlich mehr für einen Kita-Platz als in…</t>
         </is>
       </c>
       <c r="F91" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
Update adjudication rules and review process documentation; enhance partner review sheet with two-question rule and clarify reviewer role
</commit_message>
<xml_diff>
--- a/data/gold/for_partner/adjudication.xlsx
+++ b/data/gold/for_partner/adjudication.xlsx
@@ -73,7 +73,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -84,6 +84,10 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -466,28 +470,28 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>What this is: affairs where the evaluation found a disagreement (and some where it didn't), mixed and shuffled. You don't see who said what — no model answer, no PolitMonitor tag, no hint which side flagged it. Your answer decides the 'after review' numbers.</t>
+          <t>What this is: affairs where the evaluation found a disagreement (and some where it didn't), mixed and shuffled. You don't see who said what — no model answer, no PolitMonitor tag, no hint which side flagged it. Your answers decide the 'after review' numbers.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>For each row: read the title and the excerpt (open the link for the full text if needed). Decide by your definition (sheet 'Definition', = data/gold/digitalisation_definition.md as committed — the rules are fixed before you start). Choose yes / no / unsure. Add a short note if useful (e.g. 'only in passing').</t>
+          <t>Rule (fixed before you start): answer two questions per affair. 1) 'Digitale Technik drin?' — ja / nein / unsicher. 2) 'Ziel oder Nebensache?' — is the digital part the goal of the affair (Ziel) or a side matter (Nebensache)? The column 'Entscheid' fills itself: ja only if 1 = ja AND 2 = Ziel; nein if 1 = nein or 2 = Nebensache; otherwise unsicher. Question 2 can stay empty when 1 = nein.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>About 1 minute per affair. Yellow cells are for you. Please don't change the other columns or the row order.</t>
+          <t>Texts: federal affairs are shown in the official German version where the original is French or Italian (marked in the excerpt). Open the link for the full text. 'Belegsatz' (optional): the sentence that decided it.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>This file is a template until the evaluation run (S6) fills it.</t>
+          <t>About 1 minute per affair. Yellow cells are for you. Please don't change the other columns or the row order.</t>
         </is>
       </c>
     </row>
@@ -540,16 +544,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G301"/>
+  <dimension ref="A1:J91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="90" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="80" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -580,10 +587,25 @@
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t>Is this about digitalisation? (yes/no/unsure)</t>
+          <t>Digitale Technik drin?</t>
         </is>
       </c>
       <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Ziel oder Nebensache?</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Entscheid (auto)</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Belegsatz (optional)</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
@@ -613,6 +635,12 @@
       </c>
       <c r="F2" s="5" t="inlineStr"/>
       <c r="G2" s="5" t="inlineStr"/>
+      <c r="H2" s="6">
+        <f>IF(F2="nein","nein",IF(OR(F2="",G2=""),"",IF(AND(F2="ja",G2="Ziel"),"ja",IF(G2="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I2" s="7" t="inlineStr"/>
+      <c r="J2" s="5" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -638,6 +666,12 @@
       </c>
       <c r="F3" s="5" t="inlineStr"/>
       <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="6">
+        <f>IF(F3="nein","nein",IF(OR(F3="",G3=""),"",IF(AND(F3="ja",G3="Ziel"),"ja",IF(G3="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I3" s="7" t="inlineStr"/>
+      <c r="J3" s="5" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -663,6 +697,12 @@
       </c>
       <c r="F4" s="5" t="inlineStr"/>
       <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="6">
+        <f>IF(F4="nein","nein",IF(OR(F4="",G4=""),"",IF(AND(F4="ja",G4="Ziel"),"ja",IF(G4="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I4" s="7" t="inlineStr"/>
+      <c r="J4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -688,6 +728,12 @@
       </c>
       <c r="F5" s="5" t="inlineStr"/>
       <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="6">
+        <f>IF(F5="nein","nein",IF(OR(F5="",G5=""),"",IF(AND(F5="ja",G5="Ziel"),"ja",IF(G5="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I5" s="7" t="inlineStr"/>
+      <c r="J5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -713,6 +759,12 @@
       </c>
       <c r="F6" s="5" t="inlineStr"/>
       <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="6">
+        <f>IF(F6="nein","nein",IF(OR(F6="",G6=""),"",IF(AND(F6="ja",G6="Ziel"),"ja",IF(G6="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I6" s="7" t="inlineStr"/>
+      <c r="J6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -739,6 +791,12 @@
       </c>
       <c r="F7" s="5" t="inlineStr"/>
       <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="6">
+        <f>IF(F7="nein","nein",IF(OR(F7="",G7=""),"",IF(AND(F7="ja",G7="Ziel"),"ja",IF(G7="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I7" s="7" t="inlineStr"/>
+      <c r="J7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -765,6 +823,12 @@
       </c>
       <c r="F8" s="5" t="inlineStr"/>
       <c r="G8" s="5" t="inlineStr"/>
+      <c r="H8" s="6">
+        <f>IF(F8="nein","nein",IF(OR(F8="",G8=""),"",IF(AND(F8="ja",G8="Ziel"),"ja",IF(G8="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I8" s="7" t="inlineStr"/>
+      <c r="J8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -791,6 +855,12 @@
       </c>
       <c r="F9" s="5" t="inlineStr"/>
       <c r="G9" s="5" t="inlineStr"/>
+      <c r="H9" s="6">
+        <f>IF(F9="nein","nein",IF(OR(F9="",G9=""),"",IF(AND(F9="ja",G9="Ziel"),"ja",IF(G9="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I9" s="7" t="inlineStr"/>
+      <c r="J9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -817,6 +887,12 @@
       </c>
       <c r="F10" s="5" t="inlineStr"/>
       <c r="G10" s="5" t="inlineStr"/>
+      <c r="H10" s="6">
+        <f>IF(F10="nein","nein",IF(OR(F10="",G10=""),"",IF(AND(F10="ja",G10="Ziel"),"ja",IF(G10="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I10" s="7" t="inlineStr"/>
+      <c r="J10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -843,6 +919,12 @@
       </c>
       <c r="F11" s="5" t="inlineStr"/>
       <c r="G11" s="5" t="inlineStr"/>
+      <c r="H11" s="6">
+        <f>IF(F11="nein","nein",IF(OR(F11="",G11=""),"",IF(AND(F11="ja",G11="Ziel"),"ja",IF(G11="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I11" s="7" t="inlineStr"/>
+      <c r="J11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -869,6 +951,12 @@
       </c>
       <c r="F12" s="5" t="inlineStr"/>
       <c r="G12" s="5" t="inlineStr"/>
+      <c r="H12" s="6">
+        <f>IF(F12="nein","nein",IF(OR(F12="",G12=""),"",IF(AND(F12="ja",G12="Ziel"),"ja",IF(G12="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I12" s="7" t="inlineStr"/>
+      <c r="J12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -894,6 +982,12 @@
       </c>
       <c r="F13" s="5" t="inlineStr"/>
       <c r="G13" s="5" t="inlineStr"/>
+      <c r="H13" s="6">
+        <f>IF(F13="nein","nein",IF(OR(F13="",G13=""),"",IF(AND(F13="ja",G13="Ziel"),"ja",IF(G13="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I13" s="7" t="inlineStr"/>
+      <c r="J13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -920,6 +1014,12 @@
       </c>
       <c r="F14" s="5" t="inlineStr"/>
       <c r="G14" s="5" t="inlineStr"/>
+      <c r="H14" s="6">
+        <f>IF(F14="nein","nein",IF(OR(F14="",G14=""),"",IF(AND(F14="ja",G14="Ziel"),"ja",IF(G14="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I14" s="7" t="inlineStr"/>
+      <c r="J14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -946,6 +1046,12 @@
       </c>
       <c r="F15" s="5" t="inlineStr"/>
       <c r="G15" s="5" t="inlineStr"/>
+      <c r="H15" s="6">
+        <f>IF(F15="nein","nein",IF(OR(F15="",G15=""),"",IF(AND(F15="ja",G15="Ziel"),"ja",IF(G15="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I15" s="7" t="inlineStr"/>
+      <c r="J15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -971,6 +1077,12 @@
       </c>
       <c r="F16" s="5" t="inlineStr"/>
       <c r="G16" s="5" t="inlineStr"/>
+      <c r="H16" s="6">
+        <f>IF(F16="nein","nein",IF(OR(F16="",G16=""),"",IF(AND(F16="ja",G16="Ziel"),"ja",IF(G16="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I16" s="7" t="inlineStr"/>
+      <c r="J16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -997,6 +1109,12 @@
       </c>
       <c r="F17" s="5" t="inlineStr"/>
       <c r="G17" s="5" t="inlineStr"/>
+      <c r="H17" s="6">
+        <f>IF(F17="nein","nein",IF(OR(F17="",G17=""),"",IF(AND(F17="ja",G17="Ziel"),"ja",IF(G17="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I17" s="7" t="inlineStr"/>
+      <c r="J17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1022,6 +1140,12 @@
       </c>
       <c r="F18" s="5" t="inlineStr"/>
       <c r="G18" s="5" t="inlineStr"/>
+      <c r="H18" s="6">
+        <f>IF(F18="nein","nein",IF(OR(F18="",G18=""),"",IF(AND(F18="ja",G18="Ziel"),"ja",IF(G18="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I18" s="7" t="inlineStr"/>
+      <c r="J18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1047,6 +1171,12 @@
       </c>
       <c r="F19" s="5" t="inlineStr"/>
       <c r="G19" s="5" t="inlineStr"/>
+      <c r="H19" s="6">
+        <f>IF(F19="nein","nein",IF(OR(F19="",G19=""),"",IF(AND(F19="ja",G19="Ziel"),"ja",IF(G19="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I19" s="7" t="inlineStr"/>
+      <c r="J19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1073,6 +1203,12 @@
       </c>
       <c r="F20" s="5" t="inlineStr"/>
       <c r="G20" s="5" t="inlineStr"/>
+      <c r="H20" s="6">
+        <f>IF(F20="nein","nein",IF(OR(F20="",G20=""),"",IF(AND(F20="ja",G20="Ziel"),"ja",IF(G20="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I20" s="7" t="inlineStr"/>
+      <c r="J20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1099,6 +1235,12 @@
       </c>
       <c r="F21" s="5" t="inlineStr"/>
       <c r="G21" s="5" t="inlineStr"/>
+      <c r="H21" s="6">
+        <f>IF(F21="nein","nein",IF(OR(F21="",G21=""),"",IF(AND(F21="ja",G21="Ziel"),"ja",IF(G21="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I21" s="7" t="inlineStr"/>
+      <c r="J21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1124,6 +1266,12 @@
       </c>
       <c r="F22" s="5" t="inlineStr"/>
       <c r="G22" s="5" t="inlineStr"/>
+      <c r="H22" s="6">
+        <f>IF(F22="nein","nein",IF(OR(F22="",G22=""),"",IF(AND(F22="ja",G22="Ziel"),"ja",IF(G22="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I22" s="7" t="inlineStr"/>
+      <c r="J22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1149,6 +1297,12 @@
       </c>
       <c r="F23" s="5" t="inlineStr"/>
       <c r="G23" s="5" t="inlineStr"/>
+      <c r="H23" s="6">
+        <f>IF(F23="nein","nein",IF(OR(F23="",G23=""),"",IF(AND(F23="ja",G23="Ziel"),"ja",IF(G23="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I23" s="7" t="inlineStr"/>
+      <c r="J23" s="5" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1175,6 +1329,12 @@
       </c>
       <c r="F24" s="5" t="inlineStr"/>
       <c r="G24" s="5" t="inlineStr"/>
+      <c r="H24" s="6">
+        <f>IF(F24="nein","nein",IF(OR(F24="",G24=""),"",IF(AND(F24="ja",G24="Ziel"),"ja",IF(G24="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I24" s="7" t="inlineStr"/>
+      <c r="J24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1201,6 +1361,12 @@
       </c>
       <c r="F25" s="5" t="inlineStr"/>
       <c r="G25" s="5" t="inlineStr"/>
+      <c r="H25" s="6">
+        <f>IF(F25="nein","nein",IF(OR(F25="",G25=""),"",IF(AND(F25="ja",G25="Ziel"),"ja",IF(G25="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I25" s="7" t="inlineStr"/>
+      <c r="J25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1226,6 +1392,12 @@
       </c>
       <c r="F26" s="5" t="inlineStr"/>
       <c r="G26" s="5" t="inlineStr"/>
+      <c r="H26" s="6">
+        <f>IF(F26="nein","nein",IF(OR(F26="",G26=""),"",IF(AND(F26="ja",G26="Ziel"),"ja",IF(G26="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I26" s="7" t="inlineStr"/>
+      <c r="J26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1252,6 +1424,12 @@
       </c>
       <c r="F27" s="5" t="inlineStr"/>
       <c r="G27" s="5" t="inlineStr"/>
+      <c r="H27" s="6">
+        <f>IF(F27="nein","nein",IF(OR(F27="",G27=""),"",IF(AND(F27="ja",G27="Ziel"),"ja",IF(G27="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I27" s="7" t="inlineStr"/>
+      <c r="J27" s="5" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1278,6 +1456,12 @@
       </c>
       <c r="F28" s="5" t="inlineStr"/>
       <c r="G28" s="5" t="inlineStr"/>
+      <c r="H28" s="6">
+        <f>IF(F28="nein","nein",IF(OR(F28="",G28=""),"",IF(AND(F28="ja",G28="Ziel"),"ja",IF(G28="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I28" s="7" t="inlineStr"/>
+      <c r="J28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1303,6 +1487,12 @@
       </c>
       <c r="F29" s="5" t="inlineStr"/>
       <c r="G29" s="5" t="inlineStr"/>
+      <c r="H29" s="6">
+        <f>IF(F29="nein","nein",IF(OR(F29="",G29=""),"",IF(AND(F29="ja",G29="Ziel"),"ja",IF(G29="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I29" s="7" t="inlineStr"/>
+      <c r="J29" s="5" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1328,6 +1518,12 @@
       </c>
       <c r="F30" s="5" t="inlineStr"/>
       <c r="G30" s="5" t="inlineStr"/>
+      <c r="H30" s="6">
+        <f>IF(F30="nein","nein",IF(OR(F30="",G30=""),"",IF(AND(F30="ja",G30="Ziel"),"ja",IF(G30="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I30" s="7" t="inlineStr"/>
+      <c r="J30" s="5" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1354,6 +1550,12 @@
       </c>
       <c r="F31" s="5" t="inlineStr"/>
       <c r="G31" s="5" t="inlineStr"/>
+      <c r="H31" s="6">
+        <f>IF(F31="nein","nein",IF(OR(F31="",G31=""),"",IF(AND(F31="ja",G31="Ziel"),"ja",IF(G31="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I31" s="7" t="inlineStr"/>
+      <c r="J31" s="5" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1380,6 +1582,12 @@
       </c>
       <c r="F32" s="5" t="inlineStr"/>
       <c r="G32" s="5" t="inlineStr"/>
+      <c r="H32" s="6">
+        <f>IF(F32="nein","nein",IF(OR(F32="",G32=""),"",IF(AND(F32="ja",G32="Ziel"),"ja",IF(G32="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I32" s="7" t="inlineStr"/>
+      <c r="J32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1406,6 +1614,12 @@
       </c>
       <c r="F33" s="5" t="inlineStr"/>
       <c r="G33" s="5" t="inlineStr"/>
+      <c r="H33" s="6">
+        <f>IF(F33="nein","nein",IF(OR(F33="",G33=""),"",IF(AND(F33="ja",G33="Ziel"),"ja",IF(G33="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I33" s="7" t="inlineStr"/>
+      <c r="J33" s="5" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1432,6 +1646,12 @@
       </c>
       <c r="F34" s="5" t="inlineStr"/>
       <c r="G34" s="5" t="inlineStr"/>
+      <c r="H34" s="6">
+        <f>IF(F34="nein","nein",IF(OR(F34="",G34=""),"",IF(AND(F34="ja",G34="Ziel"),"ja",IF(G34="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I34" s="7" t="inlineStr"/>
+      <c r="J34" s="5" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1457,6 +1677,12 @@
       </c>
       <c r="F35" s="5" t="inlineStr"/>
       <c r="G35" s="5" t="inlineStr"/>
+      <c r="H35" s="6">
+        <f>IF(F35="nein","nein",IF(OR(F35="",G35=""),"",IF(AND(F35="ja",G35="Ziel"),"ja",IF(G35="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I35" s="7" t="inlineStr"/>
+      <c r="J35" s="5" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1482,6 +1708,12 @@
       </c>
       <c r="F36" s="5" t="inlineStr"/>
       <c r="G36" s="5" t="inlineStr"/>
+      <c r="H36" s="6">
+        <f>IF(F36="nein","nein",IF(OR(F36="",G36=""),"",IF(AND(F36="ja",G36="Ziel"),"ja",IF(G36="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I36" s="7" t="inlineStr"/>
+      <c r="J36" s="5" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1508,6 +1740,12 @@
       </c>
       <c r="F37" s="5" t="inlineStr"/>
       <c r="G37" s="5" t="inlineStr"/>
+      <c r="H37" s="6">
+        <f>IF(F37="nein","nein",IF(OR(F37="",G37=""),"",IF(AND(F37="ja",G37="Ziel"),"ja",IF(G37="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I37" s="7" t="inlineStr"/>
+      <c r="J37" s="5" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1534,6 +1772,12 @@
       </c>
       <c r="F38" s="5" t="inlineStr"/>
       <c r="G38" s="5" t="inlineStr"/>
+      <c r="H38" s="6">
+        <f>IF(F38="nein","nein",IF(OR(F38="",G38=""),"",IF(AND(F38="ja",G38="Ziel"),"ja",IF(G38="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I38" s="7" t="inlineStr"/>
+      <c r="J38" s="5" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1559,6 +1803,12 @@
       </c>
       <c r="F39" s="5" t="inlineStr"/>
       <c r="G39" s="5" t="inlineStr"/>
+      <c r="H39" s="6">
+        <f>IF(F39="nein","nein",IF(OR(F39="",G39=""),"",IF(AND(F39="ja",G39="Ziel"),"ja",IF(G39="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I39" s="7" t="inlineStr"/>
+      <c r="J39" s="5" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1585,6 +1835,12 @@
       </c>
       <c r="F40" s="5" t="inlineStr"/>
       <c r="G40" s="5" t="inlineStr"/>
+      <c r="H40" s="6">
+        <f>IF(F40="nein","nein",IF(OR(F40="",G40=""),"",IF(AND(F40="ja",G40="Ziel"),"ja",IF(G40="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I40" s="7" t="inlineStr"/>
+      <c r="J40" s="5" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1611,6 +1867,12 @@
       </c>
       <c r="F41" s="5" t="inlineStr"/>
       <c r="G41" s="5" t="inlineStr"/>
+      <c r="H41" s="6">
+        <f>IF(F41="nein","nein",IF(OR(F41="",G41=""),"",IF(AND(F41="ja",G41="Ziel"),"ja",IF(G41="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I41" s="7" t="inlineStr"/>
+      <c r="J41" s="5" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1637,6 +1899,12 @@
       </c>
       <c r="F42" s="5" t="inlineStr"/>
       <c r="G42" s="5" t="inlineStr"/>
+      <c r="H42" s="6">
+        <f>IF(F42="nein","nein",IF(OR(F42="",G42=""),"",IF(AND(F42="ja",G42="Ziel"),"ja",IF(G42="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I42" s="7" t="inlineStr"/>
+      <c r="J42" s="5" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1662,6 +1930,12 @@
       </c>
       <c r="F43" s="5" t="inlineStr"/>
       <c r="G43" s="5" t="inlineStr"/>
+      <c r="H43" s="6">
+        <f>IF(F43="nein","nein",IF(OR(F43="",G43=""),"",IF(AND(F43="ja",G43="Ziel"),"ja",IF(G43="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I43" s="7" t="inlineStr"/>
+      <c r="J43" s="5" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1688,6 +1962,12 @@
       </c>
       <c r="F44" s="5" t="inlineStr"/>
       <c r="G44" s="5" t="inlineStr"/>
+      <c r="H44" s="6">
+        <f>IF(F44="nein","nein",IF(OR(F44="",G44=""),"",IF(AND(F44="ja",G44="Ziel"),"ja",IF(G44="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I44" s="7" t="inlineStr"/>
+      <c r="J44" s="5" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1713,6 +1993,12 @@
       </c>
       <c r="F45" s="5" t="inlineStr"/>
       <c r="G45" s="5" t="inlineStr"/>
+      <c r="H45" s="6">
+        <f>IF(F45="nein","nein",IF(OR(F45="",G45=""),"",IF(AND(F45="ja",G45="Ziel"),"ja",IF(G45="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I45" s="7" t="inlineStr"/>
+      <c r="J45" s="5" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1738,6 +2024,12 @@
       </c>
       <c r="F46" s="5" t="inlineStr"/>
       <c r="G46" s="5" t="inlineStr"/>
+      <c r="H46" s="6">
+        <f>IF(F46="nein","nein",IF(OR(F46="",G46=""),"",IF(AND(F46="ja",G46="Ziel"),"ja",IF(G46="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I46" s="7" t="inlineStr"/>
+      <c r="J46" s="5" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1765,6 +2057,12 @@
       </c>
       <c r="F47" s="5" t="inlineStr"/>
       <c r="G47" s="5" t="inlineStr"/>
+      <c r="H47" s="6">
+        <f>IF(F47="nein","nein",IF(OR(F47="",G47=""),"",IF(AND(F47="ja",G47="Ziel"),"ja",IF(G47="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I47" s="7" t="inlineStr"/>
+      <c r="J47" s="5" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1790,6 +2088,12 @@
       </c>
       <c r="F48" s="5" t="inlineStr"/>
       <c r="G48" s="5" t="inlineStr"/>
+      <c r="H48" s="6">
+        <f>IF(F48="nein","nein",IF(OR(F48="",G48=""),"",IF(AND(F48="ja",G48="Ziel"),"ja",IF(G48="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I48" s="7" t="inlineStr"/>
+      <c r="J48" s="5" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1816,6 +2120,12 @@
       </c>
       <c r="F49" s="5" t="inlineStr"/>
       <c r="G49" s="5" t="inlineStr"/>
+      <c r="H49" s="6">
+        <f>IF(F49="nein","nein",IF(OR(F49="",G49=""),"",IF(AND(F49="ja",G49="Ziel"),"ja",IF(G49="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I49" s="7" t="inlineStr"/>
+      <c r="J49" s="5" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -1841,6 +2151,12 @@
       </c>
       <c r="F50" s="5" t="inlineStr"/>
       <c r="G50" s="5" t="inlineStr"/>
+      <c r="H50" s="6">
+        <f>IF(F50="nein","nein",IF(OR(F50="",G50=""),"",IF(AND(F50="ja",G50="Ziel"),"ja",IF(G50="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I50" s="7" t="inlineStr"/>
+      <c r="J50" s="5" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1866,6 +2182,12 @@
       </c>
       <c r="F51" s="5" t="inlineStr"/>
       <c r="G51" s="5" t="inlineStr"/>
+      <c r="H51" s="6">
+        <f>IF(F51="nein","nein",IF(OR(F51="",G51=""),"",IF(AND(F51="ja",G51="Ziel"),"ja",IF(G51="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I51" s="7" t="inlineStr"/>
+      <c r="J51" s="5" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -1891,6 +2213,12 @@
       </c>
       <c r="F52" s="5" t="inlineStr"/>
       <c r="G52" s="5" t="inlineStr"/>
+      <c r="H52" s="6">
+        <f>IF(F52="nein","nein",IF(OR(F52="",G52=""),"",IF(AND(F52="ja",G52="Ziel"),"ja",IF(G52="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I52" s="7" t="inlineStr"/>
+      <c r="J52" s="5" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -1917,6 +2245,12 @@
       </c>
       <c r="F53" s="5" t="inlineStr"/>
       <c r="G53" s="5" t="inlineStr"/>
+      <c r="H53" s="6">
+        <f>IF(F53="nein","nein",IF(OR(F53="",G53=""),"",IF(AND(F53="ja",G53="Ziel"),"ja",IF(G53="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I53" s="7" t="inlineStr"/>
+      <c r="J53" s="5" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -1942,6 +2276,12 @@
       </c>
       <c r="F54" s="5" t="inlineStr"/>
       <c r="G54" s="5" t="inlineStr"/>
+      <c r="H54" s="6">
+        <f>IF(F54="nein","nein",IF(OR(F54="",G54=""),"",IF(AND(F54="ja",G54="Ziel"),"ja",IF(G54="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I54" s="7" t="inlineStr"/>
+      <c r="J54" s="5" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -1968,6 +2308,12 @@
       </c>
       <c r="F55" s="5" t="inlineStr"/>
       <c r="G55" s="5" t="inlineStr"/>
+      <c r="H55" s="6">
+        <f>IF(F55="nein","nein",IF(OR(F55="",G55=""),"",IF(AND(F55="ja",G55="Ziel"),"ja",IF(G55="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I55" s="7" t="inlineStr"/>
+      <c r="J55" s="5" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -1994,6 +2340,12 @@
       </c>
       <c r="F56" s="5" t="inlineStr"/>
       <c r="G56" s="5" t="inlineStr"/>
+      <c r="H56" s="6">
+        <f>IF(F56="nein","nein",IF(OR(F56="",G56=""),"",IF(AND(F56="ja",G56="Ziel"),"ja",IF(G56="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I56" s="7" t="inlineStr"/>
+      <c r="J56" s="5" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -2020,6 +2372,12 @@
       </c>
       <c r="F57" s="5" t="inlineStr"/>
       <c r="G57" s="5" t="inlineStr"/>
+      <c r="H57" s="6">
+        <f>IF(F57="nein","nein",IF(OR(F57="",G57=""),"",IF(AND(F57="ja",G57="Ziel"),"ja",IF(G57="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I57" s="7" t="inlineStr"/>
+      <c r="J57" s="5" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -2045,6 +2403,12 @@
       </c>
       <c r="F58" s="5" t="inlineStr"/>
       <c r="G58" s="5" t="inlineStr"/>
+      <c r="H58" s="6">
+        <f>IF(F58="nein","nein",IF(OR(F58="",G58=""),"",IF(AND(F58="ja",G58="Ziel"),"ja",IF(G58="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I58" s="7" t="inlineStr"/>
+      <c r="J58" s="5" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -2071,6 +2435,12 @@
       </c>
       <c r="F59" s="5" t="inlineStr"/>
       <c r="G59" s="5" t="inlineStr"/>
+      <c r="H59" s="6">
+        <f>IF(F59="nein","nein",IF(OR(F59="",G59=""),"",IF(AND(F59="ja",G59="Ziel"),"ja",IF(G59="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I59" s="7" t="inlineStr"/>
+      <c r="J59" s="5" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -2097,6 +2467,12 @@
       </c>
       <c r="F60" s="5" t="inlineStr"/>
       <c r="G60" s="5" t="inlineStr"/>
+      <c r="H60" s="6">
+        <f>IF(F60="nein","nein",IF(OR(F60="",G60=""),"",IF(AND(F60="ja",G60="Ziel"),"ja",IF(G60="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I60" s="7" t="inlineStr"/>
+      <c r="J60" s="5" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -2123,6 +2499,12 @@
       </c>
       <c r="F61" s="5" t="inlineStr"/>
       <c r="G61" s="5" t="inlineStr"/>
+      <c r="H61" s="6">
+        <f>IF(F61="nein","nein",IF(OR(F61="",G61=""),"",IF(AND(F61="ja",G61="Ziel"),"ja",IF(G61="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I61" s="7" t="inlineStr"/>
+      <c r="J61" s="5" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -2149,6 +2531,12 @@
       </c>
       <c r="F62" s="5" t="inlineStr"/>
       <c r="G62" s="5" t="inlineStr"/>
+      <c r="H62" s="6">
+        <f>IF(F62="nein","nein",IF(OR(F62="",G62=""),"",IF(AND(F62="ja",G62="Ziel"),"ja",IF(G62="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I62" s="7" t="inlineStr"/>
+      <c r="J62" s="5" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -2174,6 +2562,12 @@
       </c>
       <c r="F63" s="5" t="inlineStr"/>
       <c r="G63" s="5" t="inlineStr"/>
+      <c r="H63" s="6">
+        <f>IF(F63="nein","nein",IF(OR(F63="",G63=""),"",IF(AND(F63="ja",G63="Ziel"),"ja",IF(G63="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I63" s="7" t="inlineStr"/>
+      <c r="J63" s="5" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -2200,6 +2594,12 @@
       </c>
       <c r="F64" s="5" t="inlineStr"/>
       <c r="G64" s="5" t="inlineStr"/>
+      <c r="H64" s="6">
+        <f>IF(F64="nein","nein",IF(OR(F64="",G64=""),"",IF(AND(F64="ja",G64="Ziel"),"ja",IF(G64="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I64" s="7" t="inlineStr"/>
+      <c r="J64" s="5" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -2226,6 +2626,12 @@
       </c>
       <c r="F65" s="5" t="inlineStr"/>
       <c r="G65" s="5" t="inlineStr"/>
+      <c r="H65" s="6">
+        <f>IF(F65="nein","nein",IF(OR(F65="",G65=""),"",IF(AND(F65="ja",G65="Ziel"),"ja",IF(G65="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I65" s="7" t="inlineStr"/>
+      <c r="J65" s="5" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -2252,6 +2658,12 @@
       </c>
       <c r="F66" s="5" t="inlineStr"/>
       <c r="G66" s="5" t="inlineStr"/>
+      <c r="H66" s="6">
+        <f>IF(F66="nein","nein",IF(OR(F66="",G66=""),"",IF(AND(F66="ja",G66="Ziel"),"ja",IF(G66="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I66" s="7" t="inlineStr"/>
+      <c r="J66" s="5" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -2277,6 +2689,12 @@
       </c>
       <c r="F67" s="5" t="inlineStr"/>
       <c r="G67" s="5" t="inlineStr"/>
+      <c r="H67" s="6">
+        <f>IF(F67="nein","nein",IF(OR(F67="",G67=""),"",IF(AND(F67="ja",G67="Ziel"),"ja",IF(G67="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I67" s="7" t="inlineStr"/>
+      <c r="J67" s="5" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -2303,6 +2721,12 @@
       </c>
       <c r="F68" s="5" t="inlineStr"/>
       <c r="G68" s="5" t="inlineStr"/>
+      <c r="H68" s="6">
+        <f>IF(F68="nein","nein",IF(OR(F68="",G68=""),"",IF(AND(F68="ja",G68="Ziel"),"ja",IF(G68="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I68" s="7" t="inlineStr"/>
+      <c r="J68" s="5" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -2324,6 +2748,12 @@
       <c r="E69" s="2" t="inlineStr"/>
       <c r="F69" s="5" t="inlineStr"/>
       <c r="G69" s="5" t="inlineStr"/>
+      <c r="H69" s="6">
+        <f>IF(F69="nein","nein",IF(OR(F69="",G69=""),"",IF(AND(F69="ja",G69="Ziel"),"ja",IF(G69="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I69" s="7" t="inlineStr"/>
+      <c r="J69" s="5" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -2350,6 +2780,12 @@
       </c>
       <c r="F70" s="5" t="inlineStr"/>
       <c r="G70" s="5" t="inlineStr"/>
+      <c r="H70" s="6">
+        <f>IF(F70="nein","nein",IF(OR(F70="",G70=""),"",IF(AND(F70="ja",G70="Ziel"),"ja",IF(G70="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I70" s="7" t="inlineStr"/>
+      <c r="J70" s="5" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -2375,6 +2811,12 @@
       </c>
       <c r="F71" s="5" t="inlineStr"/>
       <c r="G71" s="5" t="inlineStr"/>
+      <c r="H71" s="6">
+        <f>IF(F71="nein","nein",IF(OR(F71="",G71=""),"",IF(AND(F71="ja",G71="Ziel"),"ja",IF(G71="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I71" s="7" t="inlineStr"/>
+      <c r="J71" s="5" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -2401,6 +2843,12 @@
       </c>
       <c r="F72" s="5" t="inlineStr"/>
       <c r="G72" s="5" t="inlineStr"/>
+      <c r="H72" s="6">
+        <f>IF(F72="nein","nein",IF(OR(F72="",G72=""),"",IF(AND(F72="ja",G72="Ziel"),"ja",IF(G72="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I72" s="7" t="inlineStr"/>
+      <c r="J72" s="5" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -2427,6 +2875,12 @@
       </c>
       <c r="F73" s="5" t="inlineStr"/>
       <c r="G73" s="5" t="inlineStr"/>
+      <c r="H73" s="6">
+        <f>IF(F73="nein","nein",IF(OR(F73="",G73=""),"",IF(AND(F73="ja",G73="Ziel"),"ja",IF(G73="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I73" s="7" t="inlineStr"/>
+      <c r="J73" s="5" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -2453,6 +2907,12 @@
       </c>
       <c r="F74" s="5" t="inlineStr"/>
       <c r="G74" s="5" t="inlineStr"/>
+      <c r="H74" s="6">
+        <f>IF(F74="nein","nein",IF(OR(F74="",G74=""),"",IF(AND(F74="ja",G74="Ziel"),"ja",IF(G74="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I74" s="7" t="inlineStr"/>
+      <c r="J74" s="5" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -2479,6 +2939,12 @@
       </c>
       <c r="F75" s="5" t="inlineStr"/>
       <c r="G75" s="5" t="inlineStr"/>
+      <c r="H75" s="6">
+        <f>IF(F75="nein","nein",IF(OR(F75="",G75=""),"",IF(AND(F75="ja",G75="Ziel"),"ja",IF(G75="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I75" s="7" t="inlineStr"/>
+      <c r="J75" s="5" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -2504,6 +2970,12 @@
       </c>
       <c r="F76" s="5" t="inlineStr"/>
       <c r="G76" s="5" t="inlineStr"/>
+      <c r="H76" s="6">
+        <f>IF(F76="nein","nein",IF(OR(F76="",G76=""),"",IF(AND(F76="ja",G76="Ziel"),"ja",IF(G76="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I76" s="7" t="inlineStr"/>
+      <c r="J76" s="5" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -2530,6 +3002,12 @@
       </c>
       <c r="F77" s="5" t="inlineStr"/>
       <c r="G77" s="5" t="inlineStr"/>
+      <c r="H77" s="6">
+        <f>IF(F77="nein","nein",IF(OR(F77="",G77=""),"",IF(AND(F77="ja",G77="Ziel"),"ja",IF(G77="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I77" s="7" t="inlineStr"/>
+      <c r="J77" s="5" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -2555,6 +3033,12 @@
       </c>
       <c r="F78" s="5" t="inlineStr"/>
       <c r="G78" s="5" t="inlineStr"/>
+      <c r="H78" s="6">
+        <f>IF(F78="nein","nein",IF(OR(F78="",G78=""),"",IF(AND(F78="ja",G78="Ziel"),"ja",IF(G78="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I78" s="7" t="inlineStr"/>
+      <c r="J78" s="5" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -2580,6 +3064,12 @@
       </c>
       <c r="F79" s="5" t="inlineStr"/>
       <c r="G79" s="5" t="inlineStr"/>
+      <c r="H79" s="6">
+        <f>IF(F79="nein","nein",IF(OR(F79="",G79=""),"",IF(AND(F79="ja",G79="Ziel"),"ja",IF(G79="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I79" s="7" t="inlineStr"/>
+      <c r="J79" s="5" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -2605,6 +3095,12 @@
       </c>
       <c r="F80" s="5" t="inlineStr"/>
       <c r="G80" s="5" t="inlineStr"/>
+      <c r="H80" s="6">
+        <f>IF(F80="nein","nein",IF(OR(F80="",G80=""),"",IF(AND(F80="ja",G80="Ziel"),"ja",IF(G80="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I80" s="7" t="inlineStr"/>
+      <c r="J80" s="5" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -2630,6 +3126,12 @@
       </c>
       <c r="F81" s="5" t="inlineStr"/>
       <c r="G81" s="5" t="inlineStr"/>
+      <c r="H81" s="6">
+        <f>IF(F81="nein","nein",IF(OR(F81="",G81=""),"",IF(AND(F81="ja",G81="Ziel"),"ja",IF(G81="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I81" s="7" t="inlineStr"/>
+      <c r="J81" s="5" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -2656,6 +3158,12 @@
       </c>
       <c r="F82" s="5" t="inlineStr"/>
       <c r="G82" s="5" t="inlineStr"/>
+      <c r="H82" s="6">
+        <f>IF(F82="nein","nein",IF(OR(F82="",G82=""),"",IF(AND(F82="ja",G82="Ziel"),"ja",IF(G82="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I82" s="7" t="inlineStr"/>
+      <c r="J82" s="5" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -2682,6 +3190,12 @@
       </c>
       <c r="F83" s="5" t="inlineStr"/>
       <c r="G83" s="5" t="inlineStr"/>
+      <c r="H83" s="6">
+        <f>IF(F83="nein","nein",IF(OR(F83="",G83=""),"",IF(AND(F83="ja",G83="Ziel"),"ja",IF(G83="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I83" s="7" t="inlineStr"/>
+      <c r="J83" s="5" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -2708,6 +3222,12 @@
       </c>
       <c r="F84" s="5" t="inlineStr"/>
       <c r="G84" s="5" t="inlineStr"/>
+      <c r="H84" s="6">
+        <f>IF(F84="nein","nein",IF(OR(F84="",G84=""),"",IF(AND(F84="ja",G84="Ziel"),"ja",IF(G84="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I84" s="7" t="inlineStr"/>
+      <c r="J84" s="5" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -2733,6 +3253,12 @@
       </c>
       <c r="F85" s="5" t="inlineStr"/>
       <c r="G85" s="5" t="inlineStr"/>
+      <c r="H85" s="6">
+        <f>IF(F85="nein","nein",IF(OR(F85="",G85=""),"",IF(AND(F85="ja",G85="Ziel"),"ja",IF(G85="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I85" s="7" t="inlineStr"/>
+      <c r="J85" s="5" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -2758,6 +3284,12 @@
       </c>
       <c r="F86" s="5" t="inlineStr"/>
       <c r="G86" s="5" t="inlineStr"/>
+      <c r="H86" s="6">
+        <f>IF(F86="nein","nein",IF(OR(F86="",G86=""),"",IF(AND(F86="ja",G86="Ziel"),"ja",IF(G86="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I86" s="7" t="inlineStr"/>
+      <c r="J86" s="5" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -2783,6 +3315,12 @@
       </c>
       <c r="F87" s="5" t="inlineStr"/>
       <c r="G87" s="5" t="inlineStr"/>
+      <c r="H87" s="6">
+        <f>IF(F87="nein","nein",IF(OR(F87="",G87=""),"",IF(AND(F87="ja",G87="Ziel"),"ja",IF(G87="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I87" s="7" t="inlineStr"/>
+      <c r="J87" s="5" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -2809,6 +3347,12 @@
       </c>
       <c r="F88" s="5" t="inlineStr"/>
       <c r="G88" s="5" t="inlineStr"/>
+      <c r="H88" s="6">
+        <f>IF(F88="nein","nein",IF(OR(F88="",G88=""),"",IF(AND(F88="ja",G88="Ziel"),"ja",IF(G88="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I88" s="7" t="inlineStr"/>
+      <c r="J88" s="5" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -2835,6 +3379,12 @@
       </c>
       <c r="F89" s="5" t="inlineStr"/>
       <c r="G89" s="5" t="inlineStr"/>
+      <c r="H89" s="6">
+        <f>IF(F89="nein","nein",IF(OR(F89="",G89=""),"",IF(AND(F89="ja",G89="Ziel"),"ja",IF(G89="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I89" s="7" t="inlineStr"/>
+      <c r="J89" s="5" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -2860,6 +3410,12 @@
       </c>
       <c r="F90" s="5" t="inlineStr"/>
       <c r="G90" s="5" t="inlineStr"/>
+      <c r="H90" s="6">
+        <f>IF(F90="nein","nein",IF(OR(F90="",G90=""),"",IF(AND(F90="ja",G90="Ziel"),"ja",IF(G90="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I90" s="7" t="inlineStr"/>
+      <c r="J90" s="5" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -2886,851 +3442,20 @@
       </c>
       <c r="F91" s="5" t="inlineStr"/>
       <c r="G91" s="5" t="inlineStr"/>
-    </row>
-    <row r="92">
-      <c r="F92" s="5" t="n"/>
-      <c r="G92" s="5" t="n"/>
-    </row>
-    <row r="93">
-      <c r="F93" s="5" t="n"/>
-      <c r="G93" s="5" t="n"/>
-    </row>
-    <row r="94">
-      <c r="F94" s="5" t="n"/>
-      <c r="G94" s="5" t="n"/>
-    </row>
-    <row r="95">
-      <c r="F95" s="5" t="n"/>
-      <c r="G95" s="5" t="n"/>
-    </row>
-    <row r="96">
-      <c r="F96" s="5" t="n"/>
-      <c r="G96" s="5" t="n"/>
-    </row>
-    <row r="97">
-      <c r="F97" s="5" t="n"/>
-      <c r="G97" s="5" t="n"/>
-    </row>
-    <row r="98">
-      <c r="F98" s="5" t="n"/>
-      <c r="G98" s="5" t="n"/>
-    </row>
-    <row r="99">
-      <c r="F99" s="5" t="n"/>
-      <c r="G99" s="5" t="n"/>
-    </row>
-    <row r="100">
-      <c r="F100" s="5" t="n"/>
-      <c r="G100" s="5" t="n"/>
-    </row>
-    <row r="101">
-      <c r="F101" s="5" t="n"/>
-      <c r="G101" s="5" t="n"/>
-    </row>
-    <row r="102">
-      <c r="F102" s="5" t="n"/>
-      <c r="G102" s="5" t="n"/>
-    </row>
-    <row r="103">
-      <c r="F103" s="5" t="n"/>
-      <c r="G103" s="5" t="n"/>
-    </row>
-    <row r="104">
-      <c r="F104" s="5" t="n"/>
-      <c r="G104" s="5" t="n"/>
-    </row>
-    <row r="105">
-      <c r="F105" s="5" t="n"/>
-      <c r="G105" s="5" t="n"/>
-    </row>
-    <row r="106">
-      <c r="F106" s="5" t="n"/>
-      <c r="G106" s="5" t="n"/>
-    </row>
-    <row r="107">
-      <c r="F107" s="5" t="n"/>
-      <c r="G107" s="5" t="n"/>
-    </row>
-    <row r="108">
-      <c r="F108" s="5" t="n"/>
-      <c r="G108" s="5" t="n"/>
-    </row>
-    <row r="109">
-      <c r="F109" s="5" t="n"/>
-      <c r="G109" s="5" t="n"/>
-    </row>
-    <row r="110">
-      <c r="F110" s="5" t="n"/>
-      <c r="G110" s="5" t="n"/>
-    </row>
-    <row r="111">
-      <c r="F111" s="5" t="n"/>
-      <c r="G111" s="5" t="n"/>
-    </row>
-    <row r="112">
-      <c r="F112" s="5" t="n"/>
-      <c r="G112" s="5" t="n"/>
-    </row>
-    <row r="113">
-      <c r="F113" s="5" t="n"/>
-      <c r="G113" s="5" t="n"/>
-    </row>
-    <row r="114">
-      <c r="F114" s="5" t="n"/>
-      <c r="G114" s="5" t="n"/>
-    </row>
-    <row r="115">
-      <c r="F115" s="5" t="n"/>
-      <c r="G115" s="5" t="n"/>
-    </row>
-    <row r="116">
-      <c r="F116" s="5" t="n"/>
-      <c r="G116" s="5" t="n"/>
-    </row>
-    <row r="117">
-      <c r="F117" s="5" t="n"/>
-      <c r="G117" s="5" t="n"/>
-    </row>
-    <row r="118">
-      <c r="F118" s="5" t="n"/>
-      <c r="G118" s="5" t="n"/>
-    </row>
-    <row r="119">
-      <c r="F119" s="5" t="n"/>
-      <c r="G119" s="5" t="n"/>
-    </row>
-    <row r="120">
-      <c r="F120" s="5" t="n"/>
-      <c r="G120" s="5" t="n"/>
-    </row>
-    <row r="121">
-      <c r="F121" s="5" t="n"/>
-      <c r="G121" s="5" t="n"/>
-    </row>
-    <row r="122">
-      <c r="F122" s="5" t="n"/>
-      <c r="G122" s="5" t="n"/>
-    </row>
-    <row r="123">
-      <c r="F123" s="5" t="n"/>
-      <c r="G123" s="5" t="n"/>
-    </row>
-    <row r="124">
-      <c r="F124" s="5" t="n"/>
-      <c r="G124" s="5" t="n"/>
-    </row>
-    <row r="125">
-      <c r="F125" s="5" t="n"/>
-      <c r="G125" s="5" t="n"/>
-    </row>
-    <row r="126">
-      <c r="F126" s="5" t="n"/>
-      <c r="G126" s="5" t="n"/>
-    </row>
-    <row r="127">
-      <c r="F127" s="5" t="n"/>
-      <c r="G127" s="5" t="n"/>
-    </row>
-    <row r="128">
-      <c r="F128" s="5" t="n"/>
-      <c r="G128" s="5" t="n"/>
-    </row>
-    <row r="129">
-      <c r="F129" s="5" t="n"/>
-      <c r="G129" s="5" t="n"/>
-    </row>
-    <row r="130">
-      <c r="F130" s="5" t="n"/>
-      <c r="G130" s="5" t="n"/>
-    </row>
-    <row r="131">
-      <c r="F131" s="5" t="n"/>
-      <c r="G131" s="5" t="n"/>
-    </row>
-    <row r="132">
-      <c r="F132" s="5" t="n"/>
-      <c r="G132" s="5" t="n"/>
-    </row>
-    <row r="133">
-      <c r="F133" s="5" t="n"/>
-      <c r="G133" s="5" t="n"/>
-    </row>
-    <row r="134">
-      <c r="F134" s="5" t="n"/>
-      <c r="G134" s="5" t="n"/>
-    </row>
-    <row r="135">
-      <c r="F135" s="5" t="n"/>
-      <c r="G135" s="5" t="n"/>
-    </row>
-    <row r="136">
-      <c r="F136" s="5" t="n"/>
-      <c r="G136" s="5" t="n"/>
-    </row>
-    <row r="137">
-      <c r="F137" s="5" t="n"/>
-      <c r="G137" s="5" t="n"/>
-    </row>
-    <row r="138">
-      <c r="F138" s="5" t="n"/>
-      <c r="G138" s="5" t="n"/>
-    </row>
-    <row r="139">
-      <c r="F139" s="5" t="n"/>
-      <c r="G139" s="5" t="n"/>
-    </row>
-    <row r="140">
-      <c r="F140" s="5" t="n"/>
-      <c r="G140" s="5" t="n"/>
-    </row>
-    <row r="141">
-      <c r="F141" s="5" t="n"/>
-      <c r="G141" s="5" t="n"/>
-    </row>
-    <row r="142">
-      <c r="F142" s="5" t="n"/>
-      <c r="G142" s="5" t="n"/>
-    </row>
-    <row r="143">
-      <c r="F143" s="5" t="n"/>
-      <c r="G143" s="5" t="n"/>
-    </row>
-    <row r="144">
-      <c r="F144" s="5" t="n"/>
-      <c r="G144" s="5" t="n"/>
-    </row>
-    <row r="145">
-      <c r="F145" s="5" t="n"/>
-      <c r="G145" s="5" t="n"/>
-    </row>
-    <row r="146">
-      <c r="F146" s="5" t="n"/>
-      <c r="G146" s="5" t="n"/>
-    </row>
-    <row r="147">
-      <c r="F147" s="5" t="n"/>
-      <c r="G147" s="5" t="n"/>
-    </row>
-    <row r="148">
-      <c r="F148" s="5" t="n"/>
-      <c r="G148" s="5" t="n"/>
-    </row>
-    <row r="149">
-      <c r="F149" s="5" t="n"/>
-      <c r="G149" s="5" t="n"/>
-    </row>
-    <row r="150">
-      <c r="F150" s="5" t="n"/>
-      <c r="G150" s="5" t="n"/>
-    </row>
-    <row r="151">
-      <c r="F151" s="5" t="n"/>
-      <c r="G151" s="5" t="n"/>
-    </row>
-    <row r="152">
-      <c r="F152" s="5" t="n"/>
-      <c r="G152" s="5" t="n"/>
-    </row>
-    <row r="153">
-      <c r="F153" s="5" t="n"/>
-      <c r="G153" s="5" t="n"/>
-    </row>
-    <row r="154">
-      <c r="F154" s="5" t="n"/>
-      <c r="G154" s="5" t="n"/>
-    </row>
-    <row r="155">
-      <c r="F155" s="5" t="n"/>
-      <c r="G155" s="5" t="n"/>
-    </row>
-    <row r="156">
-      <c r="F156" s="5" t="n"/>
-      <c r="G156" s="5" t="n"/>
-    </row>
-    <row r="157">
-      <c r="F157" s="5" t="n"/>
-      <c r="G157" s="5" t="n"/>
-    </row>
-    <row r="158">
-      <c r="F158" s="5" t="n"/>
-      <c r="G158" s="5" t="n"/>
-    </row>
-    <row r="159">
-      <c r="F159" s="5" t="n"/>
-      <c r="G159" s="5" t="n"/>
-    </row>
-    <row r="160">
-      <c r="F160" s="5" t="n"/>
-      <c r="G160" s="5" t="n"/>
-    </row>
-    <row r="161">
-      <c r="F161" s="5" t="n"/>
-      <c r="G161" s="5" t="n"/>
-    </row>
-    <row r="162">
-      <c r="F162" s="5" t="n"/>
-      <c r="G162" s="5" t="n"/>
-    </row>
-    <row r="163">
-      <c r="F163" s="5" t="n"/>
-      <c r="G163" s="5" t="n"/>
-    </row>
-    <row r="164">
-      <c r="F164" s="5" t="n"/>
-      <c r="G164" s="5" t="n"/>
-    </row>
-    <row r="165">
-      <c r="F165" s="5" t="n"/>
-      <c r="G165" s="5" t="n"/>
-    </row>
-    <row r="166">
-      <c r="F166" s="5" t="n"/>
-      <c r="G166" s="5" t="n"/>
-    </row>
-    <row r="167">
-      <c r="F167" s="5" t="n"/>
-      <c r="G167" s="5" t="n"/>
-    </row>
-    <row r="168">
-      <c r="F168" s="5" t="n"/>
-      <c r="G168" s="5" t="n"/>
-    </row>
-    <row r="169">
-      <c r="F169" s="5" t="n"/>
-      <c r="G169" s="5" t="n"/>
-    </row>
-    <row r="170">
-      <c r="F170" s="5" t="n"/>
-      <c r="G170" s="5" t="n"/>
-    </row>
-    <row r="171">
-      <c r="F171" s="5" t="n"/>
-      <c r="G171" s="5" t="n"/>
-    </row>
-    <row r="172">
-      <c r="F172" s="5" t="n"/>
-      <c r="G172" s="5" t="n"/>
-    </row>
-    <row r="173">
-      <c r="F173" s="5" t="n"/>
-      <c r="G173" s="5" t="n"/>
-    </row>
-    <row r="174">
-      <c r="F174" s="5" t="n"/>
-      <c r="G174" s="5" t="n"/>
-    </row>
-    <row r="175">
-      <c r="F175" s="5" t="n"/>
-      <c r="G175" s="5" t="n"/>
-    </row>
-    <row r="176">
-      <c r="F176" s="5" t="n"/>
-      <c r="G176" s="5" t="n"/>
-    </row>
-    <row r="177">
-      <c r="F177" s="5" t="n"/>
-      <c r="G177" s="5" t="n"/>
-    </row>
-    <row r="178">
-      <c r="F178" s="5" t="n"/>
-      <c r="G178" s="5" t="n"/>
-    </row>
-    <row r="179">
-      <c r="F179" s="5" t="n"/>
-      <c r="G179" s="5" t="n"/>
-    </row>
-    <row r="180">
-      <c r="F180" s="5" t="n"/>
-      <c r="G180" s="5" t="n"/>
-    </row>
-    <row r="181">
-      <c r="F181" s="5" t="n"/>
-      <c r="G181" s="5" t="n"/>
-    </row>
-    <row r="182">
-      <c r="F182" s="5" t="n"/>
-      <c r="G182" s="5" t="n"/>
-    </row>
-    <row r="183">
-      <c r="F183" s="5" t="n"/>
-      <c r="G183" s="5" t="n"/>
-    </row>
-    <row r="184">
-      <c r="F184" s="5" t="n"/>
-      <c r="G184" s="5" t="n"/>
-    </row>
-    <row r="185">
-      <c r="F185" s="5" t="n"/>
-      <c r="G185" s="5" t="n"/>
-    </row>
-    <row r="186">
-      <c r="F186" s="5" t="n"/>
-      <c r="G186" s="5" t="n"/>
-    </row>
-    <row r="187">
-      <c r="F187" s="5" t="n"/>
-      <c r="G187" s="5" t="n"/>
-    </row>
-    <row r="188">
-      <c r="F188" s="5" t="n"/>
-      <c r="G188" s="5" t="n"/>
-    </row>
-    <row r="189">
-      <c r="F189" s="5" t="n"/>
-      <c r="G189" s="5" t="n"/>
-    </row>
-    <row r="190">
-      <c r="F190" s="5" t="n"/>
-      <c r="G190" s="5" t="n"/>
-    </row>
-    <row r="191">
-      <c r="F191" s="5" t="n"/>
-      <c r="G191" s="5" t="n"/>
-    </row>
-    <row r="192">
-      <c r="F192" s="5" t="n"/>
-      <c r="G192" s="5" t="n"/>
-    </row>
-    <row r="193">
-      <c r="F193" s="5" t="n"/>
-      <c r="G193" s="5" t="n"/>
-    </row>
-    <row r="194">
-      <c r="F194" s="5" t="n"/>
-      <c r="G194" s="5" t="n"/>
-    </row>
-    <row r="195">
-      <c r="F195" s="5" t="n"/>
-      <c r="G195" s="5" t="n"/>
-    </row>
-    <row r="196">
-      <c r="F196" s="5" t="n"/>
-      <c r="G196" s="5" t="n"/>
-    </row>
-    <row r="197">
-      <c r="F197" s="5" t="n"/>
-      <c r="G197" s="5" t="n"/>
-    </row>
-    <row r="198">
-      <c r="F198" s="5" t="n"/>
-      <c r="G198" s="5" t="n"/>
-    </row>
-    <row r="199">
-      <c r="F199" s="5" t="n"/>
-      <c r="G199" s="5" t="n"/>
-    </row>
-    <row r="200">
-      <c r="F200" s="5" t="n"/>
-      <c r="G200" s="5" t="n"/>
-    </row>
-    <row r="201">
-      <c r="F201" s="5" t="n"/>
-      <c r="G201" s="5" t="n"/>
-    </row>
-    <row r="202">
-      <c r="F202" s="5" t="n"/>
-      <c r="G202" s="5" t="n"/>
-    </row>
-    <row r="203">
-      <c r="F203" s="5" t="n"/>
-      <c r="G203" s="5" t="n"/>
-    </row>
-    <row r="204">
-      <c r="F204" s="5" t="n"/>
-      <c r="G204" s="5" t="n"/>
-    </row>
-    <row r="205">
-      <c r="F205" s="5" t="n"/>
-      <c r="G205" s="5" t="n"/>
-    </row>
-    <row r="206">
-      <c r="F206" s="5" t="n"/>
-      <c r="G206" s="5" t="n"/>
-    </row>
-    <row r="207">
-      <c r="F207" s="5" t="n"/>
-      <c r="G207" s="5" t="n"/>
-    </row>
-    <row r="208">
-      <c r="F208" s="5" t="n"/>
-      <c r="G208" s="5" t="n"/>
-    </row>
-    <row r="209">
-      <c r="F209" s="5" t="n"/>
-      <c r="G209" s="5" t="n"/>
-    </row>
-    <row r="210">
-      <c r="F210" s="5" t="n"/>
-      <c r="G210" s="5" t="n"/>
-    </row>
-    <row r="211">
-      <c r="F211" s="5" t="n"/>
-      <c r="G211" s="5" t="n"/>
-    </row>
-    <row r="212">
-      <c r="F212" s="5" t="n"/>
-      <c r="G212" s="5" t="n"/>
-    </row>
-    <row r="213">
-      <c r="F213" s="5" t="n"/>
-      <c r="G213" s="5" t="n"/>
-    </row>
-    <row r="214">
-      <c r="F214" s="5" t="n"/>
-      <c r="G214" s="5" t="n"/>
-    </row>
-    <row r="215">
-      <c r="F215" s="5" t="n"/>
-      <c r="G215" s="5" t="n"/>
-    </row>
-    <row r="216">
-      <c r="F216" s="5" t="n"/>
-      <c r="G216" s="5" t="n"/>
-    </row>
-    <row r="217">
-      <c r="F217" s="5" t="n"/>
-      <c r="G217" s="5" t="n"/>
-    </row>
-    <row r="218">
-      <c r="F218" s="5" t="n"/>
-      <c r="G218" s="5" t="n"/>
-    </row>
-    <row r="219">
-      <c r="F219" s="5" t="n"/>
-      <c r="G219" s="5" t="n"/>
-    </row>
-    <row r="220">
-      <c r="F220" s="5" t="n"/>
-      <c r="G220" s="5" t="n"/>
-    </row>
-    <row r="221">
-      <c r="F221" s="5" t="n"/>
-      <c r="G221" s="5" t="n"/>
-    </row>
-    <row r="222">
-      <c r="F222" s="5" t="n"/>
-      <c r="G222" s="5" t="n"/>
-    </row>
-    <row r="223">
-      <c r="F223" s="5" t="n"/>
-      <c r="G223" s="5" t="n"/>
-    </row>
-    <row r="224">
-      <c r="F224" s="5" t="n"/>
-      <c r="G224" s="5" t="n"/>
-    </row>
-    <row r="225">
-      <c r="F225" s="5" t="n"/>
-      <c r="G225" s="5" t="n"/>
-    </row>
-    <row r="226">
-      <c r="F226" s="5" t="n"/>
-      <c r="G226" s="5" t="n"/>
-    </row>
-    <row r="227">
-      <c r="F227" s="5" t="n"/>
-      <c r="G227" s="5" t="n"/>
-    </row>
-    <row r="228">
-      <c r="F228" s="5" t="n"/>
-      <c r="G228" s="5" t="n"/>
-    </row>
-    <row r="229">
-      <c r="F229" s="5" t="n"/>
-      <c r="G229" s="5" t="n"/>
-    </row>
-    <row r="230">
-      <c r="F230" s="5" t="n"/>
-      <c r="G230" s="5" t="n"/>
-    </row>
-    <row r="231">
-      <c r="F231" s="5" t="n"/>
-      <c r="G231" s="5" t="n"/>
-    </row>
-    <row r="232">
-      <c r="F232" s="5" t="n"/>
-      <c r="G232" s="5" t="n"/>
-    </row>
-    <row r="233">
-      <c r="F233" s="5" t="n"/>
-      <c r="G233" s="5" t="n"/>
-    </row>
-    <row r="234">
-      <c r="F234" s="5" t="n"/>
-      <c r="G234" s="5" t="n"/>
-    </row>
-    <row r="235">
-      <c r="F235" s="5" t="n"/>
-      <c r="G235" s="5" t="n"/>
-    </row>
-    <row r="236">
-      <c r="F236" s="5" t="n"/>
-      <c r="G236" s="5" t="n"/>
-    </row>
-    <row r="237">
-      <c r="F237" s="5" t="n"/>
-      <c r="G237" s="5" t="n"/>
-    </row>
-    <row r="238">
-      <c r="F238" s="5" t="n"/>
-      <c r="G238" s="5" t="n"/>
-    </row>
-    <row r="239">
-      <c r="F239" s="5" t="n"/>
-      <c r="G239" s="5" t="n"/>
-    </row>
-    <row r="240">
-      <c r="F240" s="5" t="n"/>
-      <c r="G240" s="5" t="n"/>
-    </row>
-    <row r="241">
-      <c r="F241" s="5" t="n"/>
-      <c r="G241" s="5" t="n"/>
-    </row>
-    <row r="242">
-      <c r="F242" s="5" t="n"/>
-      <c r="G242" s="5" t="n"/>
-    </row>
-    <row r="243">
-      <c r="F243" s="5" t="n"/>
-      <c r="G243" s="5" t="n"/>
-    </row>
-    <row r="244">
-      <c r="F244" s="5" t="n"/>
-      <c r="G244" s="5" t="n"/>
-    </row>
-    <row r="245">
-      <c r="F245" s="5" t="n"/>
-      <c r="G245" s="5" t="n"/>
-    </row>
-    <row r="246">
-      <c r="F246" s="5" t="n"/>
-      <c r="G246" s="5" t="n"/>
-    </row>
-    <row r="247">
-      <c r="F247" s="5" t="n"/>
-      <c r="G247" s="5" t="n"/>
-    </row>
-    <row r="248">
-      <c r="F248" s="5" t="n"/>
-      <c r="G248" s="5" t="n"/>
-    </row>
-    <row r="249">
-      <c r="F249" s="5" t="n"/>
-      <c r="G249" s="5" t="n"/>
-    </row>
-    <row r="250">
-      <c r="F250" s="5" t="n"/>
-      <c r="G250" s="5" t="n"/>
-    </row>
-    <row r="251">
-      <c r="F251" s="5" t="n"/>
-      <c r="G251" s="5" t="n"/>
-    </row>
-    <row r="252">
-      <c r="F252" s="5" t="n"/>
-      <c r="G252" s="5" t="n"/>
-    </row>
-    <row r="253">
-      <c r="F253" s="5" t="n"/>
-      <c r="G253" s="5" t="n"/>
-    </row>
-    <row r="254">
-      <c r="F254" s="5" t="n"/>
-      <c r="G254" s="5" t="n"/>
-    </row>
-    <row r="255">
-      <c r="F255" s="5" t="n"/>
-      <c r="G255" s="5" t="n"/>
-    </row>
-    <row r="256">
-      <c r="F256" s="5" t="n"/>
-      <c r="G256" s="5" t="n"/>
-    </row>
-    <row r="257">
-      <c r="F257" s="5" t="n"/>
-      <c r="G257" s="5" t="n"/>
-    </row>
-    <row r="258">
-      <c r="F258" s="5" t="n"/>
-      <c r="G258" s="5" t="n"/>
-    </row>
-    <row r="259">
-      <c r="F259" s="5" t="n"/>
-      <c r="G259" s="5" t="n"/>
-    </row>
-    <row r="260">
-      <c r="F260" s="5" t="n"/>
-      <c r="G260" s="5" t="n"/>
-    </row>
-    <row r="261">
-      <c r="F261" s="5" t="n"/>
-      <c r="G261" s="5" t="n"/>
-    </row>
-    <row r="262">
-      <c r="F262" s="5" t="n"/>
-      <c r="G262" s="5" t="n"/>
-    </row>
-    <row r="263">
-      <c r="F263" s="5" t="n"/>
-      <c r="G263" s="5" t="n"/>
-    </row>
-    <row r="264">
-      <c r="F264" s="5" t="n"/>
-      <c r="G264" s="5" t="n"/>
-    </row>
-    <row r="265">
-      <c r="F265" s="5" t="n"/>
-      <c r="G265" s="5" t="n"/>
-    </row>
-    <row r="266">
-      <c r="F266" s="5" t="n"/>
-      <c r="G266" s="5" t="n"/>
-    </row>
-    <row r="267">
-      <c r="F267" s="5" t="n"/>
-      <c r="G267" s="5" t="n"/>
-    </row>
-    <row r="268">
-      <c r="F268" s="5" t="n"/>
-      <c r="G268" s="5" t="n"/>
-    </row>
-    <row r="269">
-      <c r="F269" s="5" t="n"/>
-      <c r="G269" s="5" t="n"/>
-    </row>
-    <row r="270">
-      <c r="F270" s="5" t="n"/>
-      <c r="G270" s="5" t="n"/>
-    </row>
-    <row r="271">
-      <c r="F271" s="5" t="n"/>
-      <c r="G271" s="5" t="n"/>
-    </row>
-    <row r="272">
-      <c r="F272" s="5" t="n"/>
-      <c r="G272" s="5" t="n"/>
-    </row>
-    <row r="273">
-      <c r="F273" s="5" t="n"/>
-      <c r="G273" s="5" t="n"/>
-    </row>
-    <row r="274">
-      <c r="F274" s="5" t="n"/>
-      <c r="G274" s="5" t="n"/>
-    </row>
-    <row r="275">
-      <c r="F275" s="5" t="n"/>
-      <c r="G275" s="5" t="n"/>
-    </row>
-    <row r="276">
-      <c r="F276" s="5" t="n"/>
-      <c r="G276" s="5" t="n"/>
-    </row>
-    <row r="277">
-      <c r="F277" s="5" t="n"/>
-      <c r="G277" s="5" t="n"/>
-    </row>
-    <row r="278">
-      <c r="F278" s="5" t="n"/>
-      <c r="G278" s="5" t="n"/>
-    </row>
-    <row r="279">
-      <c r="F279" s="5" t="n"/>
-      <c r="G279" s="5" t="n"/>
-    </row>
-    <row r="280">
-      <c r="F280" s="5" t="n"/>
-      <c r="G280" s="5" t="n"/>
-    </row>
-    <row r="281">
-      <c r="F281" s="5" t="n"/>
-      <c r="G281" s="5" t="n"/>
-    </row>
-    <row r="282">
-      <c r="F282" s="5" t="n"/>
-      <c r="G282" s="5" t="n"/>
-    </row>
-    <row r="283">
-      <c r="F283" s="5" t="n"/>
-      <c r="G283" s="5" t="n"/>
-    </row>
-    <row r="284">
-      <c r="F284" s="5" t="n"/>
-      <c r="G284" s="5" t="n"/>
-    </row>
-    <row r="285">
-      <c r="F285" s="5" t="n"/>
-      <c r="G285" s="5" t="n"/>
-    </row>
-    <row r="286">
-      <c r="F286" s="5" t="n"/>
-      <c r="G286" s="5" t="n"/>
-    </row>
-    <row r="287">
-      <c r="F287" s="5" t="n"/>
-      <c r="G287" s="5" t="n"/>
-    </row>
-    <row r="288">
-      <c r="F288" s="5" t="n"/>
-      <c r="G288" s="5" t="n"/>
-    </row>
-    <row r="289">
-      <c r="F289" s="5" t="n"/>
-      <c r="G289" s="5" t="n"/>
-    </row>
-    <row r="290">
-      <c r="F290" s="5" t="n"/>
-      <c r="G290" s="5" t="n"/>
-    </row>
-    <row r="291">
-      <c r="F291" s="5" t="n"/>
-      <c r="G291" s="5" t="n"/>
-    </row>
-    <row r="292">
-      <c r="F292" s="5" t="n"/>
-      <c r="G292" s="5" t="n"/>
-    </row>
-    <row r="293">
-      <c r="F293" s="5" t="n"/>
-      <c r="G293" s="5" t="n"/>
-    </row>
-    <row r="294">
-      <c r="F294" s="5" t="n"/>
-      <c r="G294" s="5" t="n"/>
-    </row>
-    <row r="295">
-      <c r="F295" s="5" t="n"/>
-      <c r="G295" s="5" t="n"/>
-    </row>
-    <row r="296">
-      <c r="F296" s="5" t="n"/>
-      <c r="G296" s="5" t="n"/>
-    </row>
-    <row r="297">
-      <c r="F297" s="5" t="n"/>
-      <c r="G297" s="5" t="n"/>
-    </row>
-    <row r="298">
-      <c r="F298" s="5" t="n"/>
-      <c r="G298" s="5" t="n"/>
-    </row>
-    <row r="299">
-      <c r="F299" s="5" t="n"/>
-      <c r="G299" s="5" t="n"/>
-    </row>
-    <row r="300">
-      <c r="F300" s="5" t="n"/>
-      <c r="G300" s="5" t="n"/>
-    </row>
-    <row r="301">
-      <c r="F301" s="5" t="n"/>
-      <c r="G301" s="5" t="n"/>
+      <c r="H91" s="6">
+        <f>IF(F91="nein","nein",IF(OR(F91="",G91=""),"",IF(AND(F91="ja",G91="Ziel"),"ja",IF(G91="Nebensache","nein","unsicher"))))</f>
+        <v/>
+      </c>
+      <c r="I91" s="7" t="inlineStr"/>
+      <c r="J91" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="F2:F301" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"yes,no,unsure"</formula1>
+  <dataValidations count="2">
+    <dataValidation sqref="F2:F91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"ja,nein,unsicher"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G2:G91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Ziel,Nebensache,unsicher"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>

</xml_diff>